<commit_message>
Update competition data 2026-09-13
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
+          <t>August 6, 2026 - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -464,26 +464,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Some of our sparkling achievements during 2014 – to help the NRF and DSI grow a representative science and technology workforce in the country – SAASTA has run a number of maths and science educator development programmes and a number of learner development programmes, including maths and science camps for learners with potential, olympiads and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -491,26 +487,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -523,17 +515,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -541,22 +533,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>info@zasdc.org, user@domain.com</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -569,17 +565,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa. Find out more</t>
+          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -592,17 +588,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Eligibility Benchmark Requirements The Africa Prize is open to individuals or teams based in sub-Saharan Africa with a scalable engineering innovation that demonstrates social or environmental impact potential. Applicants must: Be citizens ordinarily residing in a sub-Saharan African country. Be over 18 years old and fluent in English.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -610,22 +606,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -633,26 +633,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://www.thecasecentre.org/products/view?id=189255</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -665,17 +661,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Astemi Sa</t>
+          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>What is ASTEMI SA? The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible. We aim to increase participation in the activities of ASTEMI SA. We will encourage our members to lower the barriers of ...</t>
+          <t>1 month ago - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -688,17 +684,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
+          <t>South Africa International Industrial Expo | Innovation Bridge</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
+          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -706,26 +702,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>enquiries@aiexpoafrica.com</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://madeinafricaevent.co.za/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Big Data and Business Analytics Innovation Conference Johannesburg, South Africa IT &amp; Technology 101 Members Tue, 22 - Thu, 24 Sep 2026</t>
+          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -738,17 +730,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
+          <t>KZN Industrial Technology Exhibition</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://www.kznindustrial.co.za/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
+          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -756,22 +748,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>john@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
+          <t>Exhibition | Innovation Festival Durban | South Africa</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/tradeshows</t>
+          <t>https://www.innovationfestival.durban/exhibition</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>South Africa trade shows, find and compare 974 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 165 upcoming expos in 2026-2027 1. NAMPO KAAP / CAPE, 2. Nampo Kaap Cape Bredasdorp, 3. KwaZulu-Natal EduXplore Expo, 4. Mining Connect Day</t>
+          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -779,22 +775,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, Erika@innovate.durban, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, sithabile@innovate.durban</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -802,26 +802,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>support@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, customerservices@informaconnect.com, dataprivacy@knect365.com, support@informaconnect.com, customerservices@knect365.com</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
+          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://expotobi.com/country/south-africa/exhibitions</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
+          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -834,17 +830,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
+          <t>Come and explore our exhibition of innovative discoveries at Science Forum South Africa 2024 | CSIR</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
+          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
+          <t>December 3, 2024 - The exhibition launch will take place on Tuesday, 3 December 2024, with the opening address by Department of Science, Technology and Innovation Minister Dr Blade Nzimande.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -857,17 +853,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>65 Trade Fairs in South Africa from September 2026</t>
+          <t>International Science, Innovation &amp; Technology Expo (INSITE)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.tradefairdates.com/Fairs-South-Africa-Z243-S1.html</t>
+          <t>https://www.dsti.gov.za/index.php/resource-center/27-temp/dst-links/3-international-science-innovation-a-technology-expo</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Exhibition calendar with 65 trade fairs from September 2026 in South Africa sorted by exhibition date. Most trade fairs in South Africa take place in Johannesburg with 31 trade fairs.</t>
+          <t>The essence of INSITE INSITE is an international, biennial must-see Science and Technology event in South Africa, the only one of its kind in Africa that creates new frontiers for global challenges · INSITE aims to assemble the worlds leading innovators and scientists in one place, stimulating ...</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -880,17 +876,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Trade Shows Worldwide - Cape Town (South Africa) - 2026/2027</t>
+          <t>AAXO - The Association of African Exhibition Organisers</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.eventseye.com/fairs/cy1_trade-shows-cape-town.html</t>
+          <t>https://www.aaxo.co.za/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Cape Town Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in Cape Town</t>
+          <t>February 20, 2026 - CAPE TOWN, South Africa – The inaugural Festival of Eventing (FOE) brought together 350 event professionals, 85 speakers, and 10 countries under one roof for a two-day showcase of innovation, inspiration, and industry connection.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -903,17 +899,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>Exhibitions in South Africa 2026, 2027 | Conference Locate (Clocate)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://www.clocate.com/exhibitions-in+south-africa/Y28temE=/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>This page outlines collaboration oppertunities whether informs of sponsorship, partnership or by being an exhibitor.</t>
+          <t>Innovations (2) Internet of Things ... (1) Sport &amp; Leisure (2) Toys &amp; Games (3) Training (1) Transport (1) Showing 23 exhibitions · 26 May 2026 · 26-27 May 2026 · Cape Town, South Africa ·...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -921,26 +917,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, sithabile@innovate.durban, 8c4075d5481d476e945486754f783364@sentry.io, Erika@innovate.durban, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community’s challenges and how community members view the impact of these challenges on their daily lives.</t>
+          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -948,26 +940,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of ...</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Aug 4, 2025 · This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
+          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -977,24 +965,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Engineering For People Design Challenge - EWBSA</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1002,26 +990,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Engineering ENGINEERING FOR PEOPLE Design challenge DESIGN ...</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/wp-content/uploads/2024/08/2024_25_Engineering_for_People_Design_Challenge_Makers_Valley.pdf</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Makers Makers Valley Valley Johannesburg, Johannesburg, South South Africa Africa The Engineering for People Design Challenge has been delivered in the UK and Ireland since 2011, South Africa and the USA since 2019, and Cameroon in 2022. It is an educational programme based on a concept developed originally by Engineers Without Borders Australia. The production of this document has been led by ...</t>
+          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1029,22 +1013,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ied@ied.org.uk</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge - Engineers Without ...</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
+          <t>... On 30-31 March 2026, 109 students from 9 schools walked into the University of Cape Town and designed a city on the Moon. They elected leaders, divided into engineering departments, and spent 24 hours responding to a professional design brief.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1052,22 +1040,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>info@zasdc.org, user@domain.com</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Oct 24, 2024 · The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
+          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1075,26 +1067,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>team@crowdsolve.net</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
+          <t>Engineers Without Borders South ...</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1107,17 +1095,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1125,22 +1113,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Engineers Without Borders launches student challenge</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://www.theconstructionindex.co.uk/news/view/engineers-without-borders-launches-student-challenge</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>September 7, 2021 - The Engineering for People Design Challenge encourages undergraduates to broaden their awareness of the social, environmental and economic implications of their engineering solutions.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1150,24 +1142,24 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ied@ied.org.uk</t>
+          <t>news@theconstructionindex.co.uk</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>... On 30-31 March 2026, 109 students from 9 schools walked into the University of Cape Town and designed a city on the Moon. They elected leaders, divided into engineering departments, and spent 24 hours responding to a professional design brief.</t>
+          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1175,26 +1167,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>user@domain.com, info@zasdc.org</t>
-        </is>
-      </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Some of our sparkling achievements ... and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation ...</t>
+          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1207,17 +1195,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1230,17 +1218,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1248,26 +1236,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1275,26 +1259,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1307,17 +1287,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Sep 4, 2025 · 3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1325,26 +1305,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>National Student Competition | ORSSA</t>
+          <t>Engineering in South Africa: 24 Best universities Ranked</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.orssa.org.za/studentcomp</t>
+          <t>https://edurank.org/engineering/za/</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>The objectives of the competitions are to propagate the use of operations research at the tertiary level of study, to encourage the inclusion of project work in operations research courses, and to bring the Operations Research Society of South Africa to the attention of students and staff at universities in South Africa.</t>
+          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1352,26 +1328,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, email@example.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
+          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1384,17 +1356,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1407,17 +1379,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;area=2200&amp;ranking=Overall&amp;country=ZAF</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1477,24 +1449,24 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>support@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, customerservices@informaconnect.com, dataprivacy@knect365.com, support@informaconnect.com, customerservices@knect365.com</t>
+          <t>support@informaconnect.com, support@knect365.com, dataprivacy@informaconnect.com, customerservices@knect365.com, customerservices@informaconnect.com, salesenquiries@africatechfestival.com, dataprivacy@knect365.com</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 - 7, 2027 ...</t>
+          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology Expo ...</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>The annual TECHSPO Cape Town 2027 Technology Expo returns October 6th to 7th, 2027 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town. TECHSPO Cape Town Technology Expo is the must-attend event to: Experience the Future of Technology &amp; Innovation Discover cutting-edge tech, game-changing tools, and innovators shaping tomorrow's digital world. See the latest advancements in ...</t>
+          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 - 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1502,26 +1474,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>info@techspocapetown.co.za</t>
-        </is>
-      </c>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology Expo ...</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 - 7, 2027 ...</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 - 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
+          <t>The annual TECHSPO Cape Town 2027 Technology Expo returns October 6th to 7th, 2027 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town. TECHSPO Cape Town Technology Expo is the must-attend event to: Experience the Future of Technology &amp; Innovation Discover cutting-edge tech, game-changing tools, and innovators shaping tomorrow's digital world. See the latest advancements in ...</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1529,22 +1497,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2026 Technology Expo (Internet ~ Mobile ~ AdTech ...</t>
+          <t>Tech Expo Africa - Enabling Development</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://allevents.in/cape-town/techspo-cape-town-2026-technology-expo-internet-~-mobile-~-adtech-~-martech-~-saas/200030358413547</t>
+          <t>https://techexpo.africa/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town Technology Expo returns October 1-2, 2026 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town, South Africa. This must-attend, two-day annual event brings together leading developers, marketers, innovators, and technology enthusiasts eager to showcase and explore the latest in tech and digital solutions.</t>
+          <t>Tech Expo Africa is a social enterprise connecting African businesses with top tech and business leaders to drive innovation.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1552,22 +1524,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>info@techexpo.africa</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~…</t>
+          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa. This must-attend, two-day annual event brings together leading developers, marketers, innovators, and technology enthusiasts eager to showcase and explore the latest in tech and digital solutions.</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1575,26 +1551,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>colleague@company.com, you@company.com, events@techspojoburg.co.za, support@industryevents.com, your@email.com</t>
-        </is>
-      </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Tech Expo Africa - Enabling Development</t>
+          <t>TECHSPO Cape Town 2026 Technology Expo (Internet ~ Mobile ~ AdTech ...</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://techexpo.africa/</t>
+          <t>https://allevents.in/cape-town/techspo-cape-town-2026-technology-expo-internet-~-mobile-~-adtech-~-martech-~-saas/200030358413547</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Tech Expo Africa is a social enterprise connecting African businesses with top tech and business leaders to drive innovation.</t>
+          <t>TECHSPO Cape Town Technology Expo returns October 1-2, 2026 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town, South Africa. This must-attend, two-day annual event brings together leading developers, marketers, innovators, and technology enthusiasts eager to showcase and explore the latest in tech and digital solutions.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1602,26 +1574,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>info@techexpo.africa</t>
-        </is>
-      </c>
+      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
+          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1634,17 +1602,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://10times.com/johannesburg-za/technology</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1657,17 +1625,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~…</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa. This must-attend, two-day annual event brings together leading developers, marketers, innovators, and technology enthusiasts eager to showcase and explore the latest in tech and digital solutions.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1675,7 +1643,11 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>support@industryevents.com, events@techspojoburg.co.za, your@email.com, you@company.com, colleague@company.com</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1690,7 +1662,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Maker Faire Africa, Cairo, October 2011 Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds (Nubian Cheetah). Maker Faire Africa aims to engage with on ...</t>
+          <t>March 7, 2025 - Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds ...</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1713,7 +1685,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
+          <t>May 3, 2026 - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1726,17 +1698,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Maker Faire |</t>
+          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/</t>
+          <t>https://makerfairecapetown.wordpress.com/about/</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1744,26 +1716,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, pr@make.co, fancybox_sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Upcoming Faires - Maker Faire</t>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/upcoming-faires/</t>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>11 hours ago · The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1771,26 +1739,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, pr@make.co, fancybox_sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire Africa — Grokipedia</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://grokipedia.com/page/maker_faire_africa</t>
+          <t>http://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Maker Faire Africa Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
+          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1798,22 +1762,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, pr@make.co, fancybox_sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Maker Faire groups | Meetup</t>
+          <t>Blog : Maker Faire Africa</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/topics/maker-faire/za/</t>
+          <t>http://makerfaireafrica.com/blog/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
+          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building his ANIMAL car, from the ground up, that means the frame and all.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1826,17 +1794,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
+          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
+          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Aug 21, 2015 · DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
+          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1849,17 +1817,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
+          <t>The Makers Hub</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://makerfairecapetown.wordpress.com/about/</t>
+          <t>https://www.decorex.co.za/cape-town/en-gb/visit/TheMakersHub.html</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
+          <t>Explore unique handmade items, take part in interactive workshops, and engage directly with Cape Town’s vibrant maker community.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1867,22 +1835,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>decorexafrica@rxglobal.com</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1895,17 +1867,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>Why Africa needs Maker Faire | ZDNET</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>http://capetown.makerfaire.com/</t>
+          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage to attend and show off their work.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1913,26 +1885,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, pr@make.co, fancybox_sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>StemCo - StemCo 2026 International Competitions</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://stemco.org/</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
+          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1945,17 +1913,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation ...</t>
+          <t>High School STEM Competition | Southafrica 2024</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1965,24 +1933,24 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>user@domain.com, info@zasdc.org</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>February 27, 2026 - Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1995,17 +1963,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
+          <t>Local, regional and national competitions with thousands of · Multi-level events of two or more rounds that become increasingly challenging and culminate in top-level Olympiads. Enrichment programmes to inspire promising young South Africans to pursue STEMI</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2013,26 +1981,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Astemi Sa</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>The ZASDC is South Africa's national Space Design Competition, part of a global network spanning six continents. Secondary school students design futuristic space settlements in a fast-paced industry simulation that builds real STEM, leadership ...</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2040,22 +2004,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>info@zasdc.org, user@domain.com</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
+          <t>ASTEMI Competitions 2022 – SAASTA</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://saasta.ac.za/astemi-competitions-2</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2068,17 +2036,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>Competition – Eskom Expo for Young Scientists</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://exposcience.co.za/category/competition/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+          <t>Aqil Variava business cities Damien ... Gray STEMI Vuyo Nzimande · Eskom Expo for Young Scientists is an exposition, or science fair, where students have a chance to show others their projects about their own scientific investigations. At the annual prestigious Eskom Expo for Young Scientists International Science Fair (ISF), selected students from 35 Expo Regions in South Africa then compete ...</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2086,22 +2054,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>support@exposcience.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Capetown 2026</t>
+          <t>Rural youth lead in robotics at national STEM competition</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
+          <t>https://iol.co.za/news/education/2025-09-15-rural-youth-lead-in-robotics-at-national-stem-competition/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
+          <t>September 15, 2025 - Discover how South Africa's brightest young minds are tackling real-world challenges with innovative solutions at the inaugural AlgoAtWork RoboRumble STEM Innovation Challenge, where ideas like autonomous robots and smart PPE systems are set ...</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2111,24 +2083,24 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>londiwe.gumede@inl.co.za, philippa.larkin@inl.co.za, nobuntu.mgijima@volt.africa, mendy.mtshali@inl.co.za, lee.rondganger@inl.co.za, ashley.lechman@inl.co.za</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>2026 Season - Africa's Global STEM Celebration</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://www.stemfestival.org/competitions/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>April 30, 2026 - ... The Elementary, Junior, and Senior Robotics categories at STEM Festival are dedicated to advancing the World Robot Olympiad (WRO) across the Niger Delta and South-South Nigeria, working with ArcLights Foundation.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2141,17 +2113,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>National Department of Basic Education</t>
+          <t>STEAM Pitch Competition - STEM AFRICA FEST 2024</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://www.education.gov.za/LinkClick.aspx?fileticket=i9GS5Atf7zo=&amp;tabid=347&amp;portalid=0&amp;mid=14629</t>
+          <t>https://stemafricafest.com/steam-pitch-competition/</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>JOHANNESBURG, South Africa - XX Month 2026 - The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries ...</t>
+          <t>Join STEM Africa Fest , celebrating science, technology, engineering, and mathematics. Experience hands-on learning, industry leaders, and innovation across Africa.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2159,11 +2131,7 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>s.ngcobo@cheil.com, ssasft@samsung.com, j.mogoeng@samsung.com</t>
-        </is>
-      </c>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2188,7 +2156,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2215,7 +2183,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, info@thecortexhub.africa, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, info@thecortexhub.africa, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2269,24 +2237,24 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>you@email.com, info@nirvanaglobalfoundation.org, coach@school.co.za</t>
+          <t>info@nirvanaglobalfoundation.org, you@email.com, coach@school.co.za</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>Roboticon 2026: South Africa Showcases Robotics for Culture, Education ...</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop their creativity and problem-solving skills through challenging and educational robotics competitions.</t>
+          <t>The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation." South Africa's robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2294,22 +2262,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>adverts@ubuntutimes.co.za, newspaper-rec300@2x.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>FIRST South Africa - Robotics Programs for School Children</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://firstsa.org/</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>FIRST® LEGO ® League FIRST® LEGO ® League guides youth through STEM learning and exploration at an early age. From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way.</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop their creativity and problem-solving skills through challenging and educational robotics competitions.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2322,17 +2294,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Roboticon 2026: South Africa Showcases Robotics for Culture, Education ...</t>
+          <t>2026 - SpringBots South Africa</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
+          <t>https://springbots.co.za/2026-2/</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation." South Africa's robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
+          <t>This approach ensures that learners are not only participants in robotics competitions but are also equipped with real-world skills in design thinking, programming, systems engineering, and collaborative problem-solving. A Unified Future for Africa SpringBots' 2026 vision extends beyond competition and education.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2340,26 +2312,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>adverts@ubuntutimes.co.za, newspaper-rec300@2x.jpg</t>
-        </is>
-      </c>
+      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Competition &amp; Judge Registration | WROSA</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://www.wrosa.co.za/teamregistration</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>JUDGES World Robot Olympiad South Africa Team Registration 2026 Physical Events - Team Registration Team Registrations are now open! Register your teams by clicking on the button below. Team registrations will close at 12:00 on the 1st of June. No Late Registrations will be accepted. Registrations Have Closed</t>
+          <t>ICS Export Are you sure you want to remove this speaker?</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2369,24 +2337,24 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
+          <t>Welcome to FIRST Tech Challenge - FIRST South Africa</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
+          <t>https://firstsa.org/welcome-to-first-tech-challenge/</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>ICS Export Are you sure you want to remove this speaker?</t>
+          <t>The robot kit is reusable from year-to-year and can be programmed using a variety of languages, including Java. Teams also must raise funds, design and market their team brand, and do community outreach for which they can win awards.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2394,26 +2362,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>name@example.com</t>
-        </is>
-      </c>
+      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>FIRST LEGO League Challenge Events - FIRST South Africa</t>
+          <t>Home | Roboticon 2026</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://firstsa.org/challenge-events/</t>
+          <t>https://roboticon.resolute.education/</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>After all teams have finished their Judging sessions and Robot Games, there will be a Closing Ceremony, where all participants will receive medals and the Awards will be handed out. Teams have the opportunity to win awards in various categories, but the FIRST LEGO League Core Values remain the focus. List of Awards Challenge Event/Tournament ...</t>
+          <t>Join us for the ultimate robotics showcase as Resolute proudly sponsors the World Robotics Olympiad (WRO) South Africa! This year, we're bringing together two worlds for the biggest robotics event of the year - Roboticon and the WRO Nationals, happening on the same day at the same venue.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2446,7 +2410,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>subscriptions@creamermedia.co.za, advertising@creamermedia.co.za, chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za, newsletters@creamermedia.co.za</t>
+          <t>subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za, newsletters@creamermedia.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za</t>
         </is>
       </c>
     </row>
@@ -2473,7 +2437,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>communications@saice.org.za, accounts@saice.org.za, civilinfo@saice.org.za, membership@saice.org.za, marketing@saice.org.za</t>
+          <t>communications@saice.org.za, membership@saice.org.za, accounts@saice.org.za, civilinfo@saice.org.za, marketing@saice.org.za</t>
         </is>
       </c>
     </row>
@@ -2523,7 +2487,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>constr@crown.co.za, ernao@crown.co.za</t>
+          <t>ernao@crown.co.za, constr@crown.co.za</t>
         </is>
       </c>
     </row>
@@ -2672,17 +2636,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Mechanical Engineering Conferences in South Africa 2026/2027/2028 - Conference Index</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/mechanical-engineering/south-africa</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Nov 04 International Conference on Tribology and Interface Engineering (ICTIE) - Cape Town, South Africa · Nov 04 International Conference on Mechanical and Systems Engineering (ICMSE) - Cape Town, South Africa</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2695,17 +2659,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>&gt;&gt; Industrial and Manufacturing Engineering · &gt;&gt; Mechanical Engineering · &gt;&gt; Ocean Engineering · Environmental Science · Mathematics · Medicine · &gt;&gt; Anatomy · &gt;&gt; Anesthesiology and Pain Medicine · &gt;&gt; Cardiology and Cardiovascular Medicine · &gt;&gt; Critical Care and Intensive Care Medicine ·</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2718,17 +2682,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Mechanical Engineering events - South Africa Group - Institution of Mechanical Engineers</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://nearyou.imeche.org/near-you/middle-east-and-africa/south-africa/events</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>For details of Mechanical Engineering events organised by South Africa Group, please click the above link.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2741,17 +2705,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Best Mechanical Engineering Companies in South Africa</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://engineeringness.com/best-mechanical-engineering-companies-in-south-africa/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>October 4, 2025 - This article showcases our top picks for the best South Africa based Mechanical Engineering companies. These startups and companies are taking a variety of approaches to innovating the Mechanical Engineering industry, but are all exceptional companies well worth a follow.</t>
+          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2759,22 +2723,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Past Mechanical Engineering events - South Africa Group - Institution of Mechanical Engineers</t>
+          <t>WorldSkills South Africa 2027 Applications Now Open - Apply Online</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://nearyou.imeche.org/near-you/middle-east-and-africa/south-africa/past-events</t>
+          <t>https://www.edupstairs.org/worldskills-south-africa-2027-applications/</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>For details of past Mechanical Engineering events organised by South Africa Group, please click the above link.</t>
+          <t>Applications are officially open for the WorldSkills South Africa 2027 National Competition, giving talented students, apprentices, learners and qualifying skilled candidates across South Africa an opportunity to demonstrate their practical abilities on a national stage.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2782,22 +2750,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>sifisomhlongo@edupstairs.org</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>7 Mechanical Engineering Degree Programs in South Africa - Study Abroad | educations.com</t>
+          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://www.educations.com/mechanical-engineering/south-africa</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>One of the main objectives of this process is to develop an advanced capability to do fundamental engineering research independently. It also promotes a lifelong learning approach. ... The Master of Mechanical Engineering (MS) program objective is to provide students with the skill sets and knowledge necessary to become a professional who can solve practical issues of the field of mechanical engineering.</t>
+          <t>The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent's largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2810,17 +2782,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10 Mechanical Engineering Competitions for High School Students — Veritas AI</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://www.veritasai.com/veritasaiblog/10-mechanical-engineering-competitions-for-high-school-students</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>October 29, 2025 - ... Competition Dates: The contest year began on April 14 and ends on May 31. Students can submit (unique) entries for each monthly contest. Eligibility: The contest is open to all students, regardless of their age or discipline.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2830,24 +2802,24 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>user@domain.com, contact@veritasai.com</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Mechanical Engineering in South Africa: 2025 Master's Guide | Mastersportal</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://www.mastersportal.com/study-options/271564839/mechanical-engineering-south-africa.html</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>The Mechanical Engineering program at the University of Pretoria is a leading source of graduates in the... ... Applied Science Metallurgy from University of Pretoria aims to be internationally competitive while... ... Holders of any other equivalent South African or international qualification may also be considered for...</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2855,22 +2827,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Mechanical Engineering in South Africa: 2026 Bachelor's Guide | Bachelorsportal</t>
+          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://www.bachelorsportal.com/study-options/271564839/mechanical-engineering-south-africa.html</t>
+          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>International students also enjoy low costs of living and have the opportunity to explore South Africa’s beautiful cities and landscape, which includes Table Mountain, the Garden Route, and gorgeous beaches. more Read more about studying abroad in South Africa ... Take the test and find out which country is your best fit. ... Mechanical Engineering is the application of physics, mathematics, and materials science to design, analyse, manufacture, and maintain mechanical systems.</t>
+          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2883,17 +2859,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Engineering Competitions - ASME</t>
+          <t>SAIMechE</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://www.asme.org/conferences-events/competitions</t>
+          <t>https://www.saimeche.org.za/</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>There are four kinds of challenges &amp; competitions held during the three-day, two-night regional events built around design, advanced manufacturing &amp; robotics technologies. HPVC, IAM3D, the student design competition &amp; the old guard competition.</t>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2906,17 +2882,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2929,17 +2905,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
+          <t>IEEE South Africa</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
+          <t>http://www.ieee.org.za/</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
+          <t>The South African Section has around 1200 members and many subsections. It was formed in 1963 by the merger of the Institute of Radio Engineers (IRE, founded 1912) and the American Institute of Electrical Engineers (AIEE, founded 1884).</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2952,17 +2928,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - IEEE ZA 5G Competition</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51397</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Form templates: Template for a Cover Sheet for the Competition on Ideas, Designs and Applications for 5G and Beyond South Africa (.docx) [Click to Download] Template for a Resume for the Student (.docx) [Click to Download] ... Help (FAQ) • Privacy Statement • Terms &amp; Conditions The SAIEE is ...</t>
+          <t>Centres South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2970,22 +2946,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - SA Computing Olympiad stars hold their own in international competition</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51457</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>July 20, 2021 - For the other three South African team members, this was their first IOI. Brent Butkow finished ranked 342, Jean Weight finished in 287th position and Faran Steenkamp was ranked 280. In addition to the serious IOI contest days, host country Singapore arranged several fun events where Faran Steenkamp was placed third in the sponsored Code Cup, and won a cash prize of 200 USD.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2998,17 +2978,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Student Design Competition | IEEE CASS</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://ieee-cas.org/society-involvement/student-design-competition</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>CASS will reimburse the travel costs for the trip to ISCAS 2026 for the four finalists, one for each region - Regions 1-7 (USA and Canada), Region 8 (Europe, Middle East, Africa), Region 9 (Latin America), and Region 10 (Asia, Australia, Pacific), as well as ISCAS registration.</t>
+          <t>IEEE-IAS Industrial Power Conversion Systems Department Serving the electrical energy conversion professional worldwide</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3021,17 +3001,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>March 12, 2026 - At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3039,22 +3019,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Top 100 Electrical Engineering Companies in South Africa (2026) | ensun</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://ensun.io/search/electrical-engineering/south-africa</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>The competitive landscape is marked by both established firms and emerging startups, driving innovation and efficiency. Additionally, South Africa’s position in the broader global market allows for potential collaborations and export opportunities, particularly in green technologies. Understanding these factors is essential for anyone looking to engage with the Electrical Engineering sector in South Africa, as they influence the overall business environment and potential for growth.</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3067,17 +3051,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>7 Electrical Engineering Degree Programs in South Africa - Study Abroad | educations.com</t>
+          <t>Competitions | ESG</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://www.educations.com/electrical-engineering/south-africa</t>
+          <t>https://za.rs-online.com/web/content/m/competition</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Find the best fit for you - Compare 7 in Engineering Programs Electrical Engineering in South Africa for 2025/2026</t>
+          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3085,22 +3069,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>example@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Electrical Engineering Conferences in South Africa 2026/2027/2028 - Conference Index</t>
+          <t>PDF WorldSkills South Africa Provincial Competitions 2025</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
+          <t>https://www.worldskillsza.dhet.gov.za/Document/WorldSkillsZA+Provincial+Competitions+2025+V1.1.pdf</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Nov 02 International Conference on Electronics, Control and Signal Processing (ICECSP) - Cape Town, South Africa · Nov 02 International Conference on Electrical, Computer, Electronics and Communication Engineering (ICECECE) - Cape Town, South Africa</t>
+          <t>higher education &amp; training Department: Higher Education and Training REPUBLIC OF SOUTH AFRICA</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3113,17 +3101,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Electrical And Electronics Engineering Conferences in South Africa 2026 | Conference Alerts</t>
+          <t>Electronics Electrical Engineering Scholarships for South African Students</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/south-africa/electrical-and-electronics-engineering</t>
+          <t>https://www.scholarshipsads.com/electronics-electrical-engineering-scholarships-for-south-african-students</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Select your participation type (in-person, virtual, or hybrid), fill in your personal and professional details, and pay the registration fee if required. After registering, you’ll receive confirmation and access instructions. Some electrical and electronics engineering conferences in south africa also allow early-bird registration with discounted fees.</t>
+          <t>A curated list of electronics electrical engineering scholarships worldwide open to South African students — with funding, eligibility and deadline detail for each. Ranked by relevance and completeness; updated for the latest intake.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3136,17 +3124,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Hackathons en South Africa</t>
+          <t>The Home of South African Hackathons</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/</t>
+          <t>https://hackon.co.za/</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Aug 22, 2025 · Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3159,17 +3147,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons</t>
+          <t>Hackathons en South Africa</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/</t>
+          <t>https://za.allhackathons.com/</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons Join South Africa’s premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
+          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3182,7 +3170,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Unisa hosts first-ever Hackathon to ignite student learning ...</t>
+          <t>Unisa hosts first-ever Hackathon to ignite student learning experience</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3192,7 +3180,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Jul 14, 2025 · Unisa’s Information and Communication Technology Portfolio, in collaboration with the College of Science, Engineering and Technology, held the first-ever Unisa Hackathon on 3 and 4 July 2025, marking a major step in the university’s journey to embed digital innovation and entrepreneurship into the students learning experience.</t>
+          <t>Unisa's Information and Communication Technology Portfolio, in collaboration with the College of Science, Engineering and Technology, held the first-ever Unisa Hackathon on 3 and 4 July 2025, marking a major step in the university's journey to embed digital innovation and entrepreneurship into the students learning experience.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3205,17 +3193,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Hackathons in South Africa: Seasonality, Cities &amp; Platforms</t>
+          <t>The Home of South African Hackathons</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://www.hackathonradar.com/discover/country/south-africa</t>
+          <t>https://hackon.co.za/partners/</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>When and where hackathons happen in South Africa, from 9 tracked events. Peak season is Jun (2 events), quietest is Mar (1). Midrand leads by volume.</t>
+          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3228,17 +3216,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+          <t>AfriCDSA Hackathon 2025</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/partners/</t>
+          <t>https://hackathon.africdsa.tech/</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
+          <t>Join us for the AfriCDSA Hackathon 2025, where top innovators, developers, and data scientists come together to tackle real-world challenges using cutting-edge AI and data-driven solutions. This is your chance to showcase your skills, collaborate with like-minded professionals, and contribute to impactful projects that drive change.</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3246,22 +3234,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>hackathon@africdsa.com</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators - Lifestyle &amp; Tech</t>
+          <t>ICEP - Tshwane Varsity Hackathon</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>https://lifestyleandtech.co.za/company-news/article/2026-06-29/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africas-next-generation-of-innovators</t>
+          <t>https://tvh.icep.co.za/</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>June 29, 2026 - After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant exhibition showcasing the remarkable ...</t>
+          <t>South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3271,24 +3263,24 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Full-Logo-2@2x-100-485x360.jpg</t>
+          <t>MagasengQM@tut.ac.za, info@tvh.co.za</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators</t>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>https://novuspressbulletin.co.za/blog/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africa-s-next-generation-of-innovators</t>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>June 30, 2026 - ... Johannesburg, June 2026 – After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant ...</t>
+          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3296,22 +3288,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Young Engineers Showcase Innovation at STEM Hackathon</t>
+          <t>CompeteHub - Where Champions Are Made</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>https://www.futuresa.co.za/education/young-engineers-movement-stem/</t>
+          <t>https://www.devpluxe.co.za/</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>June 11, 2026 - Fifty-five high school learners and 11 teachers from underserved South African schools will showcase working engineering and technology prototypes at the Young Engineers Movement (YEM) Hackathon Exhibition Day on 26 June 2026.</t>
+          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3319,26 +3315,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>info@futuresa.co.za</t>
-        </is>
-      </c>
+      <c r="E119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Budding engineers showcase innovation at YEM hackathon | ITWeb</t>
+          <t>MakeReign | Builders Table</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>https://www.itweb.co.za/article/budding-engineers-showcase-innovation-at-yem-hackathon/kYbe97XbP4ZqAWpG</t>
+          <t>https://builderstable.net/</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>June 30, 2026 - The hackathon was hosted by Johannesburg-based non-profit education and training organisation ORT South Africa, in partnership with JSE-listed industrial and engineering supplies firm Hudaco.</t>
+          <t>Builders Table is a two-day hackathon hosted by MakeReign, built around a 24-hour build sprint. It brings together South Africa's designers, developers, strategists, founders and creative technologists to build real working prototypes under real time pressure.</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3348,24 +3340,24 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>enquiries@ombudsman.org.za</t>
+          <t>sarah.chen@horizonlabs.com, liamlr95@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Houghton hackathon: Stepping stone for future engineers | Rosebank Killarney Gazette</t>
+          <t>Zindi - Join. Learn. Win!</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>https://www.citizen.co.za/rosebank-killarney-gazette/news-headlines/local-news/2026/06/23/houghton-hackathon-stepping-stone-for-future-engineers/</t>
+          <t>https://zindi.world/</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>June 23, 2026 - Hosted by ORT South Africa in partnership with Hudaco, the hackathon has brought together 55 learners from underserved communities to work together in developing solutions to challenges they face in their communities.</t>
+          <t>University Hackathon: Tourism Classification Challenge Equator University of Science and Technology Ended ~21 hours ago 500 Points Join Challenge 🗨️ How Mobile App Development Companies in South Africa Are Driving AI-Powered Digital Transformation in 2026 - Joshika Join Chat</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">

</xml_diff>

<commit_message>
Update competition data 2026-09-14
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -608,7 +608,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
         </is>
       </c>
     </row>
@@ -661,17 +661,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition – Electrical and Electronic Engineering</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
+          <t>https://ee.sun.ac.za/faculty-of-engineering-students-to-represent-south-africa-at-global-space-competition/</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1 month ago - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
+          <t>September 16, 2025 - Seven postgraduate students from the Faculty of Engineering have been selected to represent South Africa at the Mission Idea Contest (MIC), a global space engineering competition held in Tokyo, Japan.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -684,17 +684,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>South Africa International Industrial Expo | Innovation Bridge</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
+          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -702,22 +702,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>enquiries@aiexpoafrica.com</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://10times.com/southafrica/tradeshows</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>South Africa trade shows, find and compare 974 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 166 upcoming expos in 2026-2027 1. Mining Connect Day, 2. Annual ACFE Africa Conference &amp; Exhibition, 3. Annual Smart Procurement World Indaba, 4. ECM ...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -730,17 +734,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>KZN Industrial Technology Exhibition</t>
+          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://www.kznindustrial.co.za/</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -748,11 +752,7 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>john@email.com</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -767,7 +767,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
+          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms. Opportunity to network and connect with entrepreneurs, funders, investors, government departments and corporates.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -777,24 +777,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, Erika@innovate.durban, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, sithabile@innovate.durban</t>
+          <t>8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, sithabile@innovate.durban, Erika@innovate.durban, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
+          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
+          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
+          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -807,17 +807,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -825,22 +825,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>customerservices@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, support@informaconnect.com, support@knect365.com</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Come and explore our exhibition of innovative discoveries at Science Forum South Africa 2024 | CSIR</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>December 3, 2024 - The exhibition launch will take place on Tuesday, 3 December 2024, with the opening address by Department of Science, Technology and Innovation Minister Dr Blade Nzimande.</t>
+          <t>Big Data and Business Analytics Innovation Conference Johannesburg, South Africa IT &amp; Technology 101 Members Tue, 22 - Thu, 24 Sep 2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -853,17 +857,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>International Science, Innovation &amp; Technology Expo (INSITE)</t>
+          <t>ELENEX Africa Johannesburg 2026 - TradeFairDates</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.dsti.gov.za/index.php/resource-center/27-temp/dst-links/3-international-science-innovation-a-technology-expo</t>
+          <t>https://www.tradefairdates.com/ELENEX-Africa-M6915/Johannesburg.html</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>The essence of INSITE INSITE is an international, biennial must-see Science and Technology event in South Africa, the only one of its kind in Africa that creates new frontiers for global challenges · INSITE aims to assemble the worlds leading innovators and scientists in one place, stimulating ...</t>
+          <t>The fair is deeply rooted in the dynamics and industrial growth of Johannesburg and demonstrates South Africa's role as a leading center for technological innovation in Africa.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -876,17 +880,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AAXO - The Association of African Exhibition Organisers</t>
+          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.aaxo.co.za/</t>
+          <t>https://expotobi.com/country/south-africa/exhibitions</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>February 20, 2026 - CAPE TOWN, South Africa – The inaugural Festival of Eventing (FOE) brought together 350 event professionals, 85 speakers, and 10 countries under one roof for a two-day showcase of innovation, inspiration, and industry connection.</t>
+          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -899,17 +903,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Exhibitions in South Africa 2026, 2027 | Conference Locate (Clocate)</t>
+          <t>Come and explore our exhibition of innovative discoveries at Science ...</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.clocate.com/exhibitions-in+south-africa/Y28temE=/</t>
+          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Innovations (2) Internet of Things ... (1) Sport &amp; Leisure (2) Toys &amp; Games (3) Training (1) Transport (1) Showing 23 exhibitions · 26 May 2026 · 26-27 May 2026 · Cape Town, South Africa ·...</t>
+          <t>The final countdown is underway, and all roads lead to this year's Science Forum South Africa 2024 at the CSIR International Convention Centre in Pretoria. Join us as we plan to celebrate the CSIR's impactful science, technology and innovation contributions at South Africa's premier scientific pl...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -922,17 +926,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
+          <t>Engineering for People Design Challenge</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>Our flagship programme brings to life real-world design challenges in a safe and supported environment, through a project-based learning approach.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -945,17 +949,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Trimble Sponsors Global Design Challenge to Empower Future ...</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://news.trimble.com/Trimble-Sponsors-Global-Design-Challenge-to-Empower-Future-Engineers</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
+          <t>The competition challenges university students to design engineering solutions that address the complex, real-world needs of underserved communities.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -965,24 +969,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+          <t>pr@trimble.com, ian@clayanddaughter.com</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Launching at South Africa's Universities THE ENGINEERING FOR ...</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/posts/launching-at-south-africas-universitiesthe-engineering-for-people-design-challen/1463692205784449/</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>The Engineering For People Design Challenge is an initiative that aims to instil to prospective Engineers the ethical, environmental, social and cultural ...</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -995,17 +999,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Inspiring, building and shaping a future fit engineering community</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://www.ewb-international.org/home/inspiring-building-and-shaping-a-future-fit-engineering-community/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>Since 2011, the Design Challenge has been delivered in Cameroon, South Africa, the UK and Ireland and the USA to over 70,000 students. Learn more.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1015,24 +1019,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ied@ied.org.uk</t>
+          <t>admin@ewb-international.org</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>Engineering for People Design Challenge Launches in South ...</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.linkedin.com/posts/ewbsa_engineering-for-people-design-challenge-launch-activity-7485656340049231872-lSGJ</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>... On 30-31 March 2026, 109 students from 9 schools walked into the University of Cape Town and designed a city on the Moon. They elected leaders, divided into engineering departments, and spent 24 hours responding to a professional design brief.</t>
+          <t>Jul 22, 2026 · We are bringing the Engineering for People Design Challenge to universities across South Africa. 🇿🇦 This is where engineering students design ...</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1040,26 +1044,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>info@zasdc.org, user@domain.com</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>What is the Engineering Design Challenge? - Options for Youth | Blog</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://blog.ofy.org/blog/what-is-the-engineering-design-challenge</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
+          <t>This student competition is designed to get high school students interested in science, technology, engineering, and math (STEM). This challenge gives students ...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1072,17 +1072,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South ...</t>
+          <t>Engineering for People Challenge 2025 | PDF - Scribd</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
+          <t>https://www.scribd.com/document/901928332/Engineering-for-People-Design-Challenge-Leaflet</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
+          <t>The award-winning Engineering for People Design Challenge prepares the engineers of the future to be globally responsible.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1095,17 +1095,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>Engineering for People Design Challenge 2022/2023 | New ...</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://www.magonlinelibrary.com/doi/10.12968/S0047-9624(23)60847-8</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
+          <t>The awards are open to first- and second-year undergraduates as a mandatory part of their degree course. The aim is to encourage young engineers to broaden ...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1113,26 +1113,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Engineers Without Borders launches student challenge</t>
+          <t>Engineers - Facebook</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.theconstructionindex.co.uk/news/view/engineers-without-borders-launches-student-challenge</t>
+          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/-engineering-for-people-design-challenge-2025-updateall-submissions-from-student/1254992876654384/</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>September 7, 2021 - The Engineering for People Design Challenge encourages undergraduates to broaden their awareness of the social, environmental and economic implications of their engineering solutions.</t>
+          <t>Nov 17, 2025 · 🎉 Engineering for People Design Challenge 2025 Update! All submissions from student engineers across South Africa are in and under review by ...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1140,26 +1136,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>news@theconstructionindex.co.uk</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
+          <t>CIVE 103 students win first place in Engineers Without Borders ...</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
+          <t>https://www.engr.colostate.edu/ce/cive-103-students-win-first-place-in-engineers-without-borders-uk-design-competition/</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
+          <t>Four civil and environmental engineering majors won first prize in the national competition, “Engineering for People Design Challenge.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1379,17 +1371,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>Some of our sparkling achievements ... and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation ...</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1402,7 +1394,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Technology Expo · October 10 - TECHSPO Joburg 2026</t>
+          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1412,7 +1404,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>July 30, 2026 - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1439,7 +1431,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1449,24 +1441,24 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>support@informaconnect.com, support@knect365.com, dataprivacy@informaconnect.com, customerservices@knect365.com, customerservices@informaconnect.com, salesenquiries@africatechfestival.com, dataprivacy@knect365.com</t>
+          <t>customerservices@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, support@informaconnect.com, support@knect365.com</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology Expo ...</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 - 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
+          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1474,22 +1466,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 - 7, 2027 ...</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>The annual TECHSPO Cape Town 2027 Technology Expo returns October 6th to 7th, 2027 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town. TECHSPO Cape Town Technology Expo is the must-attend event to: Experience the Future of Technology &amp; Innovation Discover cutting-edge tech, game-changing tools, and innovators shaping tomorrow's digital world. See the latest advancements in ...</t>
+          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1499,24 +1495,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>info@techspocapetown.co.za</t>
+          <t>enquiries@aiexpoafrica.com</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Tech Expo Africa - Enabling Development</t>
+          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://techexpo.africa/</t>
+          <t>https://10times.com/johannesburg-za/technology</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Tech Expo Africa is a social enterprise connecting African businesses with top tech and business leaders to drive innovation.</t>
+          <t>Sep 15, 2026 · Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1524,26 +1520,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>info@techexpo.africa</t>
-        </is>
-      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
+          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1556,17 +1548,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2026 Technology Expo (Internet ~ Mobile ~ AdTech ...</t>
+          <t>World-Class Consumer Tech Show - 4,200+ Global Exhibitors</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://allevents.in/cape-town/techspo-cape-town-2026-technology-expo-internet-~-mobile-~-adtech-~-martech-~-saas/200030358413547</t>
+          <t>https://www.bing.com/aclick?ld=e87ZKcOhwamYQPx18INGy8xTVUCUzJcJoZxfs4RMDA9DU2Gx6M5LohwCVWNPlHzX1Dnq_hnF_rtOlCJFqrTgA2ODifXtqHPHDVkGk4OCLVoEzqrw0wiSt1DgNishCMuFXS-Vdc57N8aByGib5sYNzHV-7RDUgSO2ukUIpNIduwazG7EK4B11HxIfSqzujeGi6yv7dy-uBVcouStvaTf3hdmESFhYI&amp;u=aHR0cHMlM2ElMmYlMmZ3d3cuZ2xvYmFsc291cmNlcy5jb20lMmZ0cmFkZVNob3dzJTJmSEslMmZzaG9ydHJlZ2lzdGVyJTNmc291cmNlJTNkODA0NDE2NyUyNnV0bV9zb3VyY2UlM2Q4MDQ0MTY3JTI2c2hvd191dG1fc291cmNlJTNkODA0NDE2NyUyNnV0bV9jYW1wYWlnbiUzZDUzMzY1MjczNCUyNnV0bV90ZXJtJTNkYXNpYSUyNTIwdHJhZGUlMjUyMHNob3dzJTI2YWRncm91cGlkJTNkMTM0OTEwMzQ5MzM2MDM1MyUyNnRhcmdldGlkJTNka3dkLTg0MzIwMjIzMTk5NTI3JTNhbG9jLTE5MCUyNm1hdGNodHlwZSUzZHAlMjZkZXZpY2UlM2RjJTI2Y291bnRyeSUzZDQ4NzkyJTI2bmV0d29yayUzZG8lMjZwbGFjZW1lbnQlM2QlMjZtc2Nsa2lkJTNkMjlhMWFiZjNhMjkzMWM3YmJkOGNjMTU0NTk1MmZlZGY&amp;rlid=29a1abf3a2931c7bbd8cc1545952fedf</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town Technology Expo returns October 1-2, 2026 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town, South Africa. This must-attend, two-day annual event brings together leading developers, marketers, innovators, and technology enthusiasts eager to showcase and explore the latest in tech and digital solutions.</t>
+          <t>Attend Hong Kong's leading sourcing event for AI and consumer electronics. Pre-register today to meet verified suppliers at AsiaWorld-Expo, Hong Kong.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1579,17 +1571,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology ...</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1602,17 +1594,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1620,22 +1612,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>u003einfo@techspo.co, atinfo@techspo.coor</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~…</t>
+          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
+          <t>https://africatechnologyexpo.com/</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa. This must-attend, two-day annual event brings together leading developers, marketers, innovators, and technology enthusiasts eager to showcase and explore the latest in tech and digital solutions.</t>
+          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1645,24 +1641,24 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>support@industryevents.com, events@techspojoburg.co.za, your@email.com, you@company.com, colleague@company.com</t>
+          <t>partner@africatechnologyexpo.com, info@sparkafrica.co, johndoe@email.com</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Maker Faire Africa - Wikipedia</t>
+          <t>Maker Faire - Wikipedia</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Maker_Faire_Africa</t>
+          <t>https://en.wikipedia.org/wiki/Maker_Faire</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>March 7, 2025 - Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds ...</t>
+          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1675,17 +1671,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Maker Faire - Wikipedia</t>
+          <t>Maker Faire Africa - Wikipedia</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Maker_Faire</t>
+          <t>https://en.wikipedia.org/wiki/Maker_Faire_Africa</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>May 3, 2026 - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
+          <t>The aim of a Maker Faire Africa is to create a space on the African continent where Afrigadget-type innovations, inventions and initiatives can be sought, identified, brought to life, supported, amplified and propagated.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1698,17 +1694,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
+          <t>Maker Faire groups | Meetup</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://makerfairecapetown.wordpress.com/about/</t>
+          <t>https://www.meetup.com/topics/maker-faire/za/</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
+          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1721,17 +1717,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>Maker Faire |</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>https://makerfaire.com/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1739,22 +1735,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>pr@make.co, fancybox_sprite@2x.png, fancybox_loading@2x.gif, chosen-sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>http://capetown.makerfaire.com/</t>
+          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+          <t>Aug 21, 2015 · We’re delighted to present the first ever Cape Town Maker Faire, hosted by Open Design in partnership with Trimble.Maker Faire is primarily designed as a forward-looking event, showcasing makers who are exploring new forms and new technologies.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1762,26 +1762,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, pr@make.co, fancybox_sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Blog : Maker Faire Africa</t>
+          <t>Maker Faire Africa — Grokipedia</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>http://makerfaireafrica.com/blog/</t>
+          <t>https://grokipedia.com/page/maker_faire_africa</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building his ANIMAL car, from the ground up, that means the frame and all.</t>
+          <t>Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1794,17 +1790,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
+          <t>About | Maker Faire Cape Town: Make • Create • Craft</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
+          <t>https://makerfairecapetown.wordpress.com/about/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
+          <t>Maker Faire is a community-based learning event that inspires everyone to become a maker and connect to people and projects in their local community.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1817,17 +1813,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>The Makers Hub</t>
+          <t>Maker Faire Africa (@MFAJoburg) - Facebook</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.decorex.co.za/cape-town/en-gb/visit/TheMakersHub.html</t>
+          <t>https://www.facebook.com/MFAJoburg/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Explore unique handmade items, take part in interactive workshops, and engage directly with Cape Town’s vibrant maker community.</t>
+          <t>Maker Faire Africa. The Fem-In-Tech Development Programme is aimed at female-led South African start-ups in tech and tech- enabled sectors.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1835,26 +1831,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>decorexafrica@rxglobal.com</t>
-        </is>
-      </c>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
+          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
+          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
+          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will ...</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1867,17 +1859,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Why Africa needs Maker Faire | ZDNET</t>
+          <t>Maker Faire Cape Town 2015 - PlanetJune Blog</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
+          <t>https://www.planetjune.com/blog/maker-faire-cape-town-2015/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage to attend and show off their work.</t>
+          <t>Aug 24, 2015 · Yesterday, I attended the first annual Maker Faire in Cape Town and it was inspiring – there was lots to see and explore.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1890,17 +1882,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>StemCo - StemCo 2026 International Competitions</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://stemco.org/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
+          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1913,17 +1905,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1931,26 +1923,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
+          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>February 27, 2026 - Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1958,22 +1946,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>High School STEM Competition | Capetown 2026</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Local, regional and national competitions with thousands of · Multi-level events of two or more rounds that become increasingly challenging and culminate in top-level Olympiads. Enrichment programmes to inspire promising young South Africans to pursue STEMI</t>
+          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -1981,22 +1973,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>Astemi Sa</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The ZASDC is South Africa's national Space Design Competition, part of a global network spanning six continents. Secondary school students design futuristic space settlements in a fast-paced industry simulation that builds real STEM, leadership ...</t>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2004,26 +2000,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>info@zasdc.org, user@domain.com</t>
-        </is>
-      </c>
+      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions 2022 – SAASTA</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://saasta.ac.za/astemi-competitions-2</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2036,17 +2028,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Competition – Eskom Expo for Young Scientists</t>
+          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://exposcience.co.za/category/competition/</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Aqil Variava business cities Damien ... Gray STEMI Vuyo Nzimande · Eskom Expo for Young Scientists is an exposition, or science fair, where students have a chance to show others their projects about their own scientific investigations. At the annual prestigious Eskom Expo for Young Scientists International Science Fair (ISF), selected students from 35 Expo Regions in South Africa then compete ...</t>
+          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2054,26 +2046,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>support@exposcience.co.za</t>
-        </is>
-      </c>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Rural youth lead in robotics at national STEM competition</t>
+          <t>South African Space Design Competition | Inspire Space Innovation ...</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://iol.co.za/news/education/2025-09-15-rural-youth-lead-in-robotics-at-national-stem-competition/</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>September 15, 2025 - Discover how South Africa's brightest young minds are tackling real-world challenges with innovative solutions at the inaugural AlgoAtWork RoboRumble STEM Innovation Challenge, where ideas like autonomous robots and smart PPE systems are set ...</t>
+          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2083,24 +2071,24 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>londiwe.gumede@inl.co.za, philippa.larkin@inl.co.za, nobuntu.mgijima@volt.africa, mendy.mtshali@inl.co.za, lee.rondganger@inl.co.za, ashley.lechman@inl.co.za</t>
+          <t>info@zasdc.org, user@domain.com</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026 Season - Africa's Global STEM Celebration</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://www.stemfestival.org/competitions/</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>April 30, 2026 - ... The Elementary, Junior, and Senior Robotics categories at STEM Festival are dedicated to advancing the World Robot Olympiad (WRO) across the Niger Delta and South-South Nigeria, working with ArcLights Foundation.</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2113,17 +2101,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>STEAM Pitch Competition - STEM AFRICA FEST 2024</t>
+          <t>National Department of Basic Education</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://stemafricafest.com/steam-pitch-competition/</t>
+          <t>https://www.education.gov.za/LinkClick.aspx?fileticket=i9GS5Atf7zo=&amp;tabid=347&amp;portalid=0&amp;mid=14629</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Join STEM Africa Fest , celebrating science, technology, engineering, and mathematics. Experience hands-on learning, industry leaders, and innovation across Africa.</t>
+          <t>JOHANNESBURG, South Africa - XX Month 2026 - The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries ...</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2131,7 +2119,11 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>s.ngcobo@cheil.com, ssasft@samsung.com, j.mogoeng@samsung.com</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2156,24 +2148,24 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
+          <t>8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
+          <t>April 14, 2026 - This National Event, to be held at the Sandton Convention Centre in Johannesburg, South Africa, as part of AI for Good Impact Africa, at AI Expo Africa 2025, is a qualifying tournament leading to the Grand Finale in Geneva during the AI for ...</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2183,24 +2175,24 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, info@thecortexhub.africa, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
+          <t>FIRST South Africa – Robotics Programs for School Children</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
+          <t>https://firstsa.org/</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in a UN-based global robotics competition, focusing on the critical area of disaster response.</t>
+          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2208,26 +2200,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>name@example.com</t>
-        </is>
-      </c>
+      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Live Competitions — Nirvana Global Foundation</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://nirvanaglobalfoundation.org/competition.html</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Enjoy AI South Africa An international AI and robotics competition for young innovators. Teams build, program and compete with official ENJOY AI robotics kits across categories like Battle of Stars, Mining Expedition, Drone Cup and Inventions Trail — preparing learners for the global ENJOY AI stage.</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2235,26 +2223,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>info@nirvanaglobalfoundation.org, you@email.com, coach@school.co.za</t>
-        </is>
-      </c>
+      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Roboticon 2026: South Africa Showcases Robotics for Culture, Education ...</t>
+          <t>South African Robotics Competitions and Schools</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
+          <t>https://www.sciencexpo.org.za/robotics.html</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation." South Africa's robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
+          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2264,24 +2248,24 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>adverts@ubuntutimes.co.za, newspaper-rec300@2x.jpg</t>
+          <t>marna.vanzyl@imbewu.foundation, madelien@imbewu.foundation, webmaster@sciencexpo.org.za</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop their creativity and problem-solving skills through challenging and educational robotics competitions.</t>
+          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2289,22 +2273,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>NkosiN@atnews.co.za, rampedim@atnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026 - SpringBots South Africa</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://springbots.co.za/2026-2/</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>This approach ensures that learners are not only participants in robotics competitions but are also equipped with real-world skills in design thinking, programming, systems engineering, and collaborative problem-solving. A Unified Future for Africa SpringBots' 2026 vision extends beyond competition and education.</t>
+          <t>The Robotics for Good Youth Challenge national competition will be held in Johannesburg, South Africa, at the Sandton Convention Centre on the 31st October 2025.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2312,22 +2300,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, info@thecortexhub.africa, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
+          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>ICS Export Are you sure you want to remove this speaker?</t>
+          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2335,26 +2327,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>name@example.com</t>
-        </is>
-      </c>
+      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Welcome to FIRST Tech Challenge - FIRST South Africa</t>
+          <t>Robotics &amp; Coding Classes for Kids in Johannesburg | Robotics League</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://firstsa.org/welcome-to-first-tech-challenge/</t>
+          <t>https://robotics-league.co.za/</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>The robot kit is reusable from year-to-year and can be programmed using a variety of languages, including Java. Teams also must raise funds, design and market their team brand, and do community outreach for which they can win awards.</t>
+          <t>2026 Theme · Robots Meet Culture. The World Robot Olympiad is the planet's biggest student robotics competition — over 100 countries, 100,000+ students a year. South African teams compete on two tracks: Explorer, the home-grown SA challenge, ...</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2362,22 +2350,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>info@roboticsleague.co.za, you@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Home | Roboticon 2026</t>
+          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://roboticon.resolute.education/</t>
+          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Join us for the ultimate robotics showcase as Resolute proudly sponsors the World Robotics Olympiad (WRO) South Africa! This year, we're bringing together two worlds for the biggest robotics event of the year - Roboticon and the WRO Nationals, happening on the same day at the same venue.</t>
+          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2390,17 +2382,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>Bridge Building Competition (Dept of Civil Engineering)</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
+          <t>https://civilabcut.co.za/services/bridge-building-competition-dept-of-civil-engineering/</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
+          <t>Supported by SAICE (South African Institution of Civil Engineering), the competition continues to inspire the next generation of civil engineers to create, strengthen, and innovate for a sustainable future.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2410,24 +2402,24 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za, newsletters@creamermedia.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za</t>
+          <t>Civilab@CUTLogo-Transparent.png, etheron@cut.ac.za, cropped-Civilab@CUTLogo-Transparent.png</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd International Bridge Building Competition - SAICE</t>
+          <t>Non - profit SAICE launches Bridge Building Competition</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://saice.org.za/press-releases/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://www.algoafm.co.za/event/non-profit-saice-launches-bridge-building-competition</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>April 17, 2025 - The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
+          <t>Organised by SAICE, a non-profit professional body for civil engineers in South Africa, the competition promotes teamwork, creativity, problem-solving, and an interest in engineering careers while showcasing the practical application of structural design and construction concepts.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2435,26 +2427,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>communications@saice.org.za, membership@saice.org.za, accounts@saice.org.za, civilinfo@saice.org.za, marketing@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
+          <t>Engineering the future: 16 schools compete in SAICE's 33rd ...</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
+          <t>https://www.southafricanbusiness.co.za/08/2024/construction-and-engineering/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2467,17 +2455,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>SAICE's 34th International Bridge Competition Inspires Tomorrow's ...</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
+          <t>https://southafricatoday.net/lifestyle/education/saices-34th-international-bridge-competition-inspires-tomorrows-engineers/</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2485,26 +2473,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>ernao@crown.co.za, constr@crown.co.za</t>
-        </is>
-      </c>
+      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
+          <t>The South African Institution of Civil Engineering</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
+          <t>https://civils.org.za/</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>September 7, 2025 - Find the list of upcoming Civil Engineering conferences in South Africa 2025 with invitation an letter.</t>
+          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2517,17 +2501,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SWM Communications | SAICE recognises civil engineering research excellence through national student competition</t>
+          <t>Civil Engineering Conferences in South Africa 2026/2027/2028</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://swmcommunications.co.za/press-office/saice-recognises-civil-engineering-research-excellence-through-national-student-competition/</t>
+          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>April 1, 2026 - The event – which was sponsored by Sika, WorldsView, BVI, RIBCCS, and AF Consulting – was hosted at SAICE House in Midrand, Gauteng, and accredited for 0.2 CPD points. Students were invited to present their civil engineering university research and investigation project, which is part of the national curriculum for final year civil engineering undergraduate students.</t>
+          <t>Civil Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2535,26 +2519,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>nthabeleng@saice.org.za, info@swmcommunications.co.za</t>
-        </is>
-      </c>
+      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
+          <t>VUT inspires future engineers through Bridge Building Competition</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
+          <t>https://vut.ac.za/vut-inspires-future-engineers-through-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
+          <t>Supported by the ArcelorMittal Science Centre, Institution of Structural Engineers (IStructE), Fundi, South African Institution of Civil Engineering Future Leaders Panel (SAICE FLP) Vaal and maVuti Shop, the initiative challenged learners to design and construct bridge models using simple materials, including sticks, wool and glue.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2567,17 +2547,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
+          <t>Engineering the future: 16 schools compete in bridge building ...</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
+          <t>https://www.engineerit.co.za/article/engineering-the-future-16-schools-compete-in-bridge-building-competition</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Civil engineering conferences in Cape town 2025 provide an exclusive global platform to meet and engage with experts and aspirants in various fields.</t>
+          <t>The recent South African Institution of Civil Engineering (SAICE) 33 rd International Bridge Building competition at the Midrand Conference Centre showcased 16 high schools around South Africa and one in Swaziland encouraging learners to apply their knowledge of mathematics and science in practical engineering projects. Each team received 25 sticks, string and glue to construct a bridge ...</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2590,17 +2570,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>Building the future: SAICE International Bridge Building Competition ...</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
+          <t>https://journals.co.za/doi/full/10.10520/ejc-civeng_v32_n9_a22</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>SAICE hosted its 32nd International Bridge Building Competition at the Midrand Conference Centre on 23 August 2024, bringing together 16 schools from around South Africa and Swaziland to compete for the prestigious bridge building trophy.</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2613,17 +2593,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Civil Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
+          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
+          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Apr 13 International Conference on Architectural, Civil and Environmental Engineering (ICACEE) - Cape Town, South Africa</t>
+          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2636,17 +2616,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>Category:Mechanical engineering competitions - Wikipedia</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://en.wikipedia.org/wiki/Category:Mechanical_engineering_competitions</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>Engineering competitions · Mechanical engineering · Search · Category:Mechanical engineering competitions ·</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2659,17 +2639,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>Mechanical Engineering Conferences in South Africa 2026/2027/2028 - Conference Index</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://conferenceindex.org/conferences/mechanical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>Nov 04 International Conference on Tribology and Interface Engineering (ICTIE) - Cape Town, South Africa · Nov 04 International Conference on Mechanical and Systems Engineering (ICMSE) - Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2682,17 +2662,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>&gt;&gt; Industrial and Manufacturing Engineering · &gt;&gt; Mechanical Engineering · &gt;&gt; Ocean Engineering · Environmental Science · Mathematics · Medicine · &gt;&gt; Anatomy · &gt;&gt; Anesthesiology and Pain Medicine · &gt;&gt; Cardiology and Cardiovascular Medicine · &gt;&gt; Critical Care and Intensive Care Medicine ·</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2705,17 +2685,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Mechanical Engineering events - South Africa Group - Institution of Mechanical Engineers</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://nearyou.imeche.org/near-you/middle-east-and-africa/south-africa/events</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
+          <t>For details of Mechanical Engineering events organised by South Africa Group, please click the above link.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2723,26 +2703,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>WorldSkills South Africa 2027 Applications Now Open - Apply Online</t>
+          <t>Best Mechanical Engineering Companies in South Africa</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://www.edupstairs.org/worldskills-south-africa-2027-applications/</t>
+          <t>https://engineeringness.com/best-mechanical-engineering-companies-in-south-africa/</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Applications are officially open for the WorldSkills South Africa 2027 National Competition, giving talented students, apprentices, learners and qualifying skilled candidates across South Africa an opportunity to demonstrate their practical abilities on a national stage.</t>
+          <t>October 4, 2025 - This article showcases our top picks for the best South Africa based Mechanical Engineering companies. These startups and companies are taking a variety of approaches to innovating the Mechanical Engineering industry, but are all exceptional companies well worth a follow.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2750,26 +2726,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>sifisomhlongo@edupstairs.org</t>
-        </is>
-      </c>
+      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
+          <t>Past Mechanical Engineering events - South Africa Group - Institution of Mechanical Engineers</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://nearyou.imeche.org/near-you/middle-east-and-africa/south-africa/past-events</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent's largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
+          <t>For details of past Mechanical Engineering events organised by South Africa Group, please click the above link.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2782,17 +2754,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>10 Mechanical Engineering Competitions for High School Students — Veritas AI</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.veritasai.com/veritasaiblog/10-mechanical-engineering-competitions-for-high-school-students</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>October 29, 2025 - ... Competition Dates: The contest year began on April 14 and ends on May 31. Students can submit (unique) entries for each monthly contest. Eligibility: The contest is open to all students, regardless of their age or discipline.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2802,24 +2774,24 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>contact@veritasai.com, user@domain.com</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>7 Mechanical Engineering Degree Programs in South Africa - Study Abroad | educations.com</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.educations.com/mechanical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>One of the main objectives of this process is to develop an advanced capability to do fundamental engineering research independently. It also promotes a lifelong learning approach. ... The Master of Mechanical Engineering (MS) program objective is to provide students with the skill sets and knowledge necessary to become a professional who can solve practical issues of the field of mechanical engineering.</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2827,26 +2799,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
+          <t>Mechanical Engineering in South Africa: 2025 Master's Guide | Mastersportal</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
+          <t>https://www.mastersportal.com/study-options/271564839/mechanical-engineering-south-africa.html</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
+          <t>The Mechanical Engineering program at the University of Pretoria is a leading source of graduates in the... ... Applied Science Metallurgy from University of Pretoria aims to be internationally competitive while... ... Holders of any other equivalent South African or international qualification may also be considered for...</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2859,17 +2827,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>Engineering Competitions - ASME</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>https://www.asme.org/conferences-events/competitions</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>There are four kinds of challenges &amp; competitions held during the three-day, two-night regional events built around design, advanced manufacturing &amp; robotics technologies. HPVC, IAM3D, the student design competition &amp; the old guard competition.</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2882,17 +2850,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>Student Chapter Design Contest (Africa) Serving the electrical energy conversion professional worldwide. Chapter Design Contest (Africa) Deadline: April 30, ...</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2905,17 +2873,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>IEEE South Africa</t>
+          <t>WorldSkills South Africa 2027 Applications - Edupstairs</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>http://www.ieee.org.za/</t>
+          <t>https://www.edupstairs.org/worldskills-south-africa-2027-applications/</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>The South African Section has around 1200 members and many subsections. It was formed in 1963 by the merger of the Institute of Radio Engineers (IRE, founded 1912) and the American Institute of Electrical Engineers (AIEE, founded 1884).</t>
+          <t>2 days ago · WorldSkills is about identifying exceptional practical and technical talent in fields ranging from welding, electrical installations and ...</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2923,22 +2891,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>sifisomhlongo@edupstairs.org</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>CMU-Africa students shine at global electronics conference</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://www.africa.engineering.cmu.edu/news/2026/01/16-ieee-conference.html</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Centres South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits</t>
+          <t>Jan 16, 2026 · SPEC 2025, held in Johannesburg, South Africa, is part of the Power Electronics Society, in the field of electrical engineering.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2948,24 +2920,24 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
+          <t>africa-info@andrew.cmu.edu</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>Electricity challenges a top issue at African engineering ...</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://standardmicrogrid.com/content/electricity-challenges-top-issue-african-engineering-innovation-competition</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Electricity challenges a top issue at African engineering innovation competition. Engineering innovations to boost off-grid power and stop electricity theft ... Missing: electrical | Show results with: electrical</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2978,17 +2950,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
+          <t>Take a look back at day 1 of the #WorldSkillsZA competition ...</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://www.facebook.com/GovernmentZA/videos/️-take-a-look-back-at-day-1-of-the-worldskillsza-competition-where-competitors-b/1633847574552335/</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>IEEE-IAS Industrial Power Conversion Systems Department Serving the electrical energy conversion professional worldwide</t>
+          <t>Mar 10, 2026 · South African electrical engineer wins gold medal. Njabulo Mabaso ... The WorldSkills South Africa National Competition Closing Ceremony marked ...</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3001,17 +2973,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3019,26 +2991,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3051,17 +3019,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Competitions | ESG</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://za.rs-online.com/web/content/m/competition</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
+          <t>Centres South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3071,24 +3039,24 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>example@email.com</t>
+          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>PDF WorldSkills South Africa Provincial Competitions 2025</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/Document/WorldSkillsZA+Provincial+Competitions+2025+V1.1.pdf</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>higher education &amp; training Department: Higher Education and Training REPUBLIC OF SOUTH AFRICA</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3101,17 +3069,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Electronics Electrical Engineering Scholarships for South African Students</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://www.scholarshipsads.com/electronics-electrical-engineering-scholarships-for-south-african-students</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>A curated list of electronics electrical engineering scholarships worldwide open to South African students — with funding, eligibility and deadline detail for each. Ranked by relevance and completeness; updated for the latest intake.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3119,7 +3087,11 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3147,17 +3119,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Hackathons en South Africa</t>
+          <t>Hackathons in South Africa: Seasonality, Cities &amp; Platforms</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/</t>
+          <t>https://www.hackathonradar.com/discover/country/south-africa</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+          <t>When and where hackathons happen in South Africa, from 9 tracked events. Peak season is Jun (2 events), quietest is Mar (1). Midrand leads by volume.</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3170,17 +3142,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Unisa hosts first-ever Hackathon to ignite student learning experience</t>
+          <t>Hackathons en South Africa</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
+          <t>https://za.allhackathons.com/</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Unisa's Information and Communication Technology Portfolio, in collaboration with the College of Science, Engineering and Technology, held the first-ever Unisa Hackathon on 3 and 4 July 2025, marking a major step in the university's journey to embed digital innovation and entrepreneurship into the students learning experience.</t>
+          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3193,17 +3165,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>The Home of South African Hackathons</t>
+          <t>AfriHack 2026: Pan-African Hackathon for Technology Students in ...</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/partners/</t>
+          <t>https://youthopportunitieshub.com/afrihack-2026/</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
+          <t>The annual hackathon, organised by Empiras Global, is returning in 2026 for its third edition. The programme is designed to bring together technology students from South Africa, other African countries and international universities to work on authentic business challenges.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3216,17 +3188,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>AfriCDSA Hackathon 2025</t>
+          <t>The Home of South African Hackathons</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>https://hackathon.africdsa.tech/</t>
+          <t>https://hackon.co.za/partners/</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Join us for the AfriCDSA Hackathon 2025, where top innovators, developers, and data scientists come together to tackle real-world challenges using cutting-edge AI and data-driven solutions. This is your chance to showcase your skills, collaborate with like-minded professionals, and contribute to impactful projects that drive change.</t>
+          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3234,26 +3206,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>hackathon@africdsa.com</t>
-        </is>
-      </c>
+      <c r="E116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ICEP - Tshwane Varsity Hackathon</t>
+          <t>Hackathons in South Africa</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>https://tvh.icep.co.za/</t>
+          <t>https://za.allhackathons.com/hackathons/</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
+          <t>Hackathons in South Africa Verken alle hackathons in South Africa PERSOONLIK GIRLCODE GHANA HACKATHON 2025 Aug. 22, 2025 - Sept. 14, 2025 Eindig</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3261,26 +3229,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>MagasengQM@tut.ac.za, info@tvh.co.za</t>
-        </is>
-      </c>
+      <c r="E117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Young Engineers Movement (YEM) - ORT SA</t>
+          <t>Houghton hackathon: Stepping stone for future engineers</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+          <t>https://www.citizen.co.za/rosebank-killarney-gazette/news-headlines/local-news/2026/06/23/houghton-hackathon-stepping-stone-for-future-engineers/</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
+          <t>55 learners from underserved communities are developing creative solutions to everyday challenges while navigating future careers in engineering and technology at a five-day hackathon in Houghton ...</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3288,26 +3252,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
-        </is>
-      </c>
+      <c r="E118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CompeteHub - Where Champions Are Made</t>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>https://www.devpluxe.co.za/</t>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
+          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3315,22 +3275,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>MakeReign | Builders Table</t>
+          <t>CompeteHub - Where Champions Are Made</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>https://builderstable.net/</t>
+          <t>https://www.devpluxe.co.za/</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Builders Table is a two-day hackathon hosted by MakeReign, built around a 24-hour build sprint. It brings together South Africa's designers, developers, strategists, founders and creative technologists to build real working prototypes under real time pressure.</t>
+          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3338,26 +3302,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>sarah.chen@horizonlabs.com, liamlr95@gmail.com</t>
-        </is>
-      </c>
+      <c r="E120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Zindi - Join. Learn. Win!</t>
+          <t>AfriHack 2026 | Empiras Global</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>https://zindi.world/</t>
+          <t>https://www.empirasglobal.com/afrihack26</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>University Hackathon: Tourism Classification Challenge Equator University of Science and Technology Ended ~21 hours ago 500 Points Join Challenge 🗨️ How Mobile App Development Companies in South Africa Are Driving AI-Powered Digital Transformation in 2026 - Joshika Join Chat</t>
+          <t>AfriHack is an annual initiative aimed at uplifting young local, continental, and global tech students. In 2026, Empiras is thrilled to present the third edition of AfriHack. The hackathon series is designed to engage technology students from all regions of South Africa in addressing authentic business challenges, while simultaneously fostering collaboration and innovation among participants ...</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -3365,7 +3325,11 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 1eeb89147c984dc6bc3ffafd9e6cd089@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 54b4aac306184111a223c0f4aea635c3@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 98b21aa53d68482b8414e892d9af0e5f@sentry-next.wixpress.com, e40146ef843e4f9196e5d00c98ac3689@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, cd64ba1f47df485bba2b0076c0dd3b25@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, info@empirasglobal.com, a18507e8883842d8a1ba47257fee81ac@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-09-15
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>August 6, 2026 - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -492,17 +492,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -510,22 +510,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
+          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -535,24 +539,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>info@zasdc.org, user@domain.com</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -565,17 +569,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Engineering Conferences in South Africa 2025-2026</t>
+          <t>Competitions – Enactus South Africa | National Expos ...</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
+          <t>https://enactusza.org/what-we-do/competitions</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
+          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -583,22 +587,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>xmadlanga@enactus.org, liso@enactus.org, marketingsa@enactus.org, adminsa@enactus.org</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
+          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>August 6, 2026 - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -606,26 +614,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -638,17 +642,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.thecasecentre.org/products/view?id=189255</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
+          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -656,22 +660,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>info@zasdc.org, user@domain.com</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition – Electrical and Electronic Engineering</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://ee.sun.ac.za/faculty-of-engineering-students-to-represent-south-africa-at-global-space-competition/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>September 16, 2025 - Seven postgraduate students from the Faculty of Engineering have been selected to represent South Africa at the Mission Idea Contest (MIC), a global space engineering competition held in Tokyo, Japan.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -679,7 +687,11 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -734,17 +746,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -752,22 +764,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>dataprivacy@knect365.com, customerservices@knect365.com, salesenquiries@africatechfestival.com, support@informaconnect.com, dataprivacy@informaconnect.com, customerservices@informaconnect.com, support@knect365.com</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms. Opportunity to network and connect with entrepreneurs, funders, investors, government departments and corporates.</t>
+          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -775,26 +791,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, sithabile@innovate.durban, Erika@innovate.durban, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
+          <t>Exhibition | Innovation Festival Durban | South Africa</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
+          <t>https://www.innovationfestival.durban/exhibition</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
+          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms. Opportunity to network and connect with entrepreneurs, funders, investors, government departments and corporates.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -802,22 +814,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, Erika@innovate.durban, 8c4075d5481d476e945486754f783364@sentry.io, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, sithabile@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -825,11 +841,7 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>customerservices@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, support@informaconnect.com, support@knect365.com</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -857,17 +869,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ELENEX Africa Johannesburg 2026 - TradeFairDates</t>
+          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.tradefairdates.com/ELENEX-Africa-M6915/Johannesburg.html</t>
+          <t>https://expotobi.com/country/south-africa/exhibitions</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>The fair is deeply rooted in the dynamics and industrial growth of Johannesburg and demonstrates South Africa's role as a leading center for technological innovation in Africa.</t>
+          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -880,17 +892,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
+          <t>South Africa - IoT Africa Exhibition and Conference</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://expotobi.com/country/south-africa/exhibitions</t>
+          <t>https://iot-africa.com/south-africa/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
+          <t>IoT Africa Exhibition and Conference in Johannesburg, South Africa brings together leaders across IoT, data centres, cloud, telecom, AI, cybersecurity, and digital infrastructure. Connect with enterprises, government, and tech innovators shaping Africa's smart, connected future.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -898,7 +910,11 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>info@iot-africa.com</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -926,17 +942,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge</t>
+          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Our flagship programme brings to life real-world design challenges in a safe and supported environment, through a project-based learning approach.</t>
+          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -949,17 +965,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Trimble Sponsors Global Design Challenge to Empower Future ...</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://news.trimble.com/Trimble-Sponsors-Global-Design-Challenge-to-Empower-Future-Engineers</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>The competition challenges university students to design engineering solutions that address the complex, real-world needs of underserved communities.</t>
+          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -969,24 +985,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>pr@trimble.com, ian@clayanddaughter.com</t>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Launching at South Africa's Universities THE ENGINEERING FOR ...</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/posts/launching-at-south-africas-universitiesthe-engineering-for-people-design-challen/1463692205784449/</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>The Engineering For People Design Challenge is an initiative that aims to instil to prospective Engineers the ethical, environmental, social and cultural ...</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -999,17 +1015,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Inspiring, building and shaping a future fit engineering community</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.ewb-international.org/home/inspiring-building-and-shaping-a-future-fit-engineering-community/</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Since 2011, the Design Challenge has been delivered in Cameroon, South Africa, the UK and Ireland and the USA to over 70,000 students. Learn more.</t>
+          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1019,24 +1035,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>admin@ewb-international.org</t>
+          <t>ied@ied.org.uk</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge Launches in South ...</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/posts/ewbsa_engineering-for-people-design-challenge-launch-activity-7485656340049231872-lSGJ</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Jul 22, 2026 · We are bringing the Engineering for People Design Challenge to universities across South Africa. 🇿🇦 This is where engineering students design ...</t>
+          <t>... On 30-31 March 2026, 109 students from 9 schools walked into the University of Cape Town and designed a city on the Moon. They elected leaders, divided into engineering departments, and spent 24 hours responding to a professional design brief.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1044,22 +1060,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>info@zasdc.org, user@domain.com</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>What is the Engineering Design Challenge? - Options for Youth | Blog</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://blog.ofy.org/blog/what-is-the-engineering-design-challenge</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>This student competition is designed to get high school students interested in science, technology, engineering, and math (STEM). This challenge gives students ...</t>
+          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1072,17 +1092,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineering for People Challenge 2025 | PDF - Scribd</t>
+          <t>Engineers Without Borders South ...</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.scribd.com/document/901928332/Engineering-for-People-Design-Challenge-Leaflet</t>
+          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>The award-winning Engineering for People Design Challenge prepares the engineers of the future to be globally responsible.</t>
+          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1095,17 +1115,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge 2022/2023 | New ...</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.magonlinelibrary.com/doi/10.12968/S0047-9624(23)60847-8</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>The awards are open to first- and second-year undergraduates as a mandatory part of their degree course. The aim is to encourage young engineers to broaden ...</t>
+          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1118,17 +1138,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Engineers - Facebook</t>
+          <t>Engineers Without Borders launches student challenge</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/-engineering-for-people-design-challenge-2025-updateall-submissions-from-student/1254992876654384/</t>
+          <t>https://www.theconstructionindex.co.uk/news/view/engineers-without-borders-launches-student-challenge</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Nov 17, 2025 · 🎉 Engineering for People Design Challenge 2025 Update! All submissions from student engineers across South Africa are in and under review by ...</t>
+          <t>September 7, 2021 - The Engineering for People Design Challenge encourages undergraduates to broaden their awareness of the social, environmental and economic implications of their engineering solutions.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1136,22 +1156,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>news@theconstructionindex.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CIVE 103 students win first place in Engineers Without Borders ...</t>
+          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.engr.colostate.edu/ce/cive-103-students-win-first-place-in-engineers-without-borders-uk-design-competition/</t>
+          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Four civil and environmental engineering majors won first prize in the national competition, “Engineering for People Design Challenge.</t>
+          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1159,22 +1183,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>privacy@studocu.com</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
+          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1182,22 +1210,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1205,22 +1237,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1233,17 +1269,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1256,17 +1292,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
+          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1274,22 +1310,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, email@example.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Competitions - Enactus South Africa | National Expos, Challenges ...</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://enactusza.org/what-we-do/competitions</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1297,22 +1337,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>xmadlanga@enactus.org, liso@enactus.org, marketingsa@enactus.org, adminsa@enactus.org</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Engineering in South Africa: 24 Best universities Ranked</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/za/</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1325,17 +1369,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>Competitions - SABSA</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://sabsa.co.za/competitions/</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>African Business Concept Challenge ABCC is a virtual simulation-based business concept competition for African undergraduate and graduate students. The competition will challenge student teams to design a viable business concept that addresses a locally-relevant challenge or problem related to Agenda 2063, and inclusive and sustainable development.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1343,22 +1387,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>anne@sabsa.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>Competitions | ESG</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
+          <t>https://za.rs-online.com/web/content/m/competition</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1366,22 +1414,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>example@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Astemi Sa</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Some of our sparkling achievements ... and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation ...</t>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1421,17 +1473,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1439,26 +1491,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>customerservices@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, support@informaconnect.com, support@knect365.com</t>
-        </is>
-      </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
+          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1468,24 +1516,24 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>info@techspocapetown.co.za</t>
+          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
+          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://africatechnologyexpo.com/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
+          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1495,24 +1543,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>enquiries@aiexpoafrica.com</t>
+          <t>info@sparkafrica.co, johndoe@email.com, partner@africatechnologyexpo.com</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Sep 15, 2026 · Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience.</t>
+          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1520,22 +1568,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>Home - Mediatech Africa | South Africa</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://www.mediatech.co.za/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1543,22 +1595,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>World-Class Consumer Tech Show - 4,200+ Global Exhibitors</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://www.bing.com/aclick?ld=e87ZKcOhwamYQPx18INGy8xTVUCUzJcJoZxfs4RMDA9DU2Gx6M5LohwCVWNPlHzX1Dnq_hnF_rtOlCJFqrTgA2ODifXtqHPHDVkGk4OCLVoEzqrw0wiSt1DgNishCMuFXS-Vdc57N8aByGib5sYNzHV-7RDUgSO2ukUIpNIduwazG7EK4B11HxIfSqzujeGi6yv7dy-uBVcouStvaTf3hdmESFhYI&amp;u=aHR0cHMlM2ElMmYlMmZ3d3cuZ2xvYmFsc291cmNlcy5jb20lMmZ0cmFkZVNob3dzJTJmSEslMmZzaG9ydHJlZ2lzdGVyJTNmc291cmNlJTNkODA0NDE2NyUyNnV0bV9zb3VyY2UlM2Q4MDQ0MTY3JTI2c2hvd191dG1fc291cmNlJTNkODA0NDE2NyUyNnV0bV9jYW1wYWlnbiUzZDUzMzY1MjczNCUyNnV0bV90ZXJtJTNkYXNpYSUyNTIwdHJhZGUlMjUyMHNob3dzJTI2YWRncm91cGlkJTNkMTM0OTEwMzQ5MzM2MDM1MyUyNnRhcmdldGlkJTNka3dkLTg0MzIwMjIzMTk5NTI3JTNhbG9jLTE5MCUyNm1hdGNodHlwZSUzZHAlMjZkZXZpY2UlM2RjJTI2Y291bnRyeSUzZDQ4NzkyJTI2bmV0d29yayUzZG8lMjZwbGFjZW1lbnQlM2QlMjZtc2Nsa2lkJTNkMjlhMWFiZjNhMjkzMWM3YmJkOGNjMTU0NTk1MmZlZGY&amp;rlid=29a1abf3a2931c7bbd8cc1545952fedf</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Attend Hong Kong's leading sourcing event for AI and consumer electronics. Pre-register today to meet verified suppliers at AsiaWorld-Expo, Hong Kong.</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1566,22 +1622,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>dataprivacy@knect365.com, customerservices@knect365.com, salesenquiries@africatechfestival.com, support@informaconnect.com, dataprivacy@informaconnect.com, customerservices@informaconnect.com, support@knect365.com</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology ...</t>
+          <t>HOME | Africa Tech Week</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
+          <t>https://africatechweek.co.za/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
+          <t>May 11, 2026 - From sensational speakers, to top tech exhibitons, see what’s in store when you attend the 2-day Sentech Africa Tech Week Conference in 2025&gt;&gt; ... Sponsor, Speak, Attend! For more information on how you can be a part of the #ATW family, contact ...</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1594,17 +1654,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
+          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
+          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
+          <t>Save this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaShare this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1612,26 +1672,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>u003einfo@techspo.co, atinfo@techspo.coor</t>
-        </is>
-      </c>
+      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
+          <t>FinancialContent - TECHSPO Cape Town 2026 Unites Business, Tech and Marketing Leaders for High-Impact Expo</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://africatechnologyexpo.com/</t>
+          <t>https://markets.financialcontent.com/stocks/article/abnewswire-2026-4-8-techspo-cape-town-2026-unites-business-tech-and-marketing-leaders-for-high-impact-expo</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
+          <t>April 8, 2026 - Cape Town, South Africa - TECHSPO Cape Town Technology Expo returns October 1-2, 2026, to the V&amp;A Waterfront Cape Town Avenue Conference Venue, uniting business leaders, technologists, marketers, and innovators for a high-impact, two-day showcase ...</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1639,26 +1695,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>partner@africatechnologyexpo.com, info@sparkafrica.co, johndoe@email.com</t>
-        </is>
-      </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Maker Faire - Wikipedia</t>
+          <t>Maker Faire Africa - Wikipedia</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Maker_Faire</t>
+          <t>https://en.wikipedia.org/wiki/Maker_Faire_Africa</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
+          <t>March 7, 2025 - Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds ...</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1671,17 +1723,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Maker Faire Africa - Wikipedia</t>
+          <t>Maker Faire - Wikipedia</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Maker_Faire_Africa</t>
+          <t>https://en.wikipedia.org/wiki/Maker_Faire</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>The aim of a Maker Faire Africa is to create a space on the African continent where Afrigadget-type innovations, inventions and initiatives can be sought, identified, brought to life, supported, amplified and propagated.</t>
+          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1694,17 +1746,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Maker Faire groups | Meetup</t>
+          <t>Maker Faire Africa — Grokipedia</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/topics/maker-faire/za/</t>
+          <t>https://grokipedia.com/page/maker_faire_africa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
+          <t>Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1717,17 +1769,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Maker Faire |</t>
+          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/</t>
+          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>Aug 21, 2015 · We’re delighted to present the first ever Cape Town Maker Faire, hosted by Open Design in partnership with Trimble.Maker Faire is primarily designed as a forward-looking event, showcasing makers who are exploring new forms and new technologies.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1735,26 +1787,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>pr@make.co, fancybox_sprite@2x.png, fancybox_loading@2x.gif, chosen-sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
+          <t>Maker Faire groups | Meetup</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
+          <t>https://www.meetup.com/topics/maker-faire/za/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Aug 21, 2015 · We’re delighted to present the first ever Cape Town Maker Faire, hosted by Open Design in partnership with Trimble.Maker Faire is primarily designed as a forward-looking event, showcasing makers who are exploring new forms and new technologies.</t>
+          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1767,17 +1815,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Maker Faire Africa — Grokipedia</t>
+          <t>Global Faires - Maker Faire</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://grokipedia.com/page/maker_faire_africa</t>
+          <t>https://makerfaire.com/globalfaires/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
+          <t>Global Maker Faires showcase the very best of Maker innovation and creativity on a grand scale in the world's most dynamic cities.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1785,22 +1833,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>pr@make.co, fancybox_loading@2x.gif, chosen-sprite@2x.png, fancybox_sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>About | Maker Faire Cape Town: Make • Create • Craft</t>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://makerfairecapetown.wordpress.com/about/</t>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Maker Faire is a community-based learning event that inspires everyone to become a maker and connect to people and projects in their local community.</t>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1813,17 +1865,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Maker Faire Africa (@MFAJoburg) - Facebook</t>
+          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/MFAJoburg/</t>
+          <t>https://makerfairecapetown.wordpress.com/about/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Maker Faire Africa. The Fem-In-Tech Development Programme is aimed at female-led South African start-ups in tech and tech- enabled sectors.</t>
+          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1836,17 +1888,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
+          <t>http://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will ...</t>
+          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1854,22 +1906,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>pr@make.co, fancybox_loading@2x.gif, chosen-sprite@2x.png, fancybox_sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Maker Faire Cape Town 2015 - PlanetJune Blog</t>
+          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.planetjune.com/blog/maker-faire-cape-town-2015/</t>
+          <t>https://contemporaryand.com/fr/events/maker-faire-africa-comes-to-johannesburg</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Aug 24, 2015 · Yesterday, I attended the first annual Maker Faire in Cape Town and it was inspiring – there was lots to see and explore.</t>
+          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1882,17 +1938,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>StemCo - StemCo 2026 International Competitions</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://stemco.org/</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
+          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1905,17 +1961,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>High School STEM Competition | Southafrica 2024</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1923,22 +1979,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
+          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
+          <t>February 27, 2026 - Samsung Electronics South Africa has opened applications for the 2026 edition of Solve for Tomorrow (SFT), its annual science, technology, engineering, and mathematics (STEM) competition aimed at Grade 10 and 11 learners.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1946,26 +2006,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Capetown 2026</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
+          <t>Local, regional and national competitions with thousands of · Multi-level events of two or more rounds that become increasingly challenging and culminate in top-level Olympiads. Enrichment programmes to inspire promising young South Africans to pursue STEMI</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -1973,26 +2029,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Astemi Sa</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>The ZASDC is South Africa's national Space Design Competition, part of a global network spanning six continents. Secondary school students design futuristic space settlements in a fast-paced industry simulation that builds real STEM, leadership ...</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2000,22 +2052,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>info@zasdc.org, user@domain.com</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>ASTEMI Competitions 2022 – SAASTA</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://saasta.ac.za/astemi-competitions-2</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2028,17 +2084,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
+          <t>2026 Season - Africa's Global STEM Celebration</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://www.stemfestival.org/competitions/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>April 30, 2026 - ... The Elementary, Junior, and Senior Robotics categories at STEM Festival are dedicated to advancing the World Robot Olympiad (WRO) across the Niger Delta and South-South Nigeria, working with ArcLights Foundation.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2051,17 +2107,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation ...</t>
+          <t>Rural youth lead in robotics at national STEM competition</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://iol.co.za/news/education/2025-09-15-rural-youth-lead-in-robotics-at-national-stem-competition/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
+          <t>September 15, 2025 - Discover how South Africa's brightest young minds are tackling real-world challenges with innovative solutions at the inaugural AlgoAtWork RoboRumble STEM Innovation Challenge, where ideas like autonomous robots and smart PPE systems are set ...</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2071,24 +2127,24 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>info@zasdc.org, user@domain.com</t>
+          <t>philippa.larkin@inl.co.za, londiwe.gumede@inl.co.za, lee.rondganger@inl.co.za, mendy.mtshali@inl.co.za, nobuntu.mgijima@volt.africa, ashley.lechman@inl.co.za</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>Competition – Eskom Expo for Young Scientists</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://exposcience.co.za/category/competition/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>Aqil Variava business cities Damien ... Gray STEMI Vuyo Nzimande · Eskom Expo for Young Scientists is an exposition, or science fair, where students have a chance to show others their projects about their own scientific investigations. At the annual prestigious Eskom Expo for Young Scientists International Science Fair (ISF), selected students from 35 Expo Regions in South Africa then compete ...</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2096,22 +2152,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>support@exposcience.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>National Department of Basic Education</t>
+          <t>STEAM Pitch Competition - STEM AFRICA FEST 2024</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://www.education.gov.za/LinkClick.aspx?fileticket=i9GS5Atf7zo=&amp;tabid=347&amp;portalid=0&amp;mid=14629</t>
+          <t>https://stemafricafest.com/steam-pitch-competition/</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>JOHANNESBURG, South Africa - XX Month 2026 - The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries ...</t>
+          <t>Join STEM Africa Fest , celebrating science, technology, engineering, and mathematics. Experience hands-on learning, industry leaders, and innovation across Africa.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2119,11 +2179,7 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>s.ngcobo@cheil.com, ssasft@samsung.com, j.mogoeng@samsung.com</t>
-        </is>
-      </c>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2148,7 +2204,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+          <t>460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2205,17 +2261,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
+          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2228,17 +2284,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>South African Robotics Competitions and Schools</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://www.sciencexpo.org.za/robotics.html</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2246,11 +2302,7 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>marna.vanzyl@imbewu.foundation, madelien@imbewu.foundation, webmaster@sciencexpo.org.za</t>
-        </is>
-      </c>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2282,17 +2334,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+          <t>South African Robotics Competitions and Schools</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://www.sciencexpo.org.za/robotics.html</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge national competition will be held in Johannesburg, South Africa, at the Sandton Convention Centre on the 31st October 2025.</t>
+          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2302,7 +2354,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, info@thecortexhub.africa, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io</t>
+          <t>webmaster@sciencexpo.org.za, marna.vanzyl@imbewu.foundation, madelien@imbewu.foundation</t>
         </is>
       </c>
     </row>
@@ -2332,17 +2384,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Robotics &amp; Coding Classes for Kids in Johannesburg | Robotics League</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://robotics-league.co.za/</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026 Theme · Robots Meet Culture. The World Robot Olympiad is the planet's biggest student robotics competition — over 100 countries, 100,000+ students a year. South African teams compete on two tracks: Explorer, the home-grown SA challenge, ...</t>
+          <t>The Robotics for Good Youth Challenge national competition will be held in Johannesburg, South Africa, at the Sandton Convention Centre on the 31st October 2025.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2352,24 +2404,24 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>info@roboticsleague.co.za, you@email.com</t>
+          <t>info@thecortexhub.africa, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
+          <t>Robotics &amp; Coding Classes for Kids in Johannesburg | Robotics League</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
+          <t>https://robotics-league.co.za/</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
+          <t>2026 Theme · Robots Meet Culture. The World Robot Olympiad is the planet's biggest student robotics competition — over 100 countries, 100,000+ students a year. South African teams compete on two tracks: Explorer, the home-grown SA challenge, ...</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2377,22 +2429,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>you@email.com, info@roboticsleague.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Bridge Building Competition (Dept of Civil Engineering)</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://civilabcut.co.za/services/bridge-building-competition-dept-of-civil-engineering/</t>
+          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Supported by SAICE (South African Institution of Civil Engineering), the competition continues to inspire the next generation of civil engineers to create, strengthen, and innovate for a sustainable future.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2402,24 +2458,24 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Civilab@CUTLogo-Transparent.png, etheron@cut.ac.za, cropped-Civilab@CUTLogo-Transparent.png</t>
+          <t>subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za, chanel@engineeringnews.co.za</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Non - profit SAICE launches Bridge Building Competition</t>
+          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd International Bridge Building Competition - SAICE</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://www.algoafm.co.za/event/non-profit-saice-launches-bridge-building-competition</t>
+          <t>https://saice.org.za/press-releases/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Organised by SAICE, a non-profit professional body for civil engineers in South Africa, the competition promotes teamwork, creativity, problem-solving, and an interest in engineering careers while showcasing the practical application of structural design and construction concepts.</t>
+          <t>April 17, 2025 - The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2427,22 +2483,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>membership@saice.org.za, communications@saice.org.za, civilinfo@saice.org.za, accounts@saice.org.za, marketing@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Engineering the future: 16 schools compete in SAICE's 33rd ...</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://www.southafricanbusiness.co.za/08/2024/construction-and-engineering/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
+          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2455,17 +2515,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SAICE's 34th International Bridge Competition Inspires Tomorrow's ...</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/lifestyle/education/saices-34th-international-bridge-competition-inspires-tomorrows-engineers/</t>
+          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2473,22 +2533,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>ernao@crown.co.za, constr@crown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://civils.org.za/</t>
+          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
+          <t>September 7, 2025 - Find the list of upcoming Civil Engineering conferences in South Africa 2025 with invitation an letter.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2501,17 +2565,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Civil Engineering Conferences in South Africa 2026/2027/2028</t>
+          <t>SWM Communications | SAICE recognises civil engineering research excellence through national student competition</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
+          <t>https://swmcommunications.co.za/press-office/saice-recognises-civil-engineering-research-excellence-through-national-student-competition/</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Civil Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
+          <t>April 1, 2026 - The event – which was sponsored by Sika, WorldsView, BVI, RIBCCS, and AF Consulting – was hosted at SAICE House in Midrand, Gauteng, and accredited for 0.2 CPD points. Students were invited to present their civil engineering university research and investigation project, which is part of the national curriculum for final year civil engineering undergraduate students.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2519,22 +2583,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>nthabeleng@saice.org.za, info@swmcommunications.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>VUT inspires future engineers through Bridge Building Competition</t>
+          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://vut.ac.za/vut-inspires-future-engineers-through-bridge-building-competition/</t>
+          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Supported by the ArcelorMittal Science Centre, Institution of Structural Engineers (IStructE), Fundi, South African Institution of Civil Engineering Future Leaders Panel (SAICE FLP) Vaal and maVuti Shop, the initiative challenged learners to design and construct bridge models using simple materials, including sticks, wool and glue.</t>
+          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2547,17 +2615,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Engineering the future: 16 schools compete in bridge building ...</t>
+          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://www.engineerit.co.za/article/engineering-the-future-16-schools-compete-in-bridge-building-competition</t>
+          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>The recent South African Institution of Civil Engineering (SAICE) 33 rd International Bridge Building competition at the Midrand Conference Centre showcased 16 high schools around South Africa and one in Swaziland encouraging learners to apply their knowledge of mathematics and science in practical engineering projects. Each team received 25 sticks, string and glue to construct a bridge ...</t>
+          <t>Civil engineering conferences in Cape town 2025 provide an exclusive global platform to meet and engage with experts and aspirants in various fields.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2570,17 +2638,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Building the future: SAICE International Bridge Building Competition ...</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://journals.co.za/doi/full/10.10520/ejc-civeng_v32_n9_a22</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>SAICE hosted its 32nd International Bridge Building Competition at the Midrand Conference Centre on 23 August 2024, bringing together 16 schools from around South Africa and Swaziland to compete for the prestigious bridge building trophy.</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2593,17 +2661,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
+          <t>Civil Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
+          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
+          <t>Apr 13 International Conference on Architectural, Civil and Environmental Engineering (ICACEE) - Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2616,17 +2684,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Category:Mechanical engineering competitions - Wikipedia</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Category:Mechanical_engineering_competitions</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Engineering competitions · Mechanical engineering · Search · Category:Mechanical engineering competitions ·</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2639,17 +2707,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Mechanical Engineering Conferences in South Africa 2026/2027/2028 - Conference Index</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/mechanical-engineering/south-africa</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Nov 04 International Conference on Tribology and Interface Engineering (ICTIE) - Cape Town, South Africa · Nov 04 International Conference on Mechanical and Systems Engineering (ICMSE) - Cape Town, South Africa</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2662,17 +2730,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>&gt;&gt; Industrial and Manufacturing Engineering · &gt;&gt; Mechanical Engineering · &gt;&gt; Ocean Engineering · Environmental Science · Mathematics · Medicine · &gt;&gt; Anatomy · &gt;&gt; Anesthesiology and Pain Medicine · &gt;&gt; Cardiology and Cardiovascular Medicine · &gt;&gt; Critical Care and Intensive Care Medicine ·</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2685,17 +2753,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Mechanical Engineering events - South Africa Group - Institution of Mechanical Engineers</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://nearyou.imeche.org/near-you/middle-east-and-africa/south-africa/events</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>For details of Mechanical Engineering events organised by South Africa Group, please click the above link.</t>
+          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2703,22 +2771,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Best Mechanical Engineering Companies in South Africa</t>
+          <t>Hatch: Mechanical Engineering Bursary Programme 2026</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://engineeringness.com/best-mechanical-engineering-companies-in-south-africa/</t>
+          <t>https://jobs.pricesinsouthafrica.co.za/job/hatch-mechanical-engineering-bursary-programme-2026/</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>October 4, 2025 - This article showcases our top picks for the best South Africa based Mechanical Engineering companies. These startups and companies are taking a variety of approaches to innovating the Mechanical Engineering industry, but are all exceptional companies well worth a follow.</t>
+          <t>Hatch invites graduates to apply for Mechanical Engineering Bursary Programme 2026 in Johannesburg, Gauteng, South Africa. Hatch is seeking highly</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2731,17 +2803,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Past Mechanical Engineering events - South Africa Group - Institution of Mechanical Engineers</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://nearyou.imeche.org/near-you/middle-east-and-africa/south-africa/past-events</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>For details of past Mechanical Engineering events organised by South Africa Group, please click the above link.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2749,22 +2821,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>10 Mechanical Engineering Competitions for High School Students — Veritas AI</t>
+          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://www.veritasai.com/veritasaiblog/10-mechanical-engineering-competitions-for-high-school-students</t>
+          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>October 29, 2025 - ... Competition Dates: The contest year began on April 14 and ends on May 31. Students can submit (unique) entries for each monthly contest. Eligibility: The contest is open to all students, regardless of their age or discipline.</t>
+          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2772,26 +2848,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>contact@veritasai.com, user@domain.com</t>
-        </is>
-      </c>
+      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>7 Mechanical Engineering Degree Programs in South Africa - Study Abroad | educations.com</t>
+          <t>SAIMechE</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://www.educations.com/mechanical-engineering/south-africa</t>
+          <t>https://www.saimeche.org.za/</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>One of the main objectives of this process is to develop an advanced capability to do fundamental engineering research independently. It also promotes a lifelong learning approach. ... The Master of Mechanical Engineering (MS) program objective is to provide students with the skill sets and knowledge necessary to become a professional who can solve practical issues of the field of mechanical engineering.</t>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2804,17 +2876,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Mechanical Engineering in South Africa: 2025 Master's Guide | Mastersportal</t>
+          <t>merSETA Learnerships 2026: Latest Technical Training Opportunities for ...</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://www.mastersportal.com/study-options/271564839/mechanical-engineering-south-africa.html</t>
+          <t>https://www.myseta.co.za/merseta-learnership-programmes-2026/</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>The Mechanical Engineering program at the University of Pretoria is a leading source of graduates in the... ... Applied Science Metallurgy from University of Pretoria aims to be internationally competitive while... ... Holders of any other equivalent South African or international qualification may also be considered for...</t>
+          <t>Discover merSETA Learnership Programmes 2026, including apprenticeships, internships, skills programmes, eligibility, stipends, application tips and technical career opportunities in South Africa.</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2822,22 +2894,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>info@myseta.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Engineering Competitions - ASME</t>
+          <t>Apprenticeships 2025 / 2026 - StudentRoom.co.za</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://www.asme.org/conferences-events/competitions</t>
+          <t>https://www.studentroom.co.za/category/apprenticeships/</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>There are four kinds of challenges &amp; competitions held during the three-day, two-night regional events built around design, advanced manufacturing &amp; robotics technologies. HPVC, IAM3D, the student design competition &amp; the old guard competition.</t>
+          <t>Sappi offers apprenticeship and technical development opportunities for young people interested in building careers in engineering and artisan trades at its South African operations.</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2845,22 +2921,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>studentroom-logo@2x.webp</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Student Chapter Design Contest (Africa) Serving the electrical energy conversion professional worldwide. Chapter Design Contest (Africa) Deadline: April 30, ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2868,22 +2948,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>WorldSkills South Africa 2027 Applications - Edupstairs</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.edupstairs.org/worldskills-south-africa-2027-applications/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2 days ago · WorldSkills is about identifying exceptional practical and technical talent in fields ranging from welding, electrical installations and ...</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2891,26 +2975,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>sifisomhlongo@edupstairs.org</t>
-        </is>
-      </c>
+      <c r="E103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>CMU-Africa students shine at global electronics conference</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.africa.engineering.cmu.edu/news/2026/01/16-ieee-conference.html</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Jan 16, 2026 · SPEC 2025, held in Johannesburg, South Africa, is part of the Power Electronics Society, in the field of electrical engineering.</t>
+          <t>Centres South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2920,24 +3000,24 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>africa-info@andrew.cmu.edu</t>
+          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Electricity challenges a top issue at African engineering ...</t>
+          <t>ACTOM Engineering Projects and Contracts Bursaries 2027</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://standardmicrogrid.com/content/electricity-challenges-top-issue-african-engineering-innovation-competition</t>
+          <t>https://www.studentroom.co.za/actom-engineering-projects-and-contracts-bursaries-2027/</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Electricity challenges a top issue at African engineering innovation competition. Engineering innovations to boost off-grid power and stop electricity theft ... Missing: electrical | Show results with: electrical</t>
+          <t>ACTOM Engineering Projects and Contracts invites South African students to apply for the 2027 Electrical Engineering Bursary Opportunity. Applications close on 31 July 2026.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2945,22 +3025,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>epc.hc@actom.co.za, studentroom-logo@2x.webp</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Take a look back at day 1 of the #WorldSkillsZA competition ...</t>
+          <t>Competitions | ESG</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/GovernmentZA/videos/️-take-a-look-back-at-day-1-of-the-worldskillsza-competition-where-competitors-b/1633847574552335/</t>
+          <t>https://za.rs-online.com/web/content/m/competition</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Mar 10, 2026 · South African electrical engineer wins gold medal. Njabulo Mabaso ... The WorldSkills South Africa National Competition Closing Ceremony marked ...</t>
+          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -2968,22 +3052,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>example@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>Opportunities in Electrical Engineering across South Africa.</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://www.puffandpass.co.za/tag/electrical-engineering</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>Location: Johannesburg Hatch is seeking Electrical / Civil / Mechanical Engineering Graduates who will support projects globally. The engineering team is comprised of professional engineers, designers and technologists. We have experience…</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -2996,17 +3084,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>IEEE-IAS Industrial Power Conversion Systems Department Serving the electrical energy conversion professional worldwide</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3019,17 +3107,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>Eskom Bursary Programme South Africa 2026 - EduFunds SA</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://www.edufunds.co.za/eskom-bursary-programme-south-africa-2026/</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Centres South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits</t>
+          <t>Apply for the Eskom Bursary Programme South Africa 2026. Funding for BEng/BSc engineering students in Chemical, Civil, Electrical, Mechanical, Industrial, and Metallurgy disciplines. Apply by 14 November 2025.</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3039,24 +3127,24 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
+          <t>candidate.support@ci.hr, Admin@edufunds.co.za</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>Zutari Bursary Programme 2027 Opens Applications for Civil and ...</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://www.globalsouthopportunities.com/2026/08/10/zutari/</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>Zutari has opened applications for its 2027 Engineering Bursary Programme, offering financial and professional development support to South African students pursuing studies in Civil Engineering and Electrical Engineering. The engineering consulting company plans to award 10 bursaries for the 2027 academic year. The programme is aimed at young engineering talent, including matriculants and ...</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3069,17 +3157,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Eskom Bursary Programme 2027 | Apply by 22 September</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://bursaries-southafrica.co.za/eskom-bursary-programme-2027/</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>At a glance Sponsor: Eskom Academic year: 2027 Applicants: Eligible South African school-leavers and current tertiary students Institutions: Recognised public universities and universities of technology, depending on the route Application method: Online through Eskom Careers About the programme Eskom's bursary intake supports students developing skills relevant to the electricity and energy ...</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3087,16 +3175,12 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>The Home of South African Hackathons</t>
+          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3119,17 +3203,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Hackathons in South Africa: Seasonality, Cities &amp; Platforms</t>
+          <t>Hackathons en South Africa</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>https://www.hackathonradar.com/discover/country/south-africa</t>
+          <t>https://za.allhackathons.com/</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>When and where hackathons happen in South Africa, from 9 tracked events. Peak season is Jun (2 events), quietest is Mar (1). Midrand leads by volume.</t>
+          <t>Aug 22, 2025 · Join us for an electrifying hackathon where innovation meets security and finance! This event brings together developers, data scientists, cybersecurity experts, and FinTech enthusiasts to …</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3142,17 +3226,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Hackathons en South Africa</t>
+          <t>Unisa hosts first-ever Hackathon to ignite student learning ...</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/</t>
+          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+          <t>Jul 14, 2025 · The event supported key priorities of South Africa’s National Development Plan, Unisa’s Catalytic Niche Areas and the United Nations’ Sustainable Development Goals that relate to access to quality education, decent work and innovation.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3165,17 +3249,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>AfriHack 2026: Pan-African Hackathon for Technology Students in ...</t>
+          <t>Build the Future with Entelect Hackathons</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://youthopportunitieshub.com/afrihack-2026/</t>
+          <t>https://challenge.entelect.co.za/</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>The annual hackathon, organised by Empiras Global, is returning in 2026 for its third edition. The programme is designed to bring together technology students from South Africa, other African countries and international universities to work on authentic business challenges.</t>
+          <t>Instead of focusing on building a once-off project, our hackathons centre around optimisation problems. Participants develop solutions that are tested, scored, and ranked based on performance, efficiency, and strategy.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3188,7 +3272,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>The Home of South African Hackathons</t>
+          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3198,7 +3282,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
+          <t>Imagine a high-energy event where innovation and creativity collide - that’s a hackathon. Picture a whirlwind of coding, problem-solving, and brainstorming, all packed into an intense, short period.</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3211,17 +3295,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Hackathons in South Africa</t>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/hackathons/</t>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Hackathons in South Africa Verken alle hackathons in South Africa PERSOONLIK GIRLCODE GHANA HACKATHON 2025 Aug. 22, 2025 - Sept. 14, 2025 Eindig</t>
+          <t>Sep 2, 2026 · The Young Engineers Movement (YEM) is an immersive engineering and technology hackathon designed to equip young South Africans with the skills, mindset and confidence needed to solve real-world challenges.</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3229,22 +3313,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Houghton hackathon: Stepping stone for future engineers</t>
+          <t>Talks &amp; Fireside | Builders Table</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>https://www.citizen.co.za/rosebank-killarney-gazette/news-headlines/local-news/2026/06/23/houghton-hackathon-stepping-stone-for-future-engineers/</t>
+          <t>https://builderstable.net/</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>55 learners from underserved communities are developing creative solutions to everyday challenges while navigating future careers in engineering and technology at a five-day hackathon in Houghton ...</t>
+          <t>Builders Table is a two-day hackathon hosted by MakeReign, built around a 24-hour build sprint. It brings together South Africa's designers, developers, strategists, founders and creative technologists to build real working prototypes under real time pressure.</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3252,82 +3340,9 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>Young Engineers Movement (YEM) - ORT SA</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>CompeteHub - Where Champions Are Made</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>https://www.devpluxe.co.za/</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr"/>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>AfriHack 2026 | Empiras Global</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>https://www.empirasglobal.com/afrihack26</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>AfriHack is an annual initiative aimed at uplifting young local, continental, and global tech students. In 2026, Empiras is thrilled to present the third edition of AfriHack. The hackathon series is designed to engage technology students from all regions of South Africa in addressing authentic business challenges, while simultaneously fostering collaboration and innovation among participants ...</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 1eeb89147c984dc6bc3ffafd9e6cd089@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 54b4aac306184111a223c0f4aea635c3@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 98b21aa53d68482b8414e892d9af0e5f@sentry-next.wixpress.com, e40146ef843e4f9196e5d00c98ac3689@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, cd64ba1f47df485bba2b0076c0dd3b25@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, info@empirasglobal.com, a18507e8883842d8a1ba47257fee81ac@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>liamlr95@gmail.com, sarah.chen@horizonlabs.com</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update competition data 2026-09-16
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E118"/>
+  <dimension ref="A1:E121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>August 6, 2026 - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -492,17 +492,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -512,24 +512,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>info@zasdc.org, user@domain.com</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -537,26 +537,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -569,17 +565,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Competitions – Enactus South Africa | National Expos ...</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://enactusza.org/what-we-do/competitions</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -589,24 +585,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>xmadlanga@enactus.org, liso@enactus.org, marketingsa@enactus.org, adminsa@enactus.org</t>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
+          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://www.thecasecentre.org/products/view?id=189255</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>August 6, 2026 - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -619,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -642,17 +638,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
+          <t>Engineering design competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -660,26 +656,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>info@zasdc.org, user@domain.com</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
+          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>August 14, 2026 - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -687,26 +679,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
+          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://10times.com/southafrica/tradeshows</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
+          <t>South Africa trade shows, find and compare 974 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 166 upcoming expos in 2026-2027 1. Mining Connect Day, 2. Annual ACFE Africa Conference &amp; Exhibition, 3. Annual Smart Procurement World Indaba, 4. ECM ...</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -714,26 +702,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>enquiries@aiexpoafrica.com</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/tradeshows</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>South Africa trade shows, find and compare 974 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 166 upcoming expos in 2026-2027 1. Mining Connect Day, 2. Annual ACFE Africa Conference &amp; Exhibition, 3. Annual Smart Procurement World Indaba, 4. ECM ...</t>
+          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -741,22 +725,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>enquiries@aiexpoafrica.com</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>Top Expos In South Africa | Booth Exhibits™</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://boothexhibits.co.za/blog/venues-and-shows/south-africas-top-trade-shows-and-conferences/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>Explore South Africa's top expos and conferences, from Africa Tech Festival to Mining Indaba and Automechanika. Choose the right event to stand out!</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -766,24 +754,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>dataprivacy@knect365.com, customerservices@knect365.com, salesenquiries@africatechfestival.com, support@informaconnect.com, dataprivacy@informaconnect.com, customerservices@informaconnect.com, support@knect365.com</t>
+          <t>hello@boothexhibits.co.za</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
+          <t>Big Data and Business Analytics Innovation Conference Johannesburg, South Africa IT &amp; Technology 101 Members Tue, 22 - Thu, 24 Sep 2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -816,24 +804,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, Erika@innovate.durban, 8c4075d5481d476e945486754f783364@sentry.io, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, sithabile@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
+          <t>Erika@innovate.durban, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, sithabile@innovate.durban, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
+          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://expotobi.com/country/south-africa/exhibitions</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
+          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -846,17 +834,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Big Data and Business Analytics Innovation Conference Johannesburg, South Africa IT &amp; Technology 101 Members Tue, 22 - Thu, 24 Sep 2026</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -864,22 +852,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>dataprivacy@informaconnect.com, dataprivacy@knect365.com, customerservices@knect365.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, support@informaconnect.com, support@knect365.com</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
+          <t>South Africa Professional Exhibitions, Shows, Fairs</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://expotobi.com/country/south-africa/exhibitions</t>
+          <t>https://www.showsbee.com/shows-0-1-South_Africa-all_city-All_Shows.html</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
+          <t>South Africa ... First Previous , Go to page Select Shows by Industry or Country Industry Press Molecor SEA will showcase sustainable PVC-O innovations at ASIAWATER 2026 3/31/2026 Alfa Laval introduces ThinkCircularity: Closing the loop on plastic waste 2/26/2026 Vanzetti Engineering strengthens its presence in the Asian marine market 12/6/2025</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -892,17 +884,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>South Africa - IoT Africa Exhibition and Conference</t>
+          <t>Exhibitions in South Africa</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://iot-africa.com/south-africa/</t>
+          <t>https://expoonline.co.za/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>IoT Africa Exhibition and Conference in Johannesburg, South Africa brings together leaders across IoT, data centres, cloud, telecom, AI, cybersecurity, and digital infrastructure. Connect with enterprises, government, and tech innovators shaping Africa's smart, connected future.</t>
+          <t>Online Exhibition South Africa We offer a Virtual Exhibition platform for specialized trade shows and exhibitions South Africa. Browse the exhibition by Expo Categories and connect with our Exhibitors. Discover new products and suppliers for your needs and industry at our online exhibitions South Africa.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -912,24 +904,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>info@iot-africa.com</t>
+          <t>info@expoonline.co.za</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Come and explore our exhibition of innovative discoveries at Science ...</t>
+          <t>CPD Events | innovateX</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
+          <t>https://www.innovatex.biz/event-list</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>The final countdown is underway, and all roads lead to this year's Science Forum South Africa 2024 at the CSIR International Convention Centre in Pretoria. Join us as we plan to celebrate the CSIR's impactful science, technology and innovation contributions at South Africa's premier scientific pl...</t>
+          <t>The most prestigious category 1 CPD event and exhibition in South Africa, InnovateX is coming to KZN. Make sure to register today to secure your spot and valuable 1 CPD Point.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -937,7 +929,11 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -985,7 +981,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
         </is>
       </c>
     </row>
@@ -1069,17 +1065,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>Engineers Without Borders South ...</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
+          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1092,17 +1088,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South ...</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
+          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1115,17 +1111,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>Engineers Without Borders launches student challenge</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://www.theconstructionindex.co.uk/news/view/engineers-without-borders-launches-student-challenge</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
+          <t>September 7, 2021 - The Engineering for People Design Challenge encourages undergraduates to broaden their awareness of the social, environmental and economic implications of their engineering solutions.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1133,22 +1129,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>news@theconstructionindex.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Engineers Without Borders launches student challenge</t>
+          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.theconstructionindex.co.uk/news/view/engineers-without-borders-launches-student-challenge</t>
+          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>September 7, 2021 - The Engineering for People Design Challenge encourages undergraduates to broaden their awareness of the social, environmental and economic implications of their engineering solutions.</t>
+          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1156,26 +1156,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>news@theconstructionindex.co.uk</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
+          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
+          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
+          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1183,26 +1179,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>privacy@studocu.com</t>
-        </is>
-      </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
+          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1210,26 +1202,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1237,26 +1225,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1269,17 +1253,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1292,17 +1276,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>National Student Competition | ORSSA</t>
+          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://www.orssa.org.za/studentcomp</t>
+          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
+          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1310,26 +1294,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, email@example.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Competitions - Enactus South Africa | National Expos, Challenges ...</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://enactusza.org/what-we-do/competitions</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1337,26 +1317,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>xmadlanga@enactus.org, liso@enactus.org, marketingsa@enactus.org, adminsa@enactus.org</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>Engineering in South Africa: 24 Best universities Ranked</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://edurank.org/engineering/za/</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1369,17 +1345,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Competitions - SABSA</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://sabsa.co.za/competitions/</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>African Business Concept Challenge ABCC is a virtual simulation-based business concept competition for African undergraduate and graduate students. The competition will challenge student teams to design a viable business concept that addresses a locally-relevant challenge or problem related to Agenda 2063, and inclusive and sustainable development.</t>
+          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1387,26 +1363,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>anne@sabsa.co.za</t>
-        </is>
-      </c>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Competitions | ESG</t>
+          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://za.rs-online.com/web/content/m/competition</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
+          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1414,26 +1386,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>example@email.com</t>
-        </is>
-      </c>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Astemi Sa</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1516,7 +1484,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
+          <t>u003einfo@techspo.co, atinfo@techspo.coor</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1511,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>info@sparkafrica.co, johndoe@email.com, partner@africatechnologyexpo.com</t>
+          <t>johndoe@email.com, info@sparkafrica.co, partner@africatechnologyexpo.com</t>
         </is>
       </c>
     </row>
@@ -1577,17 +1545,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Home - Mediatech Africa | South Africa</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://www.mediatech.co.za/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1597,24 +1565,24 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
+          <t>dataprivacy@informaconnect.com, dataprivacy@knect365.com, customerservices@knect365.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, support@informaconnect.com, support@knect365.com</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>Home - Mediatech Africa | South Africa</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://www.mediatech.co.za/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1624,7 +1592,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>dataprivacy@knect365.com, customerservices@knect365.com, salesenquiries@africatechfestival.com, support@informaconnect.com, dataprivacy@informaconnect.com, customerservices@informaconnect.com, support@knect365.com</t>
+          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
         </is>
       </c>
     </row>
@@ -1677,17 +1645,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>FinancialContent - TECHSPO Cape Town 2026 Unites Business, Tech and Marketing Leaders for High-Impact Expo</t>
+          <t>IT &amp; Technology Events in Johannesburg, List of all Johannesburg Technology Business Expo &amp; Events in South Africa</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://markets.financialcontent.com/stocks/article/abnewswire-2026-4-8-techspo-cape-town-2026-unites-business-tech-and-marketing-leaders-for-high-impact-expo</t>
+          <t>https://10times.com/johannesburg-za/technology</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>April 8, 2026 - Cape Town, South Africa - TECHSPO Cape Town Technology Expo returns October 1-2, 2026, to the V&amp;A Waterfront Cape Town Avenue Conference Venue, uniting business leaders, technologists, marketers, and innovators for a high-impact, two-day showcase ...</t>
+          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1733,7 +1701,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
+          <t>3 days ago - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1746,17 +1714,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Maker Faire Africa — Grokipedia</t>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://grokipedia.com/page/maker_faire_africa</t>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1769,17 +1737,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
+          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
+          <t>https://makerfairecapetown.wordpress.com/about/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Aug 21, 2015 · We’re delighted to present the first ever Cape Town Maker Faire, hosted by Open Design in partnership with Trimble.Maker Faire is primarily designed as a forward-looking event, showcasing makers who are exploring new forms and new technologies.</t>
+          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1792,17 +1760,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire groups | Meetup</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/topics/maker-faire/za/</t>
+          <t>http://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
+          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1810,22 +1778,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>pr@make.co</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Global Faires - Maker Faire</t>
+          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/globalfaires/</t>
+          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Global Maker Faires showcase the very best of Maker innovation and creativity on a grand scale in the world's most dynamic cities.</t>
+          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1833,26 +1805,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>pr@make.co, fancybox_loading@2x.gif, chosen-sprite@2x.png, fancybox_sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>The Makers Hub</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>https://www.decorex.co.za/cape-town/en-gb/visit/TheMakersHub.html</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>Explore unique handmade items, take part in interactive workshops, and engage directly with Cape Town’s vibrant maker community.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1860,22 +1828,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>decorexafrica@rxglobal.com</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
+          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://makerfairecapetown.wordpress.com/about/</t>
+          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
+          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1888,17 +1860,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>Why Africa needs Maker Faire | ZDNET</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>http://capetown.makerfaire.com/</t>
+          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage to attend and show off their work.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1906,26 +1878,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>pr@make.co, fancybox_loading@2x.gif, chosen-sprite@2x.png, fancybox_sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
+          <t>HOME | MAKERS FEST</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://contemporaryand.com/fr/events/maker-faire-africa-comes-to-johannesburg</t>
+          <t>https://www.makersfestival.co.za/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
+          <t>At Makers Festival SA, you get full access to every hands-on workshop, from woodworking and ceramics to leatherwork, painting, and more.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1933,7 +1901,11 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, warren@makersfestival.co.za, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, example@mysite.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2061,17 +2033,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions 2022 – SAASTA</t>
+          <t>A first for Africa: Cape Town to host World Robot Olympiad International Final in 2028</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://saasta.ac.za/astemi-competitions-2</t>
+          <t>https://www.bizcommunity.com/article/a-first-for-africa-cape-town-to-host-world-robot-olympiad-final-in-2028-964084a</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>4 hours ago - "Bringing the International Final ... continent to discover robotics and Stem.” · Further details about the WRO International Final 2028, including confirmed competition ......</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2107,17 +2079,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Rural youth lead in robotics at national STEM competition</t>
+          <t>SA young scientists selected for global competition at Regeneron ISEF in the USA - Eskom</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://iol.co.za/news/education/2025-09-15-rural-youth-lead-in-robotics-at-national-stem-competition/</t>
+          <t>https://www.eskom.co.za/sa-young-scientists-selected-for-global-competition-at-regeneron-isef-in-the-usa/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>September 15, 2025 - Discover how South Africa's brightest young minds are tackling real-world challenges with innovative solutions at the inaugural AlgoAtWork RoboRumble STEM Innovation Challenge, where ideas like autonomous robots and smart PPE systems are set ...</t>
+          <t>May 6, 2025 - Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) competition, will take place from 10 to 16 May in Columbus, Ohio in the USA.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2127,24 +2099,24 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>philippa.larkin@inl.co.za, londiwe.gumede@inl.co.za, lee.rondganger@inl.co.za, mendy.mtshali@inl.co.za, nobuntu.mgijima@volt.africa, ashley.lechman@inl.co.za</t>
+          <t>MediaDesk@eskom.co.za</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Competition – Eskom Expo for Young Scientists</t>
+          <t>ASTEMI Competitions 2022 – SAASTA</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://exposcience.co.za/category/competition/</t>
+          <t>https://saasta.ac.za/astemi-competitions-2</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Aqil Variava business cities Damien ... Gray STEMI Vuyo Nzimande · Eskom Expo for Young Scientists is an exposition, or science fair, where students have a chance to show others their projects about their own scientific investigations. At the annual prestigious Eskom Expo for Young Scientists International Science Fair (ISF), selected students from 35 Expo Regions in South Africa then compete ...</t>
+          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2152,11 +2124,7 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>support@exposcience.co.za</t>
-        </is>
-      </c>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2202,11 +2170,7 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2261,17 +2225,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2284,17 +2248,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>A first for Africa: Cape Town to host World Robot Olympiad International Final in 2028</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://www.bizcommunity.com/article/a-first-for-africa-cape-town-to-host-world-robot-olympiad-final-in-2028-964084a</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
+          <t>4 hours ago - South Africa has been selected to host the 2028 World Robot Olympiad (WRO) International Final. The event, showing on the African continent for the first time, will take place at the Cape Town International Convention Centre (CTICC) during the ...</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2307,17 +2271,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
+          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
+          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
+          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2325,11 +2289,7 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>NkosiN@atnews.co.za, rampedim@atnews.co.za</t>
-        </is>
-      </c>
+      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2354,24 +2314,24 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>webmaster@sciencexpo.org.za, marna.vanzyl@imbewu.foundation, madelien@imbewu.foundation</t>
+          <t>madelien@imbewu.foundation, marna.vanzyl@imbewu.foundation, webmaster@sciencexpo.org.za</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
+          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
+          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
+          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2379,22 +2339,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>rampedim@atnews.co.za, NkosiN@atnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+          <t>Robotics &amp; Coding Classes for Kids in Johannesburg | Robotics League</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://robotics-league.co.za/</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge national competition will be held in Johannesburg, South Africa, at the Sandton Convention Centre on the 31st October 2025.</t>
+          <t>2026 Theme · Robots Meet Culture. The World Robot Olympiad is the planet's biggest student robotics competition — over 100 countries, 100,000+ students a year. South African teams compete on two tracks: Explorer, the home-grown SA challenge, ...</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2404,24 +2368,24 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>info@thecortexhub.africa, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io</t>
+          <t>you@email.com, info@roboticsleague.co.za</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Robotics &amp; Coding Classes for Kids in Johannesburg | Robotics League</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://robotics-league.co.za/</t>
+          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026 Theme · Robots Meet Culture. The World Robot Olympiad is the planet's biggest student robotics competition — over 100 countries, 100,000+ students a year. South African teams compete on two tracks: Explorer, the home-grown SA challenge, ...</t>
+          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2429,26 +2393,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>you@email.com, info@roboticsleague.co.za</t>
-        </is>
-      </c>
+      <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>Civil Engineering Conferences in South Africa 2026/2027/2028</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
+          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
+          <t>Civil Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2456,26 +2416,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za, chanel@engineeringnews.co.za</t>
-        </is>
-      </c>
+      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd International Bridge Building Competition - SAICE</t>
+          <t>SWM Communications | SAICE recognises civil engineering research ...</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://saice.org.za/press-releases/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://swmcommunications.co.za/press-office/saice-recognises-civil-engineering-research-excellence-through-national-student-competition/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>April 17, 2025 - The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) is a learned society and voluntary organisation that acts as a catalyst for innovation and good practice in the development of the civil engineering profession.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2485,24 +2441,24 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>membership@saice.org.za, communications@saice.org.za, civilinfo@saice.org.za, accounts@saice.org.za, marketing@saice.org.za</t>
+          <t>nthabeleng@saice.org.za, info@swmcommunications.co.za</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
+          <t>The South African Institution of Civil Engineering (SAICE)</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
+          <t>https://www.facebook.com/SAICECIVIL/posts/the-excitement-is-building-at-the-2026-saice-international-bridge-building-compe/1515152847321706/</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
+          <t>The excitement is building at the 2026 SAICE International Bridge Building Competition! The 19 finalist teams attended an official briefing with Oliver Rowe from @ECSA, where they received important information as they prepared to put their engineering knowledge, creativity, teamwork and problem-solving skills to the test.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2515,17 +2471,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>Civil Engineering Conferences In South Africa 2026-2027</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
+          <t>https://conferencenext.com/conferences/south-africa/civil-engineering</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
+          <t>Civil Engineering conference in South Africa 2026-2027 is a great opportunity to learn from the opinions of global experts and the country's growth model. These events gather members of the Civil Engineering community to share research and expertise in this field through various programs, including presentations, keynote lectures, seminars ...</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2535,24 +2491,24 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>ernao@crown.co.za, constr@crown.co.za</t>
+          <t>michaeljjacobson1@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
+          <t>Civil Engineering | Bursaries South Africa</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
+          <t>https://www.zabursaries.co.za/?s=Civil+Engineering</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>September 7, 2025 - Find the list of upcoming Civil Engineering conferences in South Africa 2025 with invitation an letter.</t>
+          <t>Bursaries are awarded each semester, for Civil Engineering studies (Degree… Read More » ENGINEERING Engineering Bursaries South Africa 2027 The Engineering sector has many sub-sectors, each of them vitally important to the functioning of various systems and industries (such as factories, motor vehicles, pharmaceuticals etc).</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2565,17 +2521,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SWM Communications | SAICE recognises civil engineering research excellence through national student competition</t>
+          <t>ICE Africa - Supporting Civil Engineers in Africa</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://swmcommunications.co.za/press-office/saice-recognises-civil-engineering-research-excellence-through-national-student-competition/</t>
+          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>April 1, 2026 - The event – which was sponsored by Sika, WorldsView, BVI, RIBCCS, and AF Consulting – was hosted at SAICE House in Midrand, Gauteng, and accredited for 0.2 CPD points. Students were invited to present their civil engineering university research and investigation project, which is part of the national curriculum for final year civil engineering undergraduate students.</t>
+          <t>ICE Africa supports civil engineers across the continent, providing access to qualifications, training, and networking opportunities for professional growth.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2583,26 +2539,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>nthabeleng@saice.org.za, info@swmcommunications.co.za</t>
-        </is>
-      </c>
+      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
+          <t>Civil Engineering Bursary - Bursaries Open Now in South Africa</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
+          <t>https://bursariesopennow.co.za/category/civil-engineering-bursary/</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
+          <t>Find Civil Engineering Bursary in South Africa. Updated bursaries with requirements, closing dates and how to apply.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2615,17 +2567,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
+          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
+          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Civil engineering conferences in Cape town 2025 provide an exclusive global platform to meet and engage with experts and aspirants in various fields.</t>
+          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2638,17 +2590,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>SAICE | Events and Awards</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
+          <t>https://members.saice.org.za/events-and-awards</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>The South African Institution Of Civil Engineering SAICE hosts the Awards Function annually to honour individuals, projects of excellence, as well as community-oriented initiatives. The annual awards function gives companies and individuals a unique opportunity to showcase their deserving projects and work to the industry.</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2661,17 +2613,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Civil Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
+          <t>Awards 2025 - SAICE</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
+          <t>https://saice.org.za/awards-2025/</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Apr 13 International Conference on Architectural, Civil and Environmental Engineering (ICACEE) - Cape Town, South Africa</t>
+          <t>Learn about SAICE's award categories, submission guidelines, key dates and how to nominate project and professionals.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2679,7 +2631,11 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>accounts@saice.org.za, marketing@saice.org.za, communications@saice.org.za, membership@saice.org.za, civilinfo@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2707,17 +2663,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2725,22 +2681,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2753,17 +2713,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
+          <t>The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent's largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2771,26 +2731,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Hatch: Mechanical Engineering Bursary Programme 2026</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://jobs.pricesinsouthafrica.co.za/job/hatch-mechanical-engineering-bursary-programme-2026/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Hatch invites graduates to apply for Mechanical Engineering Bursary Programme 2026 in Johannesburg, Gauteng, South Africa. Hatch is seeking highly</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2830,17 +2786,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2848,22 +2804,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2876,17 +2836,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>merSETA Learnerships 2026: Latest Technical Training Opportunities for ...</t>
+          <t>SAIMechE</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://www.myseta.co.za/merseta-learnership-programmes-2026/</t>
+          <t>https://www.saimeche.org.za/</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Discover merSETA Learnership Programmes 2026, including apprenticeships, internships, skills programmes, eligibility, stipends, application tips and technical career opportunities in South Africa.</t>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2894,11 +2854,7 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>info@myseta.co.za</t>
-        </is>
-      </c>
+      <c r="E100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2913,7 +2869,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Sappi offers apprenticeship and technical development opportunities for young people interested in building careers in engineering and artisan trades at its South African operations.</t>
+          <t>Tronox KZN Sands invites unemployed South African youth to apply for the Engineering Apprenticeship Programme 2026 in KwaZulu-Natal. Apprenticeship Application Closing Date: 30 September 2026 at 16:00 Apprenticeship Location: Empangeni and Mtunzini, KwaZulu-Natal, South Africa Tronox KZN Sands Engineering Apprenticeships…</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2930,17 +2886,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2948,26 +2904,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Centres South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2975,22 +2927,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>Competitions | ESG</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://za.rs-online.com/web/content/m/competition</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Centres South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits</t>
+          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -3000,24 +2956,24 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
+          <t>example@email.com</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ACTOM Engineering Projects and Contracts Bursaries 2027</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://www.studentroom.co.za/actom-engineering-projects-and-contracts-bursaries-2027/</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ACTOM Engineering Projects and Contracts invites South African students to apply for the 2027 Electrical Engineering Bursary Opportunity. Applications close on 31 July 2026.</t>
+          <t>IEEE-IAS Industrial Power Conversion Systems Department Serving the electrical energy conversion professional worldwide</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -3025,26 +2981,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>epc.hc@actom.co.za, studentroom-logo@2x.webp</t>
-        </is>
-      </c>
+      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Competitions | ESG</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://za.rs-online.com/web/content/m/competition</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3052,26 +3004,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>example@email.com</t>
-        </is>
-      </c>
+      <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Opportunities in Electrical Engineering across South Africa.</t>
+          <t>South African Institute of Electrical Engineers (SAIEE) Bursary 2027 ...</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://www.puffandpass.co.za/tag/electrical-engineering</t>
+          <t>https://www.edufunds.co.za/saiee-bursary-south-africa-2027/</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Location: Johannesburg Hatch is seeking Electrical / Civil / Mechanical Engineering Graduates who will support projects globally. The engineering team is comprised of professional engineers, designers and technologists. We have experience…</t>
+          <t>The South African Institute of Electrical Engineers (SAIEE) Bursary 2027 is now open for applications. If you are a South African citizen or permanent resident with a strong academic record, studying or intending to study Electrical Engineering, Electronics, or Computer Engineering, this opportunity could help you fund your education.</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3079,22 +3027,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Admin@edufunds.co.za, dudum@saiee.org.za, reception@saiee.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>IEEE-IAS Industrial Power Conversion Systems Department Serving the electrical energy conversion professional worldwide</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3102,22 +3054,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Eskom Bursary Programme South Africa 2026 - EduFunds SA</t>
+          <t>Masters Electrical Engineering Scholarships for South African Students</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://www.edufunds.co.za/eskom-bursary-programme-south-africa-2026/</t>
+          <t>https://www.scholarshipsads.com/masters-electrical-engineering-scholarships-for-south-african-students</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Apply for the Eskom Bursary Programme South Africa 2026. Funding for BEng/BSc engineering students in Chemical, Civil, Electrical, Mechanical, Industrial, and Metallurgy disciplines. Apply by 14 November 2025.</t>
+          <t>A curated list of masters electrical engineering scholarships worldwide open to South African students — with funding, eligibility and deadline detail for each. Ranked by relevance and completeness; updated for the latest intake.</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3125,26 +3081,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>candidate.support@ci.hr, Admin@edufunds.co.za</t>
-        </is>
-      </c>
+      <c r="E109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Zutari Bursary Programme 2027 Opens Applications for Civil and ...</t>
+          <t>IEC Young Professionals Competition | South African Bureau ... - LinkedIn</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://www.globalsouthopportunities.com/2026/08/10/zutari/</t>
+          <t>https://www.linkedin.com/posts/south-african-bureau-of-standards_iec-young-professionals-competition-activity-7322939590288240642-mm1o</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Zutari has opened applications for its 2027 Engineering Bursary Programme, offering financial and professional development support to South African students pursuing studies in Civil Engineering and Electrical Engineering. The engineering consulting company plans to award 10 bursaries for the 2027 academic year. The programme is aimed at young engineering talent, including matriculants and ...</t>
+          <t>The 2025 IEC (International Electrotechnical Commission) Young Professionals competition is here, and we are calling on all young professionals in the Electrotechnical field to jump into an ...</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3157,17 +3109,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Eskom Bursary Programme 2027 | Apply by 22 September</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://bursaries-southafrica.co.za/eskom-bursary-programme-2027/</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>At a glance Sponsor: Eskom Academic year: 2027 Applicants: Eligible South African school-leavers and current tertiary students Institutions: Recognised public universities and universities of technology, depending on the route Application method: Online through Eskom Careers About the programme Eskom's bursary intake supports students developing skills relevant to the electricity and energy ...</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3180,7 +3132,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+          <t>The Home of South African Hackathons</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3213,7 +3165,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Aug 22, 2025 · Join us for an electrifying hackathon where innovation meets security and finance! This event brings together developers, data scientists, cybersecurity experts, and FinTech enthusiasts to …</t>
+          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3226,17 +3178,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Unisa hosts first-ever Hackathon to ignite student learning ...</t>
+          <t>Build the Future with Entelect Hackathons</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
+          <t>https://challenge.entelect.co.za/</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Jul 14, 2025 · The event supported key priorities of South Africa’s National Development Plan, Unisa’s Catalytic Niche Areas and the United Nations’ Sustainable Development Goals that relate to access to quality education, decent work and innovation.</t>
+          <t>Build the Future with Entelect Hackathons Join South Africa's premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3249,17 +3201,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons</t>
+          <t>ICEP - Tshwane Varsity Hackathon</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/</t>
+          <t>https://tvh.icep.co.za/</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Instead of focusing on building a once-off project, our hackathons centre around optimisation problems. Participants develop solutions that are tested, scored, and ranked based on performance, efficiency, and strategy.</t>
+          <t>Tshwane Varsity Hackathon South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3267,12 +3219,16 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>MagasengQM@tut.ac.za, info@tvh.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+          <t>The Home of South African Hackathons</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3282,7 +3238,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Imagine a high-energy event where innovation and creativity collide - that’s a hackathon. Picture a whirlwind of coding, problem-solving, and brainstorming, all packed into an intense, short period.</t>
+          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3295,17 +3251,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Young Engineers Movement (YEM) - ORT SA</t>
+          <t>Unisa hosts first-ever Hackathon to ignite student learning experience</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Sep 2, 2026 · The Young Engineers Movement (YEM) is an immersive engineering and technology hackathon designed to equip young South Africans with the skills, mindset and confidence needed to solve real-world challenges.</t>
+          <t>Unisa's Information and Communication Technology Portfolio, in collaboration with the College of Science, Engineering and Technology, held the first-ever Unisa Hackathon on 3 and 4 July 2025, marking a major step in the university's journey to embed digital innovation and entrepreneurship into the students learning experience.</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3313,38 +3269,107 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
-        </is>
-      </c>
+      <c r="E117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
+          <t>Hackathons | Sebaka</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>https://sebakasouthafrica.co.za/hackathons.html</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
           <t>Talks &amp; Fireside | Builders Table</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr">
+      <c r="B120" t="inlineStr">
         <is>
           <t>https://builderstable.net/</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr">
+      <c r="C120" t="inlineStr">
         <is>
           <t>Builders Table is a two-day hackathon hosted by MakeReign, built around a 24-hour build sprint. It brings together South Africa's designers, developers, strategists, founders and creative technologists to build real working prototypes under real time pressure.</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr">
+      <c r="D120" t="inlineStr">
         <is>
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>liamlr95@gmail.com, sarah.chen@horizonlabs.com</t>
-        </is>
-      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>sarah.chen@horizonlabs.com, liamlr95@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>CompeteHub - Where Champions Are Made</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>https://www.devpluxe.co.za/</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-09-17
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -512,7 +512,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>info@zasdc.org, user@domain.com</t>
+          <t>user@domain.com, info@zasdc.org</t>
         </is>
       </c>
     </row>
@@ -565,17 +565,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
+          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.thecasecentre.org/products/view?id=189255</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -583,26 +583,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.thecasecentre.org/products/view?id=189255</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -610,22 +606,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>August 14, 2026 - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -638,17 +638,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Engineering design competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -661,17 +661,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>August 14, 2026 - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
+          <t>South Africa · South Korea · Spain · Sri Lanka · Sudan · Sweden · Switzerland · Syrian Arab Republic · Taiwan · Tajikistan · Tanzania · Thailand · Togo · Trinidad and Tobago · Tunisia · Turkey · Uganda · Ukraine · United Arab Emirates · United Kingdom ·</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>South Africa trade shows, find and compare 974 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 166 upcoming expos in 2026-2027 1. Mining Connect Day, 2. Annual ACFE Africa Conference &amp; Exhibition, 3. Annual Smart Procurement World Indaba, 4. ECM ...</t>
+          <t>South Africa trade shows, find and compare 971 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 164 upcoming expos in 2026-2027 1. Annual Smart Procurement World Indaba, 2. ECM Defence Symposium, 3.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -734,17 +734,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Top Expos In South Africa | Booth Exhibits™</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://boothexhibits.co.za/blog/venues-and-shows/south-africas-top-trade-shows-and-conferences/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Explore South Africa's top expos and conferences, from Africa Tech Festival to Mining Indaba and Automechanika. Choose the right event to stand out!</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -754,24 +754,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>hello@boothexhibits.co.za</t>
+          <t>customerservices@knect365.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, dataprivacy@knect365.com, salesenquiries@africatechfestival.com, support@knect365.com, support@informaconnect.com</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Big Data and Business Analytics Innovation Conference Johannesburg, South Africa IT &amp; Technology 101 Members Tue, 22 - Thu, 24 Sep 2026</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -784,17 +784,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms. Opportunity to network and connect with entrepreneurs, funders, investors, government departments and corporates.</t>
+          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -802,26 +802,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Erika@innovate.durban, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, sithabile@innovate.durban, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
+          <t>Exhibition | Innovation Festival Durban | South Africa</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://expotobi.com/country/south-africa/exhibitions</t>
+          <t>https://www.innovationfestival.durban/exhibition</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
+          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms. Opportunity to network and connect with entrepreneurs, funders, investors, government departments and corporates.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -829,22 +825,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, Erika@innovate.durban, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, sithabile@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://expotobi.com/country/south-africa/exhibitions</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -852,26 +852,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>dataprivacy@informaconnect.com, dataprivacy@knect365.com, customerservices@knect365.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, support@informaconnect.com, support@knect365.com</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>South Africa Professional Exhibitions, Shows, Fairs</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.showsbee.com/shows-0-1-South_Africa-all_city-All_Shows.html</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>South Africa ... First Previous , Go to page Select Shows by Industry or Country Industry Press Molecor SEA will showcase sustainable PVC-O innovations at ASIAWATER 2026 3/31/2026 Alfa Laval introduces ThinkCircularity: Closing the loop on plastic waste 2/26/2026 Vanzetti Engineering strengthens its presence in the Asian marine market 12/6/2025</t>
+          <t>Big Data and Business Analytics Innovation Conference Johannesburg, South Africa IT &amp; Technology 101 Members Tue, 22 - Thu, 24 Sep 2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -884,17 +880,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Exhibitions in South Africa</t>
+          <t>Trade Shows Worldwide - Cape Town (South Africa) - 2026/2027</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://expoonline.co.za/</t>
+          <t>https://www.eventseye.com/fairs/cy1_trade-shows-cape-town.html</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Online Exhibition South Africa We offer a Virtual Exhibition platform for specialized trade shows and exhibitions South Africa. Browse the exhibition by Expo Categories and connect with our Exhibitors. Discover new products and suppliers for your needs and industry at our online exhibitions South Africa.</t>
+          <t>Cape Town Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in Cape Town</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -902,26 +898,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>info@expoonline.co.za</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CPD Events | innovateX</t>
+          <t>Come and explore our exhibition of innovative discoveries at Science ...</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.innovatex.biz/event-list</t>
+          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>The most prestigious category 1 CPD event and exhibition in South Africa, InnovateX is coming to KZN. Make sure to register today to secure your spot and valuable 1 CPD Point.</t>
+          <t>The final countdown is underway, and all roads lead to this year's Science Forum South Africa 2024 at the CSIR International Convention Centre in Pretoria. Join us as we plan to celebrate the CSIR's impactful science, technology and innovation contributions at South Africa's premier scientific pl...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -929,11 +921,7 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1058,7 +1046,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>info@zasdc.org, user@domain.com</t>
+          <t>user@domain.com, info@zasdc.org</t>
         </is>
       </c>
     </row>
@@ -1088,17 +1076,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
+          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1106,22 +1094,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>privacy@studocu.com</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineers Without Borders launches student challenge</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.theconstructionindex.co.uk/news/view/engineers-without-borders-launches-student-challenge</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>September 7, 2021 - The Engineering for People Design Challenge encourages undergraduates to broaden their awareness of the social, environmental and economic implications of their engineering solutions.</t>
+          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1129,26 +1121,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>news@theconstructionindex.co.uk</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
+          <t>Engineers Without Borders launches student challenge</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
+          <t>https://www.theconstructionindex.co.uk/news/view/engineers-without-borders-launches-student-challenge</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
+          <t>September 7, 2021 - The Engineering for People Design Challenge encourages undergraduates to broaden their awareness of the social, environmental and economic implications of their engineering solutions.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1156,7 +1144,11 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>news@theconstructionindex.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1184,17 +1176,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
+          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1202,22 +1194,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1225,22 +1221,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1248,22 +1248,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, email@example.com, 8c4075d5481d476e945486754f783364@sentry.io, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1276,17 +1280,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
+          <t>Competitions - SABSA</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
+          <t>https://sabsa.co.za/competitions/</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
+          <t>African Business Concept Challenge ABCC is a virtual simulation-based business concept competition for African undergraduate and graduate students. The competition will challenge student teams to design a viable business concept that addresses a locally-relevant challenge or problem related to Agenda 2063, and inclusive and sustainable development.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1294,22 +1298,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>anne@sabsa.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1322,17 +1330,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Engineering in South Africa: 24 Best universities Ranked</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/za/</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1345,17 +1353,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>Competitions - Enactus South Africa | National Expos, Challenges ...</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://enactusza.org/what-we-do/competitions</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1363,22 +1371,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>marketingsa@enactus.org, liso@enactus.org, adminsa@enactus.org, xmadlanga@enactus.org</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>Competitions | ESG</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
+          <t>https://za.rs-online.com/web/content/m/competition</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1386,22 +1398,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>example@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1414,7 +1430,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>Technology Expo · October 10 - TECHSPO Joburg 2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1424,7 +1440,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>July 30, 2026 - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
+          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1441,17 +1457,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1459,22 +1475,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>customerservices@knect365.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, dataprivacy@knect365.com, salesenquiries@africatechfestival.com, support@knect365.com, support@informaconnect.com</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 - 7, 2027 ...</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
+          <t>The annual TECHSPO Cape Town 2027 Technology Expo returns October 6th to 7th, 2027 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town. TECHSPO Cape Town Technology Expo is the must-attend event to: Experience the Future of Technology &amp; Innovation Discover cutting-edge tech, game-changing tools, and innovators shaping tomorrow's digital world. See the latest advancements in ...</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1484,24 +1504,24 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>u003einfo@techspo.co, atinfo@techspo.coor</t>
+          <t>info@techspocapetown.co.za</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://africatechnologyexpo.com/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
+          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1511,24 +1531,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>johndoe@email.com, info@sparkafrica.co, partner@africatechnologyexpo.com</t>
+          <t>enquiries@aiexpoafrica.com</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>TECHSPO Events</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://techspo.co/events/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
+          <t>UPCOMING TECHSPO EVENTS The TECHSPO series continues to expand to multiple locations globally, to over 50 Conferences &amp; Exhibitions worldwide across 20 countries, plus an international cruise. SKIP TO REGION: Americas UK Europe Middle East Africa Asia OCEANIA SKIP TO CITY: UNITED STATES »Anaheim»Austin»Boston»Chicago»Cleveland»Dallas»Detroit»Denver»Fort Worth»Houston»Jacksonville ...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1536,26 +1556,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>info@techspocapetown.co.za</t>
-        </is>
-      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://10times.com/johannesburg-za/technology</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1563,26 +1579,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>dataprivacy@informaconnect.com, dataprivacy@knect365.com, customerservices@knect365.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, support@informaconnect.com, support@knect365.com</t>
-        </is>
-      </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Home - Mediatech Africa | South Africa</t>
+          <t>South Africa Tech Events - TECHSPO Johannesburg Technology Expo |</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://www.mediatech.co.za/</t>
+          <t>https://techspojoburg.co.za/south-africa-tech-events/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
+          <t>Welcome to the South Africa Tech Events Guide: Your number one resource to find the best, top voted, must-attend South Africa tech events online.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1592,24 +1604,24 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
+          <t>info@techspojoburg.co.za</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>HOME | Africa Tech Week</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~…</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://africatechweek.co.za/</t>
+          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>May 11, 2026 - From sensational speakers, to top tech exhibitons, see what’s in store when you attend the 2-day Sentech Africa Tech Week Conference in 2025&gt;&gt; ... Sponsor, Speak, Attend! For more information on how you can be a part of the #ATW family, contact ...</t>
+          <t>TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa. This must-attend, two-day annual event brings together leading developers, marketers, innovators, and technology enthusiasts eager to showcase and explore the latest in tech and digital solutions.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1617,22 +1629,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>support@industryevents.com, you@company.com, events@techspojoburg.co.za, colleague@company.com, your@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
+          <t>TECHSPO Cape Town 2026 Technology Expo (Internet ~ Mobile ~ AdTech ...</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
+          <t>https://allevents.in/cape-town/techspo-cape-town-2026-technology-expo-internet-~-mobile-~-adtech-~-martech-~-saas/200030358413547</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Save this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaShare this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
+          <t>TECHSPO Cape Town Technology Expo returns October 1-2, 2026 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town, South Africa. This must-attend, two-day annual event brings together leading developers, marketers, innovators, and technology enthusiasts eager to showcase and explore the latest in tech and digital solutions.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1645,17 +1661,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all Johannesburg Technology Business Expo &amp; Events in South Africa</t>
+          <t>Tech Expo Africa - Enabling Development</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://techexpo.africa/</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience.</t>
+          <t>Tech Expo Africa is a social enterprise connecting African businesses with top tech and business leaders to drive innovation.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1663,7 +1679,11 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>info@techexpo.africa</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1701,7 +1721,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>3 days ago - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
+          <t>4 days ago - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1714,17 +1734,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>https://makerfairecapetown.wordpress.com/about/</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1737,17 +1757,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://makerfairecapetown.wordpress.com/about/</t>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1780,24 +1800,24 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>pr@make.co</t>
+          <t>pr@make.co, fancybox_sprite@2x.png, fancybox_loading@2x.gif, chosen-sprite@2x.png</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
+          <t>Blog : Maker Faire Africa</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
+          <t>http://makerfaireafrica.com/blog/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
+          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building his ANIMAL car, from the ground up, that means the frame and all.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1810,17 +1830,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>The Makers Hub</t>
+          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.decorex.co.za/cape-town/en-gb/visit/TheMakersHub.html</t>
+          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Explore unique handmade items, take part in interactive workshops, and engage directly with Cape Town’s vibrant maker community.</t>
+          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1828,26 +1848,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>decorexafrica@rxglobal.com</t>
-        </is>
-      </c>
+      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
+          <t>The Makers Hub</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
+          <t>https://www.decorex.co.za/cape-town/en-gb/visit/TheMakersHub.html</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
+          <t>Explore unique handmade items, take part in interactive workshops, and engage directly with Cape Town’s vibrant maker community.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1855,22 +1871,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>decorexafrica@rxglobal.com</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Why Africa needs Maker Faire | ZDNET</t>
+          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
+          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage to attend and show off their work.</t>
+          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1883,17 +1903,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>HOME | MAKERS FEST</t>
+          <t>Why Africa needs Maker Faire | ZDNET</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.makersfestival.co.za/</t>
+          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>At Makers Festival SA, you get full access to every hands-on workshop, from woodworking and ceramics to leatherwork, painting, and more.</t>
+          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage to attend and show off their work.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1901,26 +1921,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, warren@makersfestival.co.za, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, example@mysite.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>StemCo - StemCo 2026 International Competitions</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://stemco.org/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
+          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1933,17 +1949,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024</t>
+          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
+          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1951,26 +1967,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
+          <t>High School STEM Competition | Capetown 2026</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>February 27, 2026 - Samsung Electronics South Africa has opened applications for the 2026 edition of Solve for Tomorrow (SFT), its annual science, technology, engineering, and mathematics (STEM) competition aimed at Grade 10 and 11 learners.</t>
+          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1978,22 +1990,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Local, regional and national competitions with thousands of · Multi-level events of two or more rounds that become increasingly challenging and culminate in top-level Olympiads. Enrichment programmes to inspire promising young South Africans to pursue STEMI</t>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2006,17 +2022,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The ZASDC is South Africa's national Space Design Competition, part of a global network spanning six continents. Secondary school students design futuristic space settlements in a fast-paced industry simulation that builds real STEM, leadership ...</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2024,26 +2040,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>info@zasdc.org, user@domain.com</t>
-        </is>
-      </c>
+      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>A first for Africa: Cape Town to host World Robot Olympiad International Final in 2028</t>
+          <t>Astemi Sa</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://www.bizcommunity.com/article/a-first-for-africa-cape-town-to-host-world-robot-olympiad-final-in-2028-964084a</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>4 hours ago - "Bringing the International Final ... continent to discover robotics and Stem.” · Further details about the WRO International Final 2028, including confirmed competition ......</t>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2056,17 +2068,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026 Season - Africa's Global STEM Celebration</t>
+          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://www.stemfestival.org/competitions/</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>April 30, 2026 - ... The Elementary, Junior, and Senior Robotics categories at STEM Festival are dedicated to advancing the World Robot Olympiad (WRO) across the Niger Delta and South-South Nigeria, working with ArcLights Foundation.</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2074,22 +2086,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SA young scientists selected for global competition at Regeneron ISEF in the USA - Eskom</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://www.eskom.co.za/sa-young-scientists-selected-for-global-competition-at-regeneron-isef-in-the-usa/</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>May 6, 2025 - Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) competition, will take place from 10 to 16 May in Columbus, Ohio in the USA.</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2097,26 +2113,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>MediaDesk@eskom.co.za</t>
-        </is>
-      </c>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions 2022 – SAASTA</t>
+          <t>South African Space Design Competition | Inspire Space Innovation ...</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://saasta.ac.za/astemi-competitions-2</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2124,22 +2136,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>user@domain.com, info@zasdc.org</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>STEAM Pitch Competition - STEM AFRICA FEST 2024</t>
+          <t>Imbewu Foundation</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://stemafricafest.com/steam-pitch-competition/</t>
+          <t>https://imbewu.foundation/</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Join STEM Africa Fest , celebrating science, technology, engineering, and mathematics. Experience hands-on learning, industry leaders, and innovation across Africa.</t>
+          <t>Seeding Future Scientists IMBEWU Science Foundation is a youth-focused STEMI organisation based in George, Western Cape, serving learners, educators and communities across the Eden District and Central Karoo District. We exist to nurture talent, ignite curiosity and create meaningful pathways for young South Africans to reach their full potential in science, technology, engineering ...</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2170,7 +2186,11 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2248,17 +2268,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>A first for Africa: Cape Town to host World Robot Olympiad International Final in 2028</t>
+          <t>South African Robotics Competitions and Schools</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://www.bizcommunity.com/article/a-first-for-africa-cape-town-to-host-world-robot-olympiad-final-in-2028-964084a</t>
+          <t>https://www.sciencexpo.org.za/robotics.html</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>4 hours ago - South Africa has been selected to host the 2028 World Robot Olympiad (WRO) International Final. The event, showing on the African continent for the first time, will take place at the Cape Town International Convention Centre (CTICC) during the ...</t>
+          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2266,22 +2286,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>madelien@imbewu.foundation, webmaster@sciencexpo.org.za, marna.vanzyl@imbewu.foundation</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
+          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
+          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
+          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2289,22 +2313,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>rampedim@atnews.co.za, NkosiN@atnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>South African Robotics Competitions and Schools</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://www.sciencexpo.org.za/robotics.html</t>
+          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
+          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2312,26 +2340,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>madelien@imbewu.foundation, marna.vanzyl@imbewu.foundation, webmaster@sciencexpo.org.za</t>
-        </is>
-      </c>
+      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
+          <t>The Robotics for Good Youth Challenge national competition will be held in Johannesburg, South Africa, at the Sandton Convention Centre on the 31st October 2025.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2341,7 +2365,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>rampedim@atnews.co.za, NkosiN@atnews.co.za</t>
+          <t>460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, info@thecortexhub.africa, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2375,17 +2399,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
+          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
+          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
+          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2398,17 +2422,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Civil Engineering Conferences in South Africa 2026/2027/2028</t>
+          <t>The South African Institution of Civil Engineering</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
+          <t>https://civils.org.za/</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Civil Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
+          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2421,17 +2445,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SWM Communications | SAICE recognises civil engineering research ...</t>
+          <t>Competition Ts and Cs - SAICE</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://swmcommunications.co.za/press-office/saice-recognises-civil-engineering-research-excellence-through-national-student-competition/</t>
+          <t>https://saice.org.za/competition-ts-and-cs/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) is a learned society and voluntary organisation that acts as a catalyst for innovation and good practice in the development of the civil engineering profession.</t>
+          <t>Preamble These Terms and Conditions govern participation in the Know Your Sector Competition ("the Competition") conducted by the South African Institute of Civil Engineering ("SAICE"). Definitions SAICE: Shall mean the South African Institute of Civil Engineering. The Competition: Shall mean SAICE's Know Your Sector Competition. Entrant: Shall mean any individual who enters the ...</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2441,24 +2465,24 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>nthabeleng@saice.org.za, info@swmcommunications.co.za</t>
+          <t>marketing@saice.org.za, civilinfo@saice.org.za, communications@saice.org.za, accounts@saice.org.za, membership@saice.org.za</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE)</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/SAICECIVIL/posts/the-excitement-is-building-at-the-2026-saice-international-bridge-building-compe/1515152847321706/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>The excitement is building at the 2026 SAICE International Bridge Building Competition! The 19 finalist teams attended an official briefing with Oliver Rowe from @ECSA, where they received important information as they prepared to put their engineering knowledge, creativity, teamwork and problem-solving skills to the test.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2466,22 +2490,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Civil Engineering Conferences In South Africa 2026-2027</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://conferencenext.com/conferences/south-africa/civil-engineering</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Civil Engineering conference in South Africa 2026-2027 is a great opportunity to learn from the opinions of global experts and the country's growth model. These events gather members of the Civil Engineering community to share research and expertise in this field through various programs, including presentations, keynote lectures, seminars ...</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2489,26 +2517,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>michaeljjacobson1@gmail.com</t>
-        </is>
-      </c>
+      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Civil Engineering | Bursaries South Africa</t>
+          <t>Power Construction Civil Engineering Bursary 2026: A Valuable Funding ...</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://www.zabursaries.co.za/?s=Civil+Engineering</t>
+          <t>https://www.setacareers.co.za/power-construction-civil-engineering-bursary-2026-2/</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Bursaries are awarded each semester, for Civil Engineering studies (Degree… Read More » ENGINEERING Engineering Bursaries South Africa 2027 The Engineering sector has many sub-sectors, each of them vitally important to the functioning of various systems and industries (such as factories, motor vehicles, pharmaceuticals etc).</t>
+          <t>The Power Construction Civil Engineering Bursary Programme 2026 offers qualifying students financial support linked to one of South Africa's established construction companies, with potential exposure to future work experience and career opportunities.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2516,22 +2540,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>info@setacareers.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ICE Africa - Supporting Civil Engineers in Africa</t>
+          <t>Engineering the Future: 16 schools compete in SAICE's 33rd ...</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
+          <t>https://southafricatoday.net/lifestyle/education/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ICE Africa supports civil engineers across the continent, providing access to qualifications, training, and networking opportunities for professional growth.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted its 33 rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland. The very first SAICE Bridge Building Competition was held in 1991, and it aimed to encourage high school learners to apply their knowledge of mathematics and science in a ...</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2544,17 +2572,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Civil Engineering Bursary - Bursaries Open Now in South Africa</t>
+          <t>Civil Engineering Conferences in South Africa 2026/2027/2028</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://bursariesopennow.co.za/category/civil-engineering-bursary/</t>
+          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Find Civil Engineering Bursary in South Africa. Updated bursaries with requirements, closing dates and how to apply.</t>
+          <t>Civil Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2567,17 +2595,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
+          <t>Home - SAICE</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
+          <t>https://saice.org.za/</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
+          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2585,22 +2613,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>marketing@saice.org.za, civilinfo@saice.org.za, barbara@avenue.co.za, communications@saice.org.za, executiveadmin@saice.org.za, accounts@saice.org.za, membership@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SAICE | Events and Awards</t>
+          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://members.saice.org.za/events-and-awards</t>
+          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>The South African Institution Of Civil Engineering SAICE hosts the Awards Function annually to honour individuals, projects of excellence, as well as community-oriented initiatives. The annual awards function gives companies and individuals a unique opportunity to showcase their deserving projects and work to the industry.</t>
+          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2613,17 +2645,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Awards 2025 - SAICE</t>
+          <t>SAICE Aqualibrium 2025: High School Students Rise to the Challenge in ...</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://saice.org.za/awards-2025/</t>
+          <t>https://southafricatoday.net/environment/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Learn about SAICE's award categories, submission guidelines, key dates and how to nominate project and professionals.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted the thrilling 2025 Aqualibrium Competition National Finals this past week, which brought together high school students from schools all over South Africa at the Sci-Bono Discovery Centre in Johannesburg. The event continues to be an important platform for fostering engineering talent, inspiring young minds, and raising awareness ...</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2631,11 +2663,7 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>accounts@saice.org.za, marketing@saice.org.za, communications@saice.org.za, membership@saice.org.za, civilinfo@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2690,17 +2718,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent's largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2713,17 +2741,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent's largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2736,17 +2764,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2813,17 +2841,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
+          <t>Apply Now: Africa Prize for Engineering Innovation 2026 Offers R1 ...</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
+          <t>https://stepapp.co.za/2025/08/27/apply-now-africa-prize-for-engineering-innovation-2026-offers-r1-million-top-prize/</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
+          <t>The Royal Academy of Engineering has officially launched the Africa Prize for Engineering Innovation 2026, a prestigious pan-African competition designed to support and accelerate engineering entrepreneurs who are developing scalable solutions to local challenges. This initiative, now in its 12th year, offers African innovators a unique opportunity to gain access to vital funding, mentorship ...</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2831,22 +2859,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Africa.Prize@raeng.org.uk, info@stepapp.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2859,17 +2891,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Apprenticeships 2025 / 2026 - StudentRoom.co.za</t>
+          <t>SAIMechE</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://www.studentroom.co.za/category/apprenticeships/</t>
+          <t>https://www.saimeche.org.za/</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Tronox KZN Sands invites unemployed South African youth to apply for the Engineering Apprenticeship Programme 2026 in KwaZulu-Natal. Apprenticeship Application Closing Date: 30 September 2026 at 16:00 Apprenticeship Location: Empangeni and Mtunzini, KwaZulu-Natal, South Africa Tronox KZN Sands Engineering Apprenticeships…</t>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2877,26 +2909,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>studentroom-logo@2x.webp</t>
-        </is>
-      </c>
+      <c r="E101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2909,17 +2937,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Centres South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits</t>
+          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2927,26 +2955,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
-        </is>
-      </c>
+      <c r="E103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Competitions | ESG</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - IEEE ZA 5G Competition</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://za.rs-online.com/web/content/m/competition</t>
+          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51397</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
+          <t>Form templates: Template for a Cover Sheet for the Competition on Ideas, Designs and Applications for 5G and Beyond South Africa (.docx) [Click to Download] Template for a Resume for the Student (.docx) [Click to Download] ... Help (FAQ) • Privacy Statement • Terms &amp; Conditions The SAIEE is ...</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2954,26 +2978,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>example@email.com</t>
-        </is>
-      </c>
+      <c r="E104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - SA Computing Olympiad stars hold their own in international competition</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51457</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>IEEE-IAS Industrial Power Conversion Systems Department Serving the electrical energy conversion professional worldwide</t>
+          <t>July 20, 2021 - For the other three South African team members, this was their first IOI. Brent Butkow finished ranked 342, Jean Weight finished in 287th position and Faran Steenkamp was ranked 280. In addition to the serious IOI contest days, host country Singapore arranged several fun events where Faran Steenkamp was placed third in the sponsored Code Cup, and won a cash prize of 200 USD.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2986,17 +3006,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>Student Design Competition | IEEE CASS</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://ieee-cas.org/society-involvement/student-design-competition</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>CASS will reimburse the travel costs for the trip to ISCAS 2026 for the four finalists, one for each region - Regions 1-7 (USA and Canada), Region 8 (Europe, Middle East, Africa), Region 9 (Latin America), and Region 10 (Asia, Australia, Pacific), as well as ISCAS registration.</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3009,17 +3029,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers (SAIEE) Bursary 2027 ...</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://www.edufunds.co.za/saiee-bursary-south-africa-2027/</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>The South African Institute of Electrical Engineers (SAIEE) Bursary 2027 is now open for applications. If you are a South African citizen or permanent resident with a strong academic record, studying or intending to study Electrical Engineering, Electronics, or Computer Engineering, this opportunity could help you fund your education.</t>
+          <t>March 12, 2026 - At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025.</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3027,26 +3047,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>Admin@edufunds.co.za, dudum@saiee.org.za, reception@saiee.org.za</t>
-        </is>
-      </c>
+      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Top 100 Electrical Engineering Companies in South Africa (2026) | ensun</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://ensun.io/search/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>The competitive landscape is marked by both established firms and emerging startups, driving innovation and efficiency. Additionally, South Africa’s position in the broader global market allows for potential collaborations and export opportunities, particularly in green technologies. Understanding these factors is essential for anyone looking to engage with the Electrical Engineering sector in South Africa, as they influence the overall business environment and potential for growth.</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3054,26 +3070,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Masters Electrical Engineering Scholarships for South African Students</t>
+          <t>7 Electrical Engineering Degree Programs in South Africa - Study Abroad | educations.com</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://www.scholarshipsads.com/masters-electrical-engineering-scholarships-for-south-african-students</t>
+          <t>https://www.educations.com/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>A curated list of masters electrical engineering scholarships worldwide open to South African students — with funding, eligibility and deadline detail for each. Ranked by relevance and completeness; updated for the latest intake.</t>
+          <t>Find the best fit for you - Compare 7 in Engineering Programs Electrical Engineering in South Africa for 2025/2026</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3086,17 +3098,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>IEC Young Professionals Competition | South African Bureau ... - LinkedIn</t>
+          <t>Electrical Engineering Conferences in South Africa 2026/2027/2028 - Conference Index</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/posts/south-african-bureau-of-standards_iec-young-professionals-competition-activity-7322939590288240642-mm1o</t>
+          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>The 2025 IEC (International Electrotechnical Commission) Young Professionals competition is here, and we are calling on all young professionals in the Electrotechnical field to jump into an ...</t>
+          <t>Nov 02 International Conference on Electronics, Control and Signal Processing (ICECSP) - Cape Town, South Africa · Nov 02 International Conference on Electrical, Computer, Electronics and Communication Engineering (ICECECE) - Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3109,17 +3121,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>Electrical And Electronics Engineering Conferences in South Africa 2026 | Conference Alerts</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://conferencealerts.co.in/south-africa/electrical-and-electronics-engineering</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>Select your participation type (in-person, virtual, or hybrid), fill in your personal and professional details, and pay the registration fee if required. After registering, you’ll receive confirmation and access instructions. Some electrical and electronics engineering conferences in south africa also allow early-bird registration with discounted fees.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3132,17 +3144,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>The Home of South African Hackathons</t>
+          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators - Lifestyle &amp; Tech</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/</t>
+          <t>https://lifestyleandtech.co.za/company-news/article/2026-06-29/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africas-next-generation-of-innovators</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+          <t>June 29, 2026 - After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant exhibition showcasing the remarkable ...</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3155,17 +3167,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Hackathons en South Africa</t>
+          <t>Houghton hackathon: Stepping stone for future engineers | Rosebank Killarney Gazette</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/</t>
+          <t>https://www.citizen.co.za/rosebank-killarney-gazette/news-headlines/local-news/2026/06/23/houghton-hackathon-stepping-stone-for-future-engineers/</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+          <t>June 23, 2026 - Hosted by ORT South Africa in partnership with Hudaco, the hackathon has brought together 55 learners from underserved communities to work together in developing solutions to challenges they face in their communities.</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3178,17 +3190,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons</t>
+          <t>Budding engineers showcase innovation at YEM hackathon | ITWeb</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/</t>
+          <t>https://www.itweb.co.za/article/budding-engineers-showcase-innovation-at-yem-hackathon/kYbe97XbP4ZqAWpG</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons Join South Africa's premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
+          <t>June 30, 2026 - The hackathon was hosted by Johannesburg-based non-profit education and training organisation ORT South Africa, in partnership with JSE-listed industrial and engineering supplies firm Hudaco.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3196,22 +3208,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>enquiries@ombudsman.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ICEP - Tshwane Varsity Hackathon</t>
+          <t>Young Engineers Showcase Innovation at STEM Hackathon</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://tvh.icep.co.za/</t>
+          <t>https://www.futuresa.co.za/education/young-engineers-movement-stem/</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Tshwane Varsity Hackathon South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
+          <t>June 11, 2026 - Fifty-five high school learners and 11 teachers from underserved South African schools will showcase working engineering and technology prototypes at the Young Engineers Movement (YEM) Hackathon Exhibition Day on 26 June 2026.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3221,24 +3237,24 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>MagasengQM@tut.ac.za, info@tvh.co.za</t>
+          <t>info@futuresa.co.za</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>The Home of South African Hackathons</t>
+          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/partners/</t>
+          <t>https://novuspressbulletin.co.za/blog/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africa-s-next-generation-of-innovators</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
+          <t>June 30, 2026 - ... Johannesburg, June 2026 – After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant ...</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3251,17 +3267,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Unisa hosts first-ever Hackathon to ignite student learning experience</t>
+          <t>55 learners from underserved schools showcase engineering innovations at Johannesburg hackathon</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
+          <t>https://iol.co.za/saturday-star/2026-07-01-55-learners-from-underserved-schools-showcase-engineering-innovations-at-johannesburg-hackathon/</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Unisa's Information and Communication Technology Portfolio, in collaboration with the College of Science, Engineering and Technology, held the first-ever Unisa Hackathon on 3 and 4 July 2025, marking a major step in the university's journey to embed digital innovation and entrepreneurship into the students learning experience.</t>
+          <t>July 29, 2026 - Fifty-five high school learners ... at the Young Engineers Movement (YEM) Hackathon Exhibition Day in Johannesburg last week, presenting working prototypes designed to solve real-world problems affecting their communities. The learners, accompanied by 11 teachers, took part in the five-day hackathon, hosted by ORT South Africa in partnership with Hudaco, from June 22 to 26....</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3269,22 +3285,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>yasmine.jacobs@iol.co.za, pholoso.manyama@iol.co.za, verna.vandiemen@inl.co.za, wendy.dondolo@inl.co.za, pholoso.manyama@inl.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Hackathons | Sebaka</t>
+          <t>ORT South Africa's inaugural YEM Hackathon empowers future STEM innovators</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>https://sebakasouthafrica.co.za/hackathons.html</t>
+          <t>https://www.futuresa.co.za/bursaries-and-scholarships/ort-south-africa-yem-hackathon/</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+          <t>July 30, 2026 - ORT South Africa's first Young Engineers Movement Hackathon saw 55 learners develop innovative STEM solutions during a five-day competition.</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3292,22 +3312,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>info@futuresa.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Young Engineers Movement (YEM) - ORT SA</t>
+          <t>Young Engineers Movement Hackathon opens doors to future career choices | Rosebank Killarney Gazette</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+          <t>https://www.citizen.co.za/rosebank-killarney-gazette/news-headlines/local-news/2026/07/06/hackathon-sparks-solutions/</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
+          <t>July 6, 2026 - 55 learners put ideas to paper, developing prototypes at the Young Engineers Movement (YEM) Hackathon. The ideas they came up with at the five-day hackathon in Houghton Estate, hosted by ORT South Africa, were to solve leading community issues, ...</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3315,26 +3339,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
-        </is>
-      </c>
+      <c r="E119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Talks &amp; Fireside | Builders Table</t>
+          <t>Southern Africa Digital ID Hackathon</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>https://builderstable.net/</t>
+          <t>https://www.africa.engineering.cmu.edu/events/2024/11/21-southern-digital-hackathon.html</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Builders Table is a two-day hackathon hosted by MakeReign, built around a 24-hour build sprint. It brings together South Africa's designers, developers, strategists, founders and creative technologists to build real working prototypes under real time pressure.</t>
+          <t>Learn more and register for Southern Africa Digital ID Hackathon · January 23 2026 · 12:00 PM - 1:30 PM CAT · Carnegie Mellon University Africa · Customizing the CV to the job description · Learn more about this event by contacting Paul Swaga.</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3342,26 +3362,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>sarah.chen@horizonlabs.com, liamlr95@gmail.com</t>
-        </is>
-      </c>
+      <c r="E120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CompeteHub - Where Champions Are Made</t>
+          <t>LLM Pilot Training Project 2026 | DS-I Africa</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>https://www.devpluxe.co.za/</t>
+          <t>https://dsi-africa.org/llm-pilot-training-project-2026</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
+          <t>Venue: Hackathon Professional Development Hub (PDH), University of the Witwatersrand, Johannesburg, South Africa</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -3369,7 +3385,11 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>ds-i-africa.admin@uct.ac.za</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-09-18
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -492,17 +492,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -510,26 +510,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>user@domain.com, info@zasdc.org</t>
-        </is>
-      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -537,22 +533,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>user@domain.com, info@zasdc.org</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Engineering Conferences in South Africa 2025-2026</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -565,17 +565,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
+          <t>Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.thecasecentre.org/products/view?id=189255</t>
+          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
+          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -608,24 +608,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>August 14, 2026 - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -638,17 +638,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>August 14, 2026 - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -661,17 +661,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://www.thecasecentre.org/products/view?id=189255</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>South Africa · South Korea · Spain · Sri Lanka · Sudan · Sweden · Switzerland · Syrian Arab Republic · Taiwan · Tajikistan · Tanzania · Thailand · Togo · Trinidad and Tobago · Tunisia · Turkey · Uganda · Ukraine · United Arab Emirates · United Kingdom ·</t>
+          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -684,17 +684,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/tradeshows</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>South Africa trade shows, find and compare 971 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 164 upcoming expos in 2026-2027 1. Annual Smart Procurement World Indaba, 2. ECM Defence Symposium, 3.</t>
+          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -702,22 +702,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>enquiries@aiexpoafrica.com</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
+          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://10times.com/southafrica/tradeshows</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
+          <t>South Africa trade shows, find and compare 974 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 165 upcoming expos in 2026-2027 1. NAMPO KAAP / CAPE, 2. Nampo Kaap Cape Bredasdorp, 3. KwaZulu-Natal EduXplore Expo, 4. Mining Connect Day</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -725,11 +729,7 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>enquiries@aiexpoafrica.com</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -754,24 +754,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>customerservices@knect365.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, dataprivacy@knect365.com, salesenquiries@africatechfestival.com, support@knect365.com, support@informaconnect.com</t>
+          <t>dataprivacy@knect365.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, support@knect365.com, support@informaconnect.com, customerservices@knect365.com, salesenquiries@africatechfestival.com</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
+          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
+          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -784,17 +784,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
+          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -827,24 +827,24 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, Erika@innovate.durban, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, sithabile@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com</t>
+          <t>sithabile@innovate.durban, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, Erika@innovate.durban, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://expotobi.com/country/south-africa/exhibitions</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
+          <t>Big Data and Business Analytics Innovation Conference Johannesburg, South Africa IT &amp; Technology 102 Members Tue, 22 - Thu, 24 Sep 2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -857,17 +857,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://expotobi.com/country/south-africa/exhibitions</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Big Data and Business Analytics Innovation Conference Johannesburg, South Africa IT &amp; Technology 101 Members Tue, 22 - Thu, 24 Sep 2026</t>
+          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -903,17 +903,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Come and explore our exhibition of innovative discoveries at Science ...</t>
+          <t>Manufacturing Indaba Exhibition 2027 - Manufacturing Expo</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>The final countdown is underway, and all roads lead to this year's Science Forum South Africa 2024 at the CSIR International Convention Centre in Pretoria. Join us as we plan to celebrate the CSIR's impactful science, technology and innovation contributions at South Africa's premier scientific pl...</t>
+          <t>Manufacturing Indaba Exhibition 2027: Africa's leading expo showcasing cutting-edge products, technology and innovation from manufacturers and SMEs, 13-14 July.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -926,17 +926,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
+          <t>Engineering for People Design Challenge 2024/25 - South Africa</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://crowdsolve.net/challenge/EfP-SA-25</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -944,22 +944,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>team@crowdsolve.net</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering For People Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
+          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -969,24 +973,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering for People Design Challenge - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -999,17 +1003,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>PDF Engineering ENGINEERING FOR PEOPLE Design challenge DESIGN CHALLENGE ...</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://www.ewb-uk.org/wp-content/uploads/2024/08/2024_25_Engineering_for_People_Design_Challenge_Makers_Valley.pdf</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>Makers Makers Valley Valley Johannesburg, Johannesburg, South South Africa Africa The Engineering for People Design Challenge has been delivered in the UK and Ireland since 2011, South Africa and the USA since 2019, and Cameroon in 2022. It is an educational programme based on a concept developed originally by Engineers Without Borders Australia. The production of this document has been led by ...</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1017,26 +1021,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>ied@ied.org.uk</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>... On 30-31 March 2026, 109 students from 9 schools walked into the University of Cape Town and designed a city on the Moon. They elected leaders, divided into engineering departments, and spent 24 hours responding to a professional design brief.</t>
+          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community's challenges and how community members view the impact of these challenges on their daily lives.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1046,24 +1046,24 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>user@domain.com, info@zasdc.org</t>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South ...</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
+          <t>This year's design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1071,22 +1071,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
+          <t>STEM-focused NGO Engineers Without Borders UK has launched its 2025 Engineering for People Design Challenge. Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year's challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1094,26 +1098,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>privacy@studocu.com</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>Engineers Without Borders | OU Design Show 2025</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://www.oudesignshow.org/designathon</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
+          <t>Makers Valley is a vibrant community of makers, creatives, and social enterprises in Johannesburg, South Africa. Engineers Without Borders UK has partnered with Makers Valley to engage students in design challenges focused on addressing local challenges and promoting sustainable development.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1126,17 +1126,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Engineers Without Borders launches student challenge</t>
+          <t>Engineering for People in Makers Valley | PDF | Apartheid | South Africa</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.theconstructionindex.co.uk/news/view/engineers-without-borders-launches-student-challenge</t>
+          <t>https://www.scribd.com/document/784038503/2024-25-Engineering-for-People-Design-Challenge-Makers-Valley</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>September 7, 2021 - The Engineering for People Design Challenge encourages undergraduates to broaden their awareness of the social, environmental and economic implications of their engineering solutions.</t>
+          <t>Engineering ENGINEERING for FOR people PEOPLE Design DESIGNchallenge CHALLENGE 2024-5 2024-25 Makers MakersValley Valley Johannesburg, Johannesburg,South SouthAfrica Africa fEngineering for People Design Challenge 2024-25 The Engineering for People Design Challenge contributed their time and expertise to enhance the has been delivered in the UK and Ireland since content of this design ...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1144,26 +1144,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>news@theconstructionindex.co.uk</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
+          <t>EWB-SA: Mid-Year Update - LinkedIn</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
+          <t>https://www.linkedin.com/pulse/ewb-sa-mid-year-update-ewbsa-uxo9f</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
+          <t>We wrapped up an extraordinary cycle of the 2023/24 Engineering for People Design Challenge in December 2024, with students across South Africa applying their creativity and empathy to solve real ...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1176,17 +1172,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
+          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1194,26 +1190,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1221,26 +1213,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>National Student Competition | ORSSA</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.orssa.org.za/studentcomp</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1248,26 +1236,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, email@example.com, 8c4075d5481d476e945486754f783364@sentry.io, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1280,17 +1264,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Competitions - SABSA</t>
+          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://sabsa.co.za/competitions/</t>
+          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>African Business Concept Challenge ABCC is a virtual simulation-based business concept competition for African undergraduate and graduate students. The competition will challenge student teams to design a viable business concept that addresses a locally-relevant challenge or problem related to Agenda 2063, and inclusive and sustainable development.</t>
+          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1298,26 +1282,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>anne@sabsa.co.za</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1330,17 +1310,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
+          <t>Engineering in South Africa: 24 Best universities Ranked</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://edurank.org/engineering/za/</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
+          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1353,17 +1333,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Competitions - Enactus South Africa | National Expos, Challenges ...</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://enactusza.org/what-we-do/competitions</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
+          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1371,26 +1351,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>marketingsa@enactus.org, liso@enactus.org, adminsa@enactus.org, xmadlanga@enactus.org</t>
-        </is>
-      </c>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Competitions | ESG</t>
+          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://za.rs-online.com/web/content/m/competition</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
+          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1398,26 +1374,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>example@email.com</t>
-        </is>
-      </c>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1430,7 +1402,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Technology Expo · October 10 - TECHSPO Joburg 2026</t>
+          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1440,7 +1412,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>July 30, 2026 - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1457,17 +1429,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1475,26 +1447,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>customerservices@knect365.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, dataprivacy@knect365.com, salesenquiries@africatechfestival.com, support@knect365.com, support@informaconnect.com</t>
-        </is>
-      </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 - 7, 2027 ...</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>The annual TECHSPO Cape Town 2027 Technology Expo returns October 6th to 7th, 2027 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town. TECHSPO Cape Town Technology Expo is the must-attend event to: Experience the Future of Technology &amp; Innovation Discover cutting-edge tech, game-changing tools, and innovators shaping tomorrow's digital world. See the latest advancements in ...</t>
+          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1504,24 +1472,24 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>info@techspocapetown.co.za</t>
+          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
+          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://africatechnologyexpo.com/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
+          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1531,24 +1499,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>enquiries@aiexpoafrica.com</t>
+          <t>info@sparkafrica.co, partner@africatechnologyexpo.com, johndoe@email.com</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TECHSPO Events</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://techspo.co/events/</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>UPCOMING TECHSPO EVENTS The TECHSPO series continues to expand to multiple locations globally, to over 50 Conferences &amp; Exhibitions worldwide across 20 countries, plus an international cruise. SKIP TO REGION: Americas UK Europe Middle East Africa Asia OCEANIA SKIP TO CITY: UNITED STATES »Anaheim»Austin»Boston»Chicago»Cleveland»Dallas»Detroit»Denver»Fort Worth»Houston»Jacksonville ...</t>
+          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1556,22 +1524,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1579,22 +1551,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>dataprivacy@knect365.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, support@knect365.com, support@informaconnect.com, customerservices@knect365.com, salesenquiries@africatechfestival.com</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>South Africa Tech Events - TECHSPO Johannesburg Technology Expo |</t>
+          <t>Home - Mediatech Africa | South Africa</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/south-africa-tech-events/</t>
+          <t>https://www.mediatech.co.za/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Welcome to the South Africa Tech Events Guide: Your number one resource to find the best, top voted, must-attend South Africa tech events online.</t>
+          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1604,24 +1580,24 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>info@techspojoburg.co.za</t>
+          <t>simon@mediatech.co.za, claire@mediatech.co.za</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~…</t>
+          <t>HOME | Africa Tech Week</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
+          <t>https://africatechweek.co.za/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa. This must-attend, two-day annual event brings together leading developers, marketers, innovators, and technology enthusiasts eager to showcase and explore the latest in tech and digital solutions.</t>
+          <t>May 11, 2026 - From sensational speakers, to top tech exhibitons, see what’s in store when you attend the 2-day Sentech Africa Tech Week Conference in 2025&gt;&gt; ... Sponsor, Speak, Attend! For more information on how you can be a part of the #ATW family, contact ...</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1629,26 +1605,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>support@industryevents.com, you@company.com, events@techspojoburg.co.za, colleague@company.com, your@email.com</t>
-        </is>
-      </c>
+      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2026 Technology Expo (Internet ~ Mobile ~ AdTech ...</t>
+          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://allevents.in/cape-town/techspo-cape-town-2026-technology-expo-internet-~-mobile-~-adtech-~-martech-~-saas/200030358413547</t>
+          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town Technology Expo returns October 1-2, 2026 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town, South Africa. This must-attend, two-day annual event brings together leading developers, marketers, innovators, and technology enthusiasts eager to showcase and explore the latest in tech and digital solutions.</t>
+          <t>Save this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaShare this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1661,17 +1633,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Tech Expo Africa - Enabling Development</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://techexpo.africa/</t>
+          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Tech Expo Africa is a social enterprise connecting African businesses with top tech and business leaders to drive innovation.</t>
+          <t>TECHSPO Johannesburg – Where Business, Tech and Innovation Collide in Johannesburg, South Africa. TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1681,7 +1653,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>info@techexpo.africa</t>
+          <t>support@industryevents.com, events@techspojoburg.co.za, you@company.com, colleague@company.com, your@email.com</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1670,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>March 7, 2025 - Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds ...</t>
+          <t>Maker Faire Africa, Cairo, October 2011 Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds (Nubian Cheetah). Maker Faire Africa aims to engage with on ...</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1721,7 +1693,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>4 days ago - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
+          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1734,17 +1706,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
+          <t>Upcoming Faires - Maker Faire</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://makerfairecapetown.wordpress.com/about/</t>
+          <t>https://makerfaire.com/upcoming-faires/</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1752,22 +1724,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>fancybox_sprite@2x.png, fancybox_loading@2x.gif, pr@make.co, chosen-sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>Maker Faire Africa — Grokipedia</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>https://grokipedia.com/page/maker_faire_africa</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>Maker Faire Africa Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1780,17 +1756,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>Maker Faire groups | Meetup</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>http://capetown.makerfaire.com/</t>
+          <t>https://www.meetup.com/topics/maker-faire/za/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1798,26 +1774,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>pr@make.co, fancybox_sprite@2x.png, fancybox_loading@2x.gif, chosen-sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Blog : Maker Faire Africa</t>
+          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>http://makerfaireafrica.com/blog/</t>
+          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building his ANIMAL car, from the ground up, that means the frame and all.</t>
+          <t>DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1830,17 +1802,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
+          <t>Global Faires - Maker Faire</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
+          <t>https://makerfaire.com/globalfaires/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
+          <t>Global Maker Faires showcase the very best of Maker innovation and creativity on a grand scale in the world's most dynamic cities.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1848,22 +1820,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>fancybox_sprite@2x.png, fancybox_loading@2x.gif, pr@make.co, chosen-sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>The Makers Hub</t>
+          <t>Maker Faire Africa - Facebook</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.decorex.co.za/cape-town/en-gb/visit/TheMakersHub.html</t>
+          <t>https://www.facebook.com/MFAJoburg/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Explore unique handmade items, take part in interactive workshops, and engage directly with Cape Town’s vibrant maker community.</t>
+          <t>Maker Faire Africa. 520 likes. Where Africa's future is in the making.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1871,26 +1847,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>decorexafrica@rxglobal.com</t>
-        </is>
-      </c>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
+          <t>MakeAfrica - Le festival africain de l'innovation technologique et de ...</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
+          <t>https://makeafrica.tech/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
+          <t>Le festival africain de l'innovation technologique et de la culture maker Un événement africain pensé par des africains et qui vise à partager, créer, fabriquer et apprendre les uns des autres. Il regroupe stands de démonstration, ateliers de découverte, présentations et conférences autour des sujets liés à l'innovation, la créativité, la fabrication, le numérique, les ...</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1898,22 +1870,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>contact@makeafrica.tech</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Why Africa needs Maker Faire | ZDNET</t>
+          <t>Maker Faire Africa - Wikiwand</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
+          <t>https://www.wikiwand.com/en/articles/Maker+Faire+Africa</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage to attend and show off their work.</t>
+          <t>The aim of a Maker Faire Africa is to create a space on the African continent where Afrigadget-type innovations, inventions and initiatives can be sought, identified, brought to life, supported, amplified and propagated. At the same time, Maker Faire Africa would seek to imbue creative types in science and technology with an appreciation of fabrication and by default manufacturing. The first ...</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1999,17 +1975,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2022,17 +1998,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>Astemi Sa</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2045,17 +2021,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Astemi Sa</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2118,17 +2094,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation ...</t>
+          <t>National Department of Basic Education</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.education.gov.za/LinkClick.aspx?fileticket=i9GS5Atf7zo=&amp;tabid=347&amp;portalid=0&amp;mid=14629</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Join the South African Space Design Competition to inspire space innovation, develop STEM skills, and compete for a trip to NASA. Perfect for high school students passionate about space.</t>
+          <t>JOHANNESBURG, South Africa - XX Month 2026 - The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries ...</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2138,24 +2114,24 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>user@domain.com, info@zasdc.org</t>
+          <t>ssasft@samsung.com, s.ngcobo@cheil.com, j.mogoeng@samsung.com</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Imbewu Foundation</t>
+          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://imbewu.foundation/</t>
+          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Seeding Future Scientists IMBEWU Science Foundation is a youth-focused STEMI organisation based in George, Western Cape, serving learners, educators and communities across the Eden District and Central Karoo District. We exist to nurture talent, ignite curiosity and create meaningful pathways for young South Africans to reach their full potential in science, technology, engineering ...</t>
+          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2188,7 +2164,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com</t>
+          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2222,17 +2198,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>FIRST South Africa – Robotics Programs for School Children</t>
+          <t>A first for Africa: Cape Town to host World Robot Olympiad International Final in 2028</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://firstsa.org/</t>
+          <t>https://www.bizcommunity.com/article/a-first-for-africa-cape-town-to-host-world-robot-olympiad-final-in-2028-964084a</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
+          <t>2 days ago - South Africa has been selected to host the 2028 World Robot Olympiad (WRO) International Final. The event, showing on the African continent for the first time, will take place at the Cape Town International Convention Centre (CTICC) during the ...</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2245,17 +2221,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>FIRST South Africa – Robotics Programs for School Children</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://firstsa.org/</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
+          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2268,17 +2244,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>South African Robotics Competitions and Schools</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://www.sciencexpo.org.za/robotics.html</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2286,26 +2262,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>madelien@imbewu.foundation, webmaster@sciencexpo.org.za, marna.vanzyl@imbewu.foundation</t>
-        </is>
-      </c>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
+          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
+          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
+          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2313,26 +2285,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>rampedim@atnews.co.za, NkosiN@atnews.co.za</t>
-        </is>
-      </c>
+      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
+          <t>South African Robotics Competitions and Schools</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
+          <t>https://www.sciencexpo.org.za/robotics.html</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
+          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2340,22 +2308,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>webmaster@sciencexpo.org.za, marna.vanzyl@imbewu.foundation, madelien@imbewu.foundation</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+          <t>Robotics &amp; Coding Classes for Kids in Johannesburg | Robotics League</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://robotics-league.co.za/</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge national competition will be held in Johannesburg, South Africa, at the Sandton Convention Centre on the 31st October 2025.</t>
+          <t>2026 Theme · Robots Meet Culture. The World Robot Olympiad is the planet's biggest student robotics competition — over 100 countries, 100,000+ students a year. South African teams compete on two tracks: Explorer, the home-grown SA challenge, ...</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2365,24 +2337,24 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, info@thecortexhub.africa, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com</t>
+          <t>info@roboticsleague.co.za, you@email.com</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Robotics &amp; Coding Classes for Kids in Johannesburg | Robotics League</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://robotics-league.co.za/</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026 Theme · Robots Meet Culture. The World Robot Olympiad is the planet's biggest student robotics competition — over 100 countries, 100,000+ students a year. South African teams compete on two tracks: Explorer, the home-grown SA challenge, ...</t>
+          <t>The Robotics for Good Youth Challenge national competition will be held in Johannesburg, South Africa, at the Sandton Convention Centre on the 31st October 2025.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2392,24 +2364,24 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>you@email.com, info@roboticsleague.co.za</t>
+          <t>info@thecortexhub.africa, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
+          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
+          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2465,24 +2437,24 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>marketing@saice.org.za, civilinfo@saice.org.za, communications@saice.org.za, accounts@saice.org.za, membership@saice.org.za</t>
+          <t>civilinfo@saice.org.za, communications@saice.org.za, membership@saice.org.za, accounts@saice.org.za, marketing@saice.org.za</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>The South African Institution of Civil Engineering (SAICE) - Facebook</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.facebook.com/SAICECIVIL/</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) is with Sekadi Phayane. What a night to remember! 🎉 The 2026 SAICE National Awards brought the civil engineering industry together for an evening celebrating the remarkable people and projects helping to move South Africa forward.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2490,26 +2462,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>SAICE's 34th International Bridge Competition Inspires Tomorrow's ...</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://southafricatoday.net/lifestyle/education/saices-34th-international-bridge-competition-inspires-tomorrows-engineers/</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2522,17 +2490,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Power Construction Civil Engineering Bursary 2026: A Valuable Funding ...</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://www.setacareers.co.za/power-construction-civil-engineering-bursary-2026-2/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>The Power Construction Civil Engineering Bursary Programme 2026 offers qualifying students financial support linked to one of South Africa's established construction companies, with potential exposure to future work experience and career opportunities.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2542,24 +2510,24 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>info@setacareers.co.za</t>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Engineering the Future: 16 schools compete in SAICE's 33rd ...</t>
+          <t>ICE Africa - Supporting Civil Engineers in Africa</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/lifestyle/education/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted its 33 rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland. The very first SAICE Bridge Building Competition was held in 1991, and it aimed to encourage high school learners to apply their knowledge of mathematics and science in a ...</t>
+          <t>ICE Africa supports civil engineers across the continent, providing access to qualifications, training, and networking opportunities for professional growth.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2572,17 +2540,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Civil Engineering Conferences in South Africa 2026/2027/2028</t>
+          <t>Home - SAICE</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
+          <t>https://saice.org.za/</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Civil Engineering Conferences in South Africa 2026 2027 2028 is for the researchers, scientists, scholars, engineers, academic, scientific and university practitioners to present research activities that might want to attend events, meetings, seminars, congresses, workshops, summit, and symposiums.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2590,22 +2558,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>civilinfo@saice.org.za, barbara@avenue.co.za, executiveadmin@saice.org.za, communications@saice.org.za, membership@saice.org.za, accounts@saice.org.za, marketing@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Home - SAICE</t>
+          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://saice.org.za/</t>
+          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
+          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2613,26 +2585,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>marketing@saice.org.za, civilinfo@saice.org.za, barbara@avenue.co.za, communications@saice.org.za, executiveadmin@saice.org.za, accounts@saice.org.za, membership@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
+          <t>SAICE Aqualibrium 2025: High School Students Rise to the Challenge in ...</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
+          <t>https://southafricatoday.net/environment/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted the thrilling 2025 Aqualibrium Competition National Finals this past week, which brought together high school students from schools all over South Africa at the Sci-Bono Discovery Centre in Johannesburg. The event continues to be an important platform for fostering engineering talent, inspiring young minds, and raising awareness ...</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2645,17 +2613,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>SAICE Aqualibrium 2025: High School Students Rise to the Challenge in ...</t>
+          <t>SAICE | Events and Awards</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/environment/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
+          <t>https://members.saice.org.za/events-and-awards</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted the thrilling 2025 Aqualibrium Competition National Finals this past week, which brought together high school students from schools all over South Africa at the Sci-Bono Discovery Centre in Johannesburg. The event continues to be an important platform for fostering engineering talent, inspiring young minds, and raising awareness ...</t>
+          <t>The South African Institution Of Civil Engineering SAICE hosts the Awards Function annually to honour individuals, projects of excellence, as well as community-oriented initiatives. The annual awards function gives companies and individuals a unique opportunity to showcase their deserving projects and work to the industry.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2718,17 +2686,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent's largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2741,17 +2709,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2759,22 +2727,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2787,17 +2759,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent's largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2805,11 +2777,7 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2834,7 +2802,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2829,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Africa.Prize@raeng.org.uk, info@stepapp.co.za</t>
+          <t>info@stepapp.co.za, Africa.Prize@raeng.org.uk</t>
         </is>
       </c>
     </row>
@@ -3190,17 +3158,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Budding engineers showcase innovation at YEM hackathon | ITWeb</t>
+          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://www.itweb.co.za/article/budding-engineers-showcase-innovation-at-yem-hackathon/kYbe97XbP4ZqAWpG</t>
+          <t>https://novuspressbulletin.co.za/blog/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africa-s-next-generation-of-innovators</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>June 30, 2026 - The hackathon was hosted by Johannesburg-based non-profit education and training organisation ORT South Africa, in partnership with JSE-listed industrial and engineering supplies firm Hudaco.</t>
+          <t>June 30, 2026 - ... Johannesburg, June 2026 – After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant ...</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3208,26 +3176,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>enquiries@ombudsman.org.za</t>
-        </is>
-      </c>
+      <c r="E114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Young Engineers Showcase Innovation at STEM Hackathon</t>
+          <t>Budding engineers showcase innovation at YEM hackathon | ITWeb</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://www.futuresa.co.za/education/young-engineers-movement-stem/</t>
+          <t>https://www.itweb.co.za/article/budding-engineers-showcase-innovation-at-yem-hackathon/kYbe97XbP4ZqAWpG</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>June 11, 2026 - Fifty-five high school learners and 11 teachers from underserved South African schools will showcase working engineering and technology prototypes at the Young Engineers Movement (YEM) Hackathon Exhibition Day on 26 June 2026.</t>
+          <t>June 30, 2026 - The hackathon was hosted by Johannesburg-based non-profit education and training organisation ORT South Africa, in partnership with JSE-listed industrial and engineering supplies firm Hudaco.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3237,24 +3201,24 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>info@futuresa.co.za</t>
+          <t>enquiries@ombudsman.org.za</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators</t>
+          <t>Young Engineers Showcase Innovation at STEM Hackathon</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>https://novuspressbulletin.co.za/blog/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africa-s-next-generation-of-innovators</t>
+          <t>https://www.futuresa.co.za/education/young-engineers-movement-stem/</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>June 30, 2026 - ... Johannesburg, June 2026 – After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant ...</t>
+          <t>June 11, 2026 - Fifty-five high school learners and 11 teachers from underserved South African schools will showcase working engineering and technology prototypes at the Young Engineers Movement (YEM) Hackathon Exhibition Day on 26 June 2026.</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3262,22 +3226,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>info@futuresa.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>55 learners from underserved schools showcase engineering innovations at Johannesburg hackathon</t>
+          <t>ORT South Africa's inaugural YEM Hackathon empowers future STEM innovators</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>https://iol.co.za/saturday-star/2026-07-01-55-learners-from-underserved-schools-showcase-engineering-innovations-at-johannesburg-hackathon/</t>
+          <t>https://www.futuresa.co.za/bursaries-and-scholarships/ort-south-africa-yem-hackathon/</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>July 29, 2026 - Fifty-five high school learners ... at the Young Engineers Movement (YEM) Hackathon Exhibition Day in Johannesburg last week, presenting working prototypes designed to solve real-world problems affecting their communities. The learners, accompanied by 11 teachers, took part in the five-day hackathon, hosted by ORT South Africa in partnership with Hudaco, from June 22 to 26....</t>
+          <t>July 30, 2026 - ORT South Africa's first Young Engineers Movement Hackathon saw 55 learners develop innovative STEM solutions during a five-day competition.</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3287,24 +3255,24 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>yasmine.jacobs@iol.co.za, pholoso.manyama@iol.co.za, verna.vandiemen@inl.co.za, wendy.dondolo@inl.co.za, pholoso.manyama@inl.co.za</t>
+          <t>info@futuresa.co.za</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>ORT South Africa's inaugural YEM Hackathon empowers future STEM innovators</t>
+          <t>55 learners from underserved schools showcase engineering innovations at Johannesburg hackathon</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>https://www.futuresa.co.za/bursaries-and-scholarships/ort-south-africa-yem-hackathon/</t>
+          <t>https://iol.co.za/saturday-star/2026-07-01-55-learners-from-underserved-schools-showcase-engineering-innovations-at-johannesburg-hackathon/</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>July 30, 2026 - ORT South Africa's first Young Engineers Movement Hackathon saw 55 learners develop innovative STEM solutions during a five-day competition.</t>
+          <t>July 29, 2026 - Fifty-five high school learners ... at the Young Engineers Movement (YEM) Hackathon Exhibition Day in Johannesburg last week, presenting working prototypes designed to solve real-world problems affecting their communities. The learners, accompanied by 11 teachers, took part in the five-day hackathon, hosted by ORT South Africa in partnership with Hudaco, from June 22 to 26....</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3314,7 +3282,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>info@futuresa.co.za</t>
+          <t>verna.vandiemen@inl.co.za, pholoso.manyama@iol.co.za, pholoso.manyama@inl.co.za, yasmine.jacobs@iol.co.za, wendy.dondolo@inl.co.za</t>
         </is>
       </c>
     </row>
@@ -3367,17 +3335,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>LLM Pilot Training Project 2026 | DS-I Africa</t>
+          <t>PATH South Africa co-hosts Harvard Health Hackathon | PATH</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>https://dsi-africa.org/llm-pilot-training-project-2026</t>
+          <t>https://www.path.org/our-impact/articles/path-south-africa-co-hosts-harvard-health-hackathon/</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Venue: Hackathon Professional Development Hub (PDH), University of the Witwatersrand, Johannesburg, South Africa</t>
+          <t>The South Africa hackathon location was at the University of Cape Town (UCT) and dubbed the UCT Hub. It attracted over 80 applicants from diverse fields, including medicine, engineering, research, and software development.</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -3385,11 +3353,7 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>ds-i-africa.admin@uct.ac.za</t>
-        </is>
-      </c>
+      <c r="E121" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-09-19
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -492,17 +492,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -510,22 +510,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>user@domain.com, info@zasdc.org</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -533,26 +537,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>user@domain.com, info@zasdc.org</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -565,17 +565,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Engineering Conferences in South Africa 2025-2026</t>
+          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
+          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
+          <t>August 14, 2026 - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -638,17 +638,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
+          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
+          <t>https://www.thecasecentre.org/products/view?id=189255</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>August 14, 2026 - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
+          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -661,17 +661,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.thecasecentre.org/products/view?id=189255</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
+          <t>Engineering design competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -684,17 +684,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
+          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://10times.com/southafrica/tradeshows</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
+          <t>South Africa trade shows, find and compare 971 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 162 upcoming expos in 2026-2027 1. Africa Aerospace &amp; Defence Expo, 2. Cape Town Audio Expo, 3.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -702,26 +702,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>enquiries@aiexpoafrica.com</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
+          <t>Exhibition | Innovation Festival Durban | South Africa</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/tradeshows</t>
+          <t>https://www.innovationfestival.durban/exhibition</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>South Africa trade shows, find and compare 974 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 165 upcoming expos in 2026-2027 1. NAMPO KAAP / CAPE, 2. Nampo Kaap Cape Bredasdorp, 3. KwaZulu-Natal EduXplore Expo, 4. Mining Connect Day</t>
+          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms. Opportunity to network and connect with entrepreneurs, funders, investors, government departments and corporates.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -729,22 +725,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, Erika@innovate.durban, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, sithabile@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -754,24 +754,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>dataprivacy@knect365.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, support@knect365.com, support@informaconnect.com, customerservices@knect365.com, salesenquiries@africatechfestival.com</t>
+          <t>enquiries@aiexpoafrica.com</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -779,7 +779,11 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>dataprivacy@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@knect365.com, dataprivacy@knect365.com, support@informaconnect.com, support@knect365.com, customerservices@informaconnect.com</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -807,17 +811,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms. Opportunity to network and connect with entrepreneurs, funders, investors, government departments and corporates.</t>
+          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -825,11 +829,7 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>sithabile@innovate.durban, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, Erika@innovate.durban, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -857,17 +857,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
+          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://expotobi.com/country/south-africa/exhibitions</t>
+          <t>https://innovationweek.co.za/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
+          <t>SA Innovation Week 2026 is South Africa's official national innovation platform accelerating implementation, commercialisation and impact.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -875,22 +875,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>info@pixal8media.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Trade Shows Worldwide - Cape Town (South Africa) - 2026/2027</t>
+          <t>TECHSPO Cape Town 2027 - Technology Expo · October 6</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.eventseye.com/fairs/cy1_trade-shows-cape-town.html</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Cape Town Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in Cape Town</t>
+          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -898,22 +902,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2027 - Manufacturing Expo</t>
+          <t>TECHSPO Joburg 2026 - Technology Expo · October 10</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://techspojoburg.co.za/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2027: Africa's leading expo showcasing cutting-edge products, technology and innovation from manufacturers and SMEs, 13-14 July.</t>
+          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -921,22 +929,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>info@techspojoburg.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge 2024/25 - South Africa</t>
+          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://crowdsolve.net/challenge/EfP-SA-25</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
+          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -944,26 +956,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>team@crowdsolve.net</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Engineering For People Design Challenge - EWBSA</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
+          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -980,17 +988,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge - Engineers Without Borders UK</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1003,17 +1011,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>PDF Engineering ENGINEERING FOR PEOPLE Design challenge DESIGN CHALLENGE ...</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/wp-content/uploads/2024/08/2024_25_Engineering_for_People_Design_Challenge_Makers_Valley.pdf</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Makers Makers Valley Valley Johannesburg, Johannesburg, South South Africa Africa The Engineering for People Design Challenge has been delivered in the UK and Ireland since 2011, South Africa and the USA since 2019, and Cameroon in 2022. It is an educational programme based on a concept developed originally by Engineers Without Borders Australia. The production of this document has been led by ...</t>
+          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1021,22 +1029,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ied@ied.org.uk</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community's challenges and how community members view the impact of these challenges on their daily lives.</t>
+          <t>... On 30-31 March 2026, 109 students from 9 schools walked into the University of Cape Town and designed a city on the Moon. They elected leaders, divided into engineering departments, and spent 24 hours responding to a professional design brief.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1046,24 +1058,24 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+          <t>user@domain.com, info@zasdc.org</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>Engineers Without Borders South ...</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>This year's design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
+          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1071,26 +1083,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>STEM-focused NGO Engineers Without Borders UK has launched its 2025 Engineering for People Design Challenge. Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year's challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
+          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1098,22 +1106,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineers Without Borders | OU Design Show 2025</t>
+          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.oudesignshow.org/designathon</t>
+          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Makers Valley is a vibrant community of makers, creatives, and social enterprises in Johannesburg, South Africa. Engineers Without Borders UK has partnered with Makers Valley to engage students in design challenges focused on addressing local challenges and promoting sustainable development.</t>
+          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1126,17 +1138,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Engineering for People in Makers Valley | PDF | Apartheid | South Africa</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.scribd.com/document/784038503/2024-25-Engineering-for-People-Design-Challenge-Makers-Valley</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Engineering ENGINEERING for FOR people PEOPLE Design DESIGNchallenge CHALLENGE 2024-5 2024-25 Makers MakersValley Valley Johannesburg, Johannesburg,South SouthAfrica Africa fEngineering for People Design Challenge 2024-25 The Engineering for People Design Challenge contributed their time and expertise to enhance the has been delivered in the UK and Ireland since content of this design ...</t>
+          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1149,17 +1161,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>EWB-SA: Mid-Year Update - LinkedIn</t>
+          <t>Engineers Without Borders launches student challenge</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/pulse/ewb-sa-mid-year-update-ewbsa-uxo9f</t>
+          <t>https://www.theconstructionindex.co.uk/news/view/engineers-without-borders-launches-student-challenge</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>We wrapped up an extraordinary cycle of the 2023/24 Engineering for People Design Challenge in December 2024, with students across South Africa applying their creativity and empathy to solve real ...</t>
+          <t>September 7, 2021 - The Engineering for People Design Challenge encourages undergraduates to broaden their awareness of the social, environmental and economic implications of their engineering solutions.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1167,7 +1179,11 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>news@theconstructionindex.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1310,17 +1326,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Engineering in South Africa: 24 Best universities Ranked</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/za/</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
+          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1333,17 +1349,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>Engineering in South Africa: 24 Best universities Ranked</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://edurank.org/engineering/za/</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1479,17 +1495,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://africatechnologyexpo.com/</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
+          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1499,24 +1515,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>info@sparkafrica.co, partner@africatechnologyexpo.com, johndoe@email.com</t>
+          <t>info@techspocapetown.co.za</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://africatechnologyexpo.com/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
+          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1526,7 +1542,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>info@techspocapetown.co.za</t>
+          <t>partner@africatechnologyexpo.com, johndoe@email.com, info@sparkafrica.co</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1569,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>dataprivacy@knect365.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, support@knect365.com, support@informaconnect.com, customerservices@knect365.com, salesenquiries@africatechfestival.com</t>
+          <t>dataprivacy@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@knect365.com, dataprivacy@knect365.com, support@informaconnect.com, support@knect365.com, customerservices@informaconnect.com</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1669,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>support@industryevents.com, events@techspojoburg.co.za, you@company.com, colleague@company.com, your@email.com</t>
+          <t>colleague@company.com, support@industryevents.com, events@techspojoburg.co.za, your@email.com, you@company.com</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1686,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Maker Faire Africa, Cairo, October 2011 Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds (Nubian Cheetah). Maker Faire Africa aims to engage with on ...</t>
+          <t>March 7, 2025 - Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds ...</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1693,7 +1709,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
+          <t>1 week ago - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1706,17 +1722,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Upcoming Faires - Maker Faire</t>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/upcoming-faires/</t>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1724,26 +1740,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>fancybox_sprite@2x.png, fancybox_loading@2x.gif, pr@make.co, chosen-sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Maker Faire Africa — Grokipedia</t>
+          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://grokipedia.com/page/maker_faire_africa</t>
+          <t>https://makerfairecapetown.wordpress.com/about/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Maker Faire Africa Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
+          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1756,17 +1768,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire groups | Meetup</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/topics/maker-faire/za/</t>
+          <t>http://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
+          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1774,22 +1786,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>fancybox_loading@2x.gif, fancybox_sprite@2x.png, chosen-sprite@2x.png, pr@make.co</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
+          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
+          <t>https://contemporaryand.com/fr/events/maker-faire-africa-comes-to-johannesburg</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
+          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1802,17 +1818,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Global Faires - Maker Faire</t>
+          <t>The Makers Hub</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/globalfaires/</t>
+          <t>https://www.decorex.co.za/cape-town/en-gb/visit/TheMakersHub.html</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Global Maker Faires showcase the very best of Maker innovation and creativity on a grand scale in the world's most dynamic cities.</t>
+          <t>Explore unique handmade items, take part in interactive workshops, and engage directly with Cape Town’s vibrant maker community.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1822,24 +1838,24 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>fancybox_sprite@2x.png, fancybox_loading@2x.gif, pr@make.co, chosen-sprite@2x.png</t>
+          <t>decorexafrica@rxglobal.com</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Maker Faire Africa - Facebook</t>
+          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/MFAJoburg/</t>
+          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Maker Faire Africa. 520 likes. Where Africa's future is in the making.</t>
+          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1852,17 +1868,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>MakeAfrica - Le festival africain de l'innovation technologique et de ...</t>
+          <t>Makers Festival SA 🛠️ (@makersfestival_sa) • Instagram photos ...</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://makeafrica.tech/</t>
+          <t>https://www.instagram.com/makersfestival_sa/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Le festival africain de l'innovation technologique et de la culture maker Un événement africain pensé par des africains et qui vise à partager, créer, fabriquer et apprendre les uns des autres. Il regroupe stands de démonstration, ateliers de découverte, présentations et conférences autour des sujets liés à l'innovation, la créativité, la fabrication, le numérique, les ...</t>
+          <t>8,503 Followers, 58 Following, 57 Posts - Makers Festival SA 🛠️ (@makersfestival_sa) on Instagram: "🛠️ Building Skills. Building Memories. 🏕️ 8th &amp; 9th November 2025 / Cape Town, SA 🪵 Founder @hutch_custom 📩 DM us - apply to be a MAKER 🫶🏼"</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1870,26 +1886,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>contact@makeafrica.tech</t>
-        </is>
-      </c>
+      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Maker Faire Africa - Wikiwand</t>
+          <t>Why Africa needs Maker Faire | ZDNET</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.wikiwand.com/en/articles/Maker+Faire+Africa</t>
+          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>The aim of a Maker Faire Africa is to create a space on the African continent where Afrigadget-type innovations, inventions and initiatives can be sought, identified, brought to life, supported, amplified and propagated. At the same time, Maker Faire Africa would seek to imbue creative types in science and technology with an appreciation of fabrication and by default manufacturing. The first ...</t>
+          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage ...</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1948,17 +1960,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Capetown 2026</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1966,26 +1978,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -1998,17 +2006,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Astemi Sa</t>
+          <t>High School STEM Competition | Capetown 2026</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2016,22 +2024,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>Astemi Sa</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2044,17 +2056,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2062,26 +2074,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>The IEOM High School/Middle School STEM Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2089,22 +2097,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>National Department of Basic Education</t>
+          <t>Competition - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://www.education.gov.za/LinkClick.aspx?fileticket=i9GS5Atf7zo=&amp;tabid=347&amp;portalid=0&amp;mid=14629</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/competition/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>JOHANNESBURG, South Africa - XX Month 2026 - The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries ...</t>
+          <t>Want to change the world for good? Come design the future with Samsung Solve for Tomorrow. Explore the role tech can play in solving biggest issues. No qualifications needed.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2112,11 +2124,7 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>ssasft@samsung.com, s.ngcobo@cheil.com, j.mogoeng@samsung.com</t>
-        </is>
-      </c>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2154,7 +2162,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>WRO South Africa ( World Robot Olympiad ) is a robotics competition which brings together young people from all over the world to develop their creativity and problem-solving skills.</t>
+          <t>World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop their creativity and problem-solving skills through challenging and educational ...</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2164,7 +2172,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+          <t>271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2198,17 +2206,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>A first for Africa: Cape Town to host World Robot Olympiad International Final in 2028</t>
+          <t>FIRST South Africa – Robotics Programs for School Children</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://www.bizcommunity.com/article/a-first-for-africa-cape-town-to-host-world-robot-olympiad-final-in-2028-964084a</t>
+          <t>https://firstsa.org/</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2 days ago - South Africa has been selected to host the 2028 World Robot Olympiad (WRO) International Final. The event, showing on the African continent for the first time, will take place at the Cape Town International Convention Centre (CTICC) during the ...</t>
+          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2221,17 +2229,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>FIRST South Africa – Robotics Programs for School Children</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://firstsa.org/</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2244,17 +2252,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
+          <t>The Robotics for Good Youth Challenge national competition will be held in Johannesburg, South Africa, at the Sandton Convention Centre on the 31st October 2025.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2262,22 +2270,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, info@thecortexhub.africa, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
+          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
+          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2290,17 +2302,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>South African Robotics Competitions and Schools</t>
+          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://www.sciencexpo.org.za/robotics.html</t>
+          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
+          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2310,24 +2322,24 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>webmaster@sciencexpo.org.za, marna.vanzyl@imbewu.foundation, madelien@imbewu.foundation</t>
+          <t>NkosiN@atnews.co.za, rampedim@atnews.co.za</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Robotics &amp; Coding Classes for Kids in Johannesburg | Robotics League</t>
+          <t>South African Robotics Competitions and Schools</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://robotics-league.co.za/</t>
+          <t>https://www.sciencexpo.org.za/robotics.html</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026 Theme · Robots Meet Culture. The World Robot Olympiad is the planet's biggest student robotics competition — over 100 countries, 100,000+ students a year. South African teams compete on two tracks: Explorer, the home-grown SA challenge, ...</t>
+          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2337,24 +2349,24 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>info@roboticsleague.co.za, you@email.com</t>
+          <t>webmaster@sciencexpo.org.za, marna.vanzyl@imbewu.foundation, madelien@imbewu.foundation</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+          <t>Robotics &amp; Coding Classes for Kids in Johannesburg | Robotics League</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://robotics-league.co.za/</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge national competition will be held in Johannesburg, South Africa, at the Sandton Convention Centre on the 31st October 2025.</t>
+          <t>2026 Theme · Robots Meet Culture. The World Robot Olympiad is the planet's biggest student robotics competition — over 100 countries, 100,000+ students a year. South African teams compete on two tracks: Explorer, the home-grown SA challenge, ...</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2364,24 +2376,24 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>info@thecortexhub.africa, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+          <t>you@email.com, info@roboticsleague.co.za</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
+          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
+          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
+          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2394,17 +2406,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://civils.org.za/</t>
+          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2412,22 +2424,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za, chanel@engineeringnews.co.za, advertising@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Competition Ts and Cs - SAICE</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://saice.org.za/competition-ts-and-cs/</t>
+          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Preamble These Terms and Conditions govern participation in the Know Your Sector Competition ("the Competition") conducted by the South African Institute of Civil Engineering ("SAICE"). Definitions SAICE: Shall mean the South African Institute of Civil Engineering. The Competition: Shall mean SAICE's Know Your Sector Competition. Entrant: Shall mean any individual who enters the ...</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2437,24 +2453,24 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>civilinfo@saice.org.za, communications@saice.org.za, membership@saice.org.za, accounts@saice.org.za, marketing@saice.org.za</t>
+          <t>ernao@crown.co.za, constr@crown.co.za</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) - Facebook</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/SAICECIVIL/</t>
+          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) is with Sekadi Phayane. What a night to remember! 🎉 The 2026 SAICE National Awards brought the civil engineering industry together for an evening celebrating the remarkable people and projects helping to move South Africa forward.</t>
+          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2467,17 +2483,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SAICE's 34th International Bridge Competition Inspires Tomorrow's ...</t>
+          <t>SWM Communications | SAICE recognises civil engineering research excellence through national student competition</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/lifestyle/education/saices-34th-international-bridge-competition-inspires-tomorrows-engineers/</t>
+          <t>https://swmcommunications.co.za/press-office/saice-recognises-civil-engineering-research-excellence-through-national-student-competition/</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
+          <t>April 1, 2026 - The event – which was sponsored by Sika, WorldsView, BVI, RIBCCS, and AF Consulting – was hosted at SAICE House in Midrand, Gauteng, and accredited for 0.2 CPD points. Students were invited to present their civil engineering university research and investigation project, which is part of the national curriculum for final year civil engineering undergraduate students.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2485,22 +2501,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>nthabeleng@saice.org.za, info@swmcommunications.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>September 7, 2025 - Find the list of upcoming Civil Engineering conferences in South Africa 2025 with invitation an letter.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2508,16 +2528,12 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ICE Africa - Supporting Civil Engineers in Africa</t>
+          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2527,7 +2543,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ICE Africa supports civil engineers across the continent, providing access to qualifications, training, and networking opportunities for professional growth.</t>
+          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2540,17 +2556,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Home - SAICE</t>
+          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://saice.org.za/</t>
+          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
+          <t>Civil engineering conferences in Cape town 2025 provide an exclusive global platform to meet and engage with experts and aspirants in various fields.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2558,26 +2574,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>civilinfo@saice.org.za, barbara@avenue.co.za, executiveadmin@saice.org.za, communications@saice.org.za, membership@saice.org.za, accounts@saice.org.za, marketing@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2590,17 +2602,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SAICE Aqualibrium 2025: High School Students Rise to the Challenge in ...</t>
+          <t>Civil Engineering Competition - Christian Brothers University</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/environment/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
+          <t>https://www.cbu.edu/civil-engineering-competition/</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted the thrilling 2025 Aqualibrium Competition National Finals this past week, which brought together high school students from schools all over South Africa at the Sci-Bono Discovery Centre in Johannesburg. The event continues to be an important platform for fostering engineering talent, inspiring young minds, and raising awareness ...</t>
+          <t>August 14, 2023 - Gather a team (2-5 members) to compete in CBU’s Civil Engineering Competition September 18, 2023, when up to six teams in each category will test their skills for the judges, CBU’s renowned engineering professors.</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2608,22 +2620,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>info@cbu.edu, jkaufma1@cbu.edu</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>SAICE | Events and Awards</t>
+          <t>Civil Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://members.saice.org.za/events-and-awards</t>
+          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>The South African Institution Of Civil Engineering SAICE hosts the Awards Function annually to honour individuals, projects of excellence, as well as community-oriented initiatives. The annual awards function gives companies and individuals a unique opportunity to showcase their deserving projects and work to the industry.</t>
+          <t>Apr 13 International Conference on Architectural, Civil and Environmental Engineering (ICACEE) - Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2686,17 +2702,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2709,17 +2725,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2727,26 +2743,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent's largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2759,17 +2771,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent's largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2777,7 +2789,11 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2829,7 +2845,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>info@stepapp.co.za, Africa.Prize@raeng.org.uk</t>
+          <t>Africa.Prize@raeng.org.uk, info@stepapp.co.za</t>
         </is>
       </c>
     </row>
@@ -2882,17 +2898,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2905,17 +2921,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
+          <t>South African Institute of Electrical Engineers 18a Gill Street Observatory Johannesburg South Africa Phone: +27 (0)11 487 3003 Email: reception@saiee.org.za Powered by</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2923,22 +2939,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - IEEE ZA 5G Competition</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51397</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Form templates: Template for a Cover Sheet for the Competition on Ideas, Designs and Applications for 5G and Beyond South Africa (.docx) [Click to Download] Template for a Resume for the Student (.docx) [Click to Download] ... Help (FAQ) • Privacy Statement • Terms &amp; Conditions The SAIEE is ...</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2951,17 +2971,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - SA Computing Olympiad stars hold their own in international competition</t>
+          <t>Competitions | ESG</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51457</t>
+          <t>https://za.rs-online.com/web/content/m/competition</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>July 20, 2021 - For the other three South African team members, this was their first IOI. Brent Butkow finished ranked 342, Jean Weight finished in 287th position and Faran Steenkamp was ranked 280. In addition to the serious IOI contest days, host country Singapore arranged several fun events where Faran Steenkamp was placed third in the sponsored Code Cup, and won a cash prize of 200 USD.</t>
+          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2969,22 +2989,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>example@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Student Design Competition | IEEE CASS</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://ieee-cas.org/society-involvement/student-design-competition</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>CASS will reimburse the travel costs for the trip to ISCAS 2026 for the four finalists, one for each region - Regions 1-7 (USA and Canada), Region 8 (Europe, Middle East, Africa), Region 9 (Latin America), and Region 10 (Asia, Australia, Pacific), as well as ISCAS registration.</t>
+          <t>IEEE-IAS Industrial Power Conversion Systems Department Serving the electrical energy conversion professional worldwide</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -2997,17 +3021,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>South African Institute of Electrical Engineers (SAIEE) Bursary 2027 ...</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://www.edufunds.co.za/saiee-bursary-south-africa-2027/</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>March 12, 2026 - At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025.</t>
+          <t>The South African Institute of Electrical Engineers (SAIEE) Bursary 2027 is now open for applications. If you are a South African citizen or permanent resident with a strong academic record, studying or intending to study Electrical Engineering, Electronics, or Computer Engineering, this opportunity could help you fund your education.</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3015,22 +3039,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>dudum@saiee.org.za, reception@saiee.org.za, Admin@edufunds.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Top 100 Electrical Engineering Companies in South Africa (2026) | ensun</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://ensun.io/search/electrical-engineering/south-africa</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>The competitive landscape is marked by both established firms and emerging startups, driving innovation and efficiency. Additionally, South Africa’s position in the broader global market allows for potential collaborations and export opportunities, particularly in green technologies. Understanding these factors is essential for anyone looking to engage with the Electrical Engineering sector in South Africa, as they influence the overall business environment and potential for growth.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3038,22 +3066,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>7 Electrical Engineering Degree Programs in South Africa - Study Abroad | educations.com</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://www.educations.com/electrical-engineering/south-africa</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Find the best fit for you - Compare 7 in Engineering Programs Electrical Engineering in South Africa for 2025/2026</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3066,17 +3098,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Electrical Engineering Conferences in South Africa 2026/2027/2028 - Conference Index</t>
+          <t>Engineering students compete in global high-performance computing ...</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
+          <t>https://ebe.uct.ac.za/articles/2026-05-29-engineering-students-compete-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Nov 02 International Conference on Electronics, Control and Signal Processing (ICECSP) - Cape Town, South Africa · Nov 02 International Conference on Electrical, Computer, Electronics and Communication Engineering (ICECECE) - Cape Town, South Africa</t>
+          <t>At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025. Now, Team UCT is preparing to represent South Africa at the global finals in Germany later this year.</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3084,22 +3116,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>ebe-faculty@uct.ac.za</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Electrical And Electronics Engineering Conferences in South Africa 2026 | Conference Alerts</t>
+          <t>ACTOM Engineering Projects and Contracts Bursaries 2027</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/south-africa/electrical-and-electronics-engineering</t>
+          <t>https://www.studentroom.co.za/actom-engineering-projects-and-contracts-bursaries-2027/</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Select your participation type (in-person, virtual, or hybrid), fill in your personal and professional details, and pay the registration fee if required. After registering, you’ll receive confirmation and access instructions. Some electrical and electronics engineering conferences in south africa also allow early-bird registration with discounted fees.</t>
+          <t>Bursary Location: Impala Mines, North West, South Africa About the ACTOM Engineering Projects and Contracts Bursary 2027 ACTOM Engineering Projects and Contracts has opened applications for its 2027 Bursary Opportunity for qualifying South African students studying Electrical Engineering at a University of Technology.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3107,22 +3143,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>epc.hc@actom.co.za, studentroom-logo@2x.webp</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators - Lifestyle &amp; Tech</t>
+          <t>The Home of South African Hackathons</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>https://lifestyleandtech.co.za/company-news/article/2026-06-29/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africas-next-generation-of-innovators</t>
+          <t>https://hackon.co.za/</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>June 29, 2026 - After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant exhibition showcasing the remarkable ...</t>
+          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3135,17 +3175,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Houghton hackathon: Stepping stone for future engineers | Rosebank Killarney Gazette</t>
+          <t>Hackathons en South Africa</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>https://www.citizen.co.za/rosebank-killarney-gazette/news-headlines/local-news/2026/06/23/houghton-hackathon-stepping-stone-for-future-engineers/</t>
+          <t>https://za.allhackathons.com/</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>June 23, 2026 - Hosted by ORT South Africa in partnership with Hudaco, the hackathon has brought together 55 learners from underserved communities to work together in developing solutions to challenges they face in their communities.</t>
+          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3158,17 +3198,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators</t>
+          <t>ICEP - Tshwane Varsity Hackathon</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://novuspressbulletin.co.za/blog/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africa-s-next-generation-of-innovators</t>
+          <t>https://tvh.icep.co.za/</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>June 30, 2026 - ... Johannesburg, June 2026 – After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant ...</t>
+          <t>Tshwane Varsity Hackathon South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3176,22 +3216,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>MagasengQM@tut.ac.za, info@tvh.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Budding engineers showcase innovation at YEM hackathon | ITWeb</t>
+          <t>Unisa hosts first-ever Hackathon to ignite student learning experience</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://www.itweb.co.za/article/budding-engineers-showcase-innovation-at-yem-hackathon/kYbe97XbP4ZqAWpG</t>
+          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>June 30, 2026 - The hackathon was hosted by Johannesburg-based non-profit education and training organisation ORT South Africa, in partnership with JSE-listed industrial and engineering supplies firm Hudaco.</t>
+          <t>Unisa's Information and Communication Technology Portfolio, in collaboration with the College of Science, Engineering and Technology, held the first-ever Unisa Hackathon on 3 and 4 July 2025, marking a major step in the university's journey to embed digital innovation and entrepreneurship into the students learning experience.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3199,26 +3243,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>enquiries@ombudsman.org.za</t>
-        </is>
-      </c>
+      <c r="E115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Young Engineers Showcase Innovation at STEM Hackathon</t>
+          <t>The Home of South African Hackathons</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>https://www.futuresa.co.za/education/young-engineers-movement-stem/</t>
+          <t>https://hackon.co.za/partners/</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>June 11, 2026 - Fifty-five high school learners and 11 teachers from underserved South African schools will showcase working engineering and technology prototypes at the Young Engineers Movement (YEM) Hackathon Exhibition Day on 26 June 2026.</t>
+          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3226,26 +3266,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>info@futuresa.co.za</t>
-        </is>
-      </c>
+      <c r="E116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ORT South Africa's inaugural YEM Hackathon empowers future STEM innovators</t>
+          <t>Build the Future with Entelect Hackathons</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>https://www.futuresa.co.za/bursaries-and-scholarships/ort-south-africa-yem-hackathon/</t>
+          <t>https://challenge.entelect.co.za/</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>July 30, 2026 - ORT South Africa's first Young Engineers Movement Hackathon saw 55 learners develop innovative STEM solutions during a five-day competition.</t>
+          <t>Build the Future with Entelect Hackathons Join South Africa's premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3253,26 +3289,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>info@futuresa.co.za</t>
-        </is>
-      </c>
+      <c r="E117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>55 learners from underserved schools showcase engineering innovations at Johannesburg hackathon</t>
+          <t>AfriCDSA Hackathon 2025</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>https://iol.co.za/saturday-star/2026-07-01-55-learners-from-underserved-schools-showcase-engineering-innovations-at-johannesburg-hackathon/</t>
+          <t>https://hackathon.africdsa.tech/</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>July 29, 2026 - Fifty-five high school learners ... at the Young Engineers Movement (YEM) Hackathon Exhibition Day in Johannesburg last week, presenting working prototypes designed to solve real-world problems affecting their communities. The learners, accompanied by 11 teachers, took part in the five-day hackathon, hosted by ORT South Africa in partnership with Hudaco, from June 22 to 26....</t>
+          <t>The Hackathon has begun! About the Hackathon Join us for the AfriCDSA Hackathon 2025, where top innovators, developers, and data scientists come together to tackle real-world challenges using cutting-edge AI and data-driven solutions.</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3282,24 +3314,24 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>verna.vandiemen@inl.co.za, pholoso.manyama@iol.co.za, pholoso.manyama@inl.co.za, yasmine.jacobs@iol.co.za, wendy.dondolo@inl.co.za</t>
+          <t>hackathon@africdsa.com</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Young Engineers Movement Hackathon opens doors to future career choices | Rosebank Killarney Gazette</t>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>https://www.citizen.co.za/rosebank-killarney-gazette/news-headlines/local-news/2026/07/06/hackathon-sparks-solutions/</t>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>July 6, 2026 - 55 learners put ideas to paper, developing prototypes at the Young Engineers Movement (YEM) Hackathon. The ideas they came up with at the five-day hackathon in Houghton Estate, hosted by ORT South Africa, were to solve leading community issues, ...</t>
+          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3307,22 +3339,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Southern Africa Digital ID Hackathon</t>
+          <t>Talks &amp; Fireside | Builders Table</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>https://www.africa.engineering.cmu.edu/events/2024/11/21-southern-digital-hackathon.html</t>
+          <t>https://builderstable.net/</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Learn more and register for Southern Africa Digital ID Hackathon · January 23 2026 · 12:00 PM - 1:30 PM CAT · Carnegie Mellon University Africa · Customizing the CV to the job description · Learn more about this event by contacting Paul Swaga.</t>
+          <t>Builders Table is a two-day hackathon hosted by MakeReign, built around a 24-hour build sprint. It brings together South Africa's designers, developers, strategists, founders and creative technologists to build real working prototypes under real time pressure.</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3330,22 +3366,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>sarah.chen@horizonlabs.com, liamlr95@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>PATH South Africa co-hosts Harvard Health Hackathon | PATH</t>
+          <t>CompeteHub - Where Champions Are Made</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>https://www.path.org/our-impact/articles/path-south-africa-co-hosts-harvard-health-hackathon/</t>
+          <t>https://www.devpluxe.co.za/</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>The South Africa hackathon location was at the University of Cape Town (UCT) and dubbed the UCT Hub. It attracted over 80 applicants from diverse fields, including medicine, engineering, research, and software development.</t>
+          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">

</xml_diff>

<commit_message>
Update competition data 2026-09-20
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>August 6, 2026 - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -492,17 +492,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -512,24 +512,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>user@domain.com, info@zasdc.org</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -537,22 +537,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Engineering Conferences in South Africa 2025-2026</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -565,17 +569,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
+          <t>Competitions - Prized Competitions South Africa</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
+          <t>https://www.prized.co.za/competitions/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>August 14, 2026 - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
+          <t>Prized is home to Online Competitions in South Africa. Enter any competition that peaks your interest and join the Prized community.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -588,17 +592,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
+          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>August 6, 2026 - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -606,26 +610,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -633,22 +633,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>info@zasdc.org, user@domain.com</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
+          <t>Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.thecasecentre.org/products/view?id=189255</t>
+          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
+          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -661,17 +665,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Engineering design competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -684,17 +688,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
+          <t>KZN Industrial Technology Exhibition</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/tradeshows</t>
+          <t>https://www.kznindustrial.co.za/</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>South Africa trade shows, find and compare 971 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 162 upcoming expos in 2026-2027 1. Africa Aerospace &amp; Defence Expo, 2. Cape Town Audio Expo, 3.</t>
+          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -702,22 +706,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>john@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>South Africa International Industrial Expo | Innovation Bridge</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms. Opportunity to network and connect with entrepreneurs, funders, investors, government departments and corporates.</t>
+          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -725,26 +733,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, Erika@innovate.durban, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, sithabile@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
+          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://madeinafricaevent.co.za/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
+          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -752,26 +756,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>enquiries@aiexpoafrica.com</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -779,26 +779,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>dataprivacy@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@knect365.com, dataprivacy@knect365.com, support@informaconnect.com, support@knect365.com, customerservices@informaconnect.com</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
+          <t>Exhibition | Innovation Festival Durban | South Africa</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://www.innovationfestival.durban/exhibition</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
+          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -806,22 +802,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, Erika@innovate.durban, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, sithabile@innovate.durban</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
+          <t>International Science, Innovation &amp; Technology Expo (INSITE)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
+          <t>https://www.dsti.gov.za/index.php/resource-center/27-temp/dst-links/3-international-science-innovation-a-technology-expo</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
+          <t>The essence of INSITE INSITE is an international, biennial must-see Science and Technology event in South Africa, the only one of its kind in Africa that creates new frontiers for global challenges · INSITE aims to assemble the worlds leading innovators and scientists in one place, stimulating ...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -834,17 +834,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Big Data and Business Analytics Innovation Conference Johannesburg, South Africa IT &amp; Technology 102 Members Tue, 22 - Thu, 24 Sep 2026</t>
+          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -857,17 +857,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
+          <t>Come and explore our exhibition of innovative discoveries at Science Forum South Africa 2024 | CSIR</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://innovationweek.co.za/</t>
+          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SA Innovation Week 2026 is South Africa's official national innovation platform accelerating implementation, commercialisation and impact.</t>
+          <t>December 3, 2024 - The exhibition launch will take place on Tuesday, 3 December 2024, with the opening address by Department of Science, Technology and Innovation Minister Dr Blade Nzimande.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -875,26 +875,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>info@pixal8media.co.za</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 - Technology Expo · October 6</t>
+          <t>AAXO - The Association of African Exhibition Organisers</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://www.aaxo.co.za/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology.</t>
+          <t>February 20, 2026 - CAPE TOWN, South Africa – The inaugural Festival of Eventing (FOE) brought together 350 event professionals, 85 speakers, and 10 countries under one roof for a two-day showcase of innovation, inspiration, and industry connection.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -902,26 +898,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>info@techspocapetown.co.za</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 - Technology Expo · October 10</t>
+          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/</t>
+          <t>https://10times.com/southafrica/tradeshows</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>South Africa trade shows, find ... Profile, Exhibitor Information etc. Listing of 166 upcoming expos in 2026-2027 1. Mining Connect Day, 2. Annual ACFE Africa Conference &amp; Exhibition, 3. Annual Smart Procurement World Indaba, ...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -929,26 +921,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>info@techspojoburg.co.za</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
+          <t>Engineering For People Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -956,22 +944,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>PDF Engineering ENGINEERING FOR PEOPLE Design challenge DESIGN CHALLENGE ...</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://www.ewb-uk.org/wp-content/uploads/2024/08/2024_25_Engineering_for_People_Design_Challenge_Makers_Valley.pdf</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
+          <t>Makers Makers Valley Valley Johannesburg, Johannesburg, South South Africa Africa The Engineering for People Design Challenge has been delivered in the UK and Ireland since 2011, South Africa and the USA since 2019, and Cameroon in 2022. It is an educational programme based on a concept developed originally by Engineers Without Borders Australia. The production of this document has been led by ...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -979,26 +971,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering for People Design Challenge - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1011,17 +999,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community's challenges and how community members view the impact of these challenges on their daily lives.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1031,24 +1019,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ied@ied.org.uk</t>
+          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>... On 30-31 March 2026, 109 students from 9 schools walked into the University of Cape Town and designed a city on the Moon. They elected leaders, divided into engineering departments, and spent 24 hours responding to a professional design brief.</t>
+          <t>STEM-focused NGO Engineers Without Borders UK has launched its 2025 Engineering for People Design Challenge. Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year's challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1056,26 +1044,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>user@domain.com, info@zasdc.org</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South ...</t>
+          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
+          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
+          <t>The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1083,7 +1067,11 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>team@crowdsolve.net</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1098,7 +1086,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
+          <t>This year's design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1108,24 +1096,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
+          <t>Engineers Without Borders | OU Design Show 2025</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
+          <t>https://www.oudesignshow.org/designathon</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
+          <t>Makers Valley is a vibrant community of makers, creatives, and social enterprises in Johannesburg, South Africa. Engineers Without Borders UK has partnered with Makers Valley to engage students in design challenges focused on addressing local challenges and promoting sustainable development.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1138,17 +1126,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>Bambasankhe Design Challenge: Engineering for a Prosperous South Africa</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://www.linkedin.com/posts/activity-7470764395091001345-GwCR</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
+          <t>By joining forces, student engineers have the chance to bridge societal gaps, uplift those in vulnerable positions, and contribute to building a more inclusive and prosperous South Africa.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1161,17 +1149,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Engineers Without Borders launches student challenge</t>
+          <t>EWB-SA: Mid-Year Update - LinkedIn</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.theconstructionindex.co.uk/news/view/engineers-without-borders-launches-student-challenge</t>
+          <t>https://www.linkedin.com/pulse/ewb-sa-mid-year-update-ewbsa-uxo9f</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>September 7, 2021 - The Engineering for People Design Challenge encourages undergraduates to broaden their awareness of the social, environmental and economic implications of their engineering solutions.</t>
+          <t>We wrapped up an extraordinary cycle of the 2023/24 Engineering for People Design Challenge in December 2024, with students across South Africa applying their creativity and empathy to solve real ...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1179,26 +1167,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>news@theconstructionindex.co.uk</t>
-        </is>
-      </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
+          <t>Some of our sparkling achievements ... and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1211,17 +1195,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1234,17 +1218,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1252,22 +1236,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1275,22 +1263,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
+          <t>2026 SOUTH AFRICA ENGINEERING COMPETITION</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
+          <t>https://notice.ukzn.ac.za/content/GetFile.aspx?id=96048</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
+          <t>Best Regards, The 2026 SA Engineering Competition Team University of KwaZulu-Natal • Elsevier</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1303,17 +1295,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1321,22 +1313,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, email@example.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>Competitions – Enactus South Africa | National Expos ...</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://enactusza.org/what-we-do/competitions</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1344,22 +1340,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>adminsa@enactus.org, xmadlanga@enactus.org, liso@enactus.org, marketingsa@enactus.org</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Engineering in South Africa: 24 Best universities Ranked</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/za/</t>
+          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
+          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1372,17 +1372,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1395,17 +1395,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1418,7 +1418,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>Technology Expo · October 10 - TECHSPO Joburg 2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>July 30, 2026 - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
+          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1445,17 +1445,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1463,22 +1463,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>customerservices@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, support@informaconnect.com, support@knect365.com</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
+          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology Expo ...</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
+          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
+          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 - 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1486,16 +1490,12 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
-        </is>
-      </c>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 - 7, 2027 ...</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
+          <t>The annual TECHSPO Cape Town 2027 Technology Expo returns October 6th to 7th, 2027 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town. TECHSPO Cape Town Technology Expo is the must-attend event to: Experience the Future of Technology &amp; Innovation Discover cutting-edge tech, game-changing tools, and innovators shaping tomorrow's digital world. See the latest advancements in ...</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1522,17 +1522,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://africatechnologyexpo.com/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
+          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1540,26 +1540,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>partner@africatechnologyexpo.com, johndoe@email.com, info@sparkafrica.co</t>
-        </is>
-      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1567,26 +1563,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>dataprivacy@informaconnect.com, salesenquiries@africatechfestival.com, customerservices@knect365.com, dataprivacy@knect365.com, support@informaconnect.com, support@knect365.com, customerservices@informaconnect.com</t>
-        </is>
-      </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Home - Mediatech Africa | South Africa</t>
+          <t>Tech Expo Africa - Enabling Development</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://www.mediatech.co.za/</t>
+          <t>https://techexpo.africa/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
+          <t>Tech Expo Africa is a social enterprise connecting African businesses with top tech and business leaders to drive innovation.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1596,24 +1588,24 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>simon@mediatech.co.za, claire@mediatech.co.za</t>
+          <t>info@techexpo.africa</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>HOME | Africa Tech Week</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://africatechweek.co.za/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>May 11, 2026 - From sensational speakers, to top tech exhibitons, see what’s in store when you attend the 2-day Sentech Africa Tech Week Conference in 2025&gt;&gt; ... Sponsor, Speak, Attend! For more information on how you can be a part of the #ATW family, contact ...</t>
+          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1621,22 +1613,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>enquiries@aiexpoafrica.com</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
+          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
+          <t>https://10times.com/johannesburg-za/technology</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Save this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaShare this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
+          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1649,17 +1645,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>TECHSPO Events</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
+          <t>https://techspo.co/events/</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg – Where Business, Tech and Innovation Collide in Johannesburg, South Africa. TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa.</t>
+          <t>UPCOMING TECHSPO EVENTS The TECHSPO series continues to expand to multiple locations globally, to over 50 Conferences &amp; Exhibitions worldwide across 20 countries, plus an international cruise. SKIP TO REGION: Americas UK Europe Middle East Africa Asia OCEANIA SKIP TO CITY: UNITED STATES »Anaheim»Austin»Boston»Chicago»Cleveland»Dallas»Detroit»Denver»Fort Worth»Houston»Jacksonville ...</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1667,11 +1663,7 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>colleague@company.com, support@industryevents.com, events@techspojoburg.co.za, your@email.com, you@company.com</t>
-        </is>
-      </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1686,7 +1678,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>March 7, 2025 - Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds ...</t>
+          <t>Maker Faire Africa, Cairo, October 2011 Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds (Nubian Cheetah). Maker Faire Africa aims to engage with on ...</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1709,7 +1701,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>1 week ago - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
+          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1722,17 +1714,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>Upcoming Faires - Maker Faire</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>https://makerfaire.com/upcoming-faires/</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1740,22 +1732,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif, pr@make.co</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
+          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://makerfairecapetown.wordpress.com/about/</t>
+          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
+          <t>Aug 21, 2015 · DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1768,17 +1764,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>Maker Faire groups | Meetup</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>http://capetown.makerfaire.com/</t>
+          <t>https://www.meetup.com/topics/maker-faire/za/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1786,26 +1782,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>fancybox_loading@2x.gif, fancybox_sprite@2x.png, chosen-sprite@2x.png, pr@make.co</t>
-        </is>
-      </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
+          <t>Maker Faire |</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://contemporaryand.com/fr/events/maker-faire-africa-comes-to-johannesburg</t>
+          <t>https://makerfaire.com/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1813,22 +1805,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif, pr@make.co</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>The Makers Hub</t>
+          <t>Maker Faire Africa — Grokipedia</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.decorex.co.za/cape-town/en-gb/visit/TheMakersHub.html</t>
+          <t>https://grokipedia.com/page/maker_faire_africa</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Explore unique handmade items, take part in interactive workshops, and engage directly with Cape Town’s vibrant maker community.</t>
+          <t>Maker Faire Africa Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1836,26 +1832,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>decorexafrica@rxglobal.com</t>
-        </is>
-      </c>
+      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1868,17 +1860,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Makers Festival SA 🛠️ (@makersfestival_sa) • Instagram photos ...</t>
+          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/makersfestival_sa/</t>
+          <t>https://makerfairecapetown.wordpress.com/about/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>8,503 Followers, 58 Following, 57 Posts - Makers Festival SA 🛠️ (@makersfestival_sa) on Instagram: "🛠️ Building Skills. Building Memories. 🏕️ 8th &amp; 9th November 2025 / Cape Town, SA 🪵 Founder @hutch_custom 📩 DM us - apply to be a MAKER 🫶🏼"</t>
+          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1891,17 +1883,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Why Africa needs Maker Faire | ZDNET</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
+          <t>http://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage ...</t>
+          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1909,12 +1901,16 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif, pr@make.co</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1937,7 +1933,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
+          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1947,7 +1943,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>February 27, 2026 - Samsung Electronics South Africa has opened applications for the 2026 edition of Solve for Tomorrow (SFT), its annual science, technology, engineering, and mathematics (STEM) competition aimed at Grade 10 and 11 learners.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1960,7 +1956,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2016,7 +2012,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
+          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the ‘first author’. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2033,7 +2029,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Astemi Sa</t>
+          <t>ASTEMI SA</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2056,17 +2052,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>StemCo - StemCo 2026 International Competitions</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://stemco.org/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2074,22 +2070,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>majed.ar@contestbag.com, bestyourself@stemco.org, info@eduverse.kz, support@contestbag.com</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>High School STEM Competition | Southafrica 2024</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>The IEOM High School/Middle School STEM Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects.</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2106,17 +2106,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Competition - Design The Future | Samsung South Africa</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/competition/</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Want to change the world for good? Come design the future with Samsung Solve for Tomorrow. Explore the role tech can play in solving biggest issues. No qualifications needed.</t>
+          <t>The ZASDC is South Africa's national Space Design Competition, part of a global network spanning six continents. Secondary school students design futuristic space settlements in a fast-paced industry simulation that builds real STEM, leadership ...</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2124,22 +2124,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>info@zasdc.org, user@domain.com</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
+          <t>SA young scientists selected for global competition at Regeneron ISEF in the USA - Eskom</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
+          <t>https://www.eskom.co.za/sa-young-scientists-selected-for-global-competition-at-regeneron-isef-in-the-usa/</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
+          <t>May 6, 2025 - Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) competition, will take place from 10 to 16 May in Columbus, Ohio in the USA.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2147,7 +2151,11 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>MediaDesk@eskom.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2162,7 +2170,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop their creativity and problem-solving skills through challenging and educational ...</t>
+          <t>WRO South Africa ( World Robot Olympiad ) is a robotics competition which brings together young people from all over the world to develop their creativity and problem-solving skills.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2172,7 +2180,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com</t>
+          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2197,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>April 14, 2026 - This National Event, to be held at the Sandton Convention Centre in Johannesburg, South Africa, as part of AI for Good Impact Africa, at AI Expo Africa 2025, is a qualifying tournament leading to the Grand Finale in Geneva during the AI for ...</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge, organized by ITU and The Cortex Hub, in partnership with Google.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2206,17 +2214,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>FIRST South Africa – Robotics Programs for School Children</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://firstsa.org/</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2224,22 +2232,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, info@thecortexhub.africa, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in a UN-based global robotics competition, focusing on the critical area of disaster response.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2247,22 +2259,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>name@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+          <t>VEX Events: Official Competition Website for VEX Robotics</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://events.vex.com/</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge national competition will be held in Johannesburg, South Africa, at the Sandton Convention Centre on the 31st October 2025.</t>
+          <t>Official Competition Website for VEX Robotics Robot Skills - IQ Elementary / Middle School Robot Skills - V5 Middle / High School Robot Skills - VEX U Collegiate / University</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2270,26 +2286,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, info@thecortexhub.africa, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop their creativity and problem-solving skills through challenging and educational robotics competitions.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2302,17 +2314,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
+          <t>Roboticon 2026: South Africa Showcases Robotics for Culture, Education ...</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
+          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
+          <t>The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation." South Africa's robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2322,24 +2334,24 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>NkosiN@atnews.co.za, rampedim@atnews.co.za</t>
+          <t>newspaper-rec300@2x.jpg, adverts@ubuntutimes.co.za</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>South African Robotics Competitions and Schools</t>
+          <t>World Robotics Olympiad (WRO) Cape Town 2028 | Resolute.Education</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://www.sciencexpo.org.za/robotics.html</t>
+          <t>https://wro2028.resolute.education/</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
+          <t>From Classroom To Industry Hosting the World Robot Olympiad (WRO) international final in South Africa</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2347,26 +2359,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>webmaster@sciencexpo.org.za, marna.vanzyl@imbewu.foundation, madelien@imbewu.foundation</t>
-        </is>
-      </c>
+      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Robotics &amp; Coding Classes for Kids in Johannesburg | Robotics League</t>
+          <t>Home | Roboticon 2026</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://robotics-league.co.za/</t>
+          <t>https://roboticon.resolute.education/</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026 Theme · Robots Meet Culture. The World Robot Olympiad is the planet's biggest student robotics competition — over 100 countries, 100,000+ students a year. South African teams compete on two tracks: Explorer, the home-grown SA challenge, ...</t>
+          <t>Thank you for joining us at the ultimate robotics showcase, as Resolute proudly sponsored the World Robotics Olympiad (WRO) South Africa. This year we brought together two worlds for the biggest robotics event of the year - Roboticon and the WRO Nationals, on the same day at the same venue.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2374,26 +2382,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>you@email.com, info@roboticsleague.co.za</t>
-        </is>
-      </c>
+      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
+          <t>ROBO-RUMBLE 2026 — Innovation in Motion</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
+          <t>https://roborumble.net/</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
+          <t>South Africa's premier youth robotics &amp; technology competition. Robo Wars, Drone Racing, Grand Prix &amp; Innovation Challenge. August 2026.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2426,7 +2430,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za, chanel@engineeringnews.co.za, advertising@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
+          <t>advertising@creamermedia.co.za, newsletters@creamermedia.co.za, subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za</t>
         </is>
       </c>
     </row>
@@ -2503,7 +2507,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>nthabeleng@saice.org.za, info@swmcommunications.co.za</t>
+          <t>info@swmcommunications.co.za, nthabeleng@saice.org.za</t>
         </is>
       </c>
     </row>
@@ -2622,7 +2626,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>info@cbu.edu, jkaufma1@cbu.edu</t>
+          <t>jkaufma1@cbu.edu, info@cbu.edu</t>
         </is>
       </c>
     </row>
@@ -2825,17 +2829,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Apply Now: Africa Prize for Engineering Innovation 2026 Offers R1 ...</t>
+          <t>List of ALL Engineering Bursaries South Africa 2027</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://stepapp.co.za/2025/08/27/apply-now-africa-prize-for-engineering-innovation-2026-offers-r1-million-top-prize/</t>
+          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>The Royal Academy of Engineering has officially launched the Africa Prize for Engineering Innovation 2026, a prestigious pan-African competition designed to support and accelerate engineering entrepreneurs who are developing scalable solutions to local challenges. This initiative, now in its 12th year, offers African innovators a unique opportunity to gain access to vital funding, mentorship ...</t>
+          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2843,11 +2847,7 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>Africa.Prize@raeng.org.uk, info@stepapp.co.za</t>
-        </is>
-      </c>
+      <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2898,17 +2898,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits · Become a SAIEE Member today! SAIEE Membership · Earn CPD credits · About Training Academy · Join a SAIEE Centre near you! Centres · South African Institute of Electrical Engineers (SAIEE) 01 ·</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2916,22 +2916,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>South African Institute of Electrical Engineers (SAIEE ...</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://www.edufunds.co.za/saiee-bursary-south-africa-2027/</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers 18a Gill Street Observatory Johannesburg South Africa Phone: +27 (0)11 487 3003 Email: reception@saiee.org.za Powered by</t>
+          <t>Aug 15, 2026 · Apply for the South African Institute of Electrical Engineers (SAIEE) Bursary 2027. Learn about the eligibility requirements, electrical engineering study options, bursary benefits, required documents, and how to apply before the closing date.</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2941,24 +2945,24 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
+          <t>Admin@edufunds.co.za, reception@saiee.org.za, dudum@saiee.org.za</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2971,17 +2975,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Competitions | ESG</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://za.rs-online.com/web/content/m/competition</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2991,24 +2995,24 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>example@email.com</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
+          <t>Competitions | ESG</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://za.rs-online.com/web/content/m/competition</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>IEEE-IAS Industrial Power Conversion Systems Department Serving the electrical energy conversion professional worldwide</t>
+          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3016,22 +3020,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>example@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers (SAIEE) Bursary 2027 ...</t>
+          <t>List of ALL Engineering Bursaries South Africa 2027</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://www.edufunds.co.za/saiee-bursary-south-africa-2027/</t>
+          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>The South African Institute of Electrical Engineers (SAIEE) Bursary 2027 is now open for applications. If you are a South African citizen or permanent resident with a strong academic record, studying or intending to study Electrical Engineering, Electronics, or Computer Engineering, this opportunity could help you fund your education.</t>
+          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3039,26 +3047,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>dudum@saiee.org.za, reception@saiee.org.za, Admin@edufunds.co.za</t>
-        </is>
-      </c>
+      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3066,26 +3070,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3098,17 +3098,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing ...</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://ebe.uct.ac.za/articles/2026-05-29-engineering-students-compete-global-high-performance-computing-challenge</t>
+          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025. Now, Team UCT is preparing to represent South Africa at the global finals in Germany later this year.</t>
+          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3116,26 +3116,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>ebe-faculty@uct.ac.za</t>
-        </is>
-      </c>
+      <c r="E110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ACTOM Engineering Projects and Contracts Bursaries 2027</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - IEEE ZA 5G Competition</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://www.studentroom.co.za/actom-engineering-projects-and-contracts-bursaries-2027/</t>
+          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51397</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Bursary Location: Impala Mines, North West, South Africa About the ACTOM Engineering Projects and Contracts Bursary 2027 ACTOM Engineering Projects and Contracts has opened applications for its 2027 Bursary Opportunity for qualifying South African students studying Electrical Engineering at a University of Technology.</t>
+          <t>Form templates: Template for a Cover Sheet for the Competition on Ideas, Designs and Applications for 5G and Beyond South Africa (.docx) [Click to Download] Template for a Resume for the Student (.docx) [Click to Download] ... Help (FAQ) • Privacy Statement • Terms &amp; Conditions The SAIEE is ...</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3143,11 +3139,7 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>epc.hc@actom.co.za, studentroom-logo@2x.webp</t>
-        </is>
-      </c>
+      <c r="E111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3175,17 +3167,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Hackathons en South Africa</t>
+          <t>ICEP - Tshwane Varsity Hackathon</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/</t>
+          <t>https://tvh.icep.co.za/</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+          <t>Tshwane Varsity Hackathon South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3193,22 +3185,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>MagasengQM@tut.ac.za, info@tvh.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ICEP - Tshwane Varsity Hackathon</t>
+          <t>Hackathons en South Africa</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://tvh.icep.co.za/</t>
+          <t>https://za.allhackathons.com/</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Tshwane Varsity Hackathon South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
+          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3216,11 +3212,7 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>MagasengQM@tut.ac.za, info@tvh.co.za</t>
-        </is>
-      </c>
+      <c r="E114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3294,17 +3286,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>AfriCDSA Hackathon 2025</t>
+          <t>Nedbank Hackathon</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>https://hackathon.africdsa.tech/</t>
+          <t>https://nedbankhackathon.co.za/</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>The Hackathon has begun! About the Hackathon Join us for the AfriCDSA Hackathon 2025, where top innovators, developers, and data scientists come together to tackle real-world challenges using cutting-edge AI and data-driven solutions.</t>
+          <t>The hackathon invitation is aimed at frontend, backend and full stack software developers, ideally at an intermediate or advanced levels of proficiency in either Java, C++, React, or Python.</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3312,11 +3304,7 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>hackathon@africdsa.com</t>
-        </is>
-      </c>
+      <c r="E118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3368,7 +3356,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>sarah.chen@horizonlabs.com, liamlr95@gmail.com</t>
+          <t>liamlr95@gmail.com, sarah.chen@horizonlabs.com</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update competition data 2026-09-21
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global ...</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.su.ac.za/en/faculties/engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>The competition offers the team an opportunity to showcase South African engineering talent on an international stage while benchmarking their skills against global peers. Beyond the event, the team aims to bring back new knowledge and inspiration, contributing to the growth of local expertise in space science and engineering.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -469,17 +469,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Some of our sparkling achievements during 2014 – to help the NRF and DSI grow a representative science and technology workforce in the country – SAASTA has run a number of maths and science educator development programmes and a number of learner development programmes, including maths and science camps for learners with potential, olympiads and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -487,22 +487,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -519,17 +523,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>2026 South Africa Engineering Competition</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://notices.ukzn.ac.za/content/GetFile.aspx?id=96048</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
+          <t>Best Regards, The 2026 SA Engineering Competition Team University of KwaZulu-Natal • Elsevier</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -537,26 +541,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>2026 South Africa Engineering</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://notices.ukzn.ac.za/content/GetFile.aspx?id=96047</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>UKZN and Elsevier. If you are an engineering student (undergraduate or postgraduate), don't miss joining the challenge to solve real-world cases using Engineering Village and Knovel.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -569,17 +569,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Competitions - Prized Competitions South Africa</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.prized.co.za/competitions/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Prized is home to Online Competitions in South Africa. Enter any competition that peaks your interest and join the Prized community.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -592,17 +592,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>August 6, 2026 - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -615,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa. Find out more</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -633,26 +633,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>info@zasdc.org, user@domain.com</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Engineering Conferences in South Africa 2025-2026</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -660,22 +656,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>Eligibility Benchmark Requirements The Africa Prize is open to individuals or teams based in sub-Saharan Africa with a scalable engineering innovation that demonstrates social or environmental impact potential. Applicants must: Be citizens ordinarily residing in a sub-Saharan African country. Be over 18 years old and fluent in English.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -688,17 +688,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>KZN Industrial Technology Exhibition</t>
+          <t>Exhibition | Innovation Festival Durban | South Africa</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://www.kznindustrial.co.za/</t>
+          <t>https://www.innovationfestival.durban/exhibition</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s ...</t>
+          <t>Exhibition Opportunities BENEFITS FOR YOUR PARTICIPATING IN THE EXHIBITION: An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -708,24 +708,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>john@email.com</t>
+          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, sithabile@innovate.durban, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, Erika@innovate.durban, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>South Africa International Industrial Expo | Innovation Bridge</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
+          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -733,22 +733,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>enquiries@aiexpoafrica.com</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -761,17 +765,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>Big Data and Business Analytics Innovation Conference Johannesburg, South Africa IT &amp; Technology 102 Members Tue, 22 - Thu, 24 Sep 2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -784,17 +788,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://innovationweek.co.za/</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
+          <t>SA Innovation Week 2026 is South Africa's official national innovation platform accelerating implementation, commercialisation and impact.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -804,24 +808,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, Erika@innovate.durban, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, sithabile@innovate.durban</t>
+          <t>info@pixal8media.co.za</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>International Science, Innovation &amp; Technology Expo (INSITE)</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://www.dsti.gov.za/index.php/resource-center/27-temp/dst-links/3-international-science-innovation-a-technology-expo</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The essence of INSITE INSITE is an international, biennial must-see Science and Technology event in South Africa, the only one of its kind in Africa that creates new frontiers for global challenges · INSITE aims to assemble the worlds leading innovators and scientists in one place, stimulating ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -829,22 +833,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>dataprivacy@knect365.com, support@knect365.com, customerservices@knect365.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, support@informaconnect.com</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
+          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
+          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
+          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -857,17 +865,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Come and explore our exhibition of innovative discoveries at Science Forum South Africa 2024 | CSIR</t>
+          <t>South Africa Manufacturing Show 2027 | Tech Event</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
+          <t>https://manufacturingitsummit.com/south-africa/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>December 3, 2024 - The exhibition launch will take place on Tuesday, 3 December 2024, with the opening address by Department of Science, Technology and Innovation Minister Dr Blade Nzimande.</t>
+          <t>Attend South Africa Manufacturing Show on 25 June 2027 to connect with 200+ manufacturing leaders driving AI, smart factories, automation, and innovation.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -875,22 +883,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>enquiry@exito-e.com</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AAXO - The Association of African Exhibition Organisers</t>
+          <t>TECHSPO Joburg 2026 - Technology Expo · October 10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.aaxo.co.za/</t>
+          <t>https://techspojoburg.co.za/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>February 20, 2026 - CAPE TOWN, South Africa – The inaugural Festival of Eventing (FOE) brought together 350 event professionals, 85 speakers, and 10 countries under one roof for a two-day showcase of innovation, inspiration, and industry connection.</t>
+          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -898,22 +910,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>info@techspojoburg.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
+          <t>TECHSPO Cape Town 2027 - Technology Expo · October 6</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/tradeshows</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>South Africa trade shows, find ... Profile, Exhibitor Information etc. Listing of 166 upcoming expos in 2026-2027 1. Mining Connect Day, 2. Annual ACFE Africa Conference &amp; Exhibition, 3. Annual Smart Procurement World Indaba, ...</t>
+          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -921,22 +937,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering For People Design Challenge - EWBSA</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
+          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -946,24 +966,24 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PDF Engineering ENGINEERING FOR PEOPLE Design challenge DESIGN CHALLENGE ...</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/wp-content/uploads/2024/08/2024_25_Engineering_for_People_Design_Challenge_Makers_Valley.pdf</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Makers Makers Valley Valley Johannesburg, Johannesburg, South South Africa Africa The Engineering for People Design Challenge has been delivered in the UK and Ireland since 2011, South Africa and the USA since 2019, and Cameroon in 2022. It is an educational programme based on a concept developed originally by Engineers Without Borders Australia. The production of this document has been led by ...</t>
+          <t>Oct 16, 2024 · Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -976,17 +996,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge - Engineers Without Borders UK</t>
+          <t>Engineering for People Design Challenge | Department of ...</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
+          <t>Aug 4, 2025 · The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -994,22 +1014,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering For People Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community's challenges and how community members view the impact of these challenges on their daily lives.</t>
+          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1019,24 +1043,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>robyn.clark@ewbsa.org, info@ewbsa.org</t>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>Engineering for People Design Challenge - Engineers Without ...</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>STEM-focused NGO Engineers Without Borders UK has launched its 2025 Engineering for People Design Challenge. Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year's challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
+          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1049,17 +1073,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
+          <t>Engineering ENGINEERING FOR PEOPLE Design challenge DESIGN ...</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
+          <t>https://www.ewb-uk.org/wp-content/uploads/2024/08/2024_25_Engineering_for_People_Design_Challenge_Makers_Valley.pdf</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
+          <t>These topics are at the centre of South Africa’s National Development Plan (NDP) 2030 and can provide insight into the main developmental challenges that are critical to South Africa.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1067,26 +1091,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>team@crowdsolve.net</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>This year's design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
+          <t>Oct 24, 2024 · The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1096,24 +1116,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
+          <t>team@crowdsolve.net</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineers Without Borders | OU Design Show 2025</t>
+          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.oudesignshow.org/designathon</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Makers Valley is a vibrant community of makers, creatives, and social enterprises in Johannesburg, South Africa. Engineers Without Borders UK has partnered with Makers Valley to engage students in design challenges focused on addressing local challenges and promoting sustainable development.</t>
+          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1126,17 +1146,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Bambasankhe Design Challenge: Engineering for a Prosperous South Africa</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/posts/activity-7470764395091001345-GwCR</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>By joining forces, student engineers have the chance to bridge societal gaps, uplift those in vulnerable positions, and contribute to building a more inclusive and prosperous South Africa.</t>
+          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1144,22 +1164,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ied@ied.org.uk</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>EWB-SA: Mid-Year Update - LinkedIn</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/pulse/ewb-sa-mid-year-update-ewbsa-uxo9f</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>We wrapped up an extraordinary cycle of the 2023/24 Engineering for People Design Challenge in December 2024, with students across South Africa applying their creativity and empathy to solve real ...</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1172,17 +1196,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Some of our sparkling achievements ... and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation ...</t>
+          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1195,17 +1219,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1218,17 +1242,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1236,26 +1260,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1263,26 +1283,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026 SOUTH AFRICA ENGINEERING COMPETITION</t>
+          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://notice.ukzn.ac.za/content/GetFile.aspx?id=96048</t>
+          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Best Regards, The 2026 SA Engineering Competition Team University of KwaZulu-Natal • Elsevier</t>
+          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1295,17 +1311,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>National Student Competition | ORSSA</t>
+          <t>Engineering in South Africa: 24 Best universities Ranked</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://www.orssa.org.za/studentcomp</t>
+          <t>https://edurank.org/engineering/za/</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
+          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1313,26 +1329,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, email@example.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Competitions – Enactus South Africa | National Expos ...</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://enactusza.org/what-we-do/competitions</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1340,26 +1352,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>adminsa@enactus.org, xmadlanga@enactus.org, liso@enactus.org, marketingsa@enactus.org</t>
-        </is>
-      </c>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
+          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1372,17 +1380,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1395,17 +1403,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1418,7 +1426,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Technology Expo · October 10 - TECHSPO Joburg 2026</t>
+          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1428,7 +1436,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>July 30, 2026 - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1445,17 +1453,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1463,26 +1471,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>customerservices@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, support@informaconnect.com, support@knect365.com</t>
-        </is>
-      </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology Expo ...</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
+          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 - 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
+          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1490,22 +1494,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 - 7, 2027 ...</t>
+          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://africatechnologyexpo.com/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>The annual TECHSPO Cape Town 2027 Technology Expo returns October 6th to 7th, 2027 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town. TECHSPO Cape Town Technology Expo is the must-attend event to: Experience the Future of Technology &amp; Innovation Discover cutting-edge tech, game-changing tools, and innovators shaping tomorrow's digital world. See the latest advancements in ...</t>
+          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1515,24 +1523,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>info@techspocapetown.co.za</t>
+          <t>partner@africatechnologyexpo.com, info@sparkafrica.co, johndoe@email.com</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1540,22 +1548,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026.</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1563,22 +1575,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>dataprivacy@knect365.com, support@knect365.com, customerservices@knect365.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, support@informaconnect.com</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Tech Expo Africa - Enabling Development</t>
+          <t>Home - Mediatech Africa | South Africa</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://techexpo.africa/</t>
+          <t>https://www.mediatech.co.za/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Tech Expo Africa is a social enterprise connecting African businesses with top tech and business leaders to drive innovation.</t>
+          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1588,24 +1604,24 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>info@techexpo.africa</t>
+          <t>simon@mediatech.co.za, claire@mediatech.co.za</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
+          <t>HOME | Africa Tech Week</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://africatechweek.co.za/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
+          <t>May 11, 2026 - From sensational speakers, to top tech exhibitons, see what’s in store when you attend the 2-day Sentech Africa Tech Week Conference in 2025&gt;&gt; ... Sponsor, Speak, Attend! For more information on how you can be a part of the #ATW family, contact ...</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1613,26 +1629,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>enquiries@aiexpoafrica.com</t>
-        </is>
-      </c>
+      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all ... - 10times</t>
+          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>Save this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaShare this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1645,17 +1657,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TECHSPO Events</t>
+          <t>IT &amp; Technology Events in Johannesburg, List of all Johannesburg Technology Business Expo &amp; Events in South Africa</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://techspo.co/events/</t>
+          <t>https://10times.com/johannesburg-za/technology</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>UPCOMING TECHSPO EVENTS The TECHSPO series continues to expand to multiple locations globally, to over 50 Conferences &amp; Exhibitions worldwide across 20 countries, plus an international cruise. SKIP TO REGION: Americas UK Europe Middle East Africa Asia OCEANIA SKIP TO CITY: UNITED STATES »Anaheim»Austin»Boston»Chicago»Cleveland»Dallas»Detroit»Denver»Fort Worth»Houston»Jacksonville ...</t>
+          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1678,7 +1690,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Maker Faire Africa, Cairo, October 2011 Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds (Nubian Cheetah). Maker Faire Africa aims to engage with on ...</t>
+          <t>The aim of a Maker Faire Africa is to create a space on the African continent where Afrigadget-type innovations, inventions and initiatives can be sought, identified, brought to life, supported, amplified and propagated.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1714,17 +1726,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Upcoming Faires - Maker Faire</t>
+          <t>Maker Faire Africa — Grokipedia</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/upcoming-faires/</t>
+          <t>https://grokipedia.com/page/maker_faire_africa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1732,26 +1744,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif, pr@make.co</t>
-        </is>
-      </c>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
+          <t>Maker Faire groups | Meetup</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
+          <t>https://www.meetup.com/topics/maker-faire/za/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Aug 21, 2015 · DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
+          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1764,17 +1772,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire groups | Meetup</t>
+          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/topics/maker-faire/za/</t>
+          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
+          <t>Aug 21, 2015 · We’re delighted to present the first ever Cape Town Maker Faire, hosted by Open Design in partnership with Trimble.Maker Faire is primarily designed as a forward-looking event, showcasing makers who are exploring new forms and new technologies.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1787,17 +1795,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Maker Faire |</t>
+          <t>Maker Faire Africa - Facebook</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/</t>
+          <t>https://www.facebook.com/MFAJoburg/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
+          <t>Jul 24, 2020 · Pizza, beer &amp; wine will be served during the film and a brief Q&amp;A about the Maker Movement will take place directly after the film, for anyone who wishes to participate.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1805,26 +1813,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif, pr@make.co</t>
-        </is>
-      </c>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa — Grokipedia</t>
+          <t>Upcoming Faires - Maker Faire</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://grokipedia.com/page/maker_faire_africa</t>
+          <t>https://makerfaire.com/upcoming-faires/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1832,27 +1836,31 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>chosen-sprite@2x.png, fancybox_sprite@2x.png, pr@make.co, fancybox_loading@2x.gif</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
+          <t>stem competition South Africa</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -1860,22 +1868,22 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://makerfairecapetown.wordpress.com/about/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
+          <t>stem competition South Africa</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -1883,44 +1891,44 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>High School STEM Competition | Capetown 2026</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>http://capetown.makerfaire.com/</t>
+          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>maker faire South Africa</t>
+          <t>stem competition South Africa</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif, pr@make.co</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Astemi Sa</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1933,7 +1941,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
+          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1943,7 +1951,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>February 27, 2026 - Samsung Electronics South Africa has opened applications for the 2026 edition of Solve for Tomorrow (SFT), its annual science, technology, engineering, and mathematics (STEM) competition aimed at Grade 10 and 11 learners.</t>
+          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1956,7 +1964,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1979,17 +1987,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2002,17 +2010,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Capetown 2026</t>
+          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the ‘first author’. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2029,17 +2037,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ASTEMI SA</t>
+          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2052,17 +2060,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>StemCo - StemCo 2026 International Competitions</t>
+          <t>Register your school for Samsung Solve for Tomorrow 2026</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://stemco.org/</t>
+          <t>https://www.sowetan.co.za/careers/2026-03-03-register-your-school-for-samsung-solve-for-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
+          <t>Register your school for Samsung Solve for Tomorrow 2026 STEM competition aims to transform and empower South African learners with critical skills to solve real-world challenges March 03, 2026 at 7:44 am</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2072,105 +2080,105 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>majed.ar@contestbag.com, bestyourself@stemco.org, info@eduverse.kz, support@contestbag.com</t>
+          <t>ssasft@samsung.com</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024</t>
+          <t>Robotics Competition | WRO South Africa | Gauteng</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://www.wrosa.co.za/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
+          <t>WRO South Africa ( World Robot Olympiad ) is a robotics competition which brings together young people from all over the world to develop their creativity and problem-solving skills.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
+          <t>robotics competition South Africa</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>South Africa to host first World Robot Olympiad International Final in Africa in 2028 - WRO Association</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://wro-association.org/south-africa-to-host-first-world-robot-olympiad-international-final-in-africa-in-2028/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>The ZASDC is South Africa's national Space Design Competition, part of a global network spanning six continents. Secondary school students design futuristic space settlements in a fast-paced industry simulation that builds real STEM, leadership ...</t>
+          <t>5 days ago - One of the world's largest ... South Africa, 12 September 2026 — South Africa will host the World Robot Olympiad (WRO®) International Final in 2028, bringing WRO's flagship global robotics...</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
+          <t>robotics competition South Africa</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>info@zasdc.org, user@domain.com</t>
+          <t>Prithul-3rd-place-Future-Engineers-2022-A-500x383@2x.jpg, Costa-Rica-team-Sprout-release-banner-500x383@2x.jpg, Annual-report-article-TZ-500x383@2x.jpg, 1-Team-CARED-Philippines-500x383@2x.jpg</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SA young scientists selected for global competition at Regeneron ISEF in the USA - Eskom</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://www.eskom.co.za/sa-young-scientists-selected-for-global-competition-at-regeneron-isef-in-the-usa/</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>May 6, 2025 - Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) competition, will take place from 10 to 16 May in Columbus, Ohio in the USA.</t>
+          <t>April 14, 2026 - This National Event, to be held at the Sandton Convention Centre in Johannesburg, South Africa, as part of AI for Good Impact Africa, at AI Expo Africa 2025, is a qualifying tournament leading to the Grand Finale in Geneva during the AI for ...</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
+          <t>robotics competition South Africa</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>MediaDesk@eskom.co.za</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Robotics Competition | WRO South Africa | Gauteng</t>
+          <t>Cape Town to host Africa’s first World Robot Olympiad</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>https://www.wrosa.co.za/</t>
+          <t>https://www.capetownetc.com/tech/cape-town-africas-first-world-robot-olympiad/</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>WRO South Africa ( World Robot Olympiad ) is a robotics competition which brings together young people from all over the world to develop their creativity and problem-solving skills.</t>
+          <t>5 hours ago - Cape Town will host the World Robot Olympiad (WRO) International Final in 2028, bringing one of the world’s largest youth robotics competitions to Africa for the first time, Cape {town} Etc reports.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2178,26 +2186,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
+          <t>FIRST South Africa – Robotics Programs for School Children</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
+          <t>https://firstsa.org/</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge, organized by ITU and The Cortex Hub, in partnership with Google.</t>
+          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2205,26 +2209,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>name@example.com</t>
-        </is>
-      </c>
+      <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2232,26 +2232,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, info@thecortexhub.africa, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
+          <t>South African Robotics Competitions and Schools</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
+          <t>https://www.sciencexpo.org.za/robotics.html</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in a UN-based global robotics competition, focusing on the critical area of disaster response.</t>
+          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2261,24 +2257,24 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>name@example.com</t>
+          <t>marna.vanzyl@imbewu.foundation, webmaster@sciencexpo.org.za, madelien@imbewu.foundation</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>VEX Events: Official Competition Website for VEX Robotics</t>
+          <t>Robotics &amp; Coding Classes for Kids in Johannesburg | Robotics League</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://events.vex.com/</t>
+          <t>https://robotics-league.co.za/</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Official Competition Website for VEX Robotics Robot Skills - IQ Elementary / Middle School Robot Skills - V5 Middle / High School Robot Skills - VEX U Collegiate / University</t>
+          <t>2026 Theme · Robots Meet Culture. The World Robot Olympiad is the planet's biggest student robotics competition — over 100 countries, 100,000+ students a year. South African teams compete on two tracks: Explorer, the home-grown SA challenge, ...</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2286,22 +2282,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>info@roboticsleague.co.za, you@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop their creativity and problem-solving skills through challenging and educational robotics competitions.</t>
+          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2309,22 +2309,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>rampedim@atnews.co.za, NkosiN@atnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Roboticon 2026: South Africa Showcases Robotics for Culture, Education ...</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
+          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation." South Africa's robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
+          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2332,54 +2336,54 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>newspaper-rec300@2x.jpg, adverts@ubuntutimes.co.za</t>
-        </is>
-      </c>
+      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>World Robotics Olympiad (WRO) Cape Town 2028 | Resolute.Education</t>
+          <t>Civil engineering Tenders SA - 72 Open | September 2026 ...</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://wro2028.resolute.education/</t>
+          <t>https://www.tenderflow.co.za/categories/civil-engineering/</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>From Classroom To Industry Hosting the World Robot Olympiad (WRO) international final in South Africa</t>
+          <t>3 days ago · Browse 72 active civil engineering tenders in South Africa. Updated daily with government, SOE &amp; private sector opportunities. Free alerts on TenderFlow.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr"/>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>support@tenderflow.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Home | Roboticon 2026</t>
+          <t>The South African Institution of Civil Engineering</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://roboticon.resolute.education/</t>
+          <t>https://civils.org.za/</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Thank you for joining us at the ultimate robotics showcase, as Resolute proudly sponsored the World Robotics Olympiad (WRO) South Africa. This year we brought together two worlds for the biggest robotics event of the year - Roboticon and the WRO Nationals, on the same day at the same venue.</t>
+          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -2387,22 +2391,22 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ROBO-RUMBLE 2026 — Innovation in Motion</t>
+          <t>Civil Engineering Tenders — 270 open listings, updated 21 ...</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://roborumble.net/</t>
+          <t>https://tenderbulletins.co.za/tender-category/civil-engineering/</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>South Africa's premier youth robotics &amp; technology competition. Robo Wars, Drone Racing, Grand Prix &amp; Innovation Challenge. August 2026.</t>
+          <t>Browse current and past Civil Engineering tenders published by South African government departments, municipalities, state-owned entities and private companies looking to procure civil engineering.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -2410,17 +2414,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
+          <t>https://safcec.org.za/</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
+          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2430,7 +2434,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>advertising@creamermedia.co.za, newsletters@creamermedia.co.za, subscriptions@creamermedia.co.za, chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za</t>
+          <t>communication@safcec.org.za</t>
         </is>
       </c>
     </row>
@@ -2442,12 +2446,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
+          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2457,24 +2461,24 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>ernao@crown.co.za, constr@crown.co.za</t>
+          <t>subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za, chanel@engineeringnews.co.za, newsletters@creamermedia.co.za</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
+          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd International Bridge Building Competition - SAICE</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
+          <t>https://saice.org.za/press-releases/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
+          <t>April 17, 2025 - The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2482,22 +2486,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>marketing@saice.org.za, civilinfo@saice.org.za, accounts@saice.org.za, communications@saice.org.za, membership@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SWM Communications | SAICE recognises civil engineering research excellence through national student competition</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://swmcommunications.co.za/press-office/saice-recognises-civil-engineering-research-excellence-through-national-student-competition/</t>
+          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>April 1, 2026 - The event – which was sponsored by Sika, WorldsView, BVI, RIBCCS, and AF Consulting – was hosted at SAICE House in Midrand, Gauteng, and accredited for 0.2 CPD points. Students were invited to present their civil engineering university research and investigation project, which is part of the national curriculum for final year civil engineering undergraduate students.</t>
+          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2505,26 +2513,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>info@swmcommunications.co.za, nthabeleng@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
+          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>September 7, 2025 - Find the list of upcoming Civil Engineering conferences in South Africa 2025 with invitation an letter.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2532,22 +2536,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>ernao@crown.co.za, constr@crown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
+          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
+          <t>September 7, 2025 - Find the list of upcoming Civil Engineering conferences in South Africa 2025 with invitation an letter.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2560,17 +2568,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
+          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
+          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Civil engineering conferences in Cape town 2025 provide an exclusive global platform to meet and engage with experts and aspirants in various fields.</t>
+          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2583,22 +2591,22 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -2606,49 +2614,49 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Civil Engineering Competition - Christian Brothers University</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://www.cbu.edu/civil-engineering-competition/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>August 14, 2023 - Gather a team (2-5 members) to compete in CBU’s Civil Engineering Competition September 18, 2023, when up to six teams in each category will test their skills for the judges, CBU’s renowned engineering professors.</t>
+          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>jkaufma1@cbu.edu, info@cbu.edu</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Civil Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Apr 13 International Conference on Architectural, Civil and Environmental Engineering (ICACEE) - Cape Town, South Africa</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -2656,17 +2664,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>List of ALL Engineering Bursaries South Africa 2027</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2679,17 +2687,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
+          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2706,17 +2714,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>APPLY NOW! WORLDSKILLS SOUTH AFRICA NATIONAL COMPETITION 2025</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>ndidate with an accredited qualification in the related skill - Candida. e must not turn 23 years old in 2026 for the skills required. - Candidate applying for Aircraft Maintenance, Mechatr.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2729,17 +2737,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>SAIMechE</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.saimeche.org.za/</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2752,99 +2760,95 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent's largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
+          <t>South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits · Become a SAIEE Member today! SAIEE Membership · Earn CPD credits · About Training Academy · Join a SAIEE Centre near you! Centres · South African Institute of Electrical Engineers (SAIEE) 01 ·</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr"/>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>List of ALL Engineering Bursaries South Africa 2027</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -2852,22 +2856,22 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
+          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -2875,22 +2879,22 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -2898,17 +2902,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits · Become a SAIEE Member today! SAIEE Membership · Earn CPD credits · About Training Academy · Join a SAIEE Centre near you! Centres · South African Institute of Electrical Engineers (SAIEE) 01 ·</t>
+          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2916,26 +2920,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
-        </is>
-      </c>
+      <c r="E102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers (SAIEE ...</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - IEEE ZA 5G Competition</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.edufunds.co.za/saiee-bursary-south-africa-2027/</t>
+          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51397</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Aug 15, 2026 · Apply for the South African Institute of Electrical Engineers (SAIEE) Bursary 2027. Learn about the eligibility requirements, electrical engineering study options, bursary benefits, required documents, and how to apply before the closing date.</t>
+          <t>Form templates: Template for a Cover Sheet for the Competition on Ideas, Designs and Applications for 5G and Beyond South Africa (.docx) [Click to Download] Template for a Resume for the Student (.docx) [Click to Download] ... Help (FAQ) • Privacy Statement • Terms &amp; Conditions The SAIEE is ...</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2943,26 +2943,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>Admin@edufunds.co.za, reception@saiee.org.za, dudum@saiee.org.za</t>
-        </is>
-      </c>
+      <c r="E103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>Student Design Competition | IEEE CASS</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://ieee-cas.org/society-involvement/student-design-competition</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>CASS will reimburse the travel costs for the trip to ISCAS 2026 for the four finalists, one for each region - Regions 1-7 (USA and Canada), Region 8 (Europe, Middle East, Africa), Region 9 (Latin America), and Region 10 (Asia, Australia, Pacific), as well as ISCAS registration.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2975,17 +2971,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - SA Computing Olympiad stars hold their own in international competition</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51457</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>July 20, 2021 - For the other three South African team members, this was their first IOI. Brent Butkow finished ranked 342, Jean Weight finished in 287th position and Faran Steenkamp was ranked 280. In addition to the serious IOI contest days, host country Singapore arranged several fun events where Faran Steenkamp was placed third in the sponsored Code Cup, and won a cash prize of 200 USD.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2993,58 +2989,50 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Competitions | ESG</t>
+          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators - Lifestyle &amp; Tech</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://za.rs-online.com/web/content/m/competition</t>
+          <t>https://lifestyleandtech.co.za/company-news/article/2026-06-29/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africas-next-generation-of-innovators</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
+          <t>June 29, 2026 - After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant exhibition showcasing the remarkable ...</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>example@email.com</t>
-        </is>
-      </c>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>List of ALL Engineering Bursaries South Africa 2027</t>
+          <t>Houghton hackathon: Stepping stone for future engineers | Rosebank Killarney Gazette</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
+          <t>https://www.citizen.co.za/rosebank-killarney-gazette/news-headlines/local-news/2026/06/23/houghton-hackathon-stepping-stone-for-future-engineers/</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
+          <t>June 23, 2026 - Hosted by ORT South Africa in partnership with Hudaco, the hackathon has brought together 55 learners from underserved communities to work together in developing solutions to challenges they face in their communities.</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>engineering hackathon South Africa</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
@@ -3052,68 +3040,76 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Budding engineers showcase innovation at YEM hackathon | ITWeb</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.itweb.co.za/article/budding-engineers-showcase-innovation-at-yem-hackathon/kYbe97XbP4ZqAWpG</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>June 30, 2026 - The hackathon was hosted by Johannesburg-based non-profit education and training organisation ORT South Africa, in partnership with JSE-listed industrial and engineering supplies firm Hudaco.</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr"/>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>enquiries@ombudsman.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>Young Engineers Showcase Innovation at STEM Hackathon</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://www.futuresa.co.za/education/young-engineers-movement-stem/</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>June 11, 2026 - Fifty-five high school learners and 11 teachers from underserved South African schools will showcase working engineering and technology prototypes at the Young Engineers Movement (YEM) Hackathon Exhibition Day on 26 June 2026.</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr"/>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>info@futuresa.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
+          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
+          <t>https://novuspressbulletin.co.za/blog/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africa-s-next-generation-of-innovators</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
+          <t>June 30, 2026 - ... Johannesburg, June 2026 – After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant ...</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>engineering hackathon South Africa</t>
         </is>
       </c>
       <c r="E110" t="inlineStr"/>
@@ -3121,40 +3117,44 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - IEEE ZA 5G Competition</t>
+          <t>55 learners from underserved schools showcase engineering innovations at Johannesburg hackathon</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51397</t>
+          <t>https://iol.co.za/saturday-star/2026-07-01-55-learners-from-underserved-schools-showcase-engineering-innovations-at-johannesburg-hackathon/</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Form templates: Template for a Cover Sheet for the Competition on Ideas, Designs and Applications for 5G and Beyond South Africa (.docx) [Click to Download] Template for a Resume for the Student (.docx) [Click to Download] ... Help (FAQ) • Privacy Statement • Terms &amp; Conditions The SAIEE is ...</t>
+          <t>July 29, 2026 - Fifty-five high school learners ... at the Young Engineers Movement (YEM) Hackathon Exhibition Day in Johannesburg last week, presenting working prototypes designed to solve real-world problems affecting their communities. The learners, accompanied by 11 teachers, took part in the five-day hackathon, hosted by ORT South Africa in partnership with Hudaco, from June 22 to 26....</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr"/>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>yasmine.jacobs@iol.co.za, pholoso.manyama@inl.co.za, wendy.dondolo@inl.co.za, pholoso.manyama@iol.co.za, verna.vandiemen@inl.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>The Home of South African Hackathons</t>
+          <t>ORT South Africa's inaugural YEM Hackathon empowers future STEM innovators</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/</t>
+          <t>https://www.futuresa.co.za/bursaries-and-scholarships/ort-south-africa-yem-hackathon/</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+          <t>July 30, 2026 - ORT South Africa's first Young Engineers Movement Hackathon saw 55 learners develop innovative STEM solutions during a five-day competition.</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3162,22 +3162,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>info@futuresa.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ICEP - Tshwane Varsity Hackathon</t>
+          <t>Young Engineers Movement Hackathon opens doors to future career choices | Rosebank Killarney Gazette</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>https://tvh.icep.co.za/</t>
+          <t>https://www.citizen.co.za/rosebank-killarney-gazette/news-headlines/local-news/2026/07/06/hackathon-sparks-solutions/</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Tshwane Varsity Hackathon South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
+          <t>July 6, 2026 - 55 learners put ideas to paper, developing prototypes at the Young Engineers Movement (YEM) Hackathon. The ideas they came up with at the five-day hackathon in Houghton Estate, hosted by ORT South Africa, were to solve leading community issues, ...</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3185,26 +3189,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>MagasengQM@tut.ac.za, info@tvh.co.za</t>
-        </is>
-      </c>
+      <c r="E113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Hackathons en South Africa</t>
+          <t>Southern Africa Digital ID Hackathon</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/</t>
+          <t>https://www.africa.engineering.cmu.edu/events/2024/11/21-southern-digital-hackathon.html</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+          <t>Learn more and register for Southern Africa Digital ID Hackathon · January 23 2026 · 12:00 PM - 1:30 PM CAT · Carnegie Mellon University Africa · Customizing the CV to the job description · Learn more about this event by contacting Paul Swaga.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3217,17 +3217,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Unisa hosts first-ever Hackathon to ignite student learning experience</t>
+          <t>PATH South Africa co-hosts Harvard Health Hackathon | PATH</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
+          <t>https://www.path.org/our-impact/articles/path-south-africa-co-hosts-harvard-health-hackathon/</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Unisa's Information and Communication Technology Portfolio, in collaboration with the College of Science, Engineering and Technology, held the first-ever Unisa Hackathon on 3 and 4 July 2025, marking a major step in the university's journey to embed digital innovation and entrepreneurship into the students learning experience.</t>
+          <t>The South Africa hackathon location was at the University of Cape Town (UCT) and dubbed the UCT Hub. It attracted over 80 applicants from diverse fields, including medicine, engineering, research, and software development.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3236,152 +3236,6 @@
         </is>
       </c>
       <c r="E115" t="inlineStr"/>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>The Home of South African Hackathons</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>https://hackon.co.za/partners/</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr"/>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>Build the Future with Entelect Hackathons</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>https://challenge.entelect.co.za/</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>Build the Future with Entelect Hackathons Join South Africa's premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr"/>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>Nedbank Hackathon</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>https://nedbankhackathon.co.za/</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>The hackathon invitation is aimed at frontend, backend and full stack software developers, ideally at an intermediate or advanced levels of proficiency in either Java, C++, React, or Python.</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr"/>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>Young Engineers Movement (YEM) - ORT SA</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>Talks &amp; Fireside | Builders Table</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>https://builderstable.net/</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>Builders Table is a two-day hackathon hosted by MakeReign, built around a 24-hour build sprint. It brings together South Africa's designers, developers, strategists, founders and creative technologists to build real working prototypes under real time pressure.</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>liamlr95@gmail.com, sarah.chen@horizonlabs.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>CompeteHub - Where Champions Are Made</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>https://www.devpluxe.co.za/</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-09-22
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E115"/>
+  <dimension ref="A1:E118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global ...</t>
+          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The competition offers the team an opportunity to showcase South African engineering talent on an international stage while benchmarking their skills against global peers. Beyond the event, the team aims to bring back new knowledge and inspiration, contributing to the growth of local expertise in space science and engineering.</t>
+          <t>August 6, 2026 - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -469,17 +469,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Some of our sparkling achievements during 2014 – to help the NRF and DSI grow a representative science and technology workforce in the country – SAASTA has run a number of maths and science educator development programmes and a number of learner development programmes, including maths and science camps for learners with potential, olympiads and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -487,26 +487,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>The IEOM UNDERGRADUATE Student Paper Competition Sponsored by SIEMENS will recognize outstanding papers in the field of industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management and operations management written by student(s). Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South ...</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -514,26 +510,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026 South Africa Engineering Competition</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://notices.ukzn.ac.za/content/GetFile.aspx?id=96048</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Best Regards, The 2026 SA Engineering Competition Team University of KwaZulu-Natal • Elsevier</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -546,17 +538,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026 South Africa Engineering</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://notices.ukzn.ac.za/content/GetFile.aspx?id=96047</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>UKZN and Elsevier. If you are an engineering student (undergraduate or postgraduate), don't miss joining the challenge to solve real-world cases using Engineering Village and Knovel.</t>
+          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -564,22 +556,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>user@domain.com, info@zasdc.org</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.thecasecentre.org/products/view?id=189255</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -592,17 +588,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -615,17 +611,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa. Find out more</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -633,22 +629,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -656,26 +656,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
+          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Eligibility Benchmark Requirements The Africa Prize is open to individuals or teams based in sub-Saharan Africa with a scalable engineering innovation that demonstrates social or environmental impact potential. Applicants must: Be citizens ordinarily residing in a sub-Saharan African country. Be over 18 years old and fluent in English.</t>
+          <t>August 14, 2026 - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -698,7 +694,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Exhibition Opportunities BENEFITS FOR YOUR PARTICIPATING IN THE EXHIBITION: An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms.</t>
+          <t>Apr 16, 2026 · Exhibition Opportunities BENEFITS FOR YOUR PARTICIPATING IN THE EXHIBITION: An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -708,24 +704,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, sithabile@innovate.durban, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, Erika@innovate.durban, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, sithabile@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, Erika@innovate.durban, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, c183baa23371454f99f417f6616b724d@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
+          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://10times.com/southafrica/tradeshows</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
+          <t>South Africa trade shows, find and compare 970 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 156 upcoming expos in 2026-2027 1. China Homelife Fair South Africa, 2.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -733,26 +729,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>enquiries@aiexpoafrica.com</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -760,22 +752,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>dataprivacy@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, support@informaconnect.com, customerservices@knect365.com, customerservices@informaconnect.com, support@knect365.com</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://innovationweek.co.za/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Big Data and Business Analytics Innovation Conference Johannesburg, South Africa IT &amp; Technology 102 Members Tue, 22 - Thu, 24 Sep 2026</t>
+          <t>SA Innovation Week 2026 is South Africa’s official national innovation platform accelerating implementation, commercialisation and impact.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -783,22 +779,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>info@pixal8media.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://innovationweek.co.za/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SA Innovation Week 2026 is South Africa's official national innovation platform accelerating implementation, commercialisation and impact.</t>
+          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -808,24 +808,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>info@pixal8media.co.za</t>
+          <t>enquiries@aiexpoafrica.com</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what’s next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -833,26 +833,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>dataprivacy@knect365.com, support@knect365.com, customerservices@knect365.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, support@informaconnect.com</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
+          <t>South Africa International Industrial Expo | Innovation Bridge</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
+          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
+          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -865,17 +861,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>South Africa Manufacturing Show 2027 | Tech Event</t>
+          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://manufacturingitsummit.com/south-africa/</t>
+          <t>https://madeinafricaevent.co.za/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Attend South Africa Manufacturing Show on 25 June 2027 to connect with 200+ manufacturing leaders driving AI, smart factories, automation, and innovation.</t>
+          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -883,26 +879,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>enquiry@exito-e.com</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 - Technology Expo · October 10</t>
+          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Joburg! TECHSPO Johannesburg is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology. See why people keep coming back year after year! Register and secure your pass today.</t>
+          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -910,26 +902,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>info@techspojoburg.co.za</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 - Technology Expo · October 6</t>
+          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Where Business, Tech and Innovation Collide in Cape Town! TECHSPO Cape Town is an annual 2 day Technology Expo which showcases the next generation of technology &amp; innovation, including; Internet, Mobile, AdTech, MarTech &amp; SaaS Technology.</t>
+          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -937,26 +925,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>info@techspocapetown.co.za</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
+          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -964,26 +948,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Oct 16, 2024 · Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
+          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -991,22 +971,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of ...</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Aug 4, 2025 · The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
+          <t>... On 30-31 March 2026, 109 students from 9 schools walked into the University of Cape Town and designed a city on the Moon. They elected leaders, divided into engineering departments, and spent 24 hours responding to a professional design brief.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1016,24 +1000,24 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
+          <t>user@domain.com, info@zasdc.org</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Engineering For People Design Challenge - EWBSA</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1041,26 +1025,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge - Engineers Without ...</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
+          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1068,22 +1048,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>ied@ied.org.uk</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineering ENGINEERING FOR PEOPLE Design challenge DESIGN ...</t>
+          <t>Engineers Without Borders South ...</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/wp-content/uploads/2024/08/2024_25_Engineering_for_People_Design_Challenge_Makers_Valley.pdf</t>
+          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>These topics are at the centre of South Africa’s National Development Plan (NDP) 2030 and can provide insight into the main developmental challenges that are critical to South Africa.</t>
+          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1096,17 +1080,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Oct 24, 2024 · The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
+          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1116,24 +1100,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>team@crowdsolve.net</t>
+          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
+          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1146,17 +1130,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1164,26 +1148,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>ied@ied.org.uk</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1265,17 +1245,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1288,17 +1268,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1496,7 +1476,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
+          <t>u003einfo@techspo.co, atinfo@techspo.coor</t>
         </is>
       </c>
     </row>
@@ -1523,24 +1503,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>partner@africatechnologyexpo.com, info@sparkafrica.co, johndoe@email.com</t>
+          <t>partner@africatechnologyexpo.com, johndoe@email.com, info@sparkafrica.co</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>Home - Mediatech Africa | South Africa</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://www.mediatech.co.za/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
+          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1550,24 +1530,24 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>info@techspocapetown.co.za</t>
+          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1577,24 +1557,24 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>dataprivacy@knect365.com, support@knect365.com, customerservices@knect365.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, dataprivacy@informaconnect.com, support@informaconnect.com</t>
+          <t>info@techspocapetown.co.za</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Home - Mediatech Africa | South Africa</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://www.mediatech.co.za/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1604,7 +1584,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>simon@mediatech.co.za, claire@mediatech.co.za</t>
+          <t>dataprivacy@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, support@informaconnect.com, customerservices@knect365.com, customerservices@informaconnect.com, support@knect365.com</t>
         </is>
       </c>
     </row>
@@ -1657,17 +1637,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in Johannesburg, List of all Johannesburg Technology Business Expo &amp; Events in South Africa</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://10times.com/johannesburg-za/technology</t>
+          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Explore a diverse array of IT &amp; Technology events in Johannesburg (South Africa). Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience.</t>
+          <t>TECHSPO Johannesburg – Where Business, Tech and Innovation Collide in Johannesburg, South Africa. TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1675,7 +1655,11 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>you@company.com, colleague@company.com, your@email.com, support@industryevents.com, events@techspojoburg.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1690,7 +1674,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>The aim of a Maker Faire Africa is to create a space on the African continent where Afrigadget-type innovations, inventions and initiatives can be sought, identified, brought to life, supported, amplified and propagated.</t>
+          <t>March 7, 2025 - Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds ...</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1703,17 +1687,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Maker Faire - Wikipedia</t>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Maker_Faire</t>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1726,17 +1710,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Maker Faire Africa — Grokipedia</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://grokipedia.com/page/maker_faire_africa</t>
+          <t>http://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
+          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1744,22 +1728,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>fancybox_loading@2x.gif, pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Maker Faire groups | Meetup</t>
+          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/topics/maker-faire/za/</t>
+          <t>https://makerfairecapetown.wordpress.com/about/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
+          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1772,17 +1760,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
+          <t>Blog : Maker Faire Africa</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
+          <t>http://makerfaireafrica.com/blog/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Aug 21, 2015 · We’re delighted to present the first ever Cape Town Maker Faire, hosted by Open Design in partnership with Trimble.Maker Faire is primarily designed as a forward-looking event, showcasing makers who are exploring new forms and new technologies.</t>
+          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building his ANIMAL car, from the ground up, that means the frame and all.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1795,17 +1783,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Maker Faire Africa - Facebook</t>
+          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/MFAJoburg/</t>
+          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Jul 24, 2020 · Pizza, beer &amp; wine will be served during the film and a brief Q&amp;A about the Maker Movement will take place directly after the film, for anyone who wishes to participate.</t>
+          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1813,22 +1801,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>00-Header-Bahamas-IMG_6749@a.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Upcoming Faires - Maker Faire</t>
+          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://makerfaire.com/upcoming-faires/</t>
+          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future.</t>
+          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1836,31 +1828,27 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>chosen-sprite@2x.png, fancybox_sprite@2x.png, pr@make.co, fancybox_loading@2x.gif</t>
-        </is>
-      </c>
+      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>Makers Festival SA 🛠️ (@makersfestival_sa) • Instagram photos ...</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.instagram.com/makersfestival_sa/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
+          <t>8,503 Followers, 58 Following, 57 Posts - Makers Festival SA 🛠️ (@makersfestival_sa) on Instagram: "🛠️ Building Skills. Building Memories. 🏕️ 8th &amp; 9th November 2025 / Cape Town, SA 🪵 Founder @hutch_custom 📩 DM us - apply to be a MAKER 🫶🏼"</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
+          <t>maker faire South Africa</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -1868,22 +1856,22 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>Why Africa needs Maker Faire | ZDNET</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage ...</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
+          <t>maker faire South Africa</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -1891,44 +1879,44 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Capetown 2026</t>
+          <t>HOME | MAKERS FEST</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
+          <t>https://www.makersfestival.co.za/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
+          <t>At Makers Festival SA, you get full access to every hands-on workshop, from woodworking and ceramics to leatherwork, painting, and more.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>stem competition South Africa</t>
+          <t>maker faire South Africa</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, example@mysite.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, warren@makersfestival.co.za, 8c4075d5481d476e945486754f783364@sentry.io</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Astemi Sa</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1941,17 +1929,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1964,17 +1952,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1987,17 +1975,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>Astemi Sa</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2010,17 +1998,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024 - IEOM Society</t>
+          <t>High School STEM Competition | Capetown 2026</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas.</t>
+          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2037,17 +2025,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
+          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
+          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2060,17 +2048,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Register your school for Samsung Solve for Tomorrow 2026</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://www.sowetan.co.za/careers/2026-03-03-register-your-school-for-samsung-solve-for-tomorrow-2026/</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Register your school for Samsung Solve for Tomorrow 2026 STEM competition aims to transform and empower South African learners with critical skills to solve real-world challenges March 03, 2026 at 7:44 am</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2078,107 +2066,95 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>ssasft@samsung.com</t>
-        </is>
-      </c>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Robotics Competition | WRO South Africa | Gauteng</t>
+          <t>PDF Department of Basic Education and Samsung South Africa Partner to ...</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://www.wrosa.co.za/</t>
+          <t>https://www.education.gov.za/Portals/0/Media/Preess+Releases/2026+Media+Releases/Applications+for+2026+Samsung+Solve+For+Tomorrow.pdf</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>WRO South Africa ( World Robot Olympiad ) is a robotics competition which brings together young people from all over the world to develop their creativity and problem-solving skills.</t>
+          <t>The 2026 competition is guided by the theme: "Innovate for Tomorrow: STEM Solutions for Sustainable Communities." Samsung Solve for Tomorrow is a global innovation competition that empowers Grade 10 and 11 learners in public schools to design science, technology, engineering and mathematics (STEM) solutions that address real-world challenges within their communities.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com</t>
-        </is>
-      </c>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>South Africa to host first World Robot Olympiad International Final in Africa in 2028 - WRO Association</t>
+          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://wro-association.org/south-africa-to-host-first-world-robot-olympiad-international-final-in-africa-in-2028/</t>
+          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>5 days ago - One of the world's largest ... South Africa, 12 September 2026 — South Africa will host the World Robot Olympiad (WRO®) International Final in 2028, bringing WRO's flagship global robotics...</t>
+          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Prithul-3rd-place-Future-Engineers-2022-A-500x383@2x.jpg, Costa-Rica-team-Sprout-release-banner-500x383@2x.jpg, Annual-report-article-TZ-500x383@2x.jpg, 1-Team-CARED-Philippines-500x383@2x.jpg</t>
-        </is>
-      </c>
+          <t>stem competition South Africa</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
+          <t>National Department of Basic Education</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
+          <t>https://www.education.gov.za/LinkClick.aspx?fileticket=i9GS5Atf7zo=&amp;tabid=347&amp;portalid=0&amp;mid=14629</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>April 14, 2026 - This National Event, to be held at the Sandton Convention Centre in Johannesburg, South Africa, as part of AI for Good Impact Africa, at AI Expo Africa 2025, is a qualifying tournament leading to the Grand Finale in Geneva during the AI for ...</t>
+          <t>JOHANNESBURG, South Africa - XX Month 2026 - The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries ...</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>robotics competition South Africa</t>
+          <t>stem competition South Africa</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>name@example.com</t>
+          <t>ssasft@samsung.com, s.ngcobo@cheil.com, j.mogoeng@samsung.com</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Cape Town to host Africa’s first World Robot Olympiad</t>
+          <t>Robotics Competition | WRO South Africa | Gauteng</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>https://www.capetownetc.com/tech/cape-town-africas-first-world-robot-olympiad/</t>
+          <t>https://www.wrosa.co.za/</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>5 hours ago - Cape Town will host the World Robot Olympiad (WRO) International Final in 2028, bringing one of the world’s largest youth robotics competitions to Africa for the first time, Cape {town} Etc reports.</t>
+          <t>WRO South Africa ( World Robot Olympiad ) is a robotics competition which brings together young people from all over the world to develop their creativity and problem-solving skills.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2186,22 +2162,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>FIRST South Africa – Robotics Programs for School Children</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://firstsa.org/</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
+          <t>April 14, 2026 - This National Event, to be held at the Sandton Convention Centre in Johannesburg, South Africa, as part of AI for Good Impact Africa, at AI Expo Africa 2025, is a qualifying tournament leading to the Grand Finale in Geneva during the AI for ...</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2209,22 +2189,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>name@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2232,22 +2216,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, info@thecortexhub.africa, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, c183baa23371454f99f417f6616b724d@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>South African Robotics Competitions and Schools</t>
+          <t>Robotics for Good Youth Challenge South Africa</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://www.sciencexpo.org.za/robotics.html</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
+          <t>Apr 25, 2025 · The Robotics for Good Youth Challenge South Africa is a national event in a global robotics competition on disaster response, leading to the AI for Good Summit 2025.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2257,24 +2245,24 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>marna.vanzyl@imbewu.foundation, webmaster@sciencexpo.org.za, madelien@imbewu.foundation</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Robotics &amp; Coding Classes for Kids in Johannesburg | Robotics League</t>
+          <t>VEX Events: Official Competition Website for VEX Robotics</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://robotics-league.co.za/</t>
+          <t>https://events.vex.com/</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026 Theme · Robots Meet Culture. The World Robot Olympiad is the planet's biggest student robotics competition — over 100 countries, 100,000+ students a year. South African teams compete on two tracks: Explorer, the home-grown SA challenge, ...</t>
+          <t>12 hours ago · Official Competition Website for VEX Robotics Robot Skills - IQ Elementary / Middle School Robot Skills - V5 Middle / High School Robot Skills - VEX U Collegiate / University</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2282,26 +2270,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>info@roboticsleague.co.za, you@email.com</t>
-        </is>
-      </c>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
+          <t>South Africa to host first World Robot Olympiad International Final in Africa in 2028 - WRO Association</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
+          <t>https://wro-association.org/south-africa-to-host-first-world-robot-olympiad-international-final-in-africa-in-2028/</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
+          <t>5 days ago - One of the world's largest ... South Africa, 12 September 2026 — South Africa will host the World Robot Olympiad (WRO®) International Final in 2028, bringing WRO's flagship global robotics...</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2311,24 +2295,24 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>rampedim@atnews.co.za, NkosiN@atnews.co.za</t>
+          <t>1-Team-CARED-Philippines-500x383@2x.jpg, Costa-Rica-team-Sprout-release-banner-500x383@2x.jpg, Prithul-3rd-place-Future-Engineers-2022-A-500x383@2x.jpg, Annual-report-article-TZ-500x383@2x.jpg</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
+          <t>Cape Town to host Africa’s first World Robot Olympiad</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
+          <t>https://www.capetownetc.com/tech/cape-town-africas-first-world-robot-olympiad/</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>AfrikaBot is affordable because you can build a competitive robot for a lot less with the correct advice. AfrikaBOT is South Africa's first robotics competition for high school teenagers and university undergraduates who are smart enough to build their own robots from electronic parts rather ...</t>
+          <t>1 day ago - Cape Town will host the World Robot Olympiad (WRO) International Final in 2028, bringing one of the world’s largest youth robotics competitions to Africa for the first time, Cape {town} Etc reports.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2341,49 +2325,45 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Civil engineering Tenders SA - 72 Open | September 2026 ...</t>
+          <t>FIRST South Africa – Robotics Programs for School Children</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://www.tenderflow.co.za/categories/civil-engineering/</t>
+          <t>https://firstsa.org/</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>3 days ago · Browse 72 active civil engineering tenders in South Africa. Updated daily with government, SOE &amp; private sector opportunities. Free alerts on TenderFlow.</t>
+          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>support@tenderflow.co.za</t>
-        </is>
-      </c>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://civils.org.za/</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
+          <t>robotics competition South Africa</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -2391,25 +2371,29 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Civil Engineering Tenders — 270 open listings, updated 21 ...</t>
+          <t>South African Robotics Competitions and Schools</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://tenderbulletins.co.za/tender-category/civil-engineering/</t>
+          <t>https://www.sciencexpo.org.za/robotics.html</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Browse current and past Civil Engineering tenders published by South African government departments, municipalities, state-owned entities and private companies looking to procure civil engineering.</t>
+          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr"/>
+          <t>robotics competition South Africa</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>madelien@imbewu.foundation, webmaster@sciencexpo.org.za, marna.vanzyl@imbewu.foundation</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2441,17 +2425,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>The South African Institution of Civil Engineering</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
+          <t>https://civils.org.za/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
+          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2459,26 +2443,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za, advertising@creamermedia.co.za, chanel@engineeringnews.co.za, newsletters@creamermedia.co.za</t>
-        </is>
-      </c>
+      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd International Bridge Building Competition - SAICE</t>
+          <t>ICE Africa - Supporting Civil Engineers in Africa</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://saice.org.za/press-releases/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>April 17, 2025 - The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
+          <t>ICE Africa supports civil engineers across the continent, providing access to qualifications, training, and networking opportunities for professional growth.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2486,26 +2466,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>marketing@saice.org.za, civilinfo@saice.org.za, accounts@saice.org.za, communications@saice.org.za, membership@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
+          <t>Engineering the Future: 16 schools compete in SAICE's 33rd ...</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
+          <t>https://southafricatoday.net/lifestyle/education/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted its 33 rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland. The very first SAICE Bridge Building Competition was held in 1991, and it aimed to encourage high school learners to apply their knowledge of mathematics and science in a ...</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2518,17 +2494,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>The South African Institution of Civil Engineering (SAICE)</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
+          <t>https://m.facebook.com/pages/The-South-African-Institution-of-Civil-Engineering-SAICE/92946824896/</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
+          <t>📢 Call for Abstracts: Structural Engineering Conference 2026 This inaugural conference brings together four leading industry institutions - the South African Institution of Civil Engineering (SAICE), the South African Institute of Steel Construction (SAISC), the Concrete Society of Southern Africa, and York Timbers in collaboration with the ...</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2536,26 +2512,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>ernao@crown.co.za, constr@crown.co.za</t>
-        </is>
-      </c>
+      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
+          <t>Home - SAICE</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
+          <t>https://saice.org.za/</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>September 7, 2025 - Find the list of upcoming Civil Engineering conferences in South Africa 2025 with invitation an letter.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2563,22 +2535,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>civilinfo@saice.org.za, marketing@saice.org.za, membership@saice.org.za, communications@saice.org.za, accounts@saice.org.za, barbara@avenue.co.za, executiveadmin@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
+          <t>Aqualibrium: Empowering Future Engineers Through Hands-On Water ...</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
+          <t>https://saice.org.za/press-releases/aqualibrium-empowering-future-engineers-through-hands-on-water-distribution-challenge/</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
+          <t>The recent finals of Aqualibrium, hosted by the South African Institution of Civil Engineering (SAICE), provided an exciting platform for students to immerse themselves in the world of water distribution and infrastructure. This annual event continues to highlight the significance of water management and the role of civil engineering in sustainable development. Recently held at […]</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2586,27 +2562,31 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>civilinfo@saice.org.za, marketing@saice.org.za, membership@saice.org.za, communications@saice.org.za, accounts@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
+          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -2614,49 +2594,45 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>SAICE Aqualibrium 2025: High School Students Rise to the Challenge in ...</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://southafricatoday.net/environment/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted the thrilling 2025 Aqualibrium Competition National Finals this past week, which brought together high school students from schools all over South Africa at the Sci-Bono Discovery Centre in Johannesburg. The event continues to be an important platform for fostering engineering talent, inspiring young minds, and raising awareness ...</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+          <t>civil engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>SAICE | Events and Awards</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://members.saice.org.za/events-and-awards</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>The South African Institution Of Civil Engineering SAICE hosts the Awards Function annually to honour individuals, projects of excellence, as well as community-oriented initiatives. The annual awards function gives companies and individuals a unique opportunity to showcase their deserving projects and work to the industry.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -2664,17 +2640,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>List of ALL Engineering Bursaries South Africa 2027</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2687,17 +2663,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2714,17 +2690,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>APPLY NOW! WORLDSKILLS SOUTH AFRICA NATIONAL COMPETITION 2025</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>ndidate with an accredited qualification in the related skill - Candida. e must not turn 23 years old in 2026 for the skills required. - Candidate applying for Aircraft Maintenance, Mechatr.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2737,17 +2713,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>List of ALL Engineering Bursaries South Africa 2027</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2760,49 +2736,45 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers (SAIEE) About Us See Member Benefits · Become a SAIEE Member today! SAIEE Membership · Earn CPD credits · About Training Academy · Join a SAIEE Centre near you! Centres · South African Institute of Electrical Engineers (SAIEE) 01 ·</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>Engineering Competition For African Youth In Engineering ...</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
+          <t>Aug 18, 2025 · The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent’s largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -2810,22 +2782,22 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>SAIMechE</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.saimeche.org.za/</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -2833,17 +2805,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions. Whether you're working in traditional engineering fields or applying innovation in areas like health, agriculture, or digital technology, the Africa Prize for Engineering Innovation offers a unique platform to ...</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2856,17 +2828,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
+          <t>South African Institute of Electrical Engineers 18a Gill Street Observatory Johannesburg South Africa Phone: +27 (0)11 487 3003 Email: reception@saiee.org.za Powered by</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2874,22 +2846,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2902,17 +2878,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
+          <t>IEEE-IAS Industrial Power Conversion Systems Department Serving the electrical energy conversion professional worldwide</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2925,17 +2901,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - IEEE ZA 5G Competition</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51397</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Form templates: Template for a Cover Sheet for the Competition on Ideas, Designs and Applications for 5G and Beyond South Africa (.docx) [Click to Download] Template for a Resume for the Student (.docx) [Click to Download] ... Help (FAQ) • Privacy Statement • Terms &amp; Conditions The SAIEE is ...</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2943,22 +2919,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Student Design Competition | IEEE CASS</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://ieee-cas.org/society-involvement/student-design-competition</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>CASS will reimburse the travel costs for the trip to ISCAS 2026 for the four finalists, one for each region - Regions 1-7 (USA and Canada), Region 8 (Europe, Middle East, Africa), Region 9 (Latin America), and Region 10 (Asia, Australia, Pacific), as well as ISCAS registration.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2971,17 +2951,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - SA Computing Olympiad stars hold their own in international competition</t>
+          <t>Engineering students compete in global high-performance computing ...</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51457</t>
+          <t>https://ebe.uct.ac.za/articles/2026-05-29-engineering-students-compete-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>July 20, 2021 - For the other three South African team members, this was their first IOI. Brent Butkow finished ranked 342, Jean Weight finished in 287th position and Faran Steenkamp was ranked 280. In addition to the serious IOI contest days, host country Singapore arranged several fun events where Faran Steenkamp was placed third in the sponsored Code Cup, and won a cash prize of 200 USD.</t>
+          <t>At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025. Now, Team UCT is preparing to represent South Africa at the global finals in Germany later this year.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2989,50 +2969,58 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>ebe-faculty@uct.ac.za</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators - Lifestyle &amp; Tech</t>
+          <t>Competitions | ESG</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://lifestyleandtech.co.za/company-news/article/2026-06-29/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africas-next-generation-of-innovators</t>
+          <t>https://za.rs-online.com/web/content/m/competition</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>June 29, 2026 - After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant exhibition showcasing the remarkable ...</t>
+          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr"/>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>example@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Houghton hackathon: Stepping stone for future engineers | Rosebank Killarney Gazette</t>
+          <t>List of ALL Engineering Bursaries South Africa 2027</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://www.citizen.co.za/rosebank-killarney-gazette/news-headlines/local-news/2026/06/23/houghton-hackathon-stepping-stone-for-future-engineers/</t>
+          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>June 23, 2026 - Hosted by ORT South Africa in partnership with Hudaco, the hackathon has brought together 55 learners from underserved communities to work together in developing solutions to challenges they face in their communities.</t>
+          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
@@ -3040,44 +3028,44 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Budding engineers showcase innovation at YEM hackathon | ITWeb</t>
+          <t>Apply Now: Africa Prize for Engineering Innovation 2026 Offers R1 ...</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://www.itweb.co.za/article/budding-engineers-showcase-innovation-at-yem-hackathon/kYbe97XbP4ZqAWpG</t>
+          <t>https://stepapp.co.za/2025/08/27/apply-now-africa-prize-for-engineering-innovation-2026-offers-r1-million-top-prize/</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>June 30, 2026 - The hackathon was hosted by Johannesburg-based non-profit education and training organisation ORT South Africa, in partnership with JSE-listed industrial and engineering supplies firm Hudaco.</t>
+          <t>The Royal Academy of Engineering has officially launched the Africa Prize for Engineering Innovation 2026, a prestigious pan-African competition designed to support and accelerate engineering entrepreneurs who are developing scalable solutions to local challenges. This initiative, now in its 12th year, offers African innovators a unique opportunity to gain access to vital funding, mentorship ...</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>enquiries@ombudsman.org.za</t>
+          <t>info@stepapp.co.za, Africa.Prize@raeng.org.uk</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Young Engineers Showcase Innovation at STEM Hackathon</t>
+          <t>The Home of South African Hackathons</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://www.futuresa.co.za/education/young-engineers-movement-stem/</t>
+          <t>https://hackon.co.za/</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>June 11, 2026 - Fifty-five high school learners and 11 teachers from underserved South African schools will showcase working engineering and technology prototypes at the Young Engineers Movement (YEM) Hackathon Exhibition Day on 26 June 2026.</t>
+          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3085,26 +3073,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>info@futuresa.co.za</t>
-        </is>
-      </c>
+      <c r="E109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Young Engineers Shine as Inaugural YEM Hackathon Celebrates South Africa's Next Generation of Innovators</t>
+          <t>Hackathons en South Africa</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://novuspressbulletin.co.za/blog/young-engineers-shine-as-inaugural-yem-hackathon-celebrates-south-africa-s-next-generation-of-innovators</t>
+          <t>https://za.allhackathons.com/</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>June 30, 2026 - ... Johannesburg, June 2026 – After five inspiring days of innovation, collaboration, and problem-solving, the inaugural Young Engineers Movement (YEM) Hackathon, hosted by ORT South Africa in partnership with Hudaco, concluded with a vibrant ...</t>
+          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3117,17 +3101,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>55 learners from underserved schools showcase engineering innovations at Johannesburg hackathon</t>
+          <t>Young Engineers Showcase Innovation at STEM Hackathon</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://iol.co.za/saturday-star/2026-07-01-55-learners-from-underserved-schools-showcase-engineering-innovations-at-johannesburg-hackathon/</t>
+          <t>https://www.futuresa.co.za/education/young-engineers-movement-stem/</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>July 29, 2026 - Fifty-five high school learners ... at the Young Engineers Movement (YEM) Hackathon Exhibition Day in Johannesburg last week, presenting working prototypes designed to solve real-world problems affecting their communities. The learners, accompanied by 11 teachers, took part in the five-day hackathon, hosted by ORT South Africa in partnership with Hudaco, from June 22 to 26....</t>
+          <t>Young Engineers Build Solutions for Real-World Challenges at STEM Hackathon Fifty-five high school learners and 11 teachers from underserved South African schools will showcase working engineering and technology prototypes at the Young Engineers Movement (YEM) Hackathon Exhibition Day on 26 June 2026.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3137,24 +3121,24 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>yasmine.jacobs@iol.co.za, pholoso.manyama@inl.co.za, wendy.dondolo@inl.co.za, pholoso.manyama@iol.co.za, verna.vandiemen@inl.co.za</t>
+          <t>info@futuresa.co.za</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ORT South Africa's inaugural YEM Hackathon empowers future STEM innovators</t>
+          <t>Build the Future with Entelect Hackathons</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>https://www.futuresa.co.za/bursaries-and-scholarships/ort-south-africa-yem-hackathon/</t>
+          <t>https://challenge.entelect.co.za/</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>July 30, 2026 - ORT South Africa's first Young Engineers Movement Hackathon saw 55 learners develop innovative STEM solutions during a five-day competition.</t>
+          <t>Build the Future with Entelect Hackathons Join South Africa's premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3162,26 +3146,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>info@futuresa.co.za</t>
-        </is>
-      </c>
+      <c r="E112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Young Engineers Movement Hackathon opens doors to future career choices | Rosebank Killarney Gazette</t>
+          <t>ICEP - Tshwane Varsity Hackathon</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>https://www.citizen.co.za/rosebank-killarney-gazette/news-headlines/local-news/2026/07/06/hackathon-sparks-solutions/</t>
+          <t>https://tvh.icep.co.za/</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>July 6, 2026 - 55 learners put ideas to paper, developing prototypes at the Young Engineers Movement (YEM) Hackathon. The ideas they came up with at the five-day hackathon in Houghton Estate, hosted by ORT South Africa, were to solve leading community issues, ...</t>
+          <t>Tshwane Varsity Hackathon South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3189,22 +3169,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>info@tvh.co.za, MagasengQM@tut.ac.za</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Southern Africa Digital ID Hackathon</t>
+          <t>The Home of South African Hackathons</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://www.africa.engineering.cmu.edu/events/2024/11/21-southern-digital-hackathon.html</t>
+          <t>https://hackon.co.za/partners/</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Learn more and register for Southern Africa Digital ID Hackathon · January 23 2026 · 12:00 PM - 1:30 PM CAT · Carnegie Mellon University Africa · Customizing the CV to the job description · Learn more about this event by contacting Paul Swaga.</t>
+          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3217,17 +3201,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>PATH South Africa co-hosts Harvard Health Hackathon | PATH</t>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://www.path.org/our-impact/articles/path-south-africa-co-hosts-harvard-health-hackathon/</t>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>The South Africa hackathon location was at the University of Cape Town (UCT) and dubbed the UCT Hub. It attracted over 80 applicants from diverse fields, including medicine, engineering, research, and software development.</t>
+          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3235,7 +3219,88 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Talks &amp; Fireside | Builders Table</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>https://builderstable.net/</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Builders Table is a two-day hackathon hosted by MakeReign, built around a 24-hour build sprint. It brings together South Africa's designers, developers, strategists, founders and creative technologists to build real working prototypes under real time pressure.</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>sarah.chen@horizonlabs.com, liamlr95@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>CompeteHub - Where Champions Are Made</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>https://www.devpluxe.co.za/</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Geekulcha Home of the Geeks</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>https://www.geekulcha.dev/</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>A community of tech development in Africa Geekulcha is where young, skilled, creative, and ambitious tech minds meet to connect with each other, share knowledge, collaborate on projects, network with industry leaders, obtain training to further improve an enhance their skills, and put that newly acquired skill to work.</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>name@domain.com</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-09-23
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E118"/>
+  <dimension ref="A1:E112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,24 +558,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>user@domain.com, info@zasdc.org</t>
+          <t>info@zasdc.org, user@domain.com</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
+          <t>Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.thecasecentre.org/products/view?id=189255</t>
+          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
+          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -588,17 +588,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Engineering Conferences in South Africa 2025-2026</t>
+          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
+          <t>https://www.thecasecentre.org/products/view?id=189255</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
+          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -684,17 +684,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Apr 16, 2026 · Exhibition Opportunities BENEFITS FOR YOUR PARTICIPATING IN THE EXHIBITION: An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms.</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -704,24 +704,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, sithabile@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, Erika@innovate.durban, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, c183baa23371454f99f417f6616b724d@sentry.wixpress.com</t>
+          <t>customerservices@informaconnect.com, dataprivacy@informaconnect.com, dataprivacy@knect365.com, support@knect365.com, salesenquiries@africatechfestival.com, support@informaconnect.com, customerservices@knect365.com</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/tradeshows</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>South Africa trade shows, find and compare 970 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 156 upcoming expos in 2026-2027 1. China Homelife Fair South Africa, 2.</t>
+          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -729,22 +729,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>enquiries@aiexpoafrica.com</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://10times.com/southafrica/tradeshows</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>South Africa trade shows, find and compare 970 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 156 upcoming expos in 2026-2027 1. China Homelife Fair South Africa, 2. Intex South Africa International Textile Exhibition, 3. Wine &amp; Wheels Expo, 4 ...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -752,26 +756,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>dataprivacy@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, support@informaconnect.com, customerservices@knect365.com, customerservices@informaconnect.com, support@knect365.com</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
+          <t>Exhibition | Innovation Festival Durban | South Africa</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://innovationweek.co.za/</t>
+          <t>https://www.innovationfestival.durban/exhibition</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SA Innovation Week 2026 is South Africa’s official national innovation platform accelerating implementation, commercialisation and impact.</t>
+          <t>Exhibition Opportunities BENEFITS FOR YOUR PARTICIPATING IN THE EXHIBITION: An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -781,24 +781,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>info@pixal8media.co.za</t>
+          <t>8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, Erika@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, sithabile@innovate.durban, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
+          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -806,26 +806,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>enquiries@aiexpoafrica.com</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
+          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what’s next before everyone else does. Only 2,500 ...</t>
+          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -838,17 +834,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>South Africa International Industrial Expo | Innovation Bridge</t>
+          <t>IT &amp; Technology Events in South Africa | 10times</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
+          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -861,17 +857,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://innovationweek.co.za/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>SA Innovation Week 2026 is South Africa's official national innovation platform accelerating implementation, commercialisation and impact.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -879,22 +875,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>info@pixal8media.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>Fak'ugesi Festival - African Digital &amp; Innovation Festival</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://www.fakugesi.co.za/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>Fak'ugesi is Africa's premier digital innovation festival, held annually at the Tshimologong Digital Innovation Precinct in Johannesburg. Now in its thirteenth year, it convenes creatives, technologists, researchers, policymakers, and industry practitioners across five intensive days of programme, exhibition, and exchange.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -907,17 +907,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
+          <t>Come and explore our exhibition of innovative discoveries at Science ...</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
+          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
+          <t>The final countdown is underway, and all roads lead to this year's Science Forum South Africa 2024 at the CSIR International Convention Centre in Pretoria. Join us as we plan to celebrate the CSIR's impactful science, technology and innovation contributions at South Africa's premier scientific pl...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -980,17 +980,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>... On 30-31 March 2026, 109 students from 9 schools walked into the University of Cape Town and designed a city on the Moon. They elected leaders, divided into engineering departments, and spent 24 hours responding to a professional design brief.</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -998,26 +998,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>user@domain.com, info@zasdc.org</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>... On 30-31 March 2026, 109 students from 9 schools walked into the University of Cape Town and designed a city on the Moon. They elected leaders, divided into engineering departments, and spent 24 hours responding to a professional design brief.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1025,7 +1021,11 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>info@zasdc.org, user@domain.com</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1057,17 +1057,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South ...</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
+          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1075,22 +1075,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>Engineers Without Borders South ...</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
+          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1098,26 +1102,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
+          <t>Engineers Without Borders launches student challenge</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
+          <t>https://www.theconstructionindex.co.uk/news/view/engineers-without-borders-launches-student-challenge</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
+          <t>September 7, 2021 - The Engineering for People Design Challenge encourages undergraduates to broaden their awareness of the social, environmental and economic implications of their engineering solutions.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1125,7 +1125,11 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>news@theconstructionindex.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1153,17 +1157,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Engineering for people, that’s the challenge | Engineers Without Borders</t>
+          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.rs-online.com/designspark/an-introduction-to-engineering-for-people-design-challenge</t>
+          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>That’s exactly what the annual Engineering for People Design Challenge asks participants to do. The competition, delivered in partnership by Engineers without Borders South Africa and Engineers Without Borders UK, encourages engineering students and those collaborating with engineers to broaden their awareness of how their decisions change the world.</t>
+          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1314,17 +1318,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1337,17 +1341,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1433,17 +1437,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1451,22 +1455,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>customerservices@informaconnect.com, dataprivacy@informaconnect.com, dataprivacy@knect365.com, support@knect365.com, salesenquiries@africatechfestival.com, support@informaconnect.com, customerservices@knect365.com</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
+          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1476,24 +1484,24 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>u003einfo@techspo.co, atinfo@techspo.coor</t>
+          <t>info@techspocapetown.co.za</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://africatechnologyexpo.com/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
+          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1503,24 +1511,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>partner@africatechnologyexpo.com, johndoe@email.com, info@sparkafrica.co</t>
+          <t>enquiries@aiexpoafrica.com</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Home - Mediatech Africa | South Africa</t>
+          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://www.mediatech.co.za/</t>
+          <t>https://10times.com/southafrica/tradeshows</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
+          <t>Sep 12, 2026 · TECHSPO Cape Town is an influential technology expo that serves as a hub where business, tech, and innovation converge. Taking place at the Avenue Conference and Event Venue in Cape Town, South Africa,...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1528,26 +1536,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
-        </is>
-      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology ...</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
+          <t>TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1555,26 +1559,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>info@techspocapetown.co.za</t>
-        </is>
-      </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>Explore IT &amp; Technology Trade Events in south-africa ...</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1582,26 +1582,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>dataprivacy@knect365.com, salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, support@informaconnect.com, customerservices@knect365.com, customerservices@informaconnect.com, support@knect365.com</t>
-        </is>
-      </c>
+      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>HOME | Africa Tech Week</t>
+          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://africatechweek.co.za/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>May 11, 2026 - From sensational speakers, to top tech exhibitons, see what’s in store when you attend the 2-day Sentech Africa Tech Week Conference in 2025&gt;&gt; ... Sponsor, Speak, Attend! For more information on how you can be a part of the #ATW family, contact ...</t>
+          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1614,17 +1610,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
+          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Save this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaShare this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
+          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1632,22 +1628,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>u003einfo@techspo.co, atinfo@techspo.coor</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
+          <t>https://africatechnologyexpo.com/</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg – Where Business, Tech and Innovation Collide in Johannesburg, South Africa. TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa.</t>
+          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>you@company.com, colleague@company.com, your@email.com, support@industryevents.com, events@techspojoburg.co.za</t>
+          <t>partner@africatechnologyexpo.com, info@sparkafrica.co, johndoe@email.com</t>
         </is>
       </c>
     </row>
@@ -1687,17 +1687,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>Maker Faire - Wikipedia</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>https://en.wikipedia.org/wiki/Maker_faire</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>1 week ago - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1710,17 +1710,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>http://capetown.makerfaire.com/</t>
+          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1728,11 +1728,7 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>fancybox_loading@2x.gif, pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
-        </is>
-      </c>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1760,17 +1756,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Blog : Maker Faire Africa</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>http://makerfaireafrica.com/blog/</t>
+          <t>http://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building his ANIMAL car, from the ground up, that means the frame and all.</t>
+          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1778,22 +1774,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif, pr@make.co</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
+          <t>Blog : Maker Faire Africa</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
+          <t>http://makerfaireafrica.com/blog/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
+          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building his ANIMAL car, from the ground up, that means the frame and all.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1801,26 +1801,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>00-Header-Bahamas-IMG_6749@a.jpg</t>
-        </is>
-      </c>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
+          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
+          <t>https://contemporaryand.com/fr/events/maker-faire-africa-comes-to-johannesburg</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
+          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1833,17 +1829,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Makers Festival SA 🛠️ (@makersfestival_sa) • Instagram photos ...</t>
+          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/makersfestival_sa/</t>
+          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>8,503 Followers, 58 Following, 57 Posts - Makers Festival SA 🛠️ (@makersfestival_sa) on Instagram: "🛠️ Building Skills. Building Memories. 🏕️ 8th &amp; 9th November 2025 / Cape Town, SA 🪵 Founder @hutch_custom 📩 DM us - apply to be a MAKER 🫶🏼"</t>
+          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1856,17 +1852,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Why Africa needs Maker Faire | ZDNET</t>
+          <t>Makers Festival SA 🛠️ (@makersfestival_sa) • Instagram photos ...</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
+          <t>https://www.instagram.com/makersfestival_sa/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage ...</t>
+          <t>8,503 Followers, 58 Following, 57 Posts - Makers Festival SA 🛠️ (@makersfestival_sa) on Instagram: "🛠️ Building Skills. Building Memories. 🏕️ 8th &amp; 9th November 2025 / Cape Town, SA 🪵 Founder @hutch_custom 📩 DM us - apply to be a MAKER 🫶🏼"</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1879,17 +1875,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>HOME | MAKERS FEST</t>
+          <t>Why Africa needs Maker Faire | ZDNET</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.makersfestival.co.za/</t>
+          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>At Makers Festival SA, you get full access to every hands-on workshop, from woodworking and ceramics to leatherwork, painting, and more.</t>
+          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage to attend and show off their work.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1897,26 +1893,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, example@mysite.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, warren@makersfestival.co.za, 8c4075d5481d476e945486754f783364@sentry.io</t>
-        </is>
-      </c>
+      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
+          <t>February 27, 2026 - Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1929,17 +1921,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>High School STEM Competition | Southafrica 2024</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1947,22 +1939,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>StemCo - StemCo 2026 International Competitions</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://stemco.org/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
+          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1970,22 +1966,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>bestyourself@stemco.org, majed.ar@contestbag.com, info@eduverse.kz, support@contestbag.com</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Astemi Sa</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>Local, regional and national competitions with thousands of · Multi-level events of two or more rounds that become increasingly challenging and culminate in top-level Olympiads. Enrichment programmes to inspire promising young South Africans to pursue STEMI</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -1998,17 +1998,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Capetown 2026</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
+          <t>The ZASDC is South Africa's national Space Design Competition, part of a global network spanning six continents. Secondary school students design futuristic space settlements in a fast-paced industry simulation that builds real STEM, leadership ...</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2018,24 +2018,24 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>info@zasdc.org, user@domain.com</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
+          <t>STEAM Pitch Competition - STEM AFRICA FEST 2024</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://stemafricafest.com/steam-pitch-competition/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>Join STEM Africa Fest , celebrating science, technology, engineering, and mathematics. Experience hands-on learning, industry leaders, and innovation across Africa.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2048,17 +2048,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>SA young scientists selected for global competition at Regeneron ISEF in the USA - Eskom</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://www.eskom.co.za/sa-young-scientists-selected-for-global-competition-at-regeneron-isef-in-the-usa/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>May 6, 2025 - Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) competition, will take place from 10 to 16 May in Columbus, Ohio in the USA.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2071,17 +2071,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>PDF Department of Basic Education and Samsung South Africa Partner to ...</t>
+          <t>ASTEMI Competitions 2022 – SAASTA</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://www.education.gov.za/Portals/0/Media/Preess+Releases/2026+Media+Releases/Applications+for+2026+Samsung+Solve+For+Tomorrow.pdf</t>
+          <t>https://saasta.ac.za/astemi-competitions-2</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>The 2026 competition is guided by the theme: "Innovate for Tomorrow: STEM Solutions for Sustainable Communities." Samsung Solve for Tomorrow is a global innovation competition that empowers Grade 10 and 11 learners in public schools to design science, technology, engineering and mathematics (STEM) solutions that address real-world challenges within their communities.</t>
+          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2094,17 +2094,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
+          <t>Competition – Eskom Expo for Young Scientists</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
+          <t>https://exposcience.co.za/category/competition/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries open until 06 March 2026. This is a transformative ...</t>
+          <t>Aqil Variava business cities Damien ... Gray STEMI Vuyo Nzimande · Eskom Expo for Young Scientists is an exposition, or science fair, where students have a chance to show others their projects about their own scientific investigations. At the annual prestigious Eskom Expo for Young Scientists International Science Fair (ISF), selected students from 35 Expo Regions in South Africa then compete ...</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2112,22 +2112,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>support@exposcience.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>National Department of Basic Education</t>
+          <t>SA young scientists selected for global competition at Regeneron ISEF in the USA – Eskom Expo for Young Scientists</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://www.education.gov.za/LinkClick.aspx?fileticket=i9GS5Atf7zo=&amp;tabid=347&amp;portalid=0&amp;mid=14629</t>
+          <t>https://exposcience.co.za/sa-young-scientists-selected-for-global-competition-at-regeneron-isef-in-the-usa/</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>JOHANNESBURG, South Africa - XX Month 2026 - The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries ...</t>
+          <t>Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) competition, will take place from 10 to 16 May in Columbus, Ohio in the USA.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2137,7 +2141,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>ssasft@samsung.com, s.ngcobo@cheil.com, j.mogoeng@samsung.com</t>
+          <t>support@exposcience.co.za</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2168,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2185,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>April 14, 2026 - This National Event, to be held at the Sandton Convention Centre in Johannesburg, South Africa, as part of AI for Good Impact Africa, at AI Expo Africa 2025, is a qualifying tournament leading to the Grand Finale in Geneva during the AI for ...</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge, organized by ITU and The Cortex Hub, in partnership with Google.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2218,14 +2222,14 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, info@thecortexhub.africa, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, c183baa23371454f99f417f6616b724d@sentry.wixpress.com</t>
+          <t>8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, info@thecortexhub.africa, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2235,7 +2239,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Apr 25, 2025 · The Robotics for Good Youth Challenge South Africa is a national event in a global robotics competition on disaster response, leading to the AI for Good Summit 2025.</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in a UN-based global robotics competition, focusing on the critical area of disaster response.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2252,17 +2256,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>VEX Events: Official Competition Website for VEX Robotics</t>
+          <t>Roboticon 2026: South Africa Showcases Robotics for Culture, Education ...</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://events.vex.com/</t>
+          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>12 hours ago · Official Competition Website for VEX Robotics Robot Skills - IQ Elementary / Middle School Robot Skills - V5 Middle / High School Robot Skills - VEX U Collegiate / University</t>
+          <t>The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation." South Africa's robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2270,22 +2274,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>newspaper-rec300@2x.jpg, adverts@ubuntutimes.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>South Africa to host first World Robot Olympiad International Final in Africa in 2028 - WRO Association</t>
+          <t>PARC 2026 - Pan-African Robotics Competition | Dakar Youth Olympic Games</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://wro-association.org/south-africa-to-host-first-world-robot-olympiad-international-final-in-africa-in-2028/</t>
+          <t>https://www.parcrobotics.org/</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>5 days ago - One of the world's largest ... South Africa, 12 September 2026 — South Africa will host the World Robot Olympiad (WRO®) International Final in 2028, bringing WRO's flagship global robotics...</t>
+          <t>Africa's largest robotics competition. Official side event of the Dakar 2026 Youth Olympic Games. Six leagues, November 3-7 in Dakar, Senegal.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2293,26 +2301,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>1-Team-CARED-Philippines-500x383@2x.jpg, Costa-Rica-team-Sprout-release-banner-500x383@2x.jpg, Prithul-3rd-place-Future-Engineers-2022-A-500x383@2x.jpg, Annual-report-article-TZ-500x383@2x.jpg</t>
-        </is>
-      </c>
+      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Cape Town to host Africa’s first World Robot Olympiad</t>
+          <t>2026 - SpringBots South Africa</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://www.capetownetc.com/tech/cape-town-africas-first-world-robot-olympiad/</t>
+          <t>https://springbots.co.za/2026-2/</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>1 day ago - Cape Town will host the World Robot Olympiad (WRO) International Final in 2028, bringing one of the world’s largest youth robotics competitions to Africa for the first time, Cape {town} Etc reports.</t>
+          <t>This approach ensures that learners are not only participants in robotics competitions but are also equipped with real-world skills in design thinking, programming, systems engineering, and collaborative problem-solving. A Unified Future for Africa SpringBots' 2026 vision extends beyond competition and education.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2325,17 +2329,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>FIRST South Africa – Robotics Programs for School Children</t>
+          <t>South Africa to host first World Robot Olympiad International Final in ...</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://firstsa.org/</t>
+          <t>https://wro-association.org/south-africa-to-host-first-world-robot-olympiad-international-final-in-africa-in-2028/</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
+          <t>One of the world's largest international youth robotics competitions will bring student teams from around the globe to Cape Town — the first time the event has been held in Africa. Johannesburg, South Africa, 12 September 2026 — South Africa will host the World Robot Olympiad (WRO®) International Final in 2028, bringing WRO's flagship global robotics competition to the African continent.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2343,22 +2347,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Costa-Rica-team-Sprout-release-banner-500x383@2x.jpg, 1-Team-CARED-Philippines-500x383@2x.jpg, Prithul-3rd-place-Future-Engineers-2022-A-500x383@2x.jpg, Annual-report-article-TZ-500x383@2x.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>Home | Roboticon 2026</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://roboticon.resolute.education/</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
+          <t>Thank you for joining us at the ultimate robotics showcase, as Resolute proudly sponsored the World Robotics Olympiad (WRO) South Africa. This year we brought together two worlds for the biggest robotics event of the year - Roboticon and the WRO Nationals, on the same day at the same venue.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2371,17 +2379,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>South African Robotics Competitions and Schools</t>
+          <t>ROBO-RUMBLE 2026 — Innovation in Motion</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://www.sciencexpo.org.za/robotics.html</t>
+          <t>https://roborumble.net/</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Please note that this website is not affiliated with any specific organisation or event. If you organise a science fair, Olympiad, or related competition in South Africa and would like your event listed here, we would be pleased to include a link to your website.</t>
+          <t>South Africa's premier youth robotics &amp; technology competition. Robo Wars, Drone Racing, Grand Prix &amp; Innovation Challenge. August 2026.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2389,26 +2397,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>madelien@imbewu.foundation, webmaster@sciencexpo.org.za, marna.vanzyl@imbewu.foundation</t>
-        </is>
-      </c>
+      <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://safcec.org.za/</t>
+          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2418,24 +2422,24 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>communication@safcec.org.za</t>
+          <t>advertising@creamermedia.co.za, newsletters@creamermedia.co.za, chanel@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://civils.org.za/</t>
+          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2443,22 +2447,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>constr@crown.co.za, ernao@crown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ICE Africa - Supporting Civil Engineers in Africa</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
+          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ICE Africa supports civil engineers across the continent, providing access to qualifications, training, and networking opportunities for professional growth.</t>
+          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2471,17 +2479,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Engineering the Future: 16 schools compete in SAICE's 33rd ...</t>
+          <t>SWM Communications | SAICE recognises civil engineering research excellence through national student competition</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/lifestyle/education/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://swmcommunications.co.za/press-office/saice-recognises-civil-engineering-research-excellence-through-national-student-competition/</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted its 33 rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland. The very first SAICE Bridge Building Competition was held in 1991, and it aimed to encourage high school learners to apply their knowledge of mathematics and science in a ...</t>
+          <t>April 1, 2026 - The event – which was sponsored by Sika, WorldsView, BVI, RIBCCS, and AF Consulting – was hosted at SAICE House in Midrand, Gauteng, and accredited for 0.2 CPD points. Students were invited to present their civil engineering university research and investigation project, which is part of the national curriculum for final year civil engineering undergraduate students.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2489,22 +2497,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>info@swmcommunications.co.za, nthabeleng@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE)</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://m.facebook.com/pages/The-South-African-Institution-of-Civil-Engineering-SAICE/92946824896/</t>
+          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>📢 Call for Abstracts: Structural Engineering Conference 2026 This inaugural conference brings together four leading industry institutions - the South African Institution of Civil Engineering (SAICE), the South African Institute of Steel Construction (SAISC), the Concrete Society of Southern Africa, and York Timbers in collaboration with the ...</t>
+          <t>September 7, 2025 - Find the list of upcoming Civil Engineering conferences in South Africa 2025 with invitation an letter.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2517,17 +2529,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Home - SAICE</t>
+          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://saice.org.za/</t>
+          <t>https://www.ice.org.uk/about-us/what-we-do/ice-near-you/international/ice-africa/</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
+          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2535,26 +2547,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>civilinfo@saice.org.za, marketing@saice.org.za, membership@saice.org.za, communications@saice.org.za, accounts@saice.org.za, barbara@avenue.co.za, executiveadmin@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Aqualibrium: Empowering Future Engineers Through Hands-On Water ...</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://saice.org.za/press-releases/aqualibrium-empowering-future-engineers-through-hands-on-water-distribution-challenge/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>The recent finals of Aqualibrium, hosted by the South African Institution of Civil Engineering (SAICE), provided an exciting platform for students to immerse themselves in the world of water distribution and infrastructure. This annual event continues to highlight the significance of water management and the role of civil engineering in sustainable development. Recently held at […]</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2562,26 +2570,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>civilinfo@saice.org.za, marketing@saice.org.za, membership@saice.org.za, communications@saice.org.za, accounts@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
+          <t>Civil Engineering Competition - Christian Brothers University</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
+          <t>https://www.cbu.edu/civil-engineering-competition/</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
+          <t>August 14, 2023 - Gather a team (2-5 members) to compete in CBU’s Civil Engineering Competition September 18, 2023, when up to six teams in each category will test their skills for the judges, CBU’s renowned engineering professors.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2589,22 +2593,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>jkaufma1@cbu.edu, info@cbu.edu</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SAICE Aqualibrium 2025: High School Students Rise to the Challenge in ...</t>
+          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/environment/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
+          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted the thrilling 2025 Aqualibrium Competition National Finals this past week, which brought together high school students from schools all over South Africa at the Sci-Bono Discovery Centre in Johannesburg. The event continues to be an important platform for fostering engineering talent, inspiring young minds, and raising awareness ...</t>
+          <t>Civil engineering conferences in Cape town 2025 provide an exclusive global platform to meet and engage with experts and aspirants in various fields.</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2617,17 +2625,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>SAICE | Events and Awards</t>
+          <t>Civil Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://members.saice.org.za/events-and-awards</t>
+          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>The South African Institution Of Civil Engineering SAICE hosts the Awards Function annually to honour individuals, projects of excellence, as well as community-oriented initiatives. The annual awards function gives companies and individuals a unique opportunity to showcase their deserving projects and work to the industry.</t>
+          <t>Apr 13 International Conference on Architectural, Civil and Environmental Engineering (ICACEE) - Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2650,7 +2658,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2673,7 +2681,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters’ program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2700,7 +2708,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2713,17 +2721,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>List of ALL Engineering Bursaries South Africa 2027</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
+          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2736,17 +2744,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>Competitions South Africa – Live Giveaways &amp; Prize Draws ...</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://freehub.co.za/competitions/</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+          <t>3 days ago · Browse live South African competitions, giveaways and prize draws. Find car, cash, voucher, tech and holiday competitions with clear entry rules and official source links.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2759,17 +2767,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Engineering Competition For African Youth In Engineering ...</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Aug 18, 2025 · The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent’s largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
+          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2777,7 +2785,11 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2805,17 +2817,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions. Whether you're working in traditional engineering fields or applying innovation in areas like health, agriculture, or digital technology, the Africa Prize for Engineering Innovation offers a unique platform to ...</t>
+          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2828,17 +2840,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers 18a Gill Street Observatory Johannesburg South Africa Phone: +27 (0)11 487 3003 Email: reception@saiee.org.za Powered by</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2846,26 +2858,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>IEEE South Africa</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>http://www.ieee.org.za/</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>The South African Section has around 1200 members and many subsections. It was formed in 1963 by the merger of the Institute of Radio Engineers (IRE, founded 1912) and the American Institute of Electrical Engineers (AIEE, founded 1884).</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2878,7 +2886,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2888,7 +2896,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>IEEE-IAS Industrial Power Conversion Systems Department Serving the electrical energy conversion professional worldwide</t>
+          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2901,17 +2909,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2919,26 +2927,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Join a SAIEE Centre near you! Become a SAIEE Member today! Join a SAIEE Centre near you! How can we assist you? SAIEE LAUNCHES NEW WEBSITE AND SOLUTION! The course starts with an overview of low voltage ... Earn your CPD credits today! Read it here.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2946,22 +2950,26 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing ...</t>
+          <t>Competitions | ESG</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://ebe.uct.ac.za/articles/2026-05-29-engineering-students-compete-global-high-performance-computing-challenge</t>
+          <t>https://za.rs-online.com/web/content/m/competition</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025. Now, Team UCT is preparing to represent South Africa at the global finals in Germany later this year.</t>
+          <t>Find your next opportunity below, we stagger them throughout the year so make sure to check back regularly for up to date information. Good luck! The RS Student Project Fund 2026 provides successful applicants with up to R10 000 to spend on RS products.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2971,101 +2979,97 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>ebe-faculty@uct.ac.za</t>
+          <t>example@email.com</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Competitions | ESG</t>
+          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://za.rs-online.com/web/content/m/competition</t>
+          <t>https://hackon.co.za/</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
+          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>example@email.com</t>
-        </is>
-      </c>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>List of ALL Engineering Bursaries South Africa 2027</t>
+          <t>ICEP - Tshwane Varsity Hackathon</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://www.zabursaries.co.za/engineering-bursaries-south-africa/</t>
+          <t>https://tvh.icep.co.za/</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>How much can I earn within the Engineering field in South Africa? The engineering sector in South Africa offers a wide range of career opportunities across fields such as civil, mechanical, electrical, chemical, mining, and industrial engineering. Salaries vary depending on qualifications, experience, and industry, with entry-level roles typically starting at moderate levels and increasing ...</t>
+          <t>The 8th Annual TVH will use a hackathon format, underpinned by Agile Scrum and Microsoft cloud computing practices, to deliver fresh ideas and solutions that catalyze 4IR on the African continent.</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr"/>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>info@tvh.co.za, MagasengQM@tut.ac.za</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Apply Now: Africa Prize for Engineering Innovation 2026 Offers R1 ...</t>
+          <t>Hackathons en South Africa</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://stepapp.co.za/2025/08/27/apply-now-africa-prize-for-engineering-innovation-2026-offers-r1-million-top-prize/</t>
+          <t>https://za.allhackathons.com/</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>The Royal Academy of Engineering has officially launched the Africa Prize for Engineering Innovation 2026, a prestigious pan-African competition designed to support and accelerate engineering entrepreneurs who are developing scalable solutions to local challenges. This initiative, now in its 12th year, offers African innovators a unique opportunity to gain access to vital funding, mentorship ...</t>
+          <t>Aug 22, 2025 · Join us for an electrifying hackathon where innovation meets security and finance! This event brings together developers, data scientists, cybersecurity experts, and FinTech enthusiasts to …</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>info@stepapp.co.za, Africa.Prize@raeng.org.uk</t>
-        </is>
-      </c>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>The Home of South African Hackathons</t>
+          <t>Geekulcha Annual Hackathon 2026 - Registration | Sonke Platform</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/</t>
+          <t>https://sonke.gklink.co/event/gkhack26</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+          <t>Every decision made during the hackathon weekend should be guided by one question: Would a real user trust and use this? The Geekulcha Annual Hackathon attracts a diverse, high-calibre community of technology builders and thinkers from across Africa.</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3078,17 +3082,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Hackathons en South Africa</t>
+          <t>Build the Future with Entelect Hackathons</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/</t>
+          <t>https://challenge.entelect.co.za/</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+          <t>Instead of focusing on building a once-off project, our hackathons centre around optimisation problems. Participants develop solutions that are tested, scored, and ranked based on performance, efficiency, and strategy.</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3101,17 +3105,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Young Engineers Showcase Innovation at STEM Hackathon</t>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://www.futuresa.co.za/education/young-engineers-movement-stem/</t>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Young Engineers Build Solutions for Real-World Challenges at STEM Hackathon Fifty-five high school learners and 11 teachers from underserved South African schools will showcase working engineering and technology prototypes at the Young Engineers Movement (YEM) Hackathon Exhibition Day on 26 June 2026.</t>
+          <t>Sep 2, 2026 · The Young Engineers Movement (YEM) is an immersive engineering and technology hackathon designed to equip young South Africans with the skills, mindset and confidence needed to solve real-world challenges.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3121,24 +3125,24 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>info@futuresa.co.za</t>
+          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons</t>
+          <t>Talks &amp; Fireside | Builders Table</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/</t>
+          <t>https://builderstable.net/</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons Join South Africa's premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
+          <t>Builders Table is a two-day hackathon hosted by MakeReign, built around a 24-hour build sprint. It brings together South Africa's designers, developers, strategists, founders and creative technologists to build real working prototypes under real time pressure.</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3146,159 +3150,9 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>ICEP - Tshwane Varsity Hackathon</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>https://tvh.icep.co.za/</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>Tshwane Varsity Hackathon South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>info@tvh.co.za, MagasengQM@tut.ac.za</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>The Home of South African Hackathons</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>https://hackon.co.za/partners/</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>Young Engineers Movement (YEM) - ORT SA</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>Talks &amp; Fireside | Builders Table</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>https://builderstable.net/</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>Builders Table is a two-day hackathon hosted by MakeReign, built around a 24-hour build sprint. It brings together South Africa's designers, developers, strategists, founders and creative technologists to build real working prototypes under real time pressure.</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
+      <c r="E112" t="inlineStr">
         <is>
           <t>sarah.chen@horizonlabs.com, liamlr95@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>CompeteHub - Where Champions Are Made</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>https://www.devpluxe.co.za/</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr"/>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>Geekulcha Home of the Geeks</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>https://www.geekulcha.dev/</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>A community of tech development in Africa Geekulcha is where young, skilled, creative, and ambitious tech minds meet to connect with each other, share knowledge, collaborate on projects, network with industry leaders, obtain training to further improve an enhance their skills, and put that newly acquired skill to work.</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>name@domain.com</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update competition data 2026-09-24
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E112"/>
+  <dimension ref="A1:E118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
+          <t>2026 South Africa Engineering Competition</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://notices.ukzn.ac.za/content/GetFile.aspx?id=96047</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>August 6, 2026 - Several South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>UKZN and Elsevier. If you are an engineering student (undergraduate or postgraduate), don't miss joining the challenge to solve real-world cases using Engineering Village and Knovel.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -469,17 +469,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Some of our sparkling achievements during 2014 – to help the NRF and DSI grow a representative science and technology workforce in the country – SAASTA has run a number of maths and science educator development programmes and a number of learner development programmes, including maths and science camps for learners with potential, olympiads and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -487,22 +487,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -510,22 +514,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -538,17 +546,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa. Find out more</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -556,26 +564,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>info@zasdc.org, user@domain.com</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Engineering Conferences in South Africa 2025-2026</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -588,17 +592,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.thecasecentre.org/products/view?id=189255</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -606,22 +610,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
+          <t>Team South Africa wins at NASA space engineering competition</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -629,26 +637,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>Eligibility Benchmark Requirements The Africa Prize is open to individuals or teams based in sub-Saharan Africa with a scalable engineering innovation that demonstrates social or environmental impact potential. Applicants must: Be citizens ordinarily residing in a sub-Saharan African country. Be over 18 years old and fluent in English.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -661,17 +665,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>August 14, 2026 - Ramaphosa acknowledged that manufacturers face high electricity costs, logistics constraints, infrastructure bottlenecks, weak demand and import competition. He urged government to provide certainty while industry invests, modernises, develops suppliers and trains young people. The ambition is therefore larger than rebuilding factories: it is about restoring South Africa’s industrial power and using that capability to capture a greater share of Africa’s rapidly expanding infrastructure and development market.</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -694,7 +698,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -704,14 +708,14 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>customerservices@informaconnect.com, dataprivacy@informaconnect.com, dataprivacy@knect365.com, support@knect365.com, salesenquiries@africatechfestival.com, support@informaconnect.com, customerservices@knect365.com</t>
+          <t>dataprivacy@knect365.com, support@knect365.com, customerservices@informaconnect.com, salesenquiries@africatechfestival.com, support@informaconnect.com, customerservices@knect365.com, dataprivacy@informaconnect.com</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -721,7 +725,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AI Expo Africa 2026 - Join the Largest AI Event &amp; Trade Community in Africa TODAY! Our business audience is a buyer / supplier focused community and comprised of Enterprise decision makers / CxOs, allied to AI Cloud platform providers, Tier 1 / 2 deployment &amp; service providers, AI start ups / innovators, investors, educators, government and AI ecosystem community builders.</t>
+          <t>(2 Day Event) 28th-29th October 2026 Sandton Convention Centre, JHB, South Africa AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -738,17 +742,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
+          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/tradeshows</t>
+          <t>https://innovationweek.co.za/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>South Africa trade shows, find and compare 970 expos, trade fairs and exhibitions to go in South Africa - Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Venue, Editions, Visitors Profile, Exhibitor Information etc. Listing of 156 upcoming expos in 2026-2027 1. China Homelife Fair South Africa, 2. Intex South Africa International Textile Exhibition, 3. Wine &amp; Wheels Expo, 4 ...</t>
+          <t>SA Innovation Week 2026 is South Africa’s official national innovation platform accelerating implementation, commercialisation and impact.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -756,22 +760,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>info@pixal8media.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Exhibition Opportunities BENEFITS FOR YOUR PARTICIPATING IN THE EXHIBITION: An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms.</t>
+          <t>From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what’s next before everyone else does. Only 2,500 free tickets are available.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -779,26 +787,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, Erika@innovate.durban, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, sithabile@innovate.durban, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
+          <t>Explore IT &amp; Technology Trade Events in south-africa ...</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
+          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -811,17 +815,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
+          <t>Fak'ugesi Festival – African Digital &amp; Innovation Festival</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
+          <t>https://www.fakugesi.co.za/</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
+          <t>Fak'ugesi is Africa's premier digital innovation festival, held annually at the Tshimologong Digital Innovation Precinct in Johannesburg. Now in its thirteenth year, it convenes creatives, technologists, researchers, policymakers, and industry practitioners across five intensive days of programme, exhibition, and exchange.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -834,17 +838,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa | 10times</t>
+          <t>South Africa International Industrial Expo | Innovation Bridge</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Explore a diverse array of events in South Africa. Find &amp; compare, Reviews, Ratings, Timings, Entry Ticket Fees, Schedule, Calendar, Discussion Topics, Venue, Speakers, Agenda, Visitors Profile, Exhibitor Information etc. for your convenience. Don't miss out on these exciting opportunities!</t>
+          <t>Organized by Golden Bridge Expo South Africa, Ry Agri South Africa in partnership with Small Enterprise Development Agency (Seda) Johannesburg branch – the three-day event themed ‘Together, Growing Industries’ seeks to foster network, ...</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -857,17 +861,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
+          <t>KZN Industrial Technology Exhibition</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://innovationweek.co.za/</t>
+          <t>https://www.kznindustrial.co.za/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SA Innovation Week 2026 is South Africa's official national innovation platform accelerating implementation, commercialisation and impact.</t>
+          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s leading platform for industrial innovation ...</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -877,24 +881,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>info@pixal8media.co.za</t>
+          <t>john@email.com</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Fak'ugesi Festival - African Digital &amp; Innovation Festival</t>
+          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.fakugesi.co.za/</t>
+          <t>https://madeinafricaevent.co.za/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Fak'ugesi is Africa's premier digital innovation festival, held annually at the Tshimologong Digital Innovation Precinct in Johannesburg. Now in its thirteenth year, it convenes creatives, technologists, researchers, policymakers, and industry practitioners across five intensive days of programme, exhibition, and exchange.</t>
+          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -907,17 +911,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Come and explore our exhibition of innovative discoveries at Science ...</t>
+          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>The final countdown is underway, and all roads lead to this year's Science Forum South Africa 2024 at the CSIR International Convention Centre in Pretoria. Join us as we plan to celebrate the CSIR's impactful science, technology and innovation contributions at South Africa's premier scientific pl...</t>
+          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -930,17 +934,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Engineering for People returns to Johannesburg - Engineers Without Borders UK</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>September 18, 2024 - Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>April 9, 2026 - In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community’s challenges ...</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -948,22 +952,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering for People Design Challenge returns to Johannesburg!</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>April 9, 2026 - Just as the word Bambasonke means ‘take hold together’ in IsiZulu, together, we can engineer a future that bridges gaps, uplifts vulnerable populations, and builds a more inclusive and prosperous South Africa. The Bambasonke Design Challenge ...</t>
+          <t>Sep 18, 2024 · Engineering for People Design Challenge returns to Johannesburg! Now entering its fourteenth year, we’re delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -971,26 +979,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Engineering for People Design Challenge | Department of ...</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers (WWE) came up with a siphon tank solution to tackle the water problem in the community, and Aston Without Borders (AWB) came up with a new and innovative rainwater harvesting and filter connected to a solar-powered boiler system to provide safe and clean water to households.</t>
+          <t>Aug 4, 2025 · The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -998,22 +1002,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>Engineering For People Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>... On 30-31 March 2026, 109 students from 9 schools walked into the University of Cape Town and designed a city on the Moon. They elected leaders, divided into engineering departments, and spent 24 hours responding to a professional design brief.</t>
+          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1023,24 +1031,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>info@zasdc.org, user@domain.com</t>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Engineering ENGINEERING FOR PEOPLE Design challenge DESIGN ...</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://www.ewb-uk.org/wp-content/uploads/2024/08/2024_25_Engineering_for_People_Design_Challenge_Makers_Valley.pdf</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>September 19, 2024 - Engineers Without Borders UK returns to Makers Valley, South Africa for the 2024/25 Engineering for People Design Challenge 18th September 2024: Engineers Without Borders UK, the organisation leading a movement […]</t>
+          <t>These topics are at the centre of South Africa’s National Development Plan (NDP) 2030 and can provide insight into the main developmental challenges that are critical to South Africa.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1048,26 +1056,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>ied@ied.org.uk</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>August 4, 2025 - This year’s design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but ...</t>
+          <t>Oct 24, 2024 · The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1077,24 +1081,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+          <t>team@crowdsolve.net</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South ...</t>
+          <t>EWB Design Challenge | Aston University</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
+          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
+          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers ...</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1107,17 +1111,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Engineers Without Borders launches student challenge</t>
+          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.theconstructionindex.co.uk/news/view/engineers-without-borders-launches-student-challenge</t>
+          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>September 7, 2021 - The Engineering for People Design Challenge encourages undergraduates to broaden their awareness of the social, environmental and economic implications of their engineering solutions.</t>
+          <t>September 19, 2024 - 18th September 2024: Engineers Without Borders UK, the organisation leading a movement to put global responsibility at the heart of engineering, has launched the 2024/25 cycle of the award-winning Engineering for People Design Challenge in ...</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1127,24 +1131,24 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>news@theconstructionindex.co.uk</t>
+          <t>ied@ied.org.uk</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Latest Community Engineering Design Competition Announced</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>October 16, 2024 - Organised in conjunction with sister ... Partnership, this year’s challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg....</t>
+          <t>... On 30-31 March 2026, 109 students from 9 schools walked into the University of Cape Town and designed a city on the Moon. They elected leaders, divided into engineering departments, and spent 24 hours responding to a professional design brief.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1152,22 +1156,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>user@domain.com, info@zasdc.org</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2024-25 Engineering for People Design Challenge: Solutions for Makers Valley - Studocu</t>
+          <t>Engineers Without Borders South ...</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.studocu.com/en-za/document/university-of-the-witwatersrand-johannesburg/engineering-and-analysis/2024-25-engineering-for-people-design-challenge-solutions-for-makers-valley/123144589</t>
+          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>April 7, 2025 - In engineering education, EWB-SA delivers the Engineering for People Design Challenge annually in collaboration with Engineers Without Borders- UK to over 2,000 students a year in South Africa, exposing engineering students to real-world design ...</t>
+          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1180,17 +1188,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate engineering students will represent South Africa at the global Mission Idea Contest in Tokyo with their innovative SLINQI satellite concept. Designed as a practical, real-world solution, SLINQI proposes a pair of small satellites ...</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1203,17 +1211,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1226,17 +1234,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>2026 SOUTH AFRICA ENGINEERING COMPETITION</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://notice.ukzn.ac.za/content/GetFile.aspx?id=96048</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Best Regards, The 2026 SA Engineering Competition Team University of KwaZulu-Natal • Elsevier</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1249,17 +1257,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
+          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1267,22 +1275,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1290,22 +1302,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Engineering in South Africa: 24 Best universities Ranked</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/za/</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>March 15, 2026 - Below is the list of 24 best universities for Engineering in South Africa ranked based on their research performance: a graph of 5.9M citations received by 257K academic papers made by these universities was used to calculate ratings and create the top.</t>
+          <t>The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1313,22 +1329,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, email@example.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>This competition is open to teams of engineering students from any university program in West Africa.</t>
+          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1341,17 +1361,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>April 28, 2026 - Seven postgraduate students from the Faculty of Engineering have been selected to represent South Africa at the · Mission Idea Contest (MIC), a global space engineering competition held in Tokyo, Japan.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1364,17 +1384,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2210</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Mechanical Engineering - South Africa 2026</t>
+          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1387,17 +1407,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1437,17 +1457,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Africa Tech Festival</t>
+          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://10times.com/southafrica/technology</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>South Africa · 158 EventsFollowShare · TrendingDate · Loading... Regional Advisory: Check official updates before travel. Premium · Loading... You may also like · NODES AI · 15 Apr · Online · NODES AI15 AprOnline · Intersec Shanghai · 07-09 May · Shanghai , China · Intersec Shanghai07-09 MayShanghai , China · GCCI Annual Trade Expo ·</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1455,26 +1475,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>customerservices@informaconnect.com, dataprivacy@informaconnect.com, dataprivacy@knect365.com, support@knect365.com, salesenquiries@africatechfestival.com, support@informaconnect.com, customerservices@knect365.com</t>
-        </is>
-      </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
+          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1484,24 +1500,24 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>info@techspocapetown.co.za</t>
+          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
+          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://africatechnologyexpo.com/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
+          <t>Africa Tech Expo (ATE) provides Trade Offices, Embassies, and Economic Missions with a strategic platform to present their national innovation agendas, enterprise capabilities, and cross-border investment priorities to Africa’s most influential ...</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1511,24 +1527,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>enquiries@aiexpoafrica.com</t>
+          <t>partner@africatechnologyexpo.com, info@sparkafrica.co, johndoe@email.com</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/tradeshows</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Sep 12, 2026 · TECHSPO Cape Town is an influential technology expo that serves as a hub where business, tech, and innovation converge. Taking place at the Avenue Conference and Event Venue in Cape Town, South Africa,...</t>
+          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1536,22 +1552,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>info@techspocapetown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology ...</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1559,22 +1579,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>dataprivacy@knect365.com, support@knect365.com, customerservices@informaconnect.com, salesenquiries@africatechfestival.com, support@informaconnect.com, customerservices@knect365.com, dataprivacy@informaconnect.com</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Explore IT &amp; Technology Trade Events in south-africa ...</t>
+          <t>Home - Mediatech Africa | South Africa</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
+          <t>https://www.mediatech.co.za/</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
+          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1582,22 +1606,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>simon@mediatech.co.za, claire@mediatech.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
+          <t>HOME | Africa Tech Week</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://africatechweek.co.za/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>New York Small Business Expo (Spring)07 MayNew York , USA · AFROZUM Fair · 07-09 May · Johannesburg , South Africa · AFROZUM Fair07-09 MayJohannesburg , South Africa · Nigeria Industries &amp; Manufacturing Summit · 18-20 May · Abuja , Nigeria ...</t>
+          <t>May 11, 2026 - Attend Africa Tech Week and learn first hand how to leverage technological change in order to gain the competitive edge, making you and your business relevant in an age of exponential disruption.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1610,17 +1638,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
+          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
+          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
+          <t>Share this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaSave this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1628,26 +1656,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>u003einfo@techspo.co, atinfo@techspo.coor</t>
-        </is>
-      </c>
+      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
+          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://africatechnologyexpo.com/</t>
+          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Africa Technology Expo 2026 isn’t just about discussing technology—it’s about showcasing it in action. This is your chance to present groundbreaking hardware innovations to the people who matter most: leading enterprises, strategic partners, ...</t>
+          <t>TECHSPO Johannesburg – Where Business, Tech and Innovation Collide in Johannesburg, South Africa. TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1657,7 +1681,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>partner@africatechnologyexpo.com, info@sparkafrica.co, johndoe@email.com</t>
+          <t>you@company.com, support@industryevents.com, your@email.com, colleague@company.com, events@techspojoburg.co.za</t>
         </is>
       </c>
     </row>
@@ -1692,12 +1716,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Maker_faire</t>
+          <t>https://en.wikipedia.org/wiki/Maker_Faire</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>1 week ago - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
+          <t>2 weeks ago - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1743,7 +1767,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>July 30, 2015 - About Cape Town Mini Maker Faire: Cape Town Maker Faire brings together families and individuals to celebrate the Do- It-Yourself (DIY) mindset and showcase all kinds of incredible projects.</t>
+          <t>July 30, 2015 - ... The City of Cape Town, being the World Design Capital 2014 and one of the base of a lot of Afrika Burn, is the ideal choice for celebrating the Movement Maker in South Africa...</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1766,7 +1790,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>April 20, 2026 - Makers are everywhere! Showcase the ingenuity and creativity in your community by starting a Maker Faire in your town, city or region today.</t>
+          <t>April 20, 2026 - Maker Faire is not an event that has to do strictly with people making hardware. For me it’s much more important because it opens up channels of communication between makers and the concept of making together.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1776,7 +1800,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif, pr@make.co</t>
+          <t>fancybox_loading@2x.gif, pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1817,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building his ANIMAL car, from the ground up, that means the frame and all.</t>
+          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building ...</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1811,7 +1835,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://contemporaryand.com/fr/events/maker-faire-africa-comes-to-johannesburg</t>
+          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1839,7 +1863,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Maker Faire Africa 2014 will bring together over 5,000 attendees, along with featured inventors, world-class makers, self-made entrepreneurs &amp; workshop experts from South Africa, across the continent, and around the world, to manufacture real solutions for some of Africa’s most pressing ...</t>
+          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1898,17 +1922,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
+          <t>StemCo - StemCo 2026 International Competitions</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://stemco.org/</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>February 27, 2026 - Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>June 10, 2026 - Singapore, Angola, Azerbaijan, Bahrain, Bosnia and Herzegovina, Canada, Cambodia, Czech Republic, Germany, Gibraltar, Indonesia, Iran, Japan, Kazakhstan, Kyrgyzstan, South Korea, Malawi, Mexico, Mongolia, Nigeria, Myanmar, North Macedonia, Peru, Philippines, Romania, Russia, Serbia, South Africa, Taiwan, Tajikistan, Thailand, Turkey, Turkmenistan, Ukraine, United Arab Emirates, United Kingdom, The United States of America, Uzbekistan, Vietnam</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1916,22 +1940,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>support@contestbag.com, bestyourself@stemco.org, majed.ar@contestbag.com, info@eduverse.kz</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024</t>
+          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
+          <t>February 27, 2026 - Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1939,26 +1967,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>StemCo - StemCo 2026 International Competitions</t>
+          <t>High School STEM Competition | Southafrica 2024</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://stemco.org/</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>June 10, 2026 - BEST YOURSELF WITH STEMCO! Platform for the world’s brightest. ... Thanks to the participating 25 countries in 2019. Singapore, Albania, Australia, Azerbaijan, Canada, Germany, India, Indonesia, Japan, Jordan, Kazakhstan, Kyrgyzstan, Malawi, Mongolia, Nigeria, Myanmar, South Africa, Tajikistan, Turkey, Turkmenistan, Ukraine, The United States, Uzbekistan, Vietnam</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1968,7 +1992,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>bestyourself@stemco.org, majed.ar@contestbag.com, info@eduverse.kz, support@contestbag.com</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
@@ -2018,24 +2042,24 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>info@zasdc.org, user@domain.com</t>
+          <t>user@domain.com, info@zasdc.org</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>STEAM Pitch Competition - STEM AFRICA FEST 2024</t>
+          <t>SA young scientists selected for global competition at Regeneron ISEF in the USA - Eskom</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://stemafricafest.com/steam-pitch-competition/</t>
+          <t>https://www.eskom.co.za/sa-young-scientists-selected-for-global-competition-at-regeneron-isef-in-the-usa/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Join STEM Africa Fest , celebrating science, technology, engineering, and mathematics. Experience hands-on learning, industry leaders, and innovation across Africa.</t>
+          <t>May 6, 2025 - Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) competition, will take place from 10 to 16 May in Columbus, Ohio in the USA.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2043,22 +2067,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>MediaDesk@eskom.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>SA young scientists selected for global competition at Regeneron ISEF in the USA - Eskom</t>
+          <t>Competition – Eskom Expo for Young Scientists</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://www.eskom.co.za/sa-young-scientists-selected-for-global-competition-at-regeneron-isef-in-the-usa/</t>
+          <t>https://exposcience.co.za/category/competition/</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>May 6, 2025 - Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) competition, will take place from 10 to 16 May in Columbus, Ohio in the USA.</t>
+          <t>Team South Africa made a remarkable impact at the SciFest International STEM Fair (ISF) in Dublin, Ireland, bringing home top honours for their exceptional scientific research and innovations.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2094,17 +2122,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Competition – Eskom Expo for Young Scientists</t>
+          <t>STEAM Pitch Competition - STEM AFRICA FEST 2024</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://exposcience.co.za/category/competition/</t>
+          <t>https://stemafricafest.com/steam-pitch-competition/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Aqil Variava business cities Damien ... Gray STEMI Vuyo Nzimande · Eskom Expo for Young Scientists is an exposition, or science fair, where students have a chance to show others their projects about their own scientific investigations. At the annual prestigious Eskom Expo for Young Scientists International Science Fair (ISF), selected students from 35 Expo Regions in South Africa then compete ...</t>
+          <t>Join STEM Africa Fest , celebrating science, technology, engineering, and mathematics. Experience hands-on learning, industry leaders, and innovation across Africa.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2112,11 +2140,7 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>support@exposcience.co.za</t>
-        </is>
-      </c>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2131,7 +2155,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) competition, will take place from 10 to 16 May in Columbus, Ohio in the USA.</t>
+          <t>South Africa at the prestigious ... curiosity, and global competitiveness of the country’s young scientists. Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) ...</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2168,24 +2192,24 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+          <t>78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
+          <t>South Africa to host first World Robot Olympiad International Final in Africa in 2028 - WRO Association</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
+          <t>https://wro-association.org/south-africa-to-host-first-world-robot-olympiad-international-final-in-africa-in-2028/</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge, organized by ITU and The Cortex Hub, in partnership with Google.</t>
+          <t>1 week ago - Johannesburg, South Africa, 12 September 2026 — South Africa will host the World Robot Olympiad (WRO®) International Final in 2028, bringing WRO’s flagship global robotics competition to the African continent.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2195,24 +2219,24 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>name@example.com</t>
+          <t>Costa-Rica-team-Sprout-release-banner-500x383@2x.jpg, Annual-report-article-TZ-500x383@2x.jpg, 1-Team-CARED-Philippines-500x383@2x.jpg, Prithul-3rd-place-Future-Engineers-2022-A-500x383@2x.jpg</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
+          <t>April 14, 2026 - The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge, organized by ITU and The Cortex Hub, in partnership with Google.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2222,24 +2246,24 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, info@thecortexhub.africa, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
+          <t>Cape Town to host Africa’s first World Robot Olympiad</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
+          <t>https://www.capetownetc.com/tech/cape-town-africas-first-world-robot-olympiad/</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in a UN-based global robotics competition, focusing on the critical area of disaster response.</t>
+          <t>3 days ago - Cape Town will host the World Robot Olympiad International Final in 2028, bringing top youth robotics teams from around the world to South Africa.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2247,26 +2271,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>name@example.com</t>
-        </is>
-      </c>
+      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Roboticon 2026: South Africa Showcases Robotics for Culture, Education ...</t>
+          <t>FIRST South Africa – Robotics Programs for School Children</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
+          <t>https://firstsa.org/</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation." South Africa's robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
+          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2274,26 +2294,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>newspaper-rec300@2x.jpg, adverts@ubuntutimes.co.za</t>
-        </is>
-      </c>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>PARC 2026 - Pan-African Robotics Competition | Dakar Youth Olympic Games</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://www.parcrobotics.org/</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Africa's largest robotics competition. Official side event of the Dakar 2026 Youth Olympic Games. Six leagues, November 3-7 in Dakar, Senegal.</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2306,17 +2322,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026 - SpringBots South Africa</t>
+          <t>South African Robotics Competitions and Schools</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://springbots.co.za/2026-2/</t>
+          <t>https://www.sciencexpo.org.za/robotics.html</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>This approach ensures that learners are not only participants in robotics competitions but are also equipped with real-world skills in design thinking, programming, systems engineering, and collaborative problem-solving. A Unified Future for Africa SpringBots' 2026 vision extends beyond competition and education.</t>
+          <t>North Gauteng Senior Science Fair is the oldest science fair in South Africa.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2324,22 +2340,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>marna.vanzyl@imbewu.foundation, webmaster@sciencexpo.org.za, madelien@imbewu.foundation</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>South Africa to host first World Robot Olympiad International Final in ...</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://wro-association.org/south-africa-to-host-first-world-robot-olympiad-international-final-in-africa-in-2028/</t>
+          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>One of the world's largest international youth robotics competitions will bring student teams from around the globe to Cape Town — the first time the event has been held in Africa. Johannesburg, South Africa, 12 September 2026 — South Africa will host the World Robot Olympiad (WRO®) International Final in 2028, bringing WRO's flagship global robotics competition to the African continent.</t>
+          <t>(ADDITIONAL VIDEO SUPPLIED BY UJ ... African teenagers to get early exposure to engineering concepts through involvement in AfrikaBOT 'the world's most affordable robotics competition'....</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2347,26 +2367,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Costa-Rica-team-Sprout-release-banner-500x383@2x.jpg, 1-Team-CARED-Philippines-500x383@2x.jpg, Prithul-3rd-place-Future-Engineers-2022-A-500x383@2x.jpg, Annual-report-article-TZ-500x383@2x.jpg</t>
-        </is>
-      </c>
+      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Home | Roboticon 2026</t>
+          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://roboticon.resolute.education/</t>
+          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Thank you for joining us at the ultimate robotics showcase, as Resolute proudly sponsored the World Robotics Olympiad (WRO) South Africa. This year we brought together two worlds for the biggest robotics event of the year - Roboticon and the WRO Nationals, on the same day at the same venue.</t>
+          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2379,17 +2395,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ROBO-RUMBLE 2026 — Innovation in Motion</t>
+          <t>South African Schools attend SITA Robotics Challenge</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://roborumble.net/</t>
+          <t>https://www.education.gov.za/ArchivedDocuments/ArchivedArticles/SITARoboticsChallenge.aspx</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>South Africa's premier youth robotics &amp; technology competition. Robo Wars, Drone Racing, Grand Prix &amp; Innovation Challenge. August 2026.</t>
+          <t>The 2024 SITA (State Information Technology Agency) Robotics Challenge took place in Summerstrand, Gqeberha at the Radisson Blu Hotel and Southern Sun Marine Hotel from 25 – 26 September 2024.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2397,22 +2413,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>certification@dbe.gov.za, callcentre@dbe.gov.za</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>CAD for Civil Engineering - 2D + 3D CAD, One Price</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
+          <t>https://www.bing.com/aclick?ld=e8JOgG79OW8S3K7GMl5QekNjVUCUxYZn-2-KTAaBfYHIMH_41pxBpPULA3St-qpSomz_eP24jLFSbWRgGMSxwYUb-DcGRXe9sFZwm5y1tm7S5AIr9cDDwkwrYyPFTsWEtsIkLZD5aN5sxttmrFiE7u0Kas32jLSfuFsflMxHqM2iYBycC3jgg8dwoekoA0KV1wDDtmd8BEIoNEzQUASf_3pj9gsNw&amp;u=aHR0cHMlM2ElMmYlMmZ3d3cucHJvZ2VjYWQudXMlMmZjaXZpbCUzZm1zY2xraWQlM2RmM2NiYWRjYzZjZWYxMTI2NzAxOGM3Nzk3NjA1Y2EzYiUyNnV0bV9zb3VyY2UlM2RiaW5nJTI2dXRtX21lZGl1bSUzZGNwYyUyNnV0bV9jYW1wYWlnbiUzZHByb2dlQ0FEJTI1MjAlMjU3QyUyNTIwSW5kdXN0cnklMjUyMFZlcnRpY2FscyUyNnV0bV90ZXJtJTNkY2l2aWwlMjUyMGVuZ2luZWVycyUyNnV0bV9jb250ZW50JTNkQ2l2aWw&amp;rlid=f3cbadcc6cef11267018c7797605ca3b</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
+          <t>Affordable, DWG-compatible CAD for civil engineers switching from costly subscriptions. Full 2D + 3D CAD with AutoLISP and VBA. Try it free for 30 days, no card needed. View Products · Check Blog · Get Help</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2422,24 +2442,24 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>advertising@creamermedia.co.za, newsletters@creamermedia.co.za, chanel@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za</t>
+          <t>jane@company.com, info@progecad.us</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>The South African Institution of Civil Engineering</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
+          <t>https://civils.org.za/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
+          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2447,26 +2467,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>constr@crown.co.za, ernao@crown.co.za</t>
-        </is>
-      </c>
+      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
+          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd ...</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
+          <t>https://southafricatoday.net/lifestyle/education/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
+          <t>Aug 30, 2024 · The South African Institution of Civil Engineering (SAICE) hosted its 33 rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2479,17 +2495,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SWM Communications | SAICE recognises civil engineering research excellence through national student competition</t>
+          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://swmcommunications.co.za/press-office/saice-recognises-civil-engineering-research-excellence-through-national-student-competition/</t>
+          <t>https://safcec.org.za/</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>April 1, 2026 - The event – which was sponsored by Sika, WorldsView, BVI, RIBCCS, and AF Consulting – was hosted at SAICE House in Midrand, Gauteng, and accredited for 0.2 CPD points. Students were invited to present their civil engineering university research and investigation project, which is part of the national curriculum for final year civil engineering undergraduate students.</t>
+          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2499,24 +2515,24 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>info@swmcommunications.co.za, nthabeleng@saice.org.za</t>
+          <t>communication@safcec.org.za</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
+          <t>Home - SAICE</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
+          <t>https://saice.org.za/</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>September 7, 2025 - Find the list of upcoming Civil Engineering conferences in South Africa 2025 with invitation an letter.</t>
+          <t>Through our divisions, branches and committees, we aim to advance professional knowledge and improve the practice of civil engineering in South Africa. Our purpose is to provide members with opportunities for professional development through continued learning opportunities and industry networking.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2524,22 +2540,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>communications@saice.org.za, membership@saice.org.za, accounts@saice.org.za, barbara@avenue.co.za, civilinfo@saice.org.za, executiveadmin@saice.org.za, marketing@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
+          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/what-we-do/ice-near-you/international/ice-africa/</t>
+          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
+          <t>Jul 7, 2026 · Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in a shared commitment to developing South Africa’s future engineering talent.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2552,17 +2572,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>SAICE Aqualibrium 2025: High School Students Rise to the ...</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
+          <t>https://southafricatoday.net/environment/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>May 14, 2025 · Each year, the Aqualibrium competition puts high school students in the shoes of actual civil engineers, putting their creativity and problem-solving abilities to the test by solving a challenging real-world problem.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2575,17 +2595,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Civil Engineering Competition - Christian Brothers University</t>
+          <t>Awards 2026 - SAICE</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://www.cbu.edu/civil-engineering-competition/</t>
+          <t>https://saice.org.za/awards-2026/</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>August 14, 2023 - Gather a team (2-5 members) to compete in CBU’s Civil Engineering Competition September 18, 2023, when up to six teams in each category will test their skills for the judges, CBU’s renowned engineering professors.</t>
+          <t>Learn about SAICE's award categories, submission guidelines, key dates and how to nominate project and professionals.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2595,29 +2615,29 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>jkaufma1@cbu.edu, info@cbu.edu</t>
+          <t>communications@saice.org.za, membership@saice.org.za, accounts@saice.org.za, civilinfo@saice.org.za, marketing@saice.org.za</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
+          <t>Study Mechanical Engineering - Engineering Master's Degree</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
+          <t>https://www.bing.com/aclick?ld=e8pnqL8XDnvh843Qo9xUYuCjVUCUwjxvFy4mAPNy03fv6uuaWSZSYpte_fjkGAaxpnkm5fcD9_VecdVqKk3i-vEL--ZZaW22cZ18PCuBlEUsIbDd7Yy8QJt_jjwji3mwY4IGseW-NOEkANQc-9l2psNBjDrtBvVmfscHHJmuZpI-kece3Z_NIQmbwuxCQ7XOF4-Q-uA_QiEswOwTfRSiioR824dAU&amp;u=aHR0cHMlM2ElMmYlMmZ3d3cud29ybGRjYW1wdXMucHN1LmVkdSUyZmRlZ3JlZXMtYW5kLWNlcnRpZmljYXRlcyUyZnBlbm4tc3RhdGUtb25saW5lLW1lY2hhbmljYWwtZW5naW5lZXJpbmctbWFzdGVycy1kZWdyZWUlMmYlM2ZjaWQlM2RDUEM1NDQ0NCUyNm1zY2xraWQlM2RiMDMxYTExYmVkMGExZjAyMjhiYWNiYWVmN2YxNWY0ZSUyNnV0bV9zb3VyY2UlM2RiaW5nJTI2dXRtX21lZGl1bSUzZGNwYyUyNnV0bV9jYW1wYWlnbiUzZEVuZ1BvcnRCaW5nV0MlMjZ1dG1fdGVybSUzZG1lY2hhbmljYWwlMjUyMGVuZ2luZWVyaW5nJTI2dXRtX2NvbnRlbnQlM2RNU01FLUdlbmVyYWw&amp;rlid=b031a11bed0a1f0228bacbaef7f15f4e</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Civil engineering conferences in Cape town 2025 provide an exclusive global platform to meet and engage with experts and aspirants in various fields.</t>
+          <t>Accredited Mechanical Engineering Master's Degree Program. 100% Online! Request Info. Study Mechanical Engineering at Penn State. 100% Online Courses that Fit Your Life. Degree programs: Electrical Engineering, Engineering Management, Mechanical Engineering</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -2625,22 +2645,22 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Civil Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Apr 13 International Conference on Architectural, Civil and Environmental Engineering (ICACEE) - Cape Town, South Africa</t>
+          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>civil engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -2648,17 +2668,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
+          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2666,22 +2686,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2689,26 +2713,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2721,17 +2741,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
+          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2739,22 +2759,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Competitions South Africa – Live Giveaways &amp; Prize Draws ...</t>
+          <t>APPLY NOW! WORLDSKILLS SOUTH AFRICA NATIONAL COMPETITION 2025</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://freehub.co.za/competitions/</t>
+          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>3 days ago · Browse live South African competitions, giveaways and prize draws. Find car, cash, voucher, tech and holiday competitions with clear entry rules and official source links.</t>
+          <t>ndidate with an accredited qualification in the related skill - Candida. e must not turn 23 years old in 2026 for the skills required. - Candidate applying for Aircraft Maintenance, Mechatr.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2767,17 +2791,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>SAIMechE</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.saimeche.org.za/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2785,26 +2809,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>$2,000 Scholarship - NO ESSAY - Deadline: September 30, 2026</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>https://www.bing.com/aclick?ld=e8Rz1L4iT8OPwFn3Pz3KSZHjVUCUyVji0V2Fcg5b0A7lg0gCsqGRtSlDK2S9nhH1sv3Xe3SgjiY23M1ewsRNPu1g__EVqD629U1Y3sVwALyE29u_lN30oLW-YhQhqAq0P_QQYQUDESOm6HvLRfFS7SMIIJXKkdvJSo-DxHWM7qU0xBjP-loICAK-df7Iw-18IdYBA0F-E34zxsLc6mRbHY8YyM_Fw&amp;u=aHR0cHMlM2ElMmYlMmZ3d3cuc2FsbGllLmNvbSUyZnNjaG9sYXJzaGlwcyUyZm5vLWVzc2F5JTNmdXRtX3NvdXJjZSUzZGJpbmclMjZ1dG1fbWVkaXVtJTNkY3BjJTI2dXRtX2NhbXBhaWduJTNkbGFfYWNxX3N3cF91X3VfdV9jdHJsX3UlMjZ1dG1fdGVybSUzZHNjaG9sYXJzaGlwcyUyNTIwZm9yJTI1MjB1bmRlcmdyYWR1YXRlcyUyNmhzYV9jbXAlM2Q1MjE1Njg0OTUlMjZoc2FfZ3JwJTNkMTMxNjExNzgyMDM3NTE3MSUyNmhzYV9hZCUzZCUyNmhzYV9zcmMlM2RvJTI2aHNhX3RndCUzZGt3ZC04MjI1ODk3NDc3NjY2MiUzYWxvYy0xOTAlMjZoc2FfbXQlM2RiJTI2aHNhX2JtdCUzZGJiJTI2aHNhX2R2YyUzZGMlMjZoc2FfbmV0JTNkbXNiaW5nYWRzJTI2bXNjbGtpZCUzZGQ4NjE2MGJkODcyNTFlNjA1ODg0MGEwODlkZGViZGRj&amp;rlid=d86160bd87251e6058840a089ddebddc</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>Apply Now Must be attending or planning to attend an accredited College or University. High School, Undergraduate and Graduate students are eligible.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2817,17 +2837,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2840,17 +2860,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2863,17 +2883,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>IEEE South Africa</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>http://www.ieee.org.za/</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>The South African Section has around 1200 members and many subsections. It was formed in 1963 by the merger of the Institute of Radio Engineers (IRE, founded 1912) and the American Institute of Electrical Engineers (AIEE, founded 1884).</t>
+          <t>Design Thinking and Innovation for Engineering Professional - Online Design Thinking and Innovation for Engineering Professional - Online (opens in a new window) Training Academy Earn your CPD credits today!</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2881,12 +2901,16 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2896,7 +2920,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
+          <t>IEEE-IAS Industrial Power Conversion Systems Department Serving the electrical energy conversion professional worldwide</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2932,17 +2956,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>PDF WorldSkills South Africa Provincial Competitions 2025</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/Document/WorldSkillsZA+Provincial+Competitions+2025+V1.1.pdf</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Join a SAIEE Centre near you! Become a SAIEE Member today! Join a SAIEE Centre near you! How can we assist you? SAIEE LAUNCHES NEW WEBSITE AND SOLUTION! The course starts with an overview of low voltage ... Earn your CPD credits today! Read it here.</t>
+          <t>higher education &amp; training Department: Higher Education and Training REPUBLIC OF SOUTH AFRICA</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2950,11 +2974,7 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2969,7 +2989,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Find your next opportunity below, we stagger them throughout the year so make sure to check back regularly for up to date information. Good luck! The RS Student Project Fund 2026 provides successful applicants with up to R10 000 to spend on RS products.</t>
+          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2986,22 +3006,22 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -3009,49 +3029,49 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ICEP - Tshwane Varsity Hackathon</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://tvh.icep.co.za/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>The 8th Annual TVH will use a hackathon format, underpinned by Agile Scrum and Microsoft cloud computing practices, to deliver fresh ideas and solutions that catalyze 4IR on the African continent.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>info@tvh.co.za, MagasengQM@tut.ac.za</t>
+          <t>info@ieomsociety.org</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Hackathons en South Africa</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Aug 22, 2025 · Join us for an electrifying hackathon where innovation meets security and finance! This event brings together developers, data scientists, cybersecurity experts, and FinTech enthusiasts to …</t>
+          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions. Whether you're working in traditional engineering fields or applying innovation in areas like health, agriculture, or digital technology, the Africa Prize for Engineering Innovation offers a unique platform to ...</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
@@ -3059,17 +3079,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Geekulcha Annual Hackathon 2026 - Registration | Sonke Platform</t>
+          <t>The Home of South African Hackathons</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://sonke.gklink.co/event/gkhack26</t>
+          <t>https://hackon.co.za/</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Every decision made during the hackathon weekend should be guided by one question: Would a real user trust and use this? The Geekulcha Annual Hackathon attracts a diverse, high-calibre community of technology builders and thinkers from across Africa.</t>
+          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3082,17 +3102,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons</t>
+          <t>Hackathons en South Africa</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/</t>
+          <t>https://za.allhackathons.com/</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Instead of focusing on building a once-off project, our hackathons centre around optimisation problems. Participants develop solutions that are tested, scored, and ranked based on performance, efficiency, and strategy.</t>
+          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3105,17 +3125,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Young Engineers Movement (YEM) - ORT SA</t>
+          <t>Unisa hosts first-ever Hackathon to ignite student learning experience</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Sep 2, 2026 · The Young Engineers Movement (YEM) is an immersive engineering and technology hackathon designed to equip young South Africans with the skills, mindset and confidence needed to solve real-world challenges.</t>
+          <t>Unisa's Information and Communication Technology Portfolio, in collaboration with the College of Science, Engineering and Technology, held the first-ever Unisa Hackathon on 3 and 4 July 2025, marking a major step in the university's journey to embed digital innovation and entrepreneurship into the students learning experience.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3123,36 +3143,178 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
-        </is>
-      </c>
+      <c r="E111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
+          <t>Build the Future with Entelect Hackathons</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>https://challenge.entelect.co.za/</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Build the Future with Entelect Hackathons Join South Africa's premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Young Engineers Showcase Innovation at STEM Hackathon</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>https://www.futuresa.co.za/education/young-engineers-movement-stem/</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Young Engineers Build Solutions for Real-World Challenges at STEM Hackathon Fifty-five high school learners and 11 teachers from underserved South African schools will showcase working engineering and technology prototypes at the Young Engineers Movement (YEM) Hackathon Exhibition Day on 26 June 2026.</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>info@futuresa.co.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Hackathons | Sebaka</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>https://sebakasouthafrica.co.za/hackathons.html</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>The Home of South African Hackathons</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>https://hackon.co.za/partners/</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>CompeteHub - Where Champions Are Made</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>https://www.devpluxe.co.za/</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
           <t>Talks &amp; Fireside | Builders Table</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
+      <c r="B118" t="inlineStr">
         <is>
           <t>https://builderstable.net/</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
+      <c r="C118" t="inlineStr">
         <is>
           <t>Builders Table is a two-day hackathon hosted by MakeReign, built around a 24-hour build sprint. It brings together South Africa's designers, developers, strategists, founders and creative technologists to build real working prototypes under real time pressure.</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr">
+      <c r="D118" t="inlineStr">
         <is>
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>sarah.chen@horizonlabs.com, liamlr95@gmail.com</t>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>liamlr95@gmail.com, sarah.chen@horizonlabs.com</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update competition data 2026-09-25
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E118"/>
+  <dimension ref="A1:E115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026 South Africa Engineering Competition</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://notices.ukzn.ac.za/content/GetFile.aspx?id=96047</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>UKZN and Elsevier. If you are an engineering student (undergraduate or postgraduate), don't miss joining the challenge to solve real-world cases using Engineering Village and Knovel.</t>
+          <t>ASTEMI is a collaboration that ... &amp; Competitions to a broader base of learners and educators. ASTEMI is a national non-profit organization of independent organizations; teachers, public organisations and volunteers dedicated to improving and promoting science education and providing recognition for outstanding achievement by both learners and teachers. To promote excellence in Science, Technology, Engineering, Mathematics and Innovation in South African ...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -469,17 +469,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>Some of our sparkling achievements during 2014 – to help the NRF and DSI grow a representative science and technology workforce in the country – SAASTA has run a number of maths and science educator development programmes and a number of learner development programmes, including maths and science camps for learners with potential, olympiads and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -487,26 +487,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Sep 4, 2025 · The Africa Prize for Engineering Innovation is open to individuals or teams based in sub-Saharan Africa who have a scalable engineering innovation with social or environmental impact potential.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -516,24 +512,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation Competition, a programme of the Royal Academy of Engineering Submissions are open for the 2025 Africa Prize for Engineering Innovation from Monday, 21 July 2025 to 23 September 2025. Universities South Africa (USAf), through its Entrepreneurship Development in Higher Education (EDHE) Programme, and the Royal Academy of Engineering are ...</t>
+          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -541,22 +537,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa. Find out more</t>
+          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -564,22 +564,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -592,17 +596,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>Engineering Competition For African Youth In Engineering ...</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Aug 18, 2025 · This call invites engineers and innovators from across sub-Saharan Africa to apply with scalable innovations that address pressing social and environmental challenges.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -610,16 +614,12 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>admin@sawea.co.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition</t>
+          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>August 6, 2026 - South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -642,17 +642,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Eligibility Benchmark Requirements The Africa Prize is open to individuals or teams based in sub-Saharan Africa with a scalable engineering innovation that demonstrates social or environmental impact potential. Applicants must: Be citizens ordinarily residing in a sub-Saharan African country. Be over 18 years old and fluent in English.</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -665,17 +665,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>Africa Tech Festival takes place in Cape Town and attracts attendees from across Africa, Europe, the Middle East and global technology markets. ... The festival covers telecoms, AI, cybersecurity, data centres, digital transformation, fintech, ...</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -708,24 +708,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>dataprivacy@knect365.com, support@knect365.com, customerservices@informaconnect.com, salesenquiries@africatechfestival.com, support@informaconnect.com, customerservices@knect365.com, dataprivacy@informaconnect.com</t>
+          <t>salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, support@knect365.com, customerservices@informaconnect.com, support@informaconnect.com</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
+          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://innovationweek.co.za/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>(2 Day Event) 28th-29th October 2026 Sandton Convention Centre, JHB, South Africa AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
+          <t>SAIW’ 26 is designed as a week-long national programme to feature provincial innovation engagements across South Africa. From 16 – 17 March, Provinces will showcase local innovation strengths, emerging enterprises and sectoral capabilities.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -735,24 +735,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>enquiries@aiexpoafrica.com</t>
+          <t>info@pixal8media.co.za</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://innovationweek.co.za/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SA Innovation Week 2026 is South Africa’s official national innovation platform accelerating implementation, commercialisation and impact.</t>
+          <t>(2 Day Event) 28th-29th October 2026 Sandton Convention Centre, JHB, South Africa AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>info@pixal8media.co.za</t>
+          <t>enquiries@aiexpoafrica.com</t>
         </is>
       </c>
     </row>
@@ -838,17 +838,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>South Africa International Industrial Expo | Innovation Bridge</t>
+          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
+          <t>https://madeinafricaevent.co.za/</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Organized by Golden Bridge Expo South Africa, Ry Agri South Africa in partnership with Small Enterprise Development Agency (Seda) Johannesburg branch – the three-day event themed ‘Together, Growing Industries’ seeks to foster network, ...</t>
+          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -888,17 +888,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -911,17 +911,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>South Africa International Industrial Expo | Innovation Bridge</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -934,17 +934,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>PDF Engineering ENGINEERING FOR PEOPLE Design challenge DESIGN CHALLENGE ...</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://www.ewb-uk.org/wp-content/uploads/2024/08/2024_25_Engineering_for_People_Design_Challenge_Makers_Valley.pdf</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>April 9, 2026 - In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community’s challenges ...</t>
+          <t>Makers Makers Valley Valley Johannesburg, Johannesburg, South South Africa Africa The Engineering for People Design Challenge has been delivered in the UK and Ireland since 2011, South Africa and the USA since 2019, and Cameroon in 2022. It is an educational programme based on a concept developed originally by Engineers Without Borders Australia. The production of this document has been led by ...</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -952,26 +952,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge returns to Johannesburg!</t>
+          <t>Engineering For People Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Sep 18, 2024 · Engineering for People Design Challenge returns to Johannesburg! Now entering its fourteenth year, we’re delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -979,22 +975,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of ...</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Aug 4, 2025 · The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
+          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community's challenges and how community members view the impact of these challenges on their daily lives.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1004,24 +1004,24 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Engineering For People Design Challenge - EWBSA</t>
+          <t>Engineering for People Design Challenge returns to Johannesburg!</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
+          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
+          <t>Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1029,26 +1029,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineering ENGINEERING FOR PEOPLE Design challenge DESIGN ...</t>
+          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/wp-content/uploads/2024/08/2024_25_Engineering_for_People_Design_Challenge_Makers_Valley.pdf</t>
+          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>These topics are at the centre of South Africa’s National Development Plan (NDP) 2030 and can provide insight into the main developmental challenges that are critical to South Africa.</t>
+          <t>The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1056,22 +1052,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>team@crowdsolve.net</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Oct 24, 2024 · The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
+          <t>This year's design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1081,24 +1081,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>team@crowdsolve.net</t>
+          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>EWB Design Challenge | Aston University</t>
+          <t>Bambasankhe Design Challenge: Engineering for a Prosperous South Africa</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.aston.ac.uk/eps/ewb-design-challenge</t>
+          <t>https://www.linkedin.com/posts/activity-7470764395091001345-GwCR</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Our academics who support the Design Challenge discuss the benefits of taking part · The 2019 challenge saw 46 students working in 9 multi-disciplinary teams to create solutions to the sustainable development issues and problems in the diverse community of Maker’s Valley in Johannesburg, South Africa. Two teams from Aston were shortlisted to attend the Grand Finals. Worldwide Engineers ...</t>
+          <t>By joining forces, student engineers have the chance to bridge societal gaps, uplift those in vulnerable positions, and contribute to building a more inclusive and prosperous South Africa.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1111,17 +1111,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Launching Engineering for People Design Challenge 2024/25 - Institution of Engineering Designers</t>
+          <t>Latest Community Engineering Design Competition Announced</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.ied.org.uk/launching-engineering-for-people-design-challenge-2024-25/</t>
+          <t>https://www.epdtonthenet.net/article/208944/Latest-Community-Engineering-Design-Competition-Announced.aspx</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>September 19, 2024 - 18th September 2024: Engineers Without Borders UK, the organisation leading a movement to put global responsibility at the heart of engineering, has launched the 2024/25 cycle of the award-winning Engineering for People Design Challenge in ...</t>
+          <t>STEM-focused NGO Engineers Without Borders UK has launched its 2025 Engineering for People Design Challenge. Organised in conjunction with sister organisation Engineers Without Borders South Africa, as well as the Makers Valley Partnership, this year's challenge will focus on helping the inhabitants of the economically-deprived suburbs of eastern Johannesburg.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1129,26 +1129,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>ied@ied.org.uk</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>Engineers Without Borders South Africa - Facebook</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/posts/were-building-something-bigthe-engineers-without-borders-south-africa-team-recen/1168670565286616/</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>... On 30-31 March 2026, 109 students from 9 schools walked into the University of Cape Town and designed a city on the Moon. They elected leaders, divided into engineering departments, and spent 24 hours responding to a professional design brief.</t>
+          <t>South Africa's future engineers are ready to solve real- world challenges. On 22 January 2027, the best student teams from across the country will compete at the Engineering for People Design Challenge Grand Finals, showcasing innovative solutions that place people, communities, and sustainability at the heart of engineering. 🏆 One stage.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1156,26 +1152,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>user@domain.com, info@zasdc.org</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South ...</t>
+          <t>EWB-SA: Mid-Year Update - LinkedIn</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/photos/we-have-launched-the-engineering-for-people-design-challenge-at-the-university-o/923920273094981/</t>
+          <t>https://www.linkedin.com/pulse/ewb-sa-mid-year-update-ewbsa-uxo9f</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South Africa. 2,278 likes · 1 talking about this. EWB-SA aims to provide communities and community-based organisations with access to engineering expertise, skills and...</t>
+          <t>We wrapped up an extraordinary cycle of the 2023/24 Engineering for People Design Challenge in December 2024, with students across South Africa applying their creativity and empathy to solve real ...</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1188,17 +1180,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1206,22 +1198,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>2026 South Africa Engineering Competition</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://notice.ukzn.ac.za/content/GetFile.aspx?id=96048</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Best Regards, The 2026 SA Engineering Competition Team University of KwaZulu-Natal • Elsevier</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1234,17 +1230,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026 SOUTH AFRICA ENGINEERING COMPETITION</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://notice.ukzn.ac.za/content/GetFile.aspx?id=96048</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Best Regards, The 2026 SA Engineering Competition Team University of KwaZulu-Natal • Elsevier</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1252,22 +1248,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1275,26 +1275,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1304,24 +1300,24 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, email@example.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>National Student Competition | ORSSA</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://www.orssa.org.za/studentcomp</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1329,26 +1325,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, email@example.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1356,22 +1348,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate students from the Faculty of Engineering have been selected to represent South Africa at the · Mission Idea Contest (MIC), a global space engineering competition held in Tokyo, Japan.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1384,17 +1380,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent's largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1407,17 +1403,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Competitions - Enactus South Africa | National Expos, Challenges ...</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://enactusza.org/what-we-do/competitions</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1425,7 +1421,11 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>liso@enactus.org, marketingsa@enactus.org, xmadlanga@enactus.org, adminsa@enactus.org</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
+          <t>u003einfo@techspo.co, atinfo@techspo.coor</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>partner@africatechnologyexpo.com, info@sparkafrica.co, johndoe@email.com</t>
+          <t>johndoe@email.com, info@sparkafrica.co, partner@africatechnologyexpo.com</t>
         </is>
       </c>
     </row>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>September 22, 2014 - TECHSPO Cape Town 2027 is a two day technology expo taking place October 6th - 7th, 2027 at the luxurious Westin Cape Town Hotel, Cape Town, Africa. TECHSPO Cape Town brings together developers, brands, marketers, technology providers, designers, ...</t>
+          <t>September 22, 2014 - The Westin Cape Town Hotel, Cape Town, Africa ... The annual TECHSPO Cape Town 2027 Technology Expo returns October 6th to 7th, 2027 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>dataprivacy@knect365.com, support@knect365.com, customerservices@informaconnect.com, salesenquiries@africatechfestival.com, support@informaconnect.com, customerservices@knect365.com, dataprivacy@informaconnect.com</t>
+          <t>salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, support@knect365.com, customerservices@informaconnect.com, support@informaconnect.com</t>
         </is>
       </c>
     </row>
@@ -1608,24 +1608,24 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>simon@mediatech.co.za, claire@mediatech.co.za</t>
+          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>HOME | Africa Tech Week</t>
+          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://africatechweek.co.za/</t>
+          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>May 11, 2026 - Attend Africa Tech Week and learn first hand how to leverage technological change in order to gain the competitive edge, making you and your business relevant in an age of exponential disruption.</t>
+          <t>Share this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaSave this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1638,17 +1638,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
+          <t>HOME | Africa Tech Week</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
+          <t>https://africatechweek.co.za/</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Share this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaSave this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
+          <t>May 11, 2026 - From sensational speakers, to top tech exhibitons, see what’s in store when you attend the 2-day Sentech Africa Tech Week Conference in 2025&gt;&gt; ... Sponsor, Speak, Attend! For more information on how you can be a part of the #ATW family, contact ...</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>you@company.com, support@industryevents.com, your@email.com, colleague@company.com, events@techspojoburg.co.za</t>
+          <t>you@company.com, events@techspojoburg.co.za, support@industryevents.com, your@email.com, colleague@company.com</t>
         </is>
       </c>
     </row>
@@ -1800,24 +1800,24 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>fancybox_loading@2x.gif, pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png</t>
+          <t>chosen-sprite@2x.png, fancybox_sprite@2x.png, pr@make.co, fancybox_loading@2x.gif</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Blog : Maker Faire Africa</t>
+          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>http://makerfaireafrica.com/blog/</t>
+          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building ...</t>
+          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1830,17 +1830,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
+          <t>Blog : Maker Faire Africa</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
+          <t>http://makerfaireafrica.com/blog/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
+          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building his ANIMAL car, from the ground up, that means the frame and all.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1876,17 +1876,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Makers Festival SA 🛠️ (@makersfestival_sa) • Instagram photos ...</t>
+          <t>Why Africa needs Maker Faire | ZDNET</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/makersfestival_sa/</t>
+          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>8,503 Followers, 58 Following, 57 Posts - Makers Festival SA 🛠️ (@makersfestival_sa) on Instagram: "🛠️ Building Skills. Building Memories. 🏕️ 8th &amp; 9th November 2025 / Cape Town, SA 🪵 Founder @hutch_custom 📩 DM us - apply to be a MAKER 🫶🏼"</t>
+          <t>July 24, 2014 - "This year we're looking to have Maker Faire Africa in Johannesburg," Okafor said. "We haven't been to southern Africa before, and South Africa will probably be different again to previous events.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1899,17 +1899,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Why Africa needs Maker Faire | ZDNET</t>
+          <t>Makers Festival SA 🛠️ (@makersfestival_sa) • Instagram photos ...</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
+          <t>https://www.instagram.com/makersfestival_sa/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>July 24, 2014 - Unlike other Maker Faires, Okafor said that it's not enough to simply hold the event in an African city and see who turns up. Two volunteers are currently working in South Africa to discover inventors in rural areas and neighbouring countries such as Zambia and Botswana who they can encourage to attend and show off their work.</t>
+          <t>8,503 Followers, 58 Following, 57 Posts - Makers Festival SA 🛠️ (@makersfestival_sa) on Instagram: "🛠️ Building Skills. Building Memories. 🏕️ 8th &amp; 9th November 2025 / Cape Town, SA 🪵 Founder @hutch_custom 📩 DM us - apply to be a MAKER 🫶🏼"</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1922,17 +1922,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>StemCo - StemCo 2026 International Competitions</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://stemco.org/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>June 10, 2026 - Singapore, Angola, Azerbaijan, Bahrain, Bosnia and Herzegovina, Canada, Cambodia, Czech Republic, Germany, Gibraltar, Indonesia, Iran, Japan, Kazakhstan, Kyrgyzstan, South Korea, Malawi, Mexico, Mongolia, Nigeria, Myanmar, North Macedonia, Peru, Philippines, Romania, Russia, Serbia, South Africa, Taiwan, Tajikistan, Thailand, Turkey, Turkmenistan, Ukraine, United Arab Emirates, United Kingdom, The United States of America, Uzbekistan, Vietnam</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1940,11 +1940,7 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>support@contestbag.com, bestyourself@stemco.org, majed.ar@contestbag.com, info@eduverse.kz</t>
-        </is>
-      </c>
+      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1959,7 +1955,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>February 27, 2026 - Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>February 27, 2026 - Samsung Electronics South Africa has opened applications for the 2026 edition of Solve for Tomorrow (SFT), its annual science, technology, engineering, and mathematics (STEM) competition aimed at Grade 10 and 11 learners.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1972,17 +1968,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1990,26 +1986,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>High School STEM Competition | Capetown 2026</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Local, regional and national competitions with thousands of · Multi-level events of two or more rounds that become increasingly challenging and culminate in top-level Olympiads. Enrichment programmes to inspire promising young South Africans to pursue STEMI</t>
+          <t>High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas. Each submission can provide a summary of the STEM project. All projects must be presented at the IEOM Cape Town, South Africa 2026.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2017,22 +2009,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The ZASDC is South Africa's national Space Design Competition, part of a global network spanning six continents. Secondary school students design futuristic space settlements in a fast-paced industry simulation that builds real STEM, leadership ...</t>
+          <t>Rooted in the belief that today’s youth hold the key to tomorrow’s progress, Solve for Tomorrow South Africa provides participants with the tools, mentorship, and platforms they need to turn ideas into action.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2040,26 +2036,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>user@domain.com, info@zasdc.org</t>
-        </is>
-      </c>
+      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>SA young scientists selected for global competition at Regeneron ISEF in the USA - Eskom</t>
+          <t>ASTEMI SA</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://www.eskom.co.za/sa-young-scientists-selected-for-global-competition-at-regeneron-isef-in-the-usa/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>May 6, 2025 - Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) competition, will take place from 10 to 16 May in Columbus, Ohio in the USA.</t>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2067,26 +2059,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>MediaDesk@eskom.co.za</t>
-        </is>
-      </c>
+      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Competition – Eskom Expo for Young Scientists</t>
+          <t>DEPARTMENT OF BASIC EDUCATION AND SAMSUNG SOUTH AFRICA ...</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://exposcience.co.za/category/competition/</t>
+          <t>https://www.education.gov.za/Portals/0/Media/Preess+Releases/2026+Media+Releases/Applications+for+2026+Samsung+Solve+For+Tomorrow.pdf</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Team South Africa made a remarkable impact at the SciFest International STEM Fair (ISF) in Dublin, Ireland, bringing home top honours for their exceptional scientific research and innovations.</t>
+          <t>Samsung Solve for Tomorrow is a global innovation competition that empowers Grade 10 and 11 learners in public schools to design science, technology, engineering and mathematics (STEM) solutions that address real-world challenges within their communities.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2099,17 +2087,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions 2022 – SAASTA</t>
+          <t>High School STEM Competition | Southafrica 2024</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://saasta.ac.za/astemi-competitions-2</t>
+          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2117,22 +2105,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>STEAM Pitch Competition - STEM AFRICA FEST 2024</t>
+          <t>SA young scientists selected for global competition at Regeneron ISEF in the USA - Eskom</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://stemafricafest.com/steam-pitch-competition/</t>
+          <t>https://www.eskom.co.za/sa-young-scientists-selected-for-global-competition-at-regeneron-isef-in-the-usa/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Join STEM Africa Fest , celebrating science, technology, engineering, and mathematics. Experience hands-on learning, industry leaders, and innovation across Africa.</t>
+          <t>May 6, 2025 - Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) competition, will take place from 10 to 16 May in Columbus, Ohio in the USA.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2140,22 +2132,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>MediaDesk@eskom.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SA young scientists selected for global competition at Regeneron ISEF in the USA – Eskom Expo for Young Scientists</t>
+          <t>ASTEMI Competitions 2022 – SAASTA</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://exposcience.co.za/sa-young-scientists-selected-for-global-competition-at-regeneron-isef-in-the-usa/</t>
+          <t>https://saasta.ac.za/astemi-competitions-2</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>South Africa at the prestigious ... curiosity, and global competitiveness of the country’s young scientists. Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) ...</t>
+          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2163,11 +2159,7 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>support@exposcience.co.za</t>
-        </is>
-      </c>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2192,7 +2184,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com</t>
+          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2219,7 +2211,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Costa-Rica-team-Sprout-release-banner-500x383@2x.jpg, Annual-report-article-TZ-500x383@2x.jpg, 1-Team-CARED-Philippines-500x383@2x.jpg, Prithul-3rd-place-Future-Engineers-2022-A-500x383@2x.jpg</t>
+          <t>1-Team-CARED-Philippines-500x383@2x.jpg, Prithul-3rd-place-Future-Engineers-2022-A-500x383@2x.jpg, Annual-report-article-TZ-500x383@2x.jpg, Costa-Rica-team-Sprout-release-banner-500x383@2x.jpg</t>
         </is>
       </c>
     </row>
@@ -2236,7 +2228,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>April 14, 2026 - The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge, organized by ITU and The Cortex Hub, in partnership with Google.</t>
+          <t>April 14, 2026 - Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2263,7 +2255,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>3 days ago - Cape Town will host the World Robot Olympiad International Final in 2028, bringing top youth robotics teams from around the world to South Africa.</t>
+          <t>4 days ago - Cape Town will host the World Robot Olympiad International Final in 2028, bringing top youth robotics teams from around the world to South Africa.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2342,24 +2334,24 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>marna.vanzyl@imbewu.foundation, webmaster@sciencexpo.org.za, madelien@imbewu.foundation</t>
+          <t>madelien@imbewu.foundation, marna.vanzyl@imbewu.foundation, webmaster@sciencexpo.org.za</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
+          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
+          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>(ADDITIONAL VIDEO SUPPLIED BY UJ ... African teenagers to get early exposure to engineering concepts through involvement in AfrikaBOT 'the world's most affordable robotics competition'....</t>
+          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2367,22 +2359,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>NkosiN@atnews.co.za, rampedim@atnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
+          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
+          <t>(ADDITIONAL VIDEO SUPPLIED BY UJ ... African teenagers to get early exposure to engineering concepts through involvement in AfrikaBOT 'the world's most affordable robotics competition'....</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2395,17 +2391,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>South African Schools attend SITA Robotics Challenge</t>
+          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://www.education.gov.za/ArchivedDocuments/ArchivedArticles/SITARoboticsChallenge.aspx</t>
+          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>The 2024 SITA (State Information Technology Agency) Robotics Challenge took place in Summerstrand, Gqeberha at the Radisson Blu Hotel and Southern Sun Marine Hotel from 25 – 26 September 2024.</t>
+          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2413,26 +2409,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>certification@dbe.gov.za, callcentre@dbe.gov.za</t>
-        </is>
-      </c>
+      <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAD for Civil Engineering - 2D + 3D CAD, One Price</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://www.bing.com/aclick?ld=e8JOgG79OW8S3K7GMl5QekNjVUCUxYZn-2-KTAaBfYHIMH_41pxBpPULA3St-qpSomz_eP24jLFSbWRgGMSxwYUb-DcGRXe9sFZwm5y1tm7S5AIr9cDDwkwrYyPFTsWEtsIkLZD5aN5sxttmrFiE7u0Kas32jLSfuFsflMxHqM2iYBycC3jgg8dwoekoA0KV1wDDtmd8BEIoNEzQUASf_3pj9gsNw&amp;u=aHR0cHMlM2ElMmYlMmZ3d3cucHJvZ2VjYWQudXMlMmZjaXZpbCUzZm1zY2xraWQlM2RmM2NiYWRjYzZjZWYxMTI2NzAxOGM3Nzk3NjA1Y2EzYiUyNnV0bV9zb3VyY2UlM2RiaW5nJTI2dXRtX21lZGl1bSUzZGNwYyUyNnV0bV9jYW1wYWlnbiUzZHByb2dlQ0FEJTI1MjAlMjU3QyUyNTIwSW5kdXN0cnklMjUyMFZlcnRpY2FscyUyNnV0bV90ZXJtJTNkY2l2aWwlMjUyMGVuZ2luZWVycyUyNnV0bV9jb250ZW50JTNkQ2l2aWw&amp;rlid=f3cbadcc6cef11267018c7797605ca3b</t>
+          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Affordable, DWG-compatible CAD for civil engineers switching from costly subscriptions. Full 2D + 3D CAD with AutoLISP and VBA. Try it free for 30 days, no card needed. View Products · Check Blog · Get Help</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2442,24 +2434,24 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>jane@company.com, info@progecad.us</t>
+          <t>chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za, advertising@creamermedia.co.za</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering</t>
+          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd International Bridge Building Competition - SAICE</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://civils.org.za/</t>
+          <t>https://saice.org.za/press-releases/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering, www.saice.org.za, about, mission statement, code of ethics, code of conduct, strat plan, logo, crest, financial stats, national office, office bearers, branches, divisions, colleagues and industry leaders</t>
+          <t>April 17, 2025 - The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2467,22 +2459,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>membership@saice.org.za, communications@saice.org.za, marketing@saice.org.za, civilinfo@saice.org.za, accounts@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd ...</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/lifestyle/education/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Aug 30, 2024 · The South African Institution of Civil Engineering (SAICE) hosted its 33 rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2490,22 +2486,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>constr@crown.co.za, ernao@crown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SAFCEC- South African Forum Of Civil Engineering Contractors</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://safcec.org.za/</t>
+          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Join SAFCEC - South Africa's premier civil engineering contractors association. 450+ members, tender opportunities, 85 years of industry leadership.</t>
+          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2513,26 +2513,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>communication@safcec.org.za</t>
-        </is>
-      </c>
+      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Home - SAICE</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://saice.org.za/</t>
+          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Through our divisions, branches and committees, we aim to advance professional knowledge and improve the practice of civil engineering in South Africa. Our purpose is to provide members with opportunities for professional development through continued learning opportunities and industry networking.</t>
+          <t>September 7, 2025 - Find all upcoming Civil Engineering conferences in South Africa 2025 with invitation letter. South Africa is a diverse and dynamic country that offers a wide range of opportunities for Civil Engineering conferences in topic Civil Engineering, and many more.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2540,26 +2536,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>communications@saice.org.za, membership@saice.org.za, accounts@saice.org.za, barbara@avenue.co.za, civilinfo@saice.org.za, executiveadmin@saice.org.za, marketing@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
+          <t>SWM Communications | SAICE recognises civil engineering research excellence through national student competition</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
+          <t>https://swmcommunications.co.za/press-office/saice-recognises-civil-engineering-research-excellence-through-national-student-competition/</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Jul 7, 2026 · Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in a shared commitment to developing South Africa’s future engineering talent.</t>
+          <t>April 1, 2026 - April 2022: The South African Institution of Civil Engineering (SAICE) recently joined forces with leading universities across the country to award civil engineering students for their research efforts.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2567,22 +2559,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>nthabeleng@saice.org.za, info@swmcommunications.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>SAICE Aqualibrium 2025: High School Students Rise to the ...</t>
+          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/environment/saice-aqualibrium-2025-high-school-students-rise-to-the-challenge-in-national-water-competition/</t>
+          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>May 14, 2025 · Each year, the Aqualibrium competition puts high school students in the shoes of actual civil engineers, putting their creativity and problem-solving abilities to the test by solving a challenging real-world problem.</t>
+          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2595,17 +2591,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Awards 2026 - SAICE</t>
+          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://saice.org.za/awards-2026/</t>
+          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Learn about SAICE's award categories, submission guidelines, key dates and how to nominate project and professionals.</t>
+          <t>4th International Conference on Advances in Science, Engineering &amp; Technology(ICASET-2025) [Accredited CPD Event]</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2613,31 +2609,27 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>communications@saice.org.za, membership@saice.org.za, accounts@saice.org.za, civilinfo@saice.org.za, marketing@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Study Mechanical Engineering - Engineering Master's Degree</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://www.bing.com/aclick?ld=e8pnqL8XDnvh843Qo9xUYuCjVUCUwjxvFy4mAPNy03fv6uuaWSZSYpte_fjkGAaxpnkm5fcD9_VecdVqKk3i-vEL--ZZaW22cZ18PCuBlEUsIbDd7Yy8QJt_jjwji3mwY4IGseW-NOEkANQc-9l2psNBjDrtBvVmfscHHJmuZpI-kece3Z_NIQmbwuxCQ7XOF4-Q-uA_QiEswOwTfRSiioR824dAU&amp;u=aHR0cHMlM2ElMmYlMmZ3d3cud29ybGRjYW1wdXMucHN1LmVkdSUyZmRlZ3JlZXMtYW5kLWNlcnRpZmljYXRlcyUyZnBlbm4tc3RhdGUtb25saW5lLW1lY2hhbmljYWwtZW5naW5lZXJpbmctbWFzdGVycy1kZWdyZWUlMmYlM2ZjaWQlM2RDUEM1NDQ0NCUyNm1zY2xraWQlM2RiMDMxYTExYmVkMGExZjAyMjhiYWNiYWVmN2YxNWY0ZSUyNnV0bV9zb3VyY2UlM2RiaW5nJTI2dXRtX21lZGl1bSUzZGNwYyUyNnV0bV9jYW1wYWlnbiUzZEVuZ1BvcnRCaW5nV0MlMjZ1dG1fdGVybSUzZG1lY2hhbmljYWwlMjUyMGVuZ2luZWVyaW5nJTI2dXRtX2NvbnRlbnQlM2RNU01FLUdlbmVyYWw&amp;rlid=b031a11bed0a1f0228bacbaef7f15f4e</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Accredited Mechanical Engineering Master's Degree Program. 100% Online! Request Info. Study Mechanical Engineering at Penn State. 100% Online Courses that Fit Your Life. Degree programs: Electrical Engineering, Engineering Management, Mechanical Engineering</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -2645,22 +2637,22 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>Civil Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
+          <t>Nov 03 International Conference on Civil and Environmental Engineering (ICCEE) - Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>mechanical engineering competition South Africa</t>
+          <t>civil engineering competition South Africa</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -2668,17 +2660,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2686,26 +2678,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions. Whether you're working in traditional engineering fields or applying innovation in areas like health, agriculture, or digital technology, the Africa Prize for Engineering Innovation offers a unique platform to ...</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2718,17 +2706,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2741,17 +2729,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2761,24 +2749,24 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>APPLY NOW! WORLDSKILLS SOUTH AFRICA NATIONAL COMPETITION 2025</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>ndidate with an accredited qualification in the related skill - Candida. e must not turn 23 years old in 2026 for the skills required. - Candidate applying for Aircraft Maintenance, Mechatr.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2786,22 +2774,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>Competitions South Africa - Live Giveaways &amp; Prize Draws | Freehub</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>https://freehub.co.za/competitions/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>Browse live South African competitions, giveaways and prize draws. Find car, cash, voucher, tech and holiday competitions with clear entry rules and official source links.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2814,17 +2806,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>$2,000 Scholarship - NO ESSAY - Deadline: September 30, 2026</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://www.bing.com/aclick?ld=e8Rz1L4iT8OPwFn3Pz3KSZHjVUCUyVji0V2Fcg5b0A7lg0gCsqGRtSlDK2S9nhH1sv3Xe3SgjiY23M1ewsRNPu1g__EVqD629U1Y3sVwALyE29u_lN30oLW-YhQhqAq0P_QQYQUDESOm6HvLRfFS7SMIIJXKkdvJSo-DxHWM7qU0xBjP-loICAK-df7Iw-18IdYBA0F-E34zxsLc6mRbHY8YyM_Fw&amp;u=aHR0cHMlM2ElMmYlMmZ3d3cuc2FsbGllLmNvbSUyZnNjaG9sYXJzaGlwcyUyZm5vLWVzc2F5JTNmdXRtX3NvdXJjZSUzZGJpbmclMjZ1dG1fbWVkaXVtJTNkY3BjJTI2dXRtX2NhbXBhaWduJTNkbGFfYWNxX3N3cF91X3VfdV9jdHJsX3UlMjZ1dG1fdGVybSUzZHNjaG9sYXJzaGlwcyUyNTIwZm9yJTI1MjB1bmRlcmdyYWR1YXRlcyUyNmhzYV9jbXAlM2Q1MjE1Njg0OTUlMjZoc2FfZ3JwJTNkMTMxNjExNzgyMDM3NTE3MSUyNmhzYV9hZCUzZCUyNmhzYV9zcmMlM2RvJTI2aHNhX3RndCUzZGt3ZC04MjI1ODk3NDc3NjY2MiUzYWxvYy0xOTAlMjZoc2FfbXQlM2RiJTI2aHNhX2JtdCUzZGJiJTI2aHNhX2R2YyUzZGMlMjZoc2FfbmV0JTNkbXNiaW5nYWRzJTI2bXNjbGtpZCUzZGQ4NjE2MGJkODcyNTFlNjA1ODg0MGEwODlkZGViZGRj&amp;rlid=d86160bd87251e6058840a089ddebddc</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Apply Now Must be attending or planning to attend an accredited College or University. High School, Undergraduate and Graduate students are eligible.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2832,27 +2824,31 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent's largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -2860,22 +2856,22 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
+          <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -2883,44 +2879,40 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>SAIMechE</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://www.saimeche.org.za/</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Design Thinking and Innovation for Engineering Professional - Online Design Thinking and Innovation for Engineering Professional - Online (opens in a new window) Training Academy Earn your CPD credits today!</t>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>electrical engineering competition South Africa</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>reception@saiee.org.za, glueup-logo-white@2x.png</t>
-        </is>
-      </c>
+          <t>mechanical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>IEEE-IAS Industrial Power Conversion Systems Department Serving the electrical energy conversion professional worldwide</t>
+          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2933,17 +2925,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2956,17 +2948,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>PDF WorldSkills South Africa Provincial Competitions 2025</t>
+          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/Document/WorldSkillsZA+Provincial+Competitions+2025+V1.1.pdf</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>higher education &amp; training Department: Higher Education and Training REPUBLIC OF SOUTH AFRICA</t>
+          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2979,17 +2971,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Competitions | ESG</t>
+          <t>IEEE South Africa</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://za.rs-online.com/web/content/m/competition</t>
+          <t>http://www.ieee.org.za/</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
+          <t>The South African Section has around 1200 members and many subsections. It was formed in 1963 by the merger of the Institute of Radio Engineers (IRE, founded 1912) and the American Institute of Electrical Engineers (AIEE, founded 1884).</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2997,26 +2989,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>example@email.com</t>
-        </is>
-      </c>
+      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3029,17 +3017,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Sep 4, 2025 · The Africa Prize for Engineering Innovation is open to individuals or teams based in sub-Saharan Africa who have a scalable engineering innovation with social or environmental impact potential.</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3049,24 +3037,24 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions. Whether you're working in traditional engineering fields or applying innovation in areas like health, agriculture, or digital technology, the Africa Prize for Engineering Innovation offers a unique platform to ...</t>
+          <t>Join a SAIEE Centre near you! Become a SAIEE Member today! Join a SAIEE Centre near you! How can we assist you? SAIEE LAUNCHES NEW WEBSITE AND SOLUTION! The course starts with an overview of low voltage ... Earn your CPD credits today! Read it here.</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3074,12 +3062,16 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>The Home of South African Hackathons</t>
+          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3112,7 +3104,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
+          <t>Aug 22, 2025 · Join us for an electrifying hackathon where innovation meets security and finance! This event brings together developers, data scientists, cybersecurity experts, and FinTech enthusiasts to …</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3125,17 +3117,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Unisa hosts first-ever Hackathon to ignite student learning experience</t>
+          <t>ICEP - Tshwane Varsity Hackathon</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
+          <t>https://tvh.icep.co.za/</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Unisa's Information and Communication Technology Portfolio, in collaboration with the College of Science, Engineering and Technology, held the first-ever Unisa Hackathon on 3 and 4 July 2025, marking a major step in the university's journey to embed digital innovation and entrepreneurship into the students learning experience.</t>
+          <t>The 8th Annual TVH will use a hackathon format, underpinned by Agile Scrum and Microsoft cloud computing practices, to deliver fresh ideas and solutions that catalyze 4IR on the African continent.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3143,7 +3135,11 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>info@tvh.co.za, MagasengQM@tut.ac.za</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3158,7 +3154,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons Join South Africa's premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
+          <t>Instead of focusing on building a once-off project, our hackathons centre around optimisation problems. Participants develop solutions that are tested, scored, and ranked based on performance, efficiency, and strategy.</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3171,17 +3167,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Young Engineers Showcase Innovation at STEM Hackathon</t>
+          <t>Unisa hosts first-ever Hackathon to ignite student learning ...</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>https://www.futuresa.co.za/education/young-engineers-movement-stem/</t>
+          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Young Engineers Build Solutions for Real-World Challenges at STEM Hackathon Fifty-five high school learners and 11 teachers from underserved South African schools will showcase working engineering and technology prototypes at the Young Engineers Movement (YEM) Hackathon Exhibition Day on 26 June 2026.</t>
+          <t>Jul 14, 2025 · The event supported key priorities of South Africa’s National Development Plan, Unisa’s Catalytic Niche Areas and the United Nations’ Sustainable Development Goals that relate to access to quality education, decent work and innovation.</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3189,26 +3185,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>info@futuresa.co.za</t>
-        </is>
-      </c>
+      <c r="E113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Hackathons | Sebaka</t>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://sebakasouthafrica.co.za/hackathons.html</t>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Sebaka Mentorship &amp; Hackathons — Build an AI Agent for Software Quality Engineering.</t>
+          <t>Sep 2, 2026 · The Young Engineers Movement (YEM) is an immersive engineering and technology hackathon designed to equip young South Africans with the skills, mindset and confidence needed to solve real-world challenges.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3216,22 +3208,26 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>marketing@ortsa.org.za, info@ortsa.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>The Home of South African Hackathons</t>
+          <t>CompeteHub - Where Champions Are Made</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/partners/</t>
+          <t>https://www.devpluxe.co.za/</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>South Africa Policy Hackathon Hello Ladies, Happy New Year. Some of you may be interested in this workshop. The workshop is flagged for South African nationals working at research and innovation offices, accelerators, innovation hubs and incubators, tech centers, and start-ups working on dual-use...</t>
+          <t>Join thousands of developers, designers, and innovators competing in South Africa ' s most impactful tech hackathons. We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3240,83 +3236,6 @@
         </is>
       </c>
       <c r="E115" t="inlineStr"/>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>Young Engineers Movement (YEM) - ORT SA</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>CompeteHub - Where Champions Are Made</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>https://www.devpluxe.co.za/</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>About DevPluxe Empowering South Africa ' s next generation of innovators We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr"/>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>Talks &amp; Fireside | Builders Table</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>https://builderstable.net/</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>Builders Table is a two-day hackathon hosted by MakeReign, built around a 24-hour build sprint. It brings together South Africa's designers, developers, strategists, founders and creative technologists to build real working prototypes under real time pressure.</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>liamlr95@gmail.com, sarah.chen@horizonlabs.com</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-09-26
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E115"/>
+  <dimension ref="A1:E121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Africa Prize For Engineering Innovation - Wikipedia</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://en.wikipedia.org/wiki/Africa_Prize_For_Engineering_Innovation</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ASTEMI is a collaboration that ... &amp; Competitions to a broader base of learners and educators. ASTEMI is a national non-profit organization of independent organizations; teachers, public organisations and volunteers dedicated to improving and promoting science education and providing recognition for outstanding achievement by both learners and teachers. To promote excellence in Science, Technology, Engineering, Mathematics and Innovation in South African ...</t>
+          <t>March 7, 2026 - These competitors receive training and support and they get the opportunity to improve their networking. The winner receives £25,000 and the second, third and fourth places are awarded £10,000. ... ↑ "Royal Academy of Engineering Africa Prize for Engineering Innovation 2022 in Sub-Saharan Africa (£25,000 Prize) – Opportunities For Africans" (in French). 2021-04-22. Retrieved 2024-11-10. 1 2 "First South ...</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -469,17 +469,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Some of our sparkling achievements during 2014 – to help the NRF and DSI grow a representative science and technology workforce in the country – SAASTA has run a number of maths and science educator development programmes and a number of learner development programmes, including maths and science camps for learners with potential, olympiads and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>August 6, 2026 - South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -492,17 +492,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sep 4, 2025 · The Africa Prize for Engineering Innovation is open to individuals or teams based in sub-Saharan Africa who have a scalable engineering innovation with social or environmental impact potential.</t>
+          <t>Some of our sparkling achievements during 2014 – to help the NRF and DSI grow a representative science and technology workforce in the country – SAASTA has run a number of maths and science educator development programmes and a number of learner development programmes, including maths and science camps for learners with potential, olympiads and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -510,26 +510,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the IEOM Cape Town, South Africa 2026 conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -537,26 +533,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Selected papers will be considered for the competition and must be presented at the 2024 South Africa Conference. The paper will be judged based on the technical content and presentation.</t>
+          <t>ASTEMI is a collaboration that ... &amp; Competitions to a broader base of learners and educators. ASTEMI is a national non-profit organization of independent organizations; teachers, public organisations and volunteers dedicated to improving and promoting science education and providing recognition for outstanding achievement by both learners and teachers. To promote excellence in Science, Technology, Engineering, Mathematics and Innovation in South African ...</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -564,26 +556,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
+          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -591,22 +579,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>user@domain.com, info@zasdc.org</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Engineering Competition For African Youth In Engineering ...</t>
+          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://www.thecasecentre.org/products/view?id=189255</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Aug 18, 2025 · This call invites engineers and innovators from across sub-Saharan Africa to apply with scalable innovations that address pressing social and environmental challenges.</t>
+          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -619,17 +611,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>August 6, 2026 - South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -642,17 +634,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -665,17 +657,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Engineering Conferences in South Africa 2025-2026</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -688,17 +680,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://madeinafricaevent.co.za/</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Africa Tech Festival takes place in Cape Town and attracts attendees from across Africa, Europe, the Middle East and global technology markets. ... The festival covers telecoms, AI, cybersecurity, data centres, digital transformation, fintech, ...</t>
+          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -706,26 +698,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, support@knect365.com, customerservices@informaconnect.com, support@informaconnect.com</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
+          <t>KZN Industrial Technology Exhibition</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://innovationweek.co.za/</t>
+          <t>https://www.kznindustrial.co.za/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SAIW’ 26 is designed as a week-long national programme to feature provincial innovation engagements across South Africa. From 16 – 17 March, Provinces will showcase local innovation strengths, emerging enterprises and sectoral capabilities.</t>
+          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s leading platform for industrial innovation ...</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -735,24 +723,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>info@pixal8media.co.za</t>
+          <t>john@email.com</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show ...</t>
+          <t>South Africa International Industrial Expo | Innovation Bridge</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://aiexpoafrica.com/</t>
+          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>(2 Day Event) 28th-29th October 2026 Sandton Convention Centre, JHB, South Africa AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
+          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -760,26 +748,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>enquiries@aiexpoafrica.com</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IT Indaba 2026 – Africa's biggest IT Conference and Expo</t>
+          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://it-indaba.co.za/</t>
+          <t>https://manufacturingindaba.co.za/exhibition/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what’s next before everyone else does. Only 2,500 free tickets are available.</t>
+          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -792,17 +776,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Explore IT &amp; Technology Trade Events in south-africa ...</t>
+          <t>Exhibition | Innovation Festival Durban | South Africa</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
+          <t>https://www.innovationfestival.durban/exhibition</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
+          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -810,22 +794,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Erika@innovate.durban, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, sithabile@innovate.durban, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Fak'ugesi Festival – African Digital &amp; Innovation Festival</t>
+          <t>International Science, Innovation &amp; Technology Expo (INSITE)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://www.fakugesi.co.za/</t>
+          <t>https://www.dsti.gov.za/index.php/resource-center/27-temp/dst-links/3-international-science-innovation-a-technology-expo</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fak'ugesi is Africa's premier digital innovation festival, held annually at the Tshimologong Digital Innovation Precinct in Johannesburg. Now in its thirteenth year, it convenes creatives, technologists, researchers, policymakers, and industry practitioners across five intensive days of programme, exhibition, and exchange.</t>
+          <t>The essence of INSITE INSITE is an international, biennial must-see Science and Technology event in South Africa, the only one of its kind in Africa that creates new frontiers for global challenges · INSITE aims to assemble the worlds leading innovators and scientists in one place, stimulating ...</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -838,17 +826,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -861,17 +849,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>KZN Industrial Technology Exhibition</t>
+          <t>AAXO - The Association of African Exhibition Organisers</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.kznindustrial.co.za/</t>
+          <t>https://www.aaxo.co.za/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s leading platform for industrial innovation ...</t>
+          <t>February 20, 2026 - CAPE TOWN, South Africa – The inaugural Festival of Eventing (FOE) brought together 350 event professionals, 85 speakers, and 10 countries under one roof for a two-day showcase of innovation, inspiration, and industry connection.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -879,26 +867,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>john@email.com</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://10times.com/southafrica/tradeshows</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>South Africa trade shows, find ... Profile, Exhibitor Information etc. Listing of 166 upcoming expos in 2026-2027 1. Mining Connect Day, 2. Annual ACFE Africa Conference &amp; Exhibition, 3. Annual Smart Procurement World Indaba, ...</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -911,17 +895,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>South Africa International Industrial Expo | Innovation Bridge</t>
+          <t>Come and explore our exhibition of innovative discoveries at Science Forum South Africa 2024 | CSIR</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
+          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
+          <t>December 3, 2024 - The exhibition launch will take place on Tuesday, 3 December 2024, with the opening address by Department of Science, Technology and Innovation Minister Dr Blade Nzimande.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -957,17 +941,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Engineering For People Design Challenge - EWBSA</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
+          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community's challenges and how community members view the impact of these challenges on their daily lives.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -975,26 +959,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering For People Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community's challenges and how community members view the impact of these challenges on their daily lives.</t>
+          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1002,26 +982,22 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge returns to Johannesburg!</t>
+          <t>Engineering for People Design Challenge - Engineers Without Borders UK</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.ewb-uk.org/efp-returns-to-johannesburg/</t>
+          <t>https://www.ewb-uk.org/upskill/design-challenges/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Now entering its fourteenth year, we're delighted to announce that our award-winning design challenge will be returning to Makers Valley in Johannesburg, South Africa for the 2024/25 cycle.</t>
+          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1034,17 +1010,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
+          <t>This year's design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1054,24 +1030,24 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>team@crowdsolve.net</t>
+          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>This year's design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
+          <t>The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1081,7 +1057,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>marketing@eng.cam.ac.uk, web-editor@eng.cam.ac.uk</t>
+          <t>team@crowdsolve.net</t>
         </is>
       </c>
     </row>
@@ -1134,17 +1110,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Engineers Without Borders South Africa - Facebook</t>
+          <t>Engineering for People in Makers Valley | PDF | Apartheid | South Africa</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/EngineersWithoutBordersSouthAfrica/posts/were-building-something-bigthe-engineers-without-borders-south-africa-team-recen/1168670565286616/</t>
+          <t>https://www.scribd.com/document/784038503/2024-25-Engineering-for-People-Design-Challenge-Makers-Valley</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>South Africa's future engineers are ready to solve real- world challenges. On 22 January 2027, the best student teams from across the country will compete at the Engineering for People Design Challenge Grand Finals, showcasing innovative solutions that place people, communities, and sustainability at the heart of engineering. 🏆 One stage.</t>
+          <t>Engineering ENGINEERING for FOR people PEOPLE Design DESIGNchallenge CHALLENGE 2024-5 2024-25 Makers MakersValley Valley Johannesburg, Johannesburg,South SouthAfrica Africa fEngineering for People Design Challenge 2024-25 The Engineering for People Design Challenge contributed their time and expertise to enhance the has been delivered in the UK and Ireland since content of this design ...</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1180,17 +1156,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>April 28, 2026 - Seven postgraduate students from the Faculty of Engineering have been selected to represent South Africa at the · Mission Idea Contest (MIC), a global space engineering competition held in Tokyo, Japan.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1198,26 +1174,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026 South Africa Engineering Competition</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://notice.ukzn.ac.za/content/GetFile.aspx?id=96048</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Best Regards, The 2026 SA Engineering Competition Team University of KwaZulu-Natal • Elsevier</t>
+          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1230,17 +1202,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>University Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1248,26 +1220,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
+          <t>ASTEMI brings together all role ... Olympiads in South Africa. THE UNIVERSITY OF CAPE TOWN MATHEMATICS COMPETITION ... National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology ...</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1280,17 +1248,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>National Student Competition | ORSSA</t>
+          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://www.orssa.org.za/studentcomp</t>
+          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
+          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1298,26 +1266,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, email@example.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>Engineering in South Africa: 24 Best universities Ranked</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://edurank.org/engineering/za/</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>March 15, 2026 - You can find information about ... Africa based on the number of universities and their ranks are Cape Town, Johannesburg, Stellenbosch, and Pretoria....</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1330,17 +1294,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>This Competition is for undergraduate students in the last two years of study (years 4 and 5) or recent 2021 graduates who will be required to design localized solutions addressing African challenges.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1348,26 +1312,22 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1380,17 +1340,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent's largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
+          <t>University Overall Rankings - Engineering - Africa 2025</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1403,17 +1363,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Competitions - Enactus South Africa | National Expos, Challenges ...</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://enactusza.org/what-we-do/competitions</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
+          <t>Some of our sparkling achievements ... and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation ...</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1421,11 +1381,7 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>liso@enactus.org, marketingsa@enactus.org, xmadlanga@enactus.org, adminsa@enactus.org</t>
-        </is>
-      </c>
+      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1500,7 +1456,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>u003einfo@techspo.co, atinfo@techspo.coor</t>
+          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
         </is>
       </c>
     </row>
@@ -1552,11 +1508,7 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>info@techspocapetown.co.za</t>
-        </is>
-      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1581,7 +1533,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>salesenquiries@africatechfestival.com, dataprivacy@informaconnect.com, customerservices@knect365.com, dataprivacy@knect365.com, support@knect365.com, customerservices@informaconnect.com, support@informaconnect.com</t>
+          <t>support@knect365.com, dataprivacy@informaconnect.com, dataprivacy@knect365.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, support@informaconnect.com, customerservices@knect365.com</t>
         </is>
       </c>
     </row>
@@ -1606,26 +1558,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>claire@mediatech.co.za, simon@mediatech.co.za</t>
-        </is>
-      </c>
+      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
+          <t>HOME | Africa Tech Week</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
+          <t>https://africatechweek.co.za/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Share this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaSave this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
+          <t>May 11, 2026 - From sensational speakers, to top tech exhibitons, see what’s in store when you attend the 2-day Sentech Africa Tech Week Conference in 2025&gt;&gt; ... Sponsor, Speak, Attend! For more information on how you can be a part of the #ATW family, contact ...</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1638,17 +1586,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>HOME | Africa Tech Week</t>
+          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://africatechweek.co.za/</t>
+          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>May 11, 2026 - From sensational speakers, to top tech exhibitons, see what’s in store when you attend the 2-day Sentech Africa Tech Week Conference in 2025&gt;&gt; ... Sponsor, Speak, Attend! For more information on how you can be a part of the #ATW family, contact ...</t>
+          <t>Share this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaSave this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1681,7 +1629,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>you@company.com, events@techspojoburg.co.za, support@industryevents.com, your@email.com, colleague@company.com</t>
+          <t>your@email.com, events@techspojoburg.co.za, you@company.com, colleague@company.com, support@industryevents.com</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1646,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>March 7, 2025 - Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds ...</t>
+          <t>Maker Faire Africa, Cairo, October 2011 Presently curated and organized by Emeka Okafor, Henry Barnor and Jennifer Wolfe, Maker Faire Africa is an international organization co-founded by Mark Grimes (Felonious Nun) Emeka Okafor (TED Africa), Lars Hasselblad Torres (IDEAS Global Challenge), Erik Hersman (Afrigadget) and Nii Simmonds (Nubian Cheetah). Maker Faire Africa aims to engage with on ...</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1721,7 +1669,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2 weeks ago - Maker Faires are also held in Europe, Asia, South America and Africa.</t>
+          <t>Maker Faire is a convention of do it yourself (DIY) enthusiasts established by Make magazine in 2006. Participants come from a wide variety of interests, such as robotics, 3D printing, computers, arts and crafts, and hacker culture.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1734,17 +1682,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2015 Cape Town Maker Movement | Makers Faire South Africa, Tech &amp; Innovation, Making Things, Collaboration &amp; Knowledge Sharing</t>
+          <t>Maker Faire |</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://www.capetownmagazine.com/whats-the-deal-with/how-to-survive-a-robot-uprising-hint-join-the-maker-movement/125_22_19889</t>
+          <t>https://makerfaire.com/</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>A little while ago, the Maker Faire came to Cape Town and Tom and I made a point of popping in to suss out what it’s all about. We’d been to KAT-O’s #TechTalkCPT Makers &amp; Innovators event featuring Omar-Pierre Soubra (one of the original Maker Faire initiators), and his infectious enthusiasm convinced us that the Maker Movement could be a very good thing for South Africa indeed.</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1752,22 +1700,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>pr@make.co</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>About | Maker Faire Cape Town: Make • Create • Craft • Build • Play</t>
+          <t>Upcoming Faires - Maker Faire</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://makerfairecapetown.wordpress.com/about/</t>
+          <t>https://makerfaire.com/upcoming-faires/</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>July 30, 2015 - ... The City of Cape Town, being the World Design Capital 2014 and one of the base of a lot of Afrika Burn, is the ideal choice for celebrating the Movement Maker in South Africa...</t>
+          <t>The largest celebration of invention, creativity, curiosity and hands-on learning that is inspiring the future. Showcasing the very best of the global Maker Movement represented by hundreds of makers and presenters from all over the world, World Maker Faire New York features more than 800 projects and multiple stages with latest developments in microelectronics, 3D printing, food, drones ...</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1775,22 +1727,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, pr@make.co, fancybox_sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
+          <t>Maker Faire Africa — Grokipedia</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>http://capetown.makerfaire.com/</t>
+          <t>https://grokipedia.com/page/maker_faire_africa</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>April 20, 2026 - Maker Faire is not an event that has to do strictly with people making hardware. For me it’s much more important because it opens up channels of communication between makers and the concept of making together.</t>
+          <t>Maker Faire Africa Maker Faire Africa is a pan-African series of events that celebrate local ingenuity, innovation, and invention by bringing together makers, inventors, and DIY enthusiasts to showcase practical projects addressing everyday challenges across the continent.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1798,26 +1754,22 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>chosen-sprite@2x.png, fancybox_sprite@2x.png, pr@make.co, fancybox_loading@2x.gif</t>
-        </is>
-      </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Johannesburg | Contemporary And (C&amp;)</t>
+          <t>Maker Faire | Start A Community Maker Faire - Maker Faire</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://contemporaryand.com/en/events/maker-faire-africa-comes-to-johannesburg</t>
+          <t>https://capetown.makerfaire.com/</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014. Makers from across Africa will join ZA Makers for 4-days of meet-ups, mash-ups, workshops, and seed-starting ideas for ...</t>
+          <t>Community maker faires bring maker faire to your community! Jump into the Make: community and bring a Maker Faire to your town, city, or region! Spark curiosity, rally makers of all ages, and plug your local scene into a global movement fueled by creativity, resilience, innovation, and hands-on learning.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1825,22 +1777,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, pr@make.co, fancybox_sprite@2x.png</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Blog : Maker Faire Africa</t>
+          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>http://makerfaireafrica.com/blog/</t>
+          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>December 31, 2021 - You can help them out on the new South African crowdfunding site, ThundaFund. ... One of the most ambitions items at Maker Faire Africa this year in Johannesburg, South Africa is Samuel Ngobeni’s “art car”. He’s a designer from Germinston, who has spent the last three years building his ANIMAL car, from the ground up, that means the frame and all.</t>
+          <t>DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1853,17 +1809,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Maker Faire Africa comes to Jo’Burg – AfriGadget</t>
+          <t>Maker Faire groups | Meetup</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.afrigadget.com/2014/07/08/maker-faire-africa-comes-to-joburg/</t>
+          <t>https://www.meetup.com/topics/maker-faire/za/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Maker Faire Africa was first held in Ghana in 2009, then Kenya 2010, Egypt 2011, Nigeria 2012 and now in South Africa 2014.</t>
+          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1876,17 +1832,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Why Africa needs Maker Faire | ZDNET</t>
+          <t>Maker Faire Africa - Facebook</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.zdnet.com/article/why-africa-needs-maker-faire/</t>
+          <t>https://www.facebook.com/MFAJoburg/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>July 24, 2014 - "This year we're looking to have Maker Faire Africa in Johannesburg," Okafor said. "We haven't been to southern Africa before, and South Africa will probably be different again to previous events.</t>
+          <t>Maker Faire Africa. 520 likes. Where Africa's future is in the making.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1899,17 +1855,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Makers Festival SA 🛠️ (@makersfestival_sa) • Instagram photos ...</t>
+          <t>MakeAfrica - Le festival africain de l'innovation technologique et de ...</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/makersfestival_sa/</t>
+          <t>https://makeafrica.tech/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>8,503 Followers, 58 Following, 57 Posts - Makers Festival SA 🛠️ (@makersfestival_sa) on Instagram: "🛠️ Building Skills. Building Memories. 🏕️ 8th &amp; 9th November 2025 / Cape Town, SA 🪵 Founder @hutch_custom 📩 DM us - apply to be a MAKER 🫶🏼"</t>
+          <t>Le festival africain de l'innovation technologique et de la culture maker Un événement africain pensé par des africains et qui vise à partager, créer, fabriquer et apprendre les uns des autres. Il regroupe stands de démonstration, ateliers de découverte, présentations et conférences autour des sujets liés à l'innovation, la créativité, la fabrication, le numérique, les ...</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1922,7 +1878,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1932,7 +1888,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>All these Olympiads and Competitions have a positive impact on education and on educational institutions in South Africa, but there is still a need to build stronger collaboration among teachers, schools, universities and educational authorities in order to meet the challenges of STEM education in South Africa today.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1945,17 +1901,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Samsung opens Solve for Tomorrow 2026 STEM competition to all South African public schools</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>February 27, 2026 - Samsung Electronics South Africa has opened applications for the 2026 edition of Solve for Tomorrow (SFT), its annual science, technology, engineering, and mathematics (STEM) competition aimed at Grade 10 and 11 learners.</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1968,17 +1924,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Astemi Sa</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2001,7 +1957,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>High school students can submit individual and/or team research projects in the field of Science, Technology, Engineering, Mathematics or similar areas. Each submission can provide a summary of the STEM project. All projects must be presented at the IEOM Cape Town, South Africa 2026.</t>
+          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2009,26 +1965,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://www.samsung.com/za/solvefortomorrow/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Rooted in the belief that today’s youth hold the key to tomorrow’s progress, Solve for Tomorrow South Africa provides participants with the tools, mentorship, and platforms they need to turn ideas into action.</t>
+          <t>The IEOM High School/Middle School STEM Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2041,17 +1993,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ASTEMI SA</t>
+          <t>STEM Scholars — 2026 STEM &amp; Entrepreneurship Discovery Initiative</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://stemscholars.co.za/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>Building South Africa's Next Generation of Innovators The STEM &amp; Entrepreneurship Discovery Initiative connects learners with a world that's often invisible from inside a classroom — and equips them with skills that last far beyond the competition.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2059,22 +2011,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>marushka@stemscholars.co.za, inforeg@justice.gov.za, you@school.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>DEPARTMENT OF BASIC EDUCATION AND SAMSUNG SOUTH AFRICA ...</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://www.education.gov.za/Portals/0/Media/Preess+Releases/2026+Media+Releases/Applications+for+2026+Samsung+Solve+For+Tomorrow.pdf</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Samsung Solve for Tomorrow is a global innovation competition that empowers Grade 10 and 11 learners in public schools to design science, technology, engineering and mathematics (STEM) solutions that address real-world challenges within their communities.</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2087,17 +2043,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Southafrica 2024</t>
+          <t>School Challenges - STEMLab - Coding &amp; Robotics Academy</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/high-school-stem-competition/</t>
+          <t>https://stemlab.co.za/school-challenges/</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>The IEOM High School Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects. High school students can submit individual and/or team research projects in the field of Science, ...</t>
+          <t>W elcome to the STEMLab Schools Challenge 2026, the most exciting robotics and coding competition for schools in South Africa! Starting in the Western Cape, this unique event offers learners the opportunity to showcase their skills in a fast-paced, thrilling battle of Engineering and Technology.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2107,24 +2063,24 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>info@ieomsociety.org</t>
+          <t>eltonearn9@gmail.com, noreply@stemlab.co.za, info@stemlab.co.za, elton@stemlabco.za</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>SA young scientists selected for global competition at Regeneron ISEF in the USA - Eskom</t>
+          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://www.eskom.co.za/sa-young-scientists-selected-for-global-competition-at-regeneron-isef-in-the-usa/</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>May 6, 2025 - Regeneron ISEF 2025, the world’s largest pre-college science, technology, engineering and mathematics (STEM) competition, will take place from 10 to 16 May in Columbus, Ohio in the USA.</t>
+          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2132,26 +2088,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>MediaDesk@eskom.co.za</t>
-        </is>
-      </c>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions 2022 – SAASTA</t>
+          <t>Imbewu Foundation</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://saasta.ac.za/astemi-competitions-2</t>
+          <t>https://imbewu.foundation/</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>Seeding Future Scientists IMBEWU Science Foundation is a youth-focused STEMI organisation based in George, Western Cape, serving learners, educators and communities across the Eden District and Central Karoo District. We exist to nurture talent, ignite curiosity and create meaningful pathways for young South Africans to reach their full potential in science, technology, engineering ...</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2184,24 +2136,24 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com</t>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>South Africa to host first World Robot Olympiad International Final in Africa in 2028 - WRO Association</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://wro-association.org/south-africa-to-host-first-world-robot-olympiad-international-final-in-africa-in-2028/</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>1 week ago - Johannesburg, South Africa, 12 September 2026 — South Africa will host the World Robot Olympiad (WRO®) International Final in 2028, bringing WRO’s flagship global robotics competition to the African continent.</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge, organized by ITU and The Cortex Hub, in partnership with Google.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2211,24 +2163,24 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>1-Team-CARED-Philippines-500x383@2x.jpg, Prithul-3rd-place-Future-Engineers-2022-A-500x383@2x.jpg, Annual-report-article-TZ-500x383@2x.jpg, Costa-Rica-team-Sprout-release-banner-500x383@2x.jpg</t>
+          <t>name@example.com</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
+          <t>Robotics for Good Youth Challenge | The Cortex Hub</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa-2/</t>
+          <t>https://www.thecortexhub.africa/roboticsforgoodyouthchallenge</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>April 14, 2026 - Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in the leading UN-based global robotics competition, focusing on the critical area of agriculture and food security.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2238,24 +2190,24 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>name@example.com</t>
+          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, info@thecortexhub.africa, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Cape Town to host Africa’s first World Robot Olympiad</t>
+          <t>Robotics for Good Youth Challenge South Africa - AI for Good</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://www.capetownetc.com/tech/cape-town-africas-first-world-robot-olympiad/</t>
+          <t>https://aiforgood.itu.int/event/robotics-for-good-youth-challenge-south-africa/</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>4 days ago - Cape Town will host the World Robot Olympiad International Final in 2028, bringing top youth robotics teams from around the world to South Africa.</t>
+          <t>The Robotics for Good Youth Challenge South Africa is the prestigious South African National Event of the Robotics for Good Youth Challenge. Experience the excitement as South African teams showcase their skills in a UN-based global robotics competition, focusing on the critical area of disaster response.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2263,22 +2215,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>name@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>FIRST South Africa – Robotics Programs for School Children</t>
+          <t>2026 - SpringBots South Africa</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://firstsa.org/</t>
+          <t>https://springbots.co.za/2026-2/</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>From Discover, to Explore, and then to Challenge, students will understand the basics of STEM and apply their skills in an exciting competition while building habits of learning, confidence, and teamwork skills along the way. FIRST Tech Challenge students learn to think like engineers. Teams ...</t>
+          <t>This approach ensures that learners are not only participants in robotics competitions but are also equipped with real-world skills in design thinking, programming, systems engineering, and collaborative problem-solving. A Unified Future for Africa SpringBots' 2026 vision extends beyond competition and education.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2291,17 +2247,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>Roboticon 2026: South Africa Showcases Robotics for Culture, Education ...</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop ...</t>
+          <t>The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation." South Africa's robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2309,22 +2265,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>newspaper-rec300@2x.jpg, adverts@ubuntutimes.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>South African Robotics Competitions and Schools</t>
+          <t>SpringBots South Africa</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://www.sciencexpo.org.za/robotics.html</t>
+          <t>https://springbots.co.za/</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>North Gauteng Senior Science Fair is the oldest science fair in South Africa.</t>
+          <t>SpringBots South Africa Igniting The Potential of South Africa's Next Generation By Bridging The Digital Divide Through High Impact Robotics, Immersive STEAM Initiatives and Targeted Short Courses Designed For The Future Of Work and Innovators.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2332,26 +2292,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>madelien@imbewu.foundation, marna.vanzyl@imbewu.foundation, webmaster@sciencexpo.org.za</t>
-        </is>
-      </c>
+      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Limpopo Learners Represent South Africa at Global Robotics Finals in Switzerland - African Times</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://www.atnews.co.za/limpopo-learners-represent-south-africa-at-global-robotics-finals-in-switzerland/</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>July 7, 2026 - The international competition, taking place from 7 to 10 July 2026 at the Palexpo International Exhibition and Convention Centre in Geneva, brings together some of the world’s brightest young innovators to develop technological solutions to ...</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop their creativity and problem-solving skills through challenging and educational robotics competitions.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2359,26 +2315,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>NkosiN@atnews.co.za, rampedim@atnews.co.za</t>
-        </is>
-      </c>
+      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - AfrikaBot</t>
+          <t>ROBO-RUMBLE 2026 — Innovation in Motion</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/displaycustomlink.aspx?name=AfrikaBot</t>
+          <t>https://roborumble.net/</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>(ADDITIONAL VIDEO SUPPLIED BY UJ ... African teenagers to get early exposure to engineering concepts through involvement in AfrikaBOT 'the world's most affordable robotics competition'....</t>
+          <t>South Africa's premier youth robotics &amp; technology competition. Robo Wars, Drone Racing, Grand Prix &amp; Innovation Challenge. August 2026.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2391,17 +2343,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>WorldSkillsZA Mobile Robotics Provincial Competition 2024</t>
+          <t>Home | Roboticon 2026</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://worldskillsza.dhet.gov.za/site/WSZA-Prov-Comp/Provincial-Competitions.aspx</t>
+          <t>https://roboticon.resolute.education/</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>The WorldSkills South Africa (WSZA) will be having its Mobile Robotics Combined Provincial Competitions in Lephalale TVET College from the 07th - 10th October 2023. the first 3 days will be focused on training and the last day will be the actual Mobile Robotics competition.</t>
+          <t>Thank you for joining us at the ultimate robotics showcase, as Resolute proudly sponsored the World Robotics Olympiad (WRO) South Africa. This year we brought together two worlds for the biggest robotics event of the year - Roboticon and the WRO Nationals, on the same day at the same venue.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2414,17 +2366,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>Civil Engineering Tenders - Tender Bulletins</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
+          <t>https://tenderbulletins.co.za/tender-category/civil-engineering/</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
+          <t>Browse current and past Civil Engineering tenders published by South African government departments, municipalities, state-owned entities and private companies looking to procure civil engineering. Tenders in this category ask suppliers to quote on civil engineering - anything from once-off supply contracts to multi-year service agreements, depending on the issuing organisation's needs ...</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2432,26 +2384,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>chanel@engineeringnews.co.za, newsdesk@engineeringnews.co.za, subscriptions@creamermedia.co.za, newsletters@creamermedia.co.za, advertising@creamermedia.co.za</t>
-        </is>
-      </c>
+      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd International Bridge Building Competition - SAICE</t>
+          <t>SAICE's 34th International Bridge Competition Inspires Tomorrow's ...</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://saice.org.za/press-releases/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://southafricatoday.net/lifestyle/education/saices-34th-international-bridge-competition-inspires-tomorrows-engineers/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>April 17, 2025 - The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2459,26 +2407,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>membership@saice.org.za, communications@saice.org.za, marketing@saice.org.za, civilinfo@saice.org.za, accounts@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
+          <t>Civil engineering Tenders | Business Opportunities in South Africa</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
+          <t>https://www.tenders-sa.org/sa-tenders/categories/civil-engineering</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
+          <t>Find the latest Civil engineering tenders and government contracts in South Africa. Browse active bids, view requirements, closing dates, and procurement details for Civil engineering opportunities.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2486,26 +2430,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>constr@crown.co.za, ernao@crown.co.za</t>
-        </is>
-      </c>
+      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
+          <t>Engineering the future: 16 schools compete in SAICE's 33rd ...</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
+          <t>https://www.southafricanbusiness.co.za/08/2024/construction-and-engineering/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2518,17 +2458,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
+          <t>Civil Engineering Tenders | eTender SA</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
+          <t>https://etendersa.co.za/tenders-south-africa/civil-engineering/</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>September 7, 2025 - Find all upcoming Civil Engineering conferences in South Africa 2025 with invitation letter. South Africa is a diverse and dynamic country that offers a wide range of opportunities for Civil Engineering conferences in topic Civil Engineering, and many more.</t>
+          <t>Civil Engineering Tenders in SA, Mining tenders, Road construction tenders in South Africa, and Bridge construction tenders in South Africa.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2541,17 +2481,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SWM Communications | SAICE recognises civil engineering research excellence through national student competition</t>
+          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://swmcommunications.co.za/press-office/saice-recognises-civil-engineering-research-excellence-through-national-student-competition/</t>
+          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>April 1, 2026 - April 2022: The South African Institution of Civil Engineering (SAICE) recently joined forces with leading universities across the country to award civil engineering students for their research efforts.</t>
+          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2559,26 +2499,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>nthabeleng@saice.org.za, info@swmcommunications.co.za</t>
-        </is>
-      </c>
+      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
+          <t>Home - SAICE</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
+          <t>https://saice.org.za/</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2586,22 +2522,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>barbara@avenue.co.za, executiveadmin@saice.org.za, membership@saice.org.za, communications@saice.org.za, accounts@saice.org.za, civilinfo@saice.org.za, marketing@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
+          <t>SAICE | Events and Awards</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
+          <t>https://members.saice.org.za/events-and-awards</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>4th International Conference on Advances in Science, Engineering &amp; Technology(ICASET-2025) [Accredited CPD Event]</t>
+          <t>The South African Institution Of Civil Engineering SAICE hosts the Awards Function annually to honour individuals, projects of excellence, as well as community-oriented initiatives. The annual awards function gives companies and individuals a unique opportunity to showcase their deserving projects and work to the industry.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2614,17 +2554,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>Greenovate</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
+          <t>https://greenovatecompetition.co.za/</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
+          <t>Growthpoint Properties and the Green Building Council South Africa invites you to Register for the 2026 Greenovate Awards, inspiring a new wave of industry talent to innovate for sustainability.</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2637,17 +2577,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Civil Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
+          <t>Awards 2026 - SAICE</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
+          <t>https://saice.org.za/awards-2026/</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Nov 03 International Conference on Civil and Environmental Engineering (ICCEE) - Cape Town, South Africa</t>
+          <t>Learn about SAICE's award categories, submission guidelines, key dates and how to nominate project and professionals.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2655,22 +2595,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>membership@saice.org.za, communications@saice.org.za, accounts@saice.org.za, civilinfo@saice.org.za, marketing@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2683,17 +2627,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions. Whether you're working in traditional engineering fields or applying innovation in areas like health, agriculture, or digital technology, the Africa Prize for Engineering Innovation offers a unique platform to ...</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2706,17 +2650,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2729,17 +2673,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2747,26 +2691,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>Opportunities in Mechanical Engineering across South Africa.</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.puffandpass.co.za/tag/mechanical-engineering</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>Location: Johannesburg Hatch is seeking Electrical / Civil / Mechanical Engineering Graduates who will support projects globally. The engineering team is comprised of professional engineers, designers and technologists. We have experience…</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2774,11 +2714,7 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2806,17 +2742,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Competitions - Prized Competitions South Africa</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.prized.co.za/competitions/</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Prized is home to Online Competitions in South Africa. Enter any competition that peaks your interest and join the Prized community.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2824,26 +2760,22 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>info@ieomsociety.org</t>
-        </is>
-      </c>
+      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
+          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
+          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent's largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
+          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2856,17 +2788,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
+          <t>SAIMechE</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
+          <t>https://www.saimeche.org.za/</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2879,17 +2811,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>Greenovate</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>https://greenovatecompetition.co.za/</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>Growthpoint Properties and the Green Building Council South Africa invites you to Register for the 2026 Greenovate Awards, inspiring a new wave of industry talent to innovate for sustainability.</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2902,17 +2834,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>If you applied and met all the requirements, you should not miss out on this life changing opportunity to be part of the WorldSkills South African Team that will travel to Shanghai China next year to compete with more than 1500 Competitors from over 65 countries and regions at the WorldSkills International Competition taking place from 22 - 27 ...</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2925,17 +2857,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>2026 South Africa Engineering Competition</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://notices.ukzn.ac.za/content/GetFile.aspx?id=96047</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role players in the field of Olympiads and Competitions – including professional and academic societies, universities and other tertiary institutions, private enterprise and government – to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>2026 South Africa Engineering Competition Organized by UKZN and Elsevier. If you are an engineering student (undergraduate or postgraduate), don't miss joining the challenge to solve real-world cases using Engineering Village and Knovel.</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2948,17 +2880,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Call to enter the Africa Prize for Engineering Innovation ...</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions.</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2971,17 +2903,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>IEEE South Africa</t>
+          <t>South African Institute of Electrical Engineers</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>http://www.ieee.org.za/</t>
+          <t>https://www.saiee.org.za/</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>The South African Section has around 1200 members and many subsections. It was formed in 1963 by the merger of the Institute of Radio Engineers (IRE, founded 1912) and the American Institute of Electrical Engineers (AIEE, founded 1884).</t>
+          <t>Design Thinking and Innovation for Engineering Professional - Online Design Thinking and Innovation for Engineering Professional - Online (opens in a new window) Training Academy Earn your CPD credits today!</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2994,17 +2926,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest ...</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 · IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa) Deadline: April 30, 2026 May 15, 2026</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3017,17 +2949,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants ...</t>
+          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Sep 4, 2025 · The Africa Prize for Engineering Innovation is open to individuals or teams based in sub-Saharan Africa who have a scalable engineering innovation with social or environmental impact potential.</t>
+          <t>IEEE-IAS Industrial Power Conversion Systems Department Serving the electrical energy conversion professional worldwide</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3035,26 +2967,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
-        </is>
-      </c>
+      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>WorldSkills South Africa 2027 Applications Now Open - Apply Online</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://www.edupstairs.org/worldskills-south-africa-2027-applications/</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Join a SAIEE Centre near you! Become a SAIEE Member today! Join a SAIEE Centre near you! How can we assist you? SAIEE LAUNCHES NEW WEBSITE AND SOLUTION! The course starts with an overview of low voltage ... Earn your CPD credits today! Read it here.</t>
+          <t>Applications are officially open for the WorldSkills South Africa 2027 National Competition, giving talented students, apprentices, learners and qualifying skilled candidates across South Africa an opportunity to demonstrate their practical abilities on a national stage.</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3064,29 +2992,29 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>glueup-logo-white@2x.png, reception@saiee.org.za</t>
+          <t>sifisomhlongo@edupstairs.org</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>THE HOME OF SOUTH AFRICAN HACKATHONS</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://hackon.co.za/</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
+          <t>electrical engineering competition South Africa</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
@@ -3094,67 +3022,67 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Hackathons en South Africa</t>
+          <t>Competitions | ESG</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://za.allhackathons.com/</t>
+          <t>https://za.rs-online.com/web/content/m/competition</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Aug 22, 2025 · Join us for an electrifying hackathon where innovation meets security and finance! This event brings together developers, data scientists, cybersecurity experts, and FinTech enthusiasts to …</t>
+          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr"/>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>example@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ICEP - Tshwane Varsity Hackathon</t>
+          <t>Best competitions to enter in South Africa this month</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://tvh.icep.co.za/</t>
+          <t>https://freehub.co.za/best-competitions-south-africa-this-month/</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>The 8th Annual TVH will use a hackathon format, underpinned by Agile Scrum and Microsoft cloud computing practices, to deliver fresh ideas and solutions that catalyze 4IR on the African continent.</t>
+          <t>Compare current South African competitions worth checking this month, with prize, cost, entry method and closing-date details from Freehub.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>engineering hackathon South Africa</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>info@tvh.co.za, MagasengQM@tut.ac.za</t>
-        </is>
-      </c>
+          <t>electrical engineering competition South Africa</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Build the Future with Entelect Hackathons</t>
+          <t>The Home of South African Hackathons</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>https://challenge.entelect.co.za/</t>
+          <t>https://hackon.co.za/</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Instead of focusing on building a once-off project, our hackathons centre around optimisation problems. Participants develop solutions that are tested, scored, and ranked based on performance, efficiency, and strategy.</t>
+          <t>A #SouthAfrican community driven hackathon series to showcase sustainable and innovative solutions being produced by local tech champions HackOn is your full guide to everything and anything about hackathons in South Africa.</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3167,17 +3095,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Unisa hosts first-ever Hackathon to ignite student learning ...</t>
+          <t>Hackathons in South Africa: Seasonality, Cities &amp; Platforms</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>https://www.unisa.ac.za/sites/corporate/default/Colleges/Science,-Engineering-&amp;-Technology/News-&amp;-events/Articles/Unisa-hosts-first-ever-Hackathon-to-ignite-student-learning-experience</t>
+          <t>https://www.hackathonradar.com/discover/country/south-africa</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Jul 14, 2025 · The event supported key priorities of South Africa’s National Development Plan, Unisa’s Catalytic Niche Areas and the United Nations’ Sustainable Development Goals that relate to access to quality education, decent work and innovation.</t>
+          <t>When and where hackathons happen in South Africa, from 9 tracked events. Peak season is Jun (2 events), quietest is Mar (1). Midrand leads by volume.</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3190,17 +3118,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Young Engineers Movement (YEM) - ORT SA</t>
+          <t>Hackathons en South Africa</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+          <t>https://za.allhackathons.com/</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Sep 2, 2026 · The Young Engineers Movement (YEM) is an immersive engineering and technology hackathon designed to equip young South Africans with the skills, mindset and confidence needed to solve real-world challenges.</t>
+          <t>Lees meer fintech · machine learning · Security · Midrand, Gauteng, South Africa PERSOONLIK Digital ID Hackathon - Southern Africa Nov. 21, 2024 - Feb. 8, 2025</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3208,26 +3136,22 @@
           <t>engineering hackathon South Africa</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>marketing@ortsa.org.za, info@ortsa.org.za</t>
-        </is>
-      </c>
+      <c r="E114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>CompeteHub - Where Champions Are Made</t>
+          <t>Geekulcha Annual Hackathon 2026 - Registration | Sonke Platform</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://www.devpluxe.co.za/</t>
+          <t>https://sonke.gklink.co/event/gkhack26</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Join thousands of developers, designers, and innovators competing in South Africa ' s most impactful tech hackathons. We organize and host premier hackathons across the North West Province, connecting developers, designers, and dreamers to solve real problems.</t>
+          <t>GEEKULCHA ANNUAL HACKATHON 2026 Africa's premier hackathon that drives digital innovation and empowers the next generation of tech leaders.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3236,6 +3160,156 @@
         </is>
       </c>
       <c r="E115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>GirlCode | Hackathon 2026</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>https://www.girlcode.co.za/hackathon-2026</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Building Africa's Next Generation of AI-Powered Female Innovators Join Africa's largest women-in-tech hackathon empowering innovators, creators, and future founders.</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>AfriHack 2026: Pan-African Hackathon for Technology Students in ...</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>https://youthopportunitieshub.com/afrihack-2026/</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>The annual hackathon, organised by Empiras Global, is returning in 2026 for its third edition. The programme is designed to bring together technology students from South Africa, other African countries and international universities to work on authentic business challenges.</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>ICEP - Tshwane Varsity Hackathon</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>https://tvh.icep.co.za/</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Tshwane Varsity Hackathon South Africa's premier inter-university hackathon competition. Join hundreds of students for 53 hours of coding, innovation, and`` fun!</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>MagasengQM@tut.ac.za, info@tvh.co.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Build the Future with Entelect Hackathons</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>https://challenge.entelect.co.za/</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Build the Future with Entelect Hackathons Join South Africa's premier optimisation-first developer competition platform. Compete, iterate, and outperform the best.</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Young Engineers Movement (YEM) - ORT SA</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>https://www.ortsa.org.za/young-engineers-movement-yem/</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>The Young Engineers Movement (YEM) is ORT South Africa's engineering and technology hackathon empowering learners to build innovative solutions, develop STEM skills, and become the future engineers of South Africa.</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>info@ortsa.org.za, marketing@ortsa.org.za</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>AfriHack 2026 | Empiras Global</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>https://www.empirasglobal.com/afrihack26</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>The hackathon series is designed to engage technology students from all regions of South Africa in addressing authentic business challenges, while simultaneously fostering collaboration and innovation among participants.</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>engineering hackathon South Africa</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>cd64ba1f47df485bba2b0076c0dd3b25@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, 1eeb89147c984dc6bc3ffafd9e6cd089@sentry.wixpress.com, info@empirasglobal.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, e40146ef843e4f9196e5d00c98ac3689@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, a18507e8883842d8a1ba47257fee81ac@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 98b21aa53d68482b8414e892d9af0e5f@sentry-next.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 54b4aac306184111a223c0f4aea635c3@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update competition data 2026-09-27
</commit_message>
<xml_diff>
--- a/data/competitions_with_emails.xlsx
+++ b/data/competitions_with_emails.xlsx
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Africa Prize For Engineering Innovation - Wikipedia</t>
+          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Africa_Prize_For_Engineering_Innovation</t>
+          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>March 7, 2026 - These competitors receive training and support and they get the opportunity to improve their networking. The winner receives £25,000 and the second, third and fourth places are awarded £10,000. ... ↑ "Royal Academy of Engineering Africa Prize for Engineering Innovation 2022 in Sub-Saharan Africa (£25,000 Prize) – Opportunities For Africans" (in French). 2021-04-22. Retrieved 2024-11-10. 1 2 "First South ...</t>
+          <t>August 6, 2026 - South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -469,17 +469,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Team South Africa wins at NASA space engineering competition – MyBroadband</t>
+          <t>Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://mybroadband.co.za/news/science/661508-team-south-africa-wins-at-nasa-space-engineering-competition.html</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>August 6, 2026 - South African high school learners selected to participate in the International Space Settlement Design Competition had prominent roles in the winning team, with one receiving individual recognition.</t>
+          <t>Some of our sparkling achievements during 2014 – to help the NRF and DSI grow a representative science and technology workforce in the country – SAASTA has run a number of maths and science educator development programmes and a number of learner development programmes, including maths and science camps for learners with potential, olympiads and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -492,17 +492,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>ASTEMI Competitions – SAASTA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Some of our sparkling achievements during 2014 – to help the NRF and DSI grow a representative science and technology workforce in the country – SAASTA has run a number of maths and science educator development programmes and a number of learner development programmes, including maths and science camps for learners with potential, olympiads and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>ASTEMI is a collaboration that ... &amp; Competitions to a broader base of learners and educators. ASTEMI is a national non-profit organization of independent organizations; teachers, public organisations and volunteers dedicated to improving and promoting science education and providing recognition for outstanding achievement by both learners and teachers. To promote excellence in Science, Technology, Engineering, Mathematics and Innovation in South African ...</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -515,17 +515,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
+          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
+          <t>https://www.zasdc.org/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
+          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -533,22 +533,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>info@zasdc.org, user@domain.com</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ASTEMI is a collaboration that ... &amp; Competitions to a broader base of learners and educators. ASTEMI is a national non-profit organization of independent organizations; teachers, public organisations and volunteers dedicated to improving and promoting science education and providing recognition for outstanding achievement by both learners and teachers. To promote excellence in Science, Technology, Engineering, Mathematics and Innovation in South African ...</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -556,22 +560,26 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>South African Space Design Competition | Inspire Space Innovation – Join Today</t>
+          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.zasdc.org/</t>
+          <t>https://www.poidata.io/report/engineer/south-africa</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Our inaugural National Finals took place at the University of Cape Town in March 2026, and our first Team South Africa were crowned world champions at the 2027 International Finals at Kennedy Space Center.</t>
+          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -579,26 +587,22 @@
           <t>engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>user@domain.com, info@zasdc.org</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
+          <t>Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.thecasecentre.org/products/view?id=189255</t>
+          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
+          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -611,17 +615,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>The 2026 Africa Prize for Engineering Innovation wants applications from Engineers and Innovators in South Africa | South Africa Wind Energy Association</t>
+          <t>South Africa targets African engineering dominance - CAJ News Africa</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
+          <t>https://cajnewsafrica.com/2026/08/14/south-africa-targets-african-engineering-dominance/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
+          <t>August 14, 2026 - Ramaphosa said South Africa should use its engineering capabilities to manufacture and export transformers, mining machinery, railway equipment, pumps, valves, fabricated steel and electrical equipment, while also selling engineering expertise to African markets.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -634,17 +638,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Engineering Conferences in South Africa 2025-2026</t>
+          <t>GRW Engineering in South Africa: When International Competition Arrives - The Case Centre</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://internationalconferencealerts.com/south-africa/engineering</t>
+          <t>https://www.thecasecentre.org/products/view?id=189255</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Advance your research at Engineering Conferences in South Africa, where the brightest minds in civil, mechanical, electrical, and chemical engineering converge. These conferences are crucial for presenting cutting-edge developments in sustainable design, smart materials, automation, and renewable ...</t>
+          <t>GRW Engineering (Pty) Ltd (GRW) is a road transport equipment designer, manufacturer, and servicer based in South Africa. With GRW facing increased competition in 2022 when one of GRW's major suppliers buys out a local competitor, Gerhard Van der Merwe, co-founder of GRW and chief executive officer since its inception in 1996, knows that GRW must now compete directly against a giant multinational and develop an appropriate strategy.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -657,17 +661,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Engineer in South Africa - Business Data &amp; Market Insights</t>
+          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.poidata.io/report/engineer/south-africa</t>
+          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>June 22, 2026 - Perform advanced spatial analysis to identify business clusters, service gaps, and market saturation patterns across 0 states in South Africa using precise coordinate data from 1,582 Engineers. Analyze trends, saturation, and competitor presence across 0 states in South Africa to uncover underserved areas and high-potential markets for Engineers.</t>
+          <t>This Competition is for undergraduate students in the last two years of study (years 4 and 5) or recent 2021 graduates who will be required to design localized solutions addressing African challenges.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -680,17 +684,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Made In Africa Events – A prestigious event that celebrates the best of African innovation, and entrepreneurship and craftmanship. Co-located with the AGOA (African Growth and Opportunity Act) forum and initiative.</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://madeinafricaevent.co.za/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>The primary goal of the Made in Africa Exhibition is to create a platform for key stakeholders to exchange ideas and showcase new and existing products and technologies. This Exhibition serves as a strategic tool to connect buyers and sellers in the Mining, Automotive, Textile, and Agriculture ...</t>
+          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -698,22 +702,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>enquiries@aiexpoafrica.com</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>KZN Industrial Technology Exhibition</t>
+          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://www.kznindustrial.co.za/</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>27–29 July 2027 Durban Exhibition Centre | KwaZulu-Natal, South Africa · Book a Stand (opens in a new tab) Become a Sponsor (opens in a new tab) Loading · 1 · 2 · 3 · 4 · The KZN Industrial Technology Exhibition (KITE) is KwaZulu-Natal’s leading platform for industrial innovation ...</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -723,24 +731,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>john@email.com</t>
+          <t>dataprivacy@knect365.com, support@knect365.com, dataprivacy@informaconnect.com, salesenquiries@africatechfestival.com, support@informaconnect.com, customerservices@knect365.com, customerservices@informaconnect.com</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>South Africa International Industrial Expo | Innovation Bridge</t>
+          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://innovationbridge.info/ibportal/events/south-africa-international-industrial-expo</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>The South Africa International Industrial Expo &amp; China (South Africa) International Trade Expo is an international exhibition covering various industrial categories which are dedicated to enterprises and institutions from South Africa, Southern ...</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026. From CIO strategy to hands-on innovation with 75+ exhibitors, this is where leaders come to see what's next before everyone else does. Only 2,500 ...</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -753,17 +761,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Manufacturing Indaba Exhibition 2026 – Manufacturing Expo</t>
+          <t>Exhibition | Innovation Festival Durban | South Africa</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://manufacturingindaba.co.za/exhibition/</t>
+          <t>https://www.innovationfestival.durban/exhibition</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>June 26, 2026 - Manufacturing Indaba Exhibition 2026: Africa’s leading manufacturing expo will showcase cutting-edge products, technology and innovation from manufacturers and SMEs.</t>
+          <t>Exhibition Opportunities BENEFITS FOR YOUR PARTICIPATING IN THE EXHIBITION: An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities. Opportunity to market your Brand. Exposure on print, electronic and social media platforms.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -771,22 +779,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Erika@innovate.durban, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, sithabile@innovate.durban, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Exhibition | Innovation Festival Durban | South Africa</t>
+          <t>Discover Trade Show Events in south-africa: Best Exhibitions, Expos ...</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://www.innovationfestival.durban/exhibition</t>
+          <t>https://globy.com/events-calendar/listing/country/south-africa</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>An opportunity to showcase your innovation / service to a niche target market with a potential for further commercial opportunities.</t>
+          <t>AfricaCom plays a pivotal role in positioning South Africa and the broader continent as leaders in digital transformation. By combining exhibitions, expert-led conferences, and awards, the event provides a platform for collaboration, innovation, and strategic investment.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -794,26 +806,22 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Erika@innovate.durban, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, sithabile@innovate.durban, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>International Science, Innovation &amp; Technology Expo (INSITE)</t>
+          <t>Exhibitions in South Africa 2026-2027 - ExpoTobi</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://www.dsti.gov.za/index.php/resource-center/27-temp/dst-links/3-international-science-innovation-a-technology-expo</t>
+          <t>https://expotobi.com/country/south-africa/exhibitions</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The essence of INSITE INSITE is an international, biennial must-see Science and Technology event in South Africa, the only one of its kind in Africa that creates new frontiers for global challenges · INSITE aims to assemble the worlds leading innovators and scientists in one place, stimulating ...</t>
+          <t>All Exhibitions in South Africa 2026-2027 | Full and accurate description of events for various business sectors | Schedule, tickets, travel arrangements and participation</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -826,17 +834,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Trade Shows Worldwide - South Africa - 2026/2027</t>
+          <t>Explore IT &amp; Technology Trade Events in south-africa: Exhibitions ...</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://www.eventseye.com/fairs/c1_trade-shows_south-africa.html</t>
+          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>South Africa Trade shows, fairs, exhibitions &amp; conferences - List of Trade Shows in South Africa</t>
+          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -849,17 +857,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AAXO - The Association of African Exhibition Organisers</t>
+          <t>2026 SA Innovation Week | Innovate. Connect. Transform</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.aaxo.co.za/</t>
+          <t>https://innovationweek.co.za/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>February 20, 2026 - CAPE TOWN, South Africa – The inaugural Festival of Eventing (FOE) brought together 350 event professionals, 85 speakers, and 10 countries under one roof for a two-day showcase of innovation, inspiration, and industry connection.</t>
+          <t>SA Innovation Week 2026 is South Africa's official national innovation platform accelerating implementation, commercialisation and impact.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -867,22 +875,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>info@pixal8media.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Trade Shows in South Africa - Expos, Trade Fairs &amp; Exhibitions</t>
+          <t>Exhibitions in South Africa</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/tradeshows</t>
+          <t>https://expoonline.co.za/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>South Africa trade shows, find ... Profile, Exhibitor Information etc. Listing of 166 upcoming expos in 2026-2027 1. Mining Connect Day, 2. Annual ACFE Africa Conference &amp; Exhibition, 3. Annual Smart Procurement World Indaba, ...</t>
+          <t>Online Exhibition South Africa We offer a Virtual Exhibition platform for specialized trade shows and exhibitions South Africa. Browse the exhibition by Expo Categories and connect with our Exhibitors. Discover new products and suppliers for your needs and industry at our online exhibitions South Africa.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -890,22 +902,26 @@
           <t>innovation exhibition South Africa</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>info@expoonline.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Come and explore our exhibition of innovative discoveries at Science Forum South Africa 2024 | CSIR</t>
+          <t>Exhibitions in South Africa 2026, 2027 | Conference Locate (Clocate)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.csir.co.za/come-and-explore-our-exhibition-innovative-discoveries-science-forum-south-africa-2024</t>
+          <t>https://www.clocate.com/exhibitions-in+south-africa/Y28temE=/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>December 3, 2024 - The exhibition launch will take place on Tuesday, 3 December 2024, with the opening address by Department of Science, Technology and Innovation Minister Dr Blade Nzimande.</t>
+          <t>With Conference Locate (Clocate), you can browse events by location. Find information on Exhibitions in South Africa 2026, 2027, including dates, locations, price ranges, and more.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -941,17 +957,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bambasonke Design Challenge - EWBSA</t>
+          <t>Engineering For People Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
+          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community's challenges and how community members view the impact of these challenges on their daily lives.</t>
+          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -959,22 +975,26 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Engineering For People Design Challenge - EWBSA</t>
+          <t>Bambasonke Design Challenge - EWBSA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://ewbsa.org/our-work/engineering-for-people-design-challenge/</t>
+          <t>https://ewbsa.org/our-work-4/bambasonke/</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge is run in partnership by Engineers Without Borders South Africa and Engineers Without Borders UK. Since starting in 2011, the programme has reached over 60,000 students across Cameroon, Ireland, South Africa, the UK and the USA.</t>
+          <t>In South Africa, the unique challenges faced by communities, necessitate innovative and context-specific engineering solutions. Through the Bambasonke Design Challenge, students are exposed to how engineers can understand a community's challenges and how community members view the impact of these challenges on their daily lives.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -982,7 +1002,11 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>info@ewbsa.org, robyn.clark@ewbsa.org</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1010,17 +1034,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge | Department of Engineering</t>
+          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
+          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>This year's design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
+          <t>The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1030,24 +1054,24 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
+          <t>team@crowdsolve.net</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Engineering for People Design Challenge 2023/24 - South Africa</t>
+          <t>Engineering for People Design Challenge | Department of Engineering</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://crowdsolve.net/challenge/EfP-SA-24</t>
+          <t>https://www.eng.cam.ac.uk/news/engineering-people-design-challenge</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>The Engineering for People Design Challenge, run in partnership with Engineers Without Borders South Africa, and UK, is taught through project-based learning and embeds global responsibility during a pivotal moment in students' careers.</t>
+          <t>This year's design context The 2024/25 Engineering for People Design Challenge, delivered in partnership with Makers Valley Partnership and Engineers Without Borders South Africa, invited students to explore Makers Valley, a vibrant but under-resourced neighbourhood on the eastern edge of Johannesburg. Home to around 46,000 people, Makers Valley is a community rich in creativity, activism ...</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1057,7 +1081,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>team@crowdsolve.net</t>
+          <t>web-editor@eng.cam.ac.uk, marketing@eng.cam.ac.uk</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1134,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Engineering for People in Makers Valley | PDF | Apartheid | South Africa</t>
+          <t>Inspiring, building and shaping a future fit engineering community</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.scribd.com/document/784038503/2024-25-Engineering-for-People-Design-Challenge-Makers-Valley</t>
+          <t>https://www.ewb-international.org/home/inspiring-building-and-shaping-a-future-fit-engineering-community/</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Engineering ENGINEERING for FOR people PEOPLE Design DESIGNchallenge CHALLENGE 2024-5 2024-25 Makers MakersValley Valley Johannesburg, Johannesburg,South SouthAfrica Africa fEngineering for People Design Challenge 2024-25 The Engineering for People Design Challenge contributed their time and expertise to enhance the has been delivered in the UK and Ireland since content of this design ...</t>
+          <t>The Engineering for People Design Challenge, a flagship initiative by Engineers Without Borders UK and South Africa, addresses this gap by empowering the next generation of engineers with the skills and insights needed for globally responsible engineering.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1128,7 +1152,11 @@
           <t>engineering design challenge South Africa</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>admin@ewb-international.org</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1156,17 +1184,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Faculty of Engineering Students to Represent South Africa at Global Space Competition | Stellenbosch University</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.su.ac.za/en/faculties/engineering/departments/chemical-engineering/news/faculty-engineering-students-represent-south-africa-global-space-competition</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>April 28, 2026 - Seven postgraduate students from the Faculty of Engineering have been selected to represent South Africa at the · Mission Idea Contest (MIC), a global space engineering competition held in Tokyo, Japan.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1174,22 +1202,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>March 12, 2026 - Ultimately, the Student Cluster Competition aims to elevate national engineering standards while preparing students for the demands of a rapidly evolving digital economy. With their national championship secured, team UCT now turns its focus ...</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1202,17 +1234,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2200</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - South Africa 2026</t>
+          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1220,22 +1252,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, email@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions – SAASTA</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ASTEMI brings together all role ... Olympiads in South Africa. THE UNIVERSITY OF CAPE TOWN MATHEMATICS COMPETITION ... National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology ...</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1248,17 +1284,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Top Engineering Universities in South Africa | US News Best Global Universities</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://www.usnews.com/education/best-global-universities/south-africa/engineering</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>These are the top universities in South Africa for engineering, based on their reputation and research in the field.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1266,22 +1302,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Engineering in South Africa: 24 Best universities Ranked</t>
+          <t>Competitions - SABSA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://edurank.org/engineering/za/</t>
+          <t>https://sabsa.co.za/competitions/</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>March 15, 2026 - You can find information about ... Africa based on the number of universities and their ranks are Cape Town, Johannesburg, Stellenbosch, and Pretoria....</t>
+          <t>African Business Concept Challenge ABCC is a virtual simulation-based business concept competition for African undergraduate and graduate students. The competition will challenge student teams to design a viable business concept that addresses a locally-relevant challenge or problem related to Agenda 2063, and inclusive and sustainable development.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1289,22 +1329,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>anne@sabsa.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>About the Competition - S2PAfrica Engineering Design Competition</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.s2pafrica.org/edc/about-edc.html</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>This Competition is for undergraduate students in the last two years of study (years 4 and 5) or recent 2021 graduates who will be required to design localized solutions addressing African challenges.</t>
+          <t>This programme is part of a series of significant milestones in our shared mission to develop entrepreneurial pathways for South African students, alumni and academics. The Africa Prize for Engineering Innovation, founded by the Royal Academy of Engineering, is Africa's biggest prize dedicated to engineering innovation. The Prize awards commercialisation support to African innovators ...</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1317,17 +1361,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>ASTEMI SA - Competition Directory</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?country=ZAF&amp;area=2200</t>
+          <t>https://www.astemi.co.za/competition-directory</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Research and Innovation Overall Rankings - Engineering - South Africa 2026</t>
+          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1340,17 +1384,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>Competitions - Enactus South Africa | National Expos, Challenges ...</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=Africa&amp;area=2200</t>
+          <t>https://enactusza.org/what-we-do/competitions</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>University Overall Rankings - Engineering - Africa 2025</t>
+          <t>Explore our national and international competitions that empower students to tackle challenges with entrepreneurial solutions and social impact at the core.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1358,22 +1402,26 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>xmadlanga@enactus.org, liso@enactus.org, adminsa@enactus.org, marketingsa@enactus.org</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Competitions – SAASTA</t>
+          <t>Competitions | ESG</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://za.rs-online.com/web/content/m/competition</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Some of our sparkling achievements ... and competitions. The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the · National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation ...</t>
+          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1381,12 +1429,16 @@
           <t>university engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>example@email.com</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TECHSPO Joburg 2026 · Technology Expo · October 10 - 11, 2024 (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>TECHSPO Joburg 2027 · Technology Expo · September 29 - 30, 2027 ...</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1396,7 +1448,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>July 30, 2026 - TECHSPO Johannesburg 2026 is a two day technology expo taking place September 28th to 29th, 2026 at the luxurious Hyatt Regency Johannesburg, Johannesburg, South Africa. TECHSPO Johannesburg brings together developers, brands, marketers, technology ...</t>
+          <t>The annual TECHSPO Johannesburg 2027 Technology Expo returns September 29th to 30th, 2027 to the NH Johannesburg Sandton Hotel in Johannesburg. TECHSPO Johannesburg Technology Expo is the must-attend event to: Experience the Future of Technology &amp; Innovation Discover cutting-edge tech, game-changing tools, and innovators shaping tomorrow's digital world. See the latest advancements in ...</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1413,17 +1465,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>IT &amp; Technology Events in South Africa, List of all South Africa Technology Business Expo &amp; Events</t>
+          <t>Africa Tech Festival</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://10times.com/southafrica/technology</t>
+          <t>https://africatechfestival.com/</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>South Africa · 158 EventsFollowShare · TrendingDate · Loading... Regional Advisory: Check official updates before travel. Premium · Loading... You may also like · NODES AI · 15 Apr · Online · NODES AI15 AprOnline · Intersec Shanghai · 07-09 May · Shanghai , China · Intersec Shanghai07-09 MayShanghai , China · GCCI Annual Trade Expo ·</t>
+          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa's tech future.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1431,22 +1483,26 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>dataprivacy@knect365.com, support@knect365.com, dataprivacy@informaconnect.com, salesenquiries@africatechfestival.com, support@informaconnect.com, customerservices@knect365.com, customerservices@informaconnect.com</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ AdTech ~ MarTech) Tickets, Monday, September 28-Tuesday, September 29 • 9 AM-4 PM | Eventbrite</t>
+          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 - 7, 2027 ...</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/techspo-johannesburg-2026-technology-expo-internet-adtech-martech-tickets-1653486545769</t>
+          <t>https://techspocapetown.co.za/</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS) - September 28 - 29, 2026 - Johannesburg, South Africa</t>
+          <t>The annual TECHSPO Cape Town 2027 Technology Expo returns October 6th to 7th, 2027 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town. TECHSPO Cape Town Technology Expo is the must-attend event to: Experience the Future of Technology &amp; Innovation Discover cutting-edge tech, game-changing tools, and innovators shaping tomorrow's digital world. See the latest advancements in ...</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1456,24 +1512,24 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>atinfo@techspo.coor, u003einfo@techspo.co</t>
+          <t>info@techspocapetown.co.za</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Africa Technology Expo | Annual Tech Event | June 25th &amp; 26th, 2027, 2027</t>
+          <t>AI Expo Africa | Africa's Largest Enterprise AI Trade Show &amp; Conference ...</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://africatechnologyexpo.com/</t>
+          <t>https://aiexpoafrica.com/</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Africa Tech Expo (ATE) provides Trade Offices, Embassies, and Economic Missions with a strategic platform to present their national innovation agendas, enterprise capabilities, and cross-border investment priorities to Africa’s most influential ...</t>
+          <t>AI Expo Africa, now entering its 9th successful year, is the largest business focused Artificial Intelligence (AI), Autonomous Enterprise and smart tech trade event in Africa, uniting 1000s of Enterprise buyers, suppliers &amp; innovators across the region.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1483,24 +1539,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>johndoe@email.com, info@sparkafrica.co, partner@africatechnologyexpo.com</t>
+          <t>enquiries@aiexpoafrica.com</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TECHSPO Cape Town 2027 · Technology Expo · October 6 – 7, 2027(Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>IT &amp; Technology Events in South Africa - globy.com</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://techspocapetown.co.za/</t>
+          <t>https://globy.com/events-calendar/listing/country/south-africa/industry/it--technology</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>September 22, 2014 - The Westin Cape Town Hotel, Cape Town, Africa ... The annual TECHSPO Cape Town 2027 Technology Expo returns October 6th to 7th, 2027 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town.</t>
+          <t>Discover a wide range of IT &amp; Technology events in south-africa. Find and compare different trade shows, conferences, expos, and exhibitions. Learn more about an event, access venue and schedule information, photo and video overviews, and learn about other attendees and exhibitors.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1513,17 +1569,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Africa Tech Festival: Welcome | Africa Tech Festival</t>
+          <t>TECHSPO Johannesburg Technology ExpoJohannesburg Technology Expo ...</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://africatechfestival.com/</t>
+          <t>https://techspojoburg.co.za/johannesburg-technology-expo/</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Join Africa Tech Festival in Cape Town to explore telecoms, AI, cybersecurity, startups and digital transformation with leaders shaping Africa’s tech future.</t>
+          <t>TECHSPO Johannesburg is a 2-day technology expo taking place September 28 - 29, 2026 at the luxurious NH Johannesburg Sandton Hotel, Toronto, Ontario. TECHSPO Johannesburg brings together developers, brands, marketers, technology providers, designers, innovators and evangelists looking to set the pace in our advanced world of technology.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1531,26 +1587,22 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>support@knect365.com, dataprivacy@informaconnect.com, dataprivacy@knect365.com, salesenquiries@africatechfestival.com, customerservices@informaconnect.com, support@informaconnect.com, customerservices@knect365.com</t>
-        </is>
-      </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Home - Mediatech Africa | South Africa</t>
+          <t>TECHSPO Johannesburg Technology Expo Sandton 2026 - TradeFairDates</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://www.mediatech.co.za/</t>
+          <t>https://www.tradefairdates.com/TECHSPO-Johannesburg-Technology-Expo-M13397/Sandton.html</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mediatech africa 2028 Expo 27 June – 29 June 2028 Africa’s largest technology showcase for AV Integration, Unified Communications, Broadcast &amp; Streaming, film, studio &amp; production, Pro Audio, Lighting, Staging, &amp; Display Solutions. Days Hours Minutes Seconds Kyalami Grand Prix Circuit&amp; ...</t>
+          <t>In conclusion, the TECHSPO Johannesburg Technology Expo is more than just an expo - it's an event that celebrates the tech future, bringing together the industry's top talents in one of South Africa's most dynamic cities. A must-attend for every tech enthusiast. The TECHSPO Johannesburg Technology Expo will take place on 2 days from Monday, 28.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1563,17 +1615,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>HOME | Africa Tech Week</t>
+          <t>IT Indaba 2026 - Africa's biggest IT Conference and Expo</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://africatechweek.co.za/</t>
+          <t>https://it-indaba.co.za/</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>May 11, 2026 - From sensational speakers, to top tech exhibitons, see what’s in store when you attend the 2-day Sentech Africa Tech Week Conference in 2025&gt;&gt; ... Sponsor, Speak, Attend! For more information on how you can be a part of the #ATW family, contact ...</t>
+          <t>The IT Indaba is the go-to gathering for forward-thinking tech and business leaders. Be one of the 3,000+ IT professionals in the room where you will pressure-test ideas, decode disruption, and explore the technologies redefining business in 2026.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1586,17 +1638,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Discover Tech Conferences Events &amp; Activities in South Africa | Eventbrite</t>
+          <t>TECHSPO Cape Town 2026 Technology Expo (Internet ~ Mobile ~ AdTech ...</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/d/south-africa/tech-conferences/</t>
+          <t>https://allevents.in/cape-town/techspo-cape-town-2026-technology-expo-internet-~-mobile-~-adtech-~-martech-~-saas/200030358413547</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Share this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South AfricaSave this event: Apex Tech &amp; Marketing Days | Apex Master Expos in Cape Town, South Africa</t>
+          <t>TECHSPO Cape Town Technology Expo returns October 1-2, 2026 to the V&amp;A Waterfront Cape Town Avenue Conference Venue in Cape Town, South Africa. This must-attend, two-day annual event brings together leading developers, marketers, innovators, and technology enthusiasts eager to showcase and explore the latest in tech and digital solutions.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1609,17 +1661,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg 2026 Technology Expo (Internet ~ Mobile ~ AdTech ~ MarTech ~ SaaS)</t>
+          <t>TECHSPO Cape Town Technology Expo Cape Town 2026 - TradeFairDates</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://www.industryevents.com/events/techspo-johannesburg-2026-technology-expo-internet-mobile-adtech-martech-saas</t>
+          <t>https://www.tradefairdates.com/TECHSPO-Cape-Town-Technology-Expo-M7893/Cape-Town.html</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>TECHSPO Johannesburg – Where Business, Tech and Innovation Collide in Johannesburg, South Africa. TECHSPO Johannesburg Technology Expo returns September 28-29, 2026 to the NH Johannesburg Sandton Hotel in Johannesburg, South Africa.</t>
+          <t>In conclusion, the TECHSPO Cape Town Technology Expo is not just an exhibition - it's an experience that celebrates the future of technology and brings together the industry's best in one of Africa's most vibrant cities. A must-attend event for all tech aficionados. The TECHSPO Cape Town Technology Expo will take place on 2 days from Thursday ...</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1627,11 +1679,7 @@
           <t>tech expo South Africa</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>your@email.com, events@techspojoburg.co.za, you@company.com, colleague@company.com, support@industryevents.com</t>
-        </is>
-      </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1702,7 +1750,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>pr@make.co</t>
+          <t>pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1777,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, pr@make.co, fancybox_sprite@2x.png</t>
+          <t>pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif</t>
         </is>
       </c>
     </row>
@@ -1779,24 +1827,24 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>fancybox_loading@2x.gif, chosen-sprite@2x.png, pr@make.co, fancybox_sprite@2x.png</t>
+          <t>pr@make.co, fancybox_sprite@2x.png, chosen-sprite@2x.png, fancybox_loading@2x.gif</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
+          <t>Maker Faire Africa - Facebook</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
+          <t>https://www.facebook.com/MFAJoburg/</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
+          <t>Maker Faire Africa. 520 likes. Where Africa's future is in the making.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1809,17 +1857,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Maker Faire groups | Meetup</t>
+          <t>Book tickets for THE CAPE TOWN MAKER FAIRE</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/topics/maker-faire/za/</t>
+          <t>https://www.quicket.co.za/events/11399-the-cape-town-maker-faire/</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>What maker faire events are happening this week? Discover all the maker faire events taking place this week here. Plan ahead and join exciting meetups throughout the week. Are there maker faire events near me? Absolutely! Find maker faire events near your location here. Connect with your local community and discover events within your area.</t>
+          <t>DIRECTIONS THE CAPE TOWN MAKER FAIRE The Lookout, V&amp;A Waterfront Granger Bay Boulevard, V &amp; A Waterfront, Cape Town, 8002, South Africa Get Directions Fri Aug 21, 13:00 - Sun Aug 23, 17:00 The Lookout, V&amp;A Waterfront View Map Payments are secure and encrypted</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1832,17 +1880,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Maker Faire Africa - Facebook</t>
+          <t>MakeAfrica - Le festival africain de l'innovation technologique et de ...</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/MFAJoburg/</t>
+          <t>https://makeafrica.tech/</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Maker Faire Africa. 520 likes. Where Africa's future is in the making.</t>
+          <t>Le festival africain de l'innovation technologique et de la culture maker Un événement africain pensé par des africains et qui vise à partager, créer, fabriquer et apprendre les uns des autres. Il regroupe stands de démonstration, ateliers de découverte, présentations et conférences autour des sujets liés à l'innovation, la créativité, la fabrication, le numérique, les ...</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1850,22 +1898,26 @@
           <t>maker faire South Africa</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>contact@makeafrica.tech</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MakeAfrica - Le festival africain de l'innovation technologique et de ...</t>
+          <t>Maker Faire groups | Meetup</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://makeafrica.tech/</t>
+          <t>https://www.meetup.com/topics/maker-faire/za/</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Le festival africain de l'innovation technologique et de la culture maker Un événement africain pensé par des africains et qui vise à partager, créer, fabriquer et apprendre les uns des autres. Il regroupe stands de démonstration, ateliers de découverte, présentations et conférences autour des sujets liés à l'innovation, la créativité, la fabrication, le numérique, les ...</t>
+          <t>Find Meetup events so you can do more of what matters to you. Or create your own group and meet people near you who share your interests.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1901,17 +1953,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Competitions - SAASTA</t>
+          <t>High School STEM Competition | Capetown 2026</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/competitions/</t>
+          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
+          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1919,22 +1971,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Astemi Sa</t>
+          <t>Solve For Tomorrow - Design The Future | Samsung South Africa</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/</t>
+          <t>https://www.samsung.com/za/solvefortomorrow/</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
+          <t>About Solve for Tomorrow South Africa Solve for Tomorrow South Africa is an innovation and education initiative that empowers young people to become problem-solvers, innovators, and future leaders. The programme challenges learners and students to identify real issues in their communities and develop practical, technology-driven solutions that create meaningful social impact. Rooted in the ...</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1947,17 +2003,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>High School STEM Competition | Capetown 2026</t>
+          <t>Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/high-school-stem-competition/</t>
+          <t>https://www.saasta.ac.za/competitions/</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>The projects should be related on STEM or similar fields. Individual or team projects can be submitted. One or more teachers may appear as co-authors of a submission, but the student must be the 'first author'. The project must be presented at the IEOM Cape Town, South Africa 2026. IEOM Competition Rubrics Overall content: 1-5 points</t>
+          <t>The South Africa Agency for Science and Technology Advancement (SAASTA) is a business unit of the National Research Foundation (NRF) with the mandate to advance public awareness, appreciation and engagement of science, engineering, innovation and technology in South Africa.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -1970,17 +2026,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The IEOM High School/Middle School STEM Competition recognizes the outstanding students for their accomplishment in Science, Technology, Engineering, and Math (STEM) for their innovative and creative projects.</t>
+          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -1993,17 +2049,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>STEM Scholars — 2026 STEM &amp; Entrepreneurship Discovery Initiative</t>
+          <t>Astemi Sa</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://stemscholars.co.za/</t>
+          <t>https://www.astemi.co.za/</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Building South Africa's Next Generation of Innovators The STEM &amp; Entrepreneurship Discovery Initiative connects learners with a world that's often invisible from inside a classroom — and equips them with skills that last far beyond the competition.</t>
+          <t>The Association for Science, Technology, Engineering, Mathematics &amp; Innovation of Southern Africa was formed in 2016. We are a collection of STEMI based organizations that have formed a community of practice to promote STEMI as far and wide as possible.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2011,26 +2067,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>marushka@stemscholars.co.za, inforeg@justice.gov.za, you@school.co.za</t>
-        </is>
-      </c>
+      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>PDF Department of Basic Education and Samsung South Africa Partner to ...</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://www.education.gov.za/Portals/0/Media/Preess+Releases/2026+Media+Releases/Applications+for+2026+Samsung+Solve+For+Tomorrow.pdf</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>The 2026 competition is guided by the theme: "Innovate for Tomorrow: STEM Solutions for Sustainable Communities." Samsung Solve for Tomorrow is a global innovation competition that empowers Grade 10 and 11 learners in public schools to design science, technology, engineering and mathematics (STEM) solutions that address real-world challenges within their communities.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2043,17 +2095,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>School Challenges - STEMLab - Coding &amp; Robotics Academy</t>
+          <t>Applications for 2026 Samsung Solve For Tomorrow Now Open!</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://stemlab.co.za/school-challenges/</t>
+          <t>https://news.samsung.com/za/applications-for-2026-samsung-solve-for-tomorrow-now-open</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>W elcome to the STEMLab Schools Challenge 2026, the most exciting robotics and coding competition for schools in South Africa! Starting in the Western Cape, this unique event offers learners the opportunity to showcase their skills in a fast-paced, thrilling battle of Engineering and Technology.</t>
+          <t>First, at the heart of South Africa's education policy is the goal of strengthening science, technology, engineering and mathematics education because these subjects are essential for the current jobs market. The SFT competition does exactly that: it gives learners practical, hands-on STEM experience.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2061,26 +2113,22 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>eltonearn9@gmail.com, noreply@stemlab.co.za, info@stemlab.co.za, elton@stemlabco.za</t>
-        </is>
-      </c>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Samsung Solve for Tomorrow 2026: STEM contest opens</t>
+          <t>Register your school for Samsung Solve for Tomorrow 2026</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://tech.africa/samsung-solve-tomorrow-2026/</t>
+          <t>https://www.sowetan.co.za/careers/2026-03-03-register-your-school-for-samsung-solve-for-tomorrow-2026/</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Samsung South Africa opens Solve for Tomorrow 2026, expanding its STEM competition to all public schools including quintile 5 for the first time.</t>
+          <t>Register your school for Samsung Solve for Tomorrow 2026 STEM competition aims to transform and empower South African learners with critical skills to solve real-world challenges March 03, 2026 at 7:44 am</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2088,22 +2136,26 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ssasft@samsung.com</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Imbewu Foundation</t>
+          <t>National Department of Basic Education</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://imbewu.foundation/</t>
+          <t>https://www.education.gov.za/LinkClick.aspx?fileticket=i9GS5Atf7zo=&amp;tabid=347&amp;portalid=0&amp;mid=14629</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Seeding Future Scientists IMBEWU Science Foundation is a youth-focused STEMI organisation based in George, Western Cape, serving learners, educators and communities across the Eden District and Central Karoo District. We exist to nurture talent, ignite curiosity and create meaningful pathways for young South Africans to reach their full potential in science, technology, engineering ...</t>
+          <t>JOHANNESBURG, South Africa - XX Month 2026 - The applications for the 2026 Samsung Solve for Tomorrow (SFT) competition are now open. This unique, global competition is inviting Grade 10 and 11 learners from public schools in South Africa to submit innovative STEM-based (Science, Technology, Engineering and Mathematics) solutions that can help tackle community challenges - with entries ...</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2111,7 +2163,11 @@
           <t>stem competition South Africa</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>j.mogoeng@samsung.com, s.ngcobo@cheil.com, ssasft@samsung.com</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2136,7 +2192,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
+          <t>8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 8c30b2581acc426badc414e8a5dc04ef@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2190,7 +2246,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, info@thecortexhub.africa, 8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com</t>
+          <t>8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, info@thecortexhub.africa, 79baaa8e09c746d2b7401643b99792e0@sentry.wixpress.com, c183baa23371454f99f417f6616b724d@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 78f7996315bc402f9dcb8a2f974b82d1@sentry.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, dd0a55ccb8124b9c9d938e3acf41f8aa@sentry.wixpress.com</t>
         </is>
       </c>
     </row>
@@ -2224,17 +2280,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026 - SpringBots South Africa</t>
+          <t>South Africa to host first World Robot Olympiad International Final in ...</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://springbots.co.za/2026-2/</t>
+          <t>https://wro-association.org/south-africa-to-host-first-world-robot-olympiad-international-final-in-africa-in-2028/</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>This approach ensures that learners are not only participants in robotics competitions but are also equipped with real-world skills in design thinking, programming, systems engineering, and collaborative problem-solving. A Unified Future for Africa SpringBots' 2026 vision extends beyond competition and education.</t>
+          <t>Johannesburg, South Africa, 12 September 2026 — South Africa will host the World Robot Olympiad (WRO®) International Final in 2028, bringing WRO's flagship global robotics competition to the African continent.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2242,22 +2298,26 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>1-Team-CARED-Philippines-500x383@2x.jpg, Costa-Rica-team-Sprout-release-banner-500x383@2x.jpg, Prithul-3rd-place-Future-Engineers-2022-A-500x383@2x.jpg, Annual-report-article-TZ-500x383@2x.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Roboticon 2026: South Africa Showcases Robotics for Culture, Education ...</t>
+          <t>SpringBots South Africa</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://www.ubuntutimes.co.za/roboticon-2026-south-africa-showcases-robotics-for-culture-education-and-innovation/</t>
+          <t>https://springbots.co.za/</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>The event, partnered with the World Robotics Olympiad, positions South Africa as a leader in educational robotics and entrepreneurial innovation." South Africa's robotics landscape reached a milestone today with the launch of Roboticon 2026, a national competition that merges creativity, technology, and cultural preservation.</t>
+          <t>SpringBots South Africa Igniting The Potential of South Africa's Next Generation By Bridging The Digital Divide Through High Impact Robotics, Immersive STEAM Initiatives and Targeted Short Courses Designed For The Future Of Work and Innovators.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2265,26 +2325,22 @@
           <t>robotics competition South Africa</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>newspaper-rec300@2x.jpg, adverts@ubuntutimes.co.za</t>
-        </is>
-      </c>
+      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SpringBots South Africa</t>
+          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://springbots.co.za/</t>
+          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>SpringBots South Africa Igniting The Potential of South Africa's Next Generation By Bridging The Digital Divide Through High Impact Robotics, Immersive STEAM Initiatives and Targeted Short Courses Designed For The Future Of Work and Innovators.</t>
+          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop their creativity and problem-solving skills through challenging and educational robotics competitions.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2297,17 +2353,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Robotics Competitions - HANDS ON TECH | LEGO Education Reseller</t>
+          <t>PARC 2026 - Pan-African Robotics Competition | Dakar Youth Olympic Games</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://www.handsontech.co.za/robotics-competitions.html</t>
+          <t>https://www.parcrobotics.org/</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>A truly global competition dedicated to science, technology and education World Robot Olympiad™ (WRO) is an event incorporating science, technology, education and robotics which brings together young people from all over the world to develop their creativity and problem-solving skills through challenging and educational robotics competitions.</t>
+          <t>Africa's largest robotics competition. Official side event of the Dakar 2026 Youth Olympic Games. Six leagues, November 3-7 in Dakar, Senegal.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2366,17 +2422,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Civil Engineering Tenders - Tender Bulletins</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://tenderbulletins.co.za/tender-category/civil-engineering/</t>
+          <t>https://www.engineeringnews.co.za/article/saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini-2022-09-13</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Browse current and past Civil Engineering tenders published by South African government departments, municipalities, state-owned entities and private companies looking to procure civil engineering. Tenders in this category ask suppliers to quote on civil engineering - anything from once-off supply contracts to multi-year service agreements, depending on the issuing organisation's needs ...</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng. Twelve schools participated in the grand finale, which saw great, ...</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2384,22 +2440,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>advertising@creamermedia.co.za, subscriptions@creamermedia.co.za, newsdesk@engineeringnews.co.za, newsletters@creamermedia.co.za, chanel@engineeringnews.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SAICE's 34th International Bridge Competition Inspires Tomorrow's ...</t>
+          <t>Engineering the Future: 16 schools compete in SAICE’s 33rd International Bridge Building Competition - SAICE</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://southafricatoday.net/lifestyle/education/saices-34th-international-bridge-competition-inspires-tomorrows-engineers/</t>
+          <t>https://saice.org.za/press-releases/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted its 34th International Bridge Building Competition at the Midrand Conference Centre, bringing together 21 teams of high school learners from across South Africa, alongside international participants from Eswatini, Uganda, and Zimbabwe.</t>
+          <t>April 17, 2025 - The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2407,22 +2467,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>civilinfo@saice.org.za, communications@saice.org.za, membership@saice.org.za, marketing@saice.org.za, accounts@saice.org.za</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Civil engineering Tenders | Business Opportunities in South Africa</t>
+          <t>SAICE Bridge Building Competition showcases the bright minds of civil engineering in South Africa, Eswatini</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://www.tenders-sa.org/sa-tenders/categories/civil-engineering</t>
+          <t>https://www.crown.co.za/construction-world/marketplace/22289-saice-bridge-building-competition-showcases-the-bright-minds-of-civil-engineering-in-south-africa-eswatini</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Find the latest Civil engineering tenders and government contracts in South Africa. Browse active bids, view requirements, closing dates, and procurement details for Civil engineering opportunities.</t>
+          <t>The South African Institution of Civil Engineering (SAICE) recently held its yearly SAICE International Bridge Building competition at the Midrand Conference Centre in Gauteng.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2430,22 +2494,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>constr@crown.co.za, ernao@crown.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Engineering the future: 16 schools compete in SAICE's 33rd ...</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025-2026</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://www.southafricanbusiness.co.za/08/2024/construction-and-engineering/engineering-the-future-16-schools-compete-in-saices-33rd-international-bridge-building-competition/</t>
+          <t>https://conferencealerts.co.in/south-africa/civil-engineering</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) hosted its 33rd International Bridge Building Competition at the Midrand Conference Centre, showcasing 16 schools from around South Africa, with one from Swaziland.</t>
+          <t>International Civil engineering conferences in South africa 2025-2026 with invitation letter. A great opportunity to meet and learn from experts in your field.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2458,17 +2526,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Civil Engineering Tenders | eTender SA</t>
+          <t>Upcoming Civil Engineering Conferences in South Africa 2025</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://etendersa.co.za/tenders-south-africa/civil-engineering/</t>
+          <t>https://www.allconferencealert.com/south-africa/civil-engineering-conference.html</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Civil Engineering Tenders in SA, Mining tenders, Road construction tenders in South Africa, and Bridge construction tenders in South Africa.</t>
+          <t>September 7, 2025 - Find all upcoming Civil Engineering conferences in South Africa 2025 with invitation letter. South Africa is a diverse and dynamic country that offers a wide range of opportunities for Civil Engineering conferences in topic Civil Engineering, and many more.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2481,17 +2549,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Inspiring the Next Generation of Engineers at the 2026 SAICE ...</t>
+          <t>ICE Africa – Supporting Civil Engineers in Africa | Institution of Civil Engineers (ICE)</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://nsbe.org.za/inspiring-the-next-generation-of-engineers-at-the-2026-saice-johannesburg-bridge-building-competition/</t>
+          <t>https://www.ice.org.uk/about-us/ice-near-you/africa</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>19 June 2026 marked an exciting celebration of Youth Month as aspiring young engineers from across Gauteng gathered for the 2026 SAICE Johannesburg Branch Schools Bridge Building Competition. Hosted by the South African Institution of Civil Engineering (SAICE) Johannesburg Branch, the event brought together learners, educators, universities, engineering professionals, and industry partners in ...</t>
+          <t>March 19, 2026 - organise seminars, workshops, visits and inter-universities competitions regarding civil engineering projects · For more information or to get involved please contact [email protected]. We have a volunteer member in South Africa who helps arrange ICE activities and promote our work.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2504,17 +2572,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Home - SAICE</t>
+          <t>Upcoming Civil engineering Conferences in Cape town 2025</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://saice.org.za/</t>
+          <t>https://conferencealerts.co.in/cape-town/civil-engineering</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>The South African Institution of Civil Engineering (SAICE) is the industry body for civil engineering professionals in South Africa. Our aim is to, promote growth, excellence and sustainability in the industry.</t>
+          <t>4th International Conference on Advances in Science, Engineering &amp; Technology(ICASET-2025) [Accredited CPD Event]</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2522,26 +2590,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>barbara@avenue.co.za, executiveadmin@saice.org.za, membership@saice.org.za, communications@saice.org.za, accounts@saice.org.za, civilinfo@saice.org.za, marketing@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>SAICE | Events and Awards</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://members.saice.org.za/events-and-awards</t>
+          <t>https://www.scimagoir.com/rankings.php?sector=Higher+educ.&amp;country=ZAF&amp;area=2205</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>The South African Institution Of Civil Engineering SAICE hosts the Awards Function annually to honour individuals, projects of excellence, as well as community-oriented initiatives. The annual awards function gives companies and individuals a unique opportunity to showcase their deserving projects and work to the industry.</t>
+          <t>University Overall Rankings - Civil and Structural Engineering - South Africa 2025</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2554,17 +2618,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Greenovate</t>
+          <t>Civil Engineering Competition - Christian Brothers University</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://greenovatecompetition.co.za/</t>
+          <t>https://www.cbu.edu/civil-engineering-competition/</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Growthpoint Properties and the Green Building Council South Africa invites you to Register for the 2026 Greenovate Awards, inspiring a new wave of industry talent to innovate for sustainability.</t>
+          <t>August 14, 2023 - Gather a team (2-5 members) to compete in CBU’s Civil Engineering Competition September 18, 2023, when up to six teams in each category will test their skills for the judges, CBU’s renowned engineering professors.</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2572,22 +2636,26 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>info@cbu.edu, jkaufma1@cbu.edu</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Awards 2026 - SAICE</t>
+          <t>Civil Engineering Conferences in South Africa 2025/2026/2027 - Conference Index</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://saice.org.za/awards-2026/</t>
+          <t>https://conferenceindex.org/conferences/civil-engineering/south-africa</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Learn about SAICE's award categories, submission guidelines, key dates and how to nominate project and professionals.</t>
+          <t>Nov 03 International Conference on Civil and Environmental Engineering (ICCEE) - Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2595,26 +2663,22 @@
           <t>civil engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>membership@saice.org.za, communications@saice.org.za, accounts@saice.org.za, civilinfo@saice.org.za, marketing@saice.org.za</t>
-        </is>
-      </c>
+      <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Competitions | Capetown 2026</t>
+          <t>How to compete at the WSZA National Competitions 2025</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/capetown2026/competitions/</t>
+          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
+          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2627,17 +2691,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>ASTEMI Competitions - SAASTA</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.saasta.ac.za/astemi-competitions/</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2650,17 +2714,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>Competitions | Capetown 2026</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://ieomsociety.org/capetown2026/competitions/</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the IEOM Cape Town, South ...</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2668,22 +2732,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>PDF Call to enter the Africa Prize for Engineering Innovation Competition ...</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://edhe.co.za/wp-content/uploads/Africa-Prize-Call-for-Applications.pdf</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>We encourage all eligible South African students, academics, and innovators to take full advantage of this incredible opportunity to showcase and scale their engineering solutions. Whether you're working in traditional engineering fields or applying innovation in areas like health, agriculture, or digital technology, the Africa Prize for Engineering Innovation offers a unique platform to ...</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2696,17 +2764,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Opportunities in Mechanical Engineering across South Africa.</t>
+          <t>Competitions | Southafrica 2024 - IEOM Society</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://www.puffandpass.co.za/tag/mechanical-engineering</t>
+          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Location: Johannesburg Hatch is seeking Electrical / Civil / Mechanical Engineering Graduates who will support projects globally. The engineering team is comprised of professional engineers, designers and technologists. We have experience…</t>
+          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2714,22 +2782,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>info@ieomsociety.org</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Competitions South Africa - Live Giveaways &amp; Prize Draws | Freehub</t>
+          <t>Engineering Competition for African Youth in Engineering Innovation ...</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://freehub.co.za/competitions/</t>
+          <t>https://daadscholarship.com/engineering-competition-for-african-youth-in-engineering-innovation-2026-open/</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Browse live South African competitions, giveaways and prize draws. Find car, cash, voucher, tech and holiday competitions with clear entry rules and official source links.</t>
+          <t>The Royal Academy of Engineering has officially launched the 2026 Africa Prize for Engineering Innovation, the continent's largest award dedicated to fostering engineering ingenuity and entrepreneurship.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2742,17 +2814,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Competitions - Prized Competitions South Africa</t>
+          <t>The 2026 Africa Prize for Engineering Innovation wants applications ...</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://www.prized.co.za/competitions/</t>
+          <t>https://sawea.org.za/news/2026-africa-prize-engineering-innovation-wants-applications-engineers-and-innovators-south</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Prized is home to Online Competitions in South Africa. Enter any competition that peaks your interest and join the Prized community.</t>
+          <t>3 September 2025: The Royal Academy of Engineering has launched its 2026 Africa Prize for Engineering Innovation with a special call out to engineers and innovators in South Africa.</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2760,22 +2832,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>glueup-logo-white@2x.png, admin@sawea.co.za</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
+          <t>National Student Competition | ORSSA</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
+          <t>https://www.orssa.org.za/studentcomp</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
+          <t>National Student Competitions The Operations Research Society of South Africa The home of decision intelligence The Society organises student competitions in two independent categories on an annual basis, namely a competition at the honours or fourth-year level of study and a competition at the master's level of study.</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2783,22 +2859,26 @@
           <t>mechanical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>8eb368c655b84e029ed79ad7a5c1718e@sentry.wixpress.com, 18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 460ff4620fa44cba8df530afde949785@sentry.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 88170cb0c9d64f94b5821ca7fd2d55a4@sentry-next.wixpress.com, 605a7baede844d278b89dc95ae0a9123@sentry-next.wixpress.com, 8c4075d5481d476e945486754f783364@sentry.io, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com, 9a65e97ebe8141fca0c4fd686f70996b@sentry.wixpress.com, 271e9fa3230b4eec94b02bf95780f5f2@sentry.wixpress.com, f36cc48fb72b4d298c835f2793cf3b84@sentry-next.wixpress.com, ed436f5053144538958ad06a5005e99a@sentry.wixpress.com, email@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SAIMechE</t>
+          <t>PDF Apply Now! Worldskills South Africa National Competition 2025</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://www.saimeche.org.za/</t>
+          <t>https://ewseta.org.za/wp-content/uploads/2021/02/WorldSkills-South-Africa-National-Competition-Registration.pdf</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
+          <t>- A student undertaking studies towards a qualification related to the skill at a University, TVET College, Private Skills Development Provider, CET College, or a Technical High School</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2811,17 +2891,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Greenovate</t>
+          <t>SAIMechE</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://greenovatecompetition.co.za/</t>
+          <t>https://www.saimeche.org.za/</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Growthpoint Properties and the Green Building Council South Africa invites you to Register for the 2026 Greenovate Awards, inspiring a new wave of industry talent to innovate for sustainability.</t>
+          <t>The pre-eminent body for the Mechanical Engineering profession! SAIMechE exists to serve the interests and needs of its members, to advance the science and practise of mechanical engineering, and to promote high standards in the profession.</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2834,17 +2914,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ASTEMI Competitions - SAASTA</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - National Student Project Competition</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://www.saasta.ac.za/astemi-competitions/</t>
+          <t>https://www.saiee.org.za/EventOrganisers/EventDetailsCorp.aspx?eeid=16485</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Organisation of international Olympiads in South Africa. ASTEMI brings together all role players in the field of Olympiads and Competitions - including professional and academic societies, universities and other tertiary institutions, private enterprise and government - to promote, coordinate and extend STEMI Olympiads in South Africa.</t>
+          <t>Every year, final year students ... nominated by these educational institutes competes against ±15or other presentations in the SAIEE National Student Project Competition, and prizes are awarded to the adjudicated winners....</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2857,17 +2937,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026 South Africa Engineering Competition</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - SAIEE National Student Project Competition</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://notices.ukzn.ac.za/content/GetFile.aspx?id=96047</t>
+          <t>https://www.saiee.org.za/calendar/EventDetails.aspx?eeid=29281</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026 South Africa Engineering Competition Organized by UKZN and Elsevier. If you are an engineering student (undergraduate or postgraduate), don't miss joining the challenge to solve real-world cases using Engineering Village and Knovel.</t>
+          <t>The SAIEE National Students Project Competition will be held at the North-West University (Potchefstroom Campus) on 21 November 2019</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2880,17 +2960,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ASTEMI SA - Competition Directory</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - IEEE ZA 5G Competition</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://www.astemi.co.za/competition-directory</t>
+          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51397</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>We have a wide range of Olympiads, Competitions ,Expos and activities that cater to a variety of age groups and offer these events in different formats at at different costs.</t>
+          <t>The IEEE South Africa Section, South African Institute of Electrical Engineers (SAIEE), the National Science and Technology Forum (NSTF), and University of Pretoria (UP) invite undergraduate and graduate students to submit essays on the topic "5G and Beyond for South Africa and Africa".</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2903,17 +2983,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>South African Institute of Electrical Engineers</t>
+          <t>Top 100 Electrical Engineering Companies in South Africa (2026) | ensun</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://www.saiee.org.za/</t>
+          <t>https://ensun.io/search/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Design Thinking and Innovation for Engineering Professional - Online Design Thinking and Innovation for Engineering Professional - Online (opens in a new window) Training Academy Earn your CPD credits today!</t>
+          <t>Their work enhances the efficiency and livability of communities in Southern Africa. ... Devcotech specializes in Electrical Engineering and Industrial Automation, providing EC&amp;I turnkey project solutions that enhance productivity through intelligent automation and SCADA software design.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2926,17 +3006,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025</t>
+          <t>Student Design Competition | IEEE CASS</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://www.worldskillsza.dhet.gov.za/24+Skills/WSZA-Promotions.aspx</t>
+          <t>https://ieee-cas.org/society-involvement/student-design-competition</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>How to compete at the WSZA National Competitions 2025 In order for you to compete at the WorldSkills South Africa National Competitions, you should be a student in an apprenticeship or learnership related to the skill.</t>
+          <t>CASS will reimburse the travel costs for the trip to ISCAS 2026 for the four finalists, one for each region - Regions 1-7 (USA and Canada), Region 8 (Europe, Middle East, Africa), Region 9 (Latin America), and Region 10 (Asia, Australia, Pacific), as well as ISCAS registration.</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -2949,17 +3029,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>IEEE IAS-IPCSD Engineering Student Chapter Design Contest (Africa)</t>
+          <t>SAIEE | The South African Institute Of Electrical Engineers - SA Computing Olympiad stars hold their own in international competition</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://site.ieee.org/ias-ipcsd/scdc-africa/</t>
+          <t>https://www.saiee.org.za/News/DisplayNewsItem.aspx?niid=51457</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>IEEE-IAS Industrial Power Conversion Systems Department Serving the electrical energy conversion professional worldwide</t>
+          <t>July 20, 2021 - South Africa’s team of four was selected from among the top participants in the South African Computing Olympiads, a key project of the Institute of Information Technology Professionals South Africa (IITPSA).</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -2972,17 +3052,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>WorldSkills South Africa 2027 Applications Now Open - Apply Online</t>
+          <t>Engineering students compete in global high-performance computing challenge | UCT News</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://www.edupstairs.org/worldskills-south-africa-2027-applications/</t>
+          <t>https://www.news.uct.ac.za/article/-2026-03-12-engineering-students-compete-in-global-high-performance-computing-challenge</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Applications are officially open for the WorldSkills South Africa 2027 National Competition, giving talented students, apprentices, learners and qualifying skilled candidates across South Africa an opportunity to demonstrate their practical abilities on a national stage.</t>
+          <t>March 12, 2026 - At the Centre for High Performance Computing (CHPC) Conference hosted in Cape Town at the end of last year, four current fourth-year electrical engineering students were crowned national champions in the Student Cluster Competition for 2025.</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -2990,26 +3070,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>sifisomhlongo@edupstairs.org</t>
-        </is>
-      </c>
+      <c r="E108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Competitions | Southafrica 2024 - IEOM Society</t>
+          <t>7 Electrical Engineering Degree Programs in South Africa - Study Abroad | educations.com</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://ieomsociety.org/southafrica2024/competitions/</t>
+          <t>https://www.educations.com/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Master Thesis Competition IEOM Master Thesis Presentation Award recognizes outstanding research in industrial engineering, manufacturing engineering, systems engineering, operations research, engineering management, operations management and related areas. Students must enroll in the masters' program during the current academic year. These awards are presented at the 2024 IEOM South Africa ...</t>
+          <t>As electronics and digital devices proliferate in the population, electrical engineers are needed to maintain and develop them. A country situated to the southern tip of Africa, South Africa has a rich culture that you will never get enough of while touring or studying here.</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3022,17 +3098,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Competitions | ESG</t>
+          <t>Electrical Engineering Conferences in South Africa 2026/2027/2028 - Conference Index</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://za.rs-online.com/web/content/m/competition</t>
+          <t>https://conferenceindex.org/conferences/electrical-engineering/south-africa</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Competitions and Awards Taking part in competitions and applying for awards is a brilliant way to enhance your CV. Participation in such activities will highlight your capabilities and enable you to include relevant achievements on applications for employment. Develop and flex your skills, gain experience and make some great connections!</t>
+          <t>Nov 02 International Conference on Electronics, Control and Signal Processing (ICECSP) - Cape Town, South Africa · Nov 02 International Conference on Electrical, Computer, Electronics and Communication Engineering (ICECECE) - Cape Town, South Africa</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3040,26 +3116,22 @@
           <t>electrical engineering competition South Africa</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>example@email.com</t>
-        </is>
-      </c>
+      <c r="E110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Best competitions to enter in South Africa this month</t>
+          <t>Electrical And Electronics Engineering Conferences in South Africa 2026 | Conference Alerts</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://freehub.co.za/best-competitions-south-africa-this-month/</t>
+          <t>https://conferencealerts.co.in/south-africa/electrical-and-electronics-engineering</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Compare current South African competitions worth checking this month, with prize, cost, entry method and closing-date details from Freehub.</t>
+          <t>Yes most academic and professional electrical and electronics engineering conferences in south africa have a Call for Papers (CFP) 